<commit_message>
Seed V3.2.0 reproducible release artifacts
</commit_message>
<xml_diff>
--- a/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
+++ b/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rfdbafa86db0c4d45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R557e234717c54f15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="Rc2d87bfa84774834"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="R3a2616d157cb4c3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R50018a0d49364b1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R45e4892ae38b4f35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R72f967c8e14945ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="R037d16771cf04e63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R179f8167b7ec45ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R15d3f61a9f564706"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Ra1182a63c5894c67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R448d143ca02b418c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="R4fa6f96291d74d3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Raf050af4020f48df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="Rc1ad0475627043e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R4ae43fe769874c98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Rb31cfb05154f48eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="R72998ff4388441f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R9c4233326ec74bde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="Rd4f648fe156f49b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,88 +19,88 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={AD76C85B-D33E-BD60-615F-7CE5ACBB1507}</x:author>
-    <x:author>tc={A89C0A60-29CB-BCB1-C24E-756EBBD610BD}</x:author>
-    <x:author>tc={749C636E-7A7E-44AE-C575-6C967A103843}</x:author>
-    <x:author>tc={7FE82A63-FFDB-5C1F-7539-D7FF41424EFB}</x:author>
-    <x:author>tc={BB5F2C3B-1762-02AC-3678-B827F2CD81AD}</x:author>
-    <x:author>tc={27080485-9683-E160-FF00-3CC16D512FF2}</x:author>
-    <x:author>tc={DFACCDE4-7ED8-D622-88B3-344385AC3840}</x:author>
-    <x:author>tc={176ABCFB-F4B7-F2A0-6CFF-72FCA064BD19}</x:author>
-    <x:author>tc={EBD22EC7-7EDE-503C-6C11-C70A8AC85292}</x:author>
-    <x:author>tc={A3AB71C1-2A40-68B1-A5CD-30E6E071B7DC}</x:author>
-    <x:author>tc={9278D5CC-0435-3F11-26AA-50760EA88AE2}</x:author>
-    <x:author>tc={C5548CA7-37D6-14DD-75DC-5D6ABA3C43C2}</x:author>
-    <x:author>tc={64547889-9E0A-2B22-DD82-0C778954A87F}</x:author>
-    <x:author>tc={32875CDC-1D01-748F-3FEF-B564BCC4F6CF}</x:author>
-    <x:author>tc={B08242B1-EF53-9913-910B-C22C411341F5}</x:author>
-    <x:author>tc={92B968CD-6246-8C17-8389-D6C45A3CAE69}</x:author>
-    <x:author>tc={AEFDF43C-FBE8-658F-E8C3-082FBEF1FF40}</x:author>
-    <x:author>tc={C477C0D5-6519-22F1-33A2-8CBFC5557854}</x:author>
-    <x:author>tc={2A8F1AF0-22C9-EDA3-08C4-FFFAA399F3C7}</x:author>
-    <x:author>tc={8BF756B5-5E00-0DE9-09F9-77907D4C9B27}</x:author>
-    <x:author>tc={3FD75A8B-4721-240C-1725-93E3EE1EB986}</x:author>
-    <x:author>tc={3F9811A0-E684-E246-E214-8C12573FC814}</x:author>
-    <x:author>tc={4F9A5689-95B3-30CB-7405-FABFDB180CF4}</x:author>
-    <x:author>tc={E4D609D7-5387-D1AF-381B-4001D4950E09}</x:author>
-    <x:author>tc={67656F98-6111-B2AA-2CAB-FA2A95D68C3B}</x:author>
-    <x:author>tc={EAC88F74-D1D2-F311-7967-60FEFDCFB860}</x:author>
-    <x:author>tc={3CFF812D-C7C6-99A0-97E8-633388370E81}</x:author>
-    <x:author>tc={CFC63739-B318-9DB1-19F0-ABD1F0E2BD96}</x:author>
-    <x:author>tc={95EE700C-5315-DC89-F405-B99C0C27E763}</x:author>
-    <x:author>tc={A530B548-98B2-1B6B-D236-DD4C0D304C21}</x:author>
-    <x:author>tc={4A572411-B39B-EF39-03F1-2EFD1E160F62}</x:author>
-    <x:author>tc={45916D39-67A3-C79F-ACE1-95D427374BBA}</x:author>
-    <x:author>tc={BD825591-F743-259C-A52D-AF796642E59E}</x:author>
-    <x:author>tc={B8F05642-8361-695B-E2C3-D72F79D4922A}</x:author>
-    <x:author>tc={E508EB94-396C-1034-1316-58874D6E8BC9}</x:author>
-    <x:author>tc={1793642E-C2C1-DAAC-7003-1FCD16D9A995}</x:author>
-    <x:author>tc={F5E05C9C-40FB-C157-CA88-5B258C461C5C}</x:author>
-    <x:author>tc={86D52D69-2BD9-5726-B3DD-8E6158F10E4C}</x:author>
-    <x:author>tc={75BAA52B-52EB-8817-C639-C9790E51E370}</x:author>
-    <x:author>tc={D514FC67-0E8C-8F25-EDF2-E61B9654E20D}</x:author>
-    <x:author>tc={E1C9BA7F-CA9B-C28D-CDFC-F17719A0EBB2}</x:author>
-    <x:author>tc={057F447F-84A0-FE01-54A6-E5B1957E058E}</x:author>
-    <x:author>tc={8FF56FC9-DE0E-E4F8-D33E-05FC6B5D72A5}</x:author>
-    <x:author>tc={9C8A34A8-8CB0-CB37-B659-2765B7286F51}</x:author>
-    <x:author>tc={A52F21B2-F7F1-89FB-088A-6B573542A95A}</x:author>
-    <x:author>tc={B3D29C51-43CA-18B8-F661-9AC7B04E76C2}</x:author>
-    <x:author>tc={895E733F-9450-F643-A586-C9778BCFEF53}</x:author>
-    <x:author>tc={E6634DA4-21AA-05EC-F06D-B9D5A9029DF0}</x:author>
-    <x:author>tc={41664D94-9B65-23EB-6D48-DE9DB5D48E7E}</x:author>
-    <x:author>tc={D8706B28-69B3-9F03-9DD7-886259DD8C69}</x:author>
-    <x:author>tc={D4F74F82-BBBB-6122-E9FE-F14DAE37B14A}</x:author>
-    <x:author>tc={67A80EB2-6450-F365-0B53-F66EF759A5B2}</x:author>
-    <x:author>tc={63BE2D86-BC91-9099-14D4-20CA68378DC7}</x:author>
-    <x:author>tc={DE361AF7-1C5C-532F-D7E1-1E40636E490B}</x:author>
-    <x:author>tc={0E8348F2-AC6D-4391-024E-2BB4B1396566}</x:author>
-    <x:author>tc={5297095B-D43A-8FE6-6F7E-CD5A9B27EA97}</x:author>
-    <x:author>tc={DA505CEF-AD44-D5D1-9EBC-8FBF8727A618}</x:author>
-    <x:author>tc={D310B17F-864A-65D6-C23B-18D651A1BCA9}</x:author>
-    <x:author>tc={99302A77-FD55-DE9E-B462-BC716BFA9BB5}</x:author>
-    <x:author>tc={E66C77C3-9DB9-77B6-0264-53B6C1B54F2D}</x:author>
-    <x:author>tc={DC9B3809-0C62-C255-8FE9-E64A74085043}</x:author>
-    <x:author>tc={2B3B55AF-EB7A-60A7-0288-A2A428FD6C08}</x:author>
-    <x:author>tc={276AFF59-0B12-12D0-1431-5C76483864FF}</x:author>
-    <x:author>tc={D0D0533F-41FA-AB3B-9E96-F9659D12551B}</x:author>
-    <x:author>tc={CA5C3F8B-3FB1-F256-BF7C-CF6073C0018C}</x:author>
-    <x:author>tc={323181B4-321D-C42A-1A18-A4AEC9952C57}</x:author>
-    <x:author>tc={4CF5C5D2-52D9-A3C3-9A30-81F574BE209A}</x:author>
-    <x:author>tc={3E520E3F-3E8D-0F95-D221-C87981A69FF7}</x:author>
-    <x:author>tc={F7DB273B-83BD-C7BB-95C1-735B3AF1B205}</x:author>
-    <x:author>tc={22866379-A890-E2D9-0B92-FACDCC7AB0BC}</x:author>
-    <x:author>tc={6D8065DD-C4EF-A377-7BFD-3DEDCF918431}</x:author>
-    <x:author>tc={A39373E7-D5D7-F8D4-9E1F-40821AB51A56}</x:author>
-    <x:author>tc={0A44F521-9201-C9A1-7C6D-695551F24ABE}</x:author>
-    <x:author>tc={786A3C30-A168-1FE7-0EF4-AFE4E8F47993}</x:author>
-    <x:author>tc={68A7284C-A659-0183-CDD3-AEE90897FAAE}</x:author>
-    <x:author>tc={E10ADEC7-AB15-EC53-EDE8-D3A26CA60955}</x:author>
-    <x:author>tc={42F3A693-983F-A53F-D994-965ABBF672D0}</x:author>
-    <x:author>tc={40E2782A-C3CC-2E07-7DE1-DB388D05A7A8}</x:author>
-    <x:author>tc={E50522DB-6CC5-0301-2314-72EC58FE6953}</x:author>
-    <x:author>tc={58739544-7137-FB67-590F-28D001FB2D1D}</x:author>
-    <x:author>tc={AD0E6454-9F8B-B5E0-95B7-AFEDC038B461}</x:author>
-    <x:author>tc={1C8AD75C-462E-DBCB-8E4B-37D4695C94F8}</x:author>
+    <x:author>tc={D7179BD9-5380-A2BE-37A2-542620D11FD6}</x:author>
+    <x:author>tc={F5D5EA40-9C27-8916-42CA-9F80A998B239}</x:author>
+    <x:author>tc={F4A30194-1A72-1C1B-D3D1-88F0876A8B1C}</x:author>
+    <x:author>tc={058CC015-9E61-4F60-3707-3AA969865D33}</x:author>
+    <x:author>tc={0EA9266E-93A4-B7F3-00BA-8A7A79DFC82B}</x:author>
+    <x:author>tc={E0C25A1B-6CEF-EF90-AC34-65B59EB516C3}</x:author>
+    <x:author>tc={D3577678-9795-3AEE-F6E6-5B7E42106D9E}</x:author>
+    <x:author>tc={741168DD-C778-7C15-2B65-17B7C07ED33D}</x:author>
+    <x:author>tc={95736628-F1F7-FE17-043B-CA174AE01EDE}</x:author>
+    <x:author>tc={829B1B69-69D1-E6CE-9B21-D90E9F236E79}</x:author>
+    <x:author>tc={E10C328C-B958-A22D-795B-86894E174992}</x:author>
+    <x:author>tc={275B946E-B475-F338-1312-E8A66EEE3FB6}</x:author>
+    <x:author>tc={25671AA7-6F50-28BD-184D-157B185AC6A1}</x:author>
+    <x:author>tc={7A90692C-D081-3F82-41F4-9D743B5AB740}</x:author>
+    <x:author>tc={4027D3F6-5103-811E-9867-0F88B7313B4E}</x:author>
+    <x:author>tc={5452B241-D82F-7E23-08FB-0FF6597AF014}</x:author>
+    <x:author>tc={846887CC-6779-2558-F219-69B7F4C9101A}</x:author>
+    <x:author>tc={4F0D7BAC-731A-10AB-17F0-CF67BEA1E0C5}</x:author>
+    <x:author>tc={71806FB6-0323-8EF2-734E-695EBE8E5C19}</x:author>
+    <x:author>tc={8C6DD087-476A-4C57-960D-E2895732691A}</x:author>
+    <x:author>tc={B47EBC4F-9B31-E559-6ED9-AAC1C334946A}</x:author>
+    <x:author>tc={58727869-8ACA-389D-CD7D-8FBA1F5DE493}</x:author>
+    <x:author>tc={62B5311B-9855-6101-F68A-04824B833B3D}</x:author>
+    <x:author>tc={BBE37CF9-417B-8492-B4BC-F67A0FB38F22}</x:author>
+    <x:author>tc={11CAB389-76D8-7602-E738-77CB6C823411}</x:author>
+    <x:author>tc={53C4CB1B-0E8D-3634-8EB7-DFF2141C14F3}</x:author>
+    <x:author>tc={52C4F871-DAB1-FC43-B689-E83208D5BDC2}</x:author>
+    <x:author>tc={5A8F28C0-DCAF-9B4F-60C2-B5519288078D}</x:author>
+    <x:author>tc={BC440591-751F-ADDA-3E20-D28B53716826}</x:author>
+    <x:author>tc={129D4D19-7FD2-1FAB-C3F2-3D85C2143407}</x:author>
+    <x:author>tc={C00BE146-1A1C-DE84-6CEC-66E28A34FB62}</x:author>
+    <x:author>tc={B2453065-6EF2-25EE-C743-1AF12D44A7E2}</x:author>
+    <x:author>tc={42F5722C-BA58-306D-7716-E7DB46B06E1C}</x:author>
+    <x:author>tc={308E1DA8-4C3B-C720-C61A-B4FD5B863D5A}</x:author>
+    <x:author>tc={575A735C-1490-C525-7FDA-D0D6CC2167F3}</x:author>
+    <x:author>tc={F04ECB4C-E296-D7B7-16F0-976919B7E452}</x:author>
+    <x:author>tc={890C7111-93D9-523E-D457-71A4254BA046}</x:author>
+    <x:author>tc={73A6DDDE-3DDB-F0A0-8427-697A1F7CA9D6}</x:author>
+    <x:author>tc={F8EC0B12-3474-AF0F-5A97-A40007A76C72}</x:author>
+    <x:author>tc={835BEA1E-53F0-17E6-E7D7-DBD14ED53706}</x:author>
+    <x:author>tc={CA531C19-FD45-25C9-0D70-197E1279C769}</x:author>
+    <x:author>tc={8774F1F6-5214-2114-2D61-8456D5360289}</x:author>
+    <x:author>tc={30902EAC-5720-96A7-8284-3D2CCAB7443B}</x:author>
+    <x:author>tc={0CB4A533-3016-5908-0FCF-23076D4239A8}</x:author>
+    <x:author>tc={E740C3D1-D9F7-5D7D-AFF3-68BEEEF5AFB6}</x:author>
+    <x:author>tc={F69FF8B4-C804-AEE4-CB67-276CB58FECC3}</x:author>
+    <x:author>tc={C43B89C3-9376-EAD3-76C9-17647D15CCF5}</x:author>
+    <x:author>tc={E454CB3F-C1C8-45BE-B525-60EFF4CDE1A6}</x:author>
+    <x:author>tc={676951D3-752E-15EF-F207-A9C4AD907FBD}</x:author>
+    <x:author>tc={B43928D3-C753-0831-5261-410F7BBF0732}</x:author>
+    <x:author>tc={7AEC7DF7-C2FC-5FD1-43E7-E31427E0CB4D}</x:author>
+    <x:author>tc={483F7CB9-A550-4C88-F30A-79F3465B8236}</x:author>
+    <x:author>tc={57E4D7D6-EAC9-3255-FC08-228D23302E84}</x:author>
+    <x:author>tc={63285F2A-DBA1-0A5B-0BD2-5CF8872592B7}</x:author>
+    <x:author>tc={5E490997-C386-5F07-4415-3BF718F6583D}</x:author>
+    <x:author>tc={530EEE62-CA06-D2AD-47F5-B427C42F71A7}</x:author>
+    <x:author>tc={D3192F1B-D4AE-761E-78F3-B7200E4D78DD}</x:author>
+    <x:author>tc={5ECB39A3-6CD9-BC08-DE2C-8BC987C1390A}</x:author>
+    <x:author>tc={83C028C4-B49A-845A-F950-45971513DB9D}</x:author>
+    <x:author>tc={14DD0686-1E74-4983-CD5F-91C8010BF879}</x:author>
+    <x:author>tc={42144CB2-40A1-FE82-EC8C-D7B918D43B31}</x:author>
+    <x:author>tc={175AC13F-5A05-534D-C6C5-368C220513B3}</x:author>
+    <x:author>tc={98B1FE03-8508-60EB-FB28-AC6EB4FF17EC}</x:author>
+    <x:author>tc={CA1C4C92-831F-ADC4-1168-DE41412AB513}</x:author>
+    <x:author>tc={66D08A53-A46F-B39D-BF8B-2F91FA5544EC}</x:author>
+    <x:author>tc={8253EE86-7926-8F10-8D36-CD8E983846E3}</x:author>
+    <x:author>tc={63C5B54E-3382-3032-03BC-A4D566E81015}</x:author>
+    <x:author>tc={19946973-1CB9-F97A-932A-4CDC93DA4076}</x:author>
+    <x:author>tc={502F2BD0-069C-A1CB-BE2A-316524EA0FE7}</x:author>
+    <x:author>tc={8D3E5E07-996C-6FA2-B7D2-F0A38B3ECA78}</x:author>
+    <x:author>tc={8E3F859E-A8E6-CD0C-796D-3ABA463D042C}</x:author>
+    <x:author>tc={7598B2B6-A8FF-7FC1-B339-88714951EF7C}</x:author>
+    <x:author>tc={C5D97150-6CE8-0ED7-9C73-F66D04986243}</x:author>
+    <x:author>tc={18CF715D-516E-7251-B463-8CC3AF4028CF}</x:author>
+    <x:author>tc={75B47754-69C2-3985-00C8-8438A73DE06D}</x:author>
+    <x:author>tc={F799C9D6-E29B-DA0B-A2F7-63ADB832072B}</x:author>
+    <x:author>tc={2387B878-7100-9F16-32DA-86297144DD8C}</x:author>
+    <x:author>tc={059C83C8-6D8C-66EA-6ABF-D9624BFBCF3A}</x:author>
+    <x:author>tc={63C2F3AB-4FB1-6250-E0A7-BE401E20C4CB}</x:author>
+    <x:author>tc={162FEE63-E7EE-3E1C-C9D1-370CE352712E}</x:author>
+    <x:author>tc={E1DE05A5-76A2-0262-A273-87EDC9B8395D}</x:author>
+    <x:author>tc={EEA21B70-769F-D42F-BB3B-483AAC8DA47C}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="P5" authorId="0">
@@ -1176,26 +1176,26 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={2E8BB02A-3139-CD3C-5D0E-AC88CA8F2019}</x:author>
-    <x:author>tc={3DDB81FF-15FD-E60F-489B-1575646D8469}</x:author>
-    <x:author>tc={0B5932A0-8591-84E1-4B70-F63B49F3453B}</x:author>
-    <x:author>tc={85C98FD3-C693-02C5-3332-CF1177B551E1}</x:author>
-    <x:author>tc={AF6C3FB9-AED5-75A6-14A0-709E8AB91D48}</x:author>
-    <x:author>tc={4772060B-833A-E9E9-3AFE-49A8716C7E71}</x:author>
-    <x:author>tc={463A4A0F-682B-B1D6-D77A-560A23DBEFDF}</x:author>
-    <x:author>tc={01F27E2A-6725-0C5C-B670-5509C805B925}</x:author>
-    <x:author>tc={D34C2E48-D415-F647-028A-2040DCF81395}</x:author>
-    <x:author>tc={DF49BA02-A9B1-2100-E76D-0280662C0C24}</x:author>
-    <x:author>tc={887B564B-6DF2-1A16-A87D-1690562134E3}</x:author>
-    <x:author>tc={A9408D64-360A-F652-AEBE-EA30854B6D47}</x:author>
-    <x:author>tc={CFA78485-73F2-87C3-2112-AECA95F2BC16}</x:author>
-    <x:author>tc={ACDF2784-4668-8932-E7E5-FED5F88FC129}</x:author>
-    <x:author>tc={8E8819F0-B3BC-BADA-0386-C459F25795B7}</x:author>
-    <x:author>tc={6AEB76BF-D747-D827-DA1F-1DFFC2C9ABE1}</x:author>
-    <x:author>tc={42395BE8-EFDC-96FB-9DDC-BBE06E46377B}</x:author>
-    <x:author>tc={BAC90213-71EA-9619-CF8B-747A266CC1BE}</x:author>
-    <x:author>tc={6832C9B6-023D-39E0-35B5-084E38F583BC}</x:author>
-    <x:author>tc={7993912D-A7F7-7C1A-88A0-D39B35A8B006}</x:author>
+    <x:author>tc={84E13648-C7F0-652B-D6D1-50FB9ABCAD46}</x:author>
+    <x:author>tc={BAE23548-9F72-6653-9CCE-AB5D6CE12D22}</x:author>
+    <x:author>tc={7F7FC2C5-35C0-7E18-21CF-E7ABD151C178}</x:author>
+    <x:author>tc={1C87D2BD-002E-EFEC-6449-F4CC621DAF19}</x:author>
+    <x:author>tc={D82E1942-60FB-A94F-1231-55C186DFE77A}</x:author>
+    <x:author>tc={8C7CBC23-095B-389F-1CE9-66A020ED5F65}</x:author>
+    <x:author>tc={FE08B92E-A8FF-1755-3A77-7296DB082B8F}</x:author>
+    <x:author>tc={17E4C51A-99FC-A26E-FA58-241D1896C185}</x:author>
+    <x:author>tc={EB6DCDB8-08F5-2F6B-58D9-D67FEBC4BF08}</x:author>
+    <x:author>tc={D1283C43-349C-5B77-B9BC-15E4F74CDBF7}</x:author>
+    <x:author>tc={22CEF8D1-497B-0746-E712-0902C2295F03}</x:author>
+    <x:author>tc={80D5AC2B-9FE7-A4E9-D58C-4B8B483C5C5C}</x:author>
+    <x:author>tc={335B0CFE-336B-8BFF-E374-338B849103E5}</x:author>
+    <x:author>tc={1A55DFCA-C281-6722-8F99-5EBA993935F7}</x:author>
+    <x:author>tc={ED05C87E-0A75-049A-05E7-96420E3A1BAD}</x:author>
+    <x:author>tc={5CCA1910-7668-C27B-F4A8-D382B08AB157}</x:author>
+    <x:author>tc={66930877-5ABE-EA1E-A91D-1E239C1A010D}</x:author>
+    <x:author>tc={BA48A1C2-E567-A40A-25BB-8868A2F95826}</x:author>
+    <x:author>tc={5362AA48-E0BF-4B27-6BFF-54D0DEDB7AE8}</x:author>
+    <x:author>tc={3831B5BD-3244-FA9B-D90E-2023EACB683C}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="J5" authorId="0">
@@ -2060,7 +2060,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R225506968cc64361"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb2a91248ccaa4d79"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2071,7 +2071,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{98806F8D-1B23-42E5-B5EC-41B17E56C056}"/>
+  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}"/>
 </xltc:personList>
 </file>
 
@@ -2268,493 +2268,493 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="P5" dT="2026-08-14T20:48:54.584" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{AD76C85B-D33E-BD60-615F-7CE5ACBB1507}">
+  <xltc:threadedComment ref="P5" dT="2026-08-15T06:47:05.396" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{D7179BD9-5380-A2BE-37A2-542620D11FD6}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P6" dT="2026-08-14T20:48:54.596" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{A89C0A60-29CB-BCB1-C24E-756EBBD610BD}">
+  <xltc:threadedComment ref="P6" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{F5D5EA40-9C27-8916-42CA-9F80A998B239}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P7" dT="2026-08-14T20:48:54.596" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{749C636E-7A7E-44AE-C575-6C967A103843}">
+  <xltc:threadedComment ref="P7" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{F4A30194-1A72-1C1B-D3D1-88F0876A8B1C}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P8" dT="2026-08-14T20:48:54.597" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{7FE82A63-FFDB-5C1F-7539-D7FF41424EFB}">
+  <xltc:threadedComment ref="P8" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{058CC015-9E61-4F60-3707-3AA969865D33}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P9" dT="2026-08-14T20:48:54.597" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{BB5F2C3B-1762-02AC-3678-B827F2CD81AD}">
+  <xltc:threadedComment ref="P9" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{0EA9266E-93A4-B7F3-00BA-8A7A79DFC82B}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P10" dT="2026-08-14T20:48:54.597" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{27080485-9683-E160-FF00-3CC16D512FF2}">
+  <xltc:threadedComment ref="P10" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{E0C25A1B-6CEF-EF90-AC34-65B59EB516C3}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 119
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P11" dT="2026-08-14T20:48:54.597" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{DFACCDE4-7ED8-D622-88B3-344385AC3840}">
+  <xltc:threadedComment ref="P11" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{D3577678-9795-3AEE-F6E6-5B7E42106D9E}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 160
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P12" dT="2026-08-14T20:48:54.597" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{176ABCFB-F4B7-F2A0-6CFF-72FCA064BD19}">
+  <xltc:threadedComment ref="P12" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{741168DD-C778-7C15-2B65-17B7C07ED33D}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P13" dT="2026-08-14T20:48:54.597" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{EBD22EC7-7EDE-503C-6C11-C70A8AC85292}">
+  <xltc:threadedComment ref="P13" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{95736628-F1F7-FE17-043B-CA174AE01EDE}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P14" dT="2026-08-14T20:48:54.598" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{A3AB71C1-2A40-68B1-A5CD-30E6E071B7DC}">
+  <xltc:threadedComment ref="P14" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{829B1B69-69D1-E6CE-9B21-D90E9F236E79}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P15" dT="2026-08-14T20:48:54.598" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{9278D5CC-0435-3F11-26AA-50760EA88AE2}">
+  <xltc:threadedComment ref="P15" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{E10C328C-B958-A22D-795B-86894E174992}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P16" dT="2026-08-14T20:48:54.598" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{C5548CA7-37D6-14DD-75DC-5D6ABA3C43C2}">
+  <xltc:threadedComment ref="P16" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{275B946E-B475-F338-1312-E8A66EEE3FB6}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P17" dT="2026-08-14T20:48:54.598" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{64547889-9E0A-2B22-DD82-0C778954A87F}">
+  <xltc:threadedComment ref="P17" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{25671AA7-6F50-28BD-184D-157B185AC6A1}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P18" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{32875CDC-1D01-748F-3FEF-B564BCC4F6CF}">
+  <xltc:threadedComment ref="P18" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{7A90692C-D081-3F82-41F4-9D743B5AB740}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P19" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{B08242B1-EF53-9913-910B-C22C411341F5}">
+  <xltc:threadedComment ref="P19" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{4027D3F6-5103-811E-9867-0F88B7313B4E}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P20" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{92B968CD-6246-8C17-8389-D6C45A3CAE69}">
+  <xltc:threadedComment ref="P20" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{5452B241-D82F-7E23-08FB-0FF6597AF014}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 138
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P21" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{AEFDF43C-FBE8-658F-E8C3-082FBEF1FF40}">
+  <xltc:threadedComment ref="P21" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{846887CC-6779-2558-F219-69B7F4C9101A}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 212
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P22" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{C477C0D5-6519-22F1-33A2-8CBFC5557854}">
+  <xltc:threadedComment ref="P22" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{4F0D7BAC-731A-10AB-17F0-CF67BEA1E0C5}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P23" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{2A8F1AF0-22C9-EDA3-08C4-FFFAA399F3C7}">
+  <xltc:threadedComment ref="P23" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{71806FB6-0323-8EF2-734E-695EBE8E5C19}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P24" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{8BF756B5-5E00-0DE9-09F9-77907D4C9B27}">
+  <xltc:threadedComment ref="P24" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{8C6DD087-476A-4C57-960D-E2895732691A}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P25" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{3FD75A8B-4721-240C-1725-93E3EE1EB986}">
+  <xltc:threadedComment ref="P25" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{B47EBC4F-9B31-E559-6ED9-AAC1C334946A}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P26" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{3F9811A0-E684-E246-E214-8C12573FC814}">
+  <xltc:threadedComment ref="P26" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{58727869-8ACA-389D-CD7D-8FBA1F5DE493}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P27" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{4F9A5689-95B3-30CB-7405-FABFDB180CF4}">
+  <xltc:threadedComment ref="P27" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{62B5311B-9855-6101-F68A-04824B833B3D}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 272
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P28" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{E4D609D7-5387-D1AF-381B-4001D4950E09}">
+  <xltc:threadedComment ref="P28" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{BBE37CF9-417B-8492-B4BC-F67A0FB38F22}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P29" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{67656F98-6111-B2AA-2CAB-FA2A95D68C3B}">
+  <xltc:threadedComment ref="P29" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{11CAB389-76D8-7602-E738-77CB6C823411}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P30" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{EAC88F74-D1D2-F311-7967-60FEFDCFB860}">
+  <xltc:threadedComment ref="P30" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{53C4CB1B-0E8D-3634-8EB7-DFF2141C14F3}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 158
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P31" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{3CFF812D-C7C6-99A0-97E8-633388370E81}">
+  <xltc:threadedComment ref="P31" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{52C4F871-DAB1-FC43-B689-E83208D5BDC2}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P32" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{CFC63739-B318-9DB1-19F0-ABD1F0E2BD96}">
+  <xltc:threadedComment ref="P32" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{5A8F28C0-DCAF-9B4F-60C2-B5519288078D}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P33" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{95EE700C-5315-DC89-F405-B99C0C27E763}">
+  <xltc:threadedComment ref="P33" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{BC440591-751F-ADDA-3E20-D28B53716826}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 72
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P34" dT="2026-08-14T20:48:54.599" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{A530B548-98B2-1B6B-D236-DD4C0D304C21}">
+  <xltc:threadedComment ref="P34" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{129D4D19-7FD2-1FAB-C3F2-3D85C2143407}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P35" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{4A572411-B39B-EF39-03F1-2EFD1E160F62}">
+  <xltc:threadedComment ref="P35" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{C00BE146-1A1C-DE84-6CEC-66E28A34FB62}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P36" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{45916D39-67A3-C79F-ACE1-95D427374BBA}">
+  <xltc:threadedComment ref="P36" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{B2453065-6EF2-25EE-C743-1AF12D44A7E2}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 24
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P37" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{BD825591-F743-259C-A52D-AF796642E59E}">
+  <xltc:threadedComment ref="P37" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{42F5722C-BA58-306D-7716-E7DB46B06E1C}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P38" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{B8F05642-8361-695B-E2C3-D72F79D4922A}">
+  <xltc:threadedComment ref="P38" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{308E1DA8-4C3B-C720-C61A-B4FD5B863D5A}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P39" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{E508EB94-396C-1034-1316-58874D6E8BC9}">
+  <xltc:threadedComment ref="P39" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{575A735C-1490-C525-7FDA-D0D6CC2167F3}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 19
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P40" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{1793642E-C2C1-DAAC-7003-1FCD16D9A995}">
+  <xltc:threadedComment ref="P40" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{F04ECB4C-E296-D7B7-16F0-976919B7E452}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P41" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{F5E05C9C-40FB-C157-CA88-5B258C461C5C}">
+  <xltc:threadedComment ref="P41" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{890C7111-93D9-523E-D457-71A4254BA046}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P42" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{86D52D69-2BD9-5726-B3DD-8E6158F10E4C}">
+  <xltc:threadedComment ref="P42" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{73A6DDDE-3DDB-F0A0-8427-697A1F7CA9D6}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P43" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{75BAA52B-52EB-8817-C639-C9790E51E370}">
+  <xltc:threadedComment ref="P43" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{F8EC0B12-3474-AF0F-5A97-A40007A76C72}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P44" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{D514FC67-0E8C-8F25-EDF2-E61B9654E20D}">
+  <xltc:threadedComment ref="P44" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{835BEA1E-53F0-17E6-E7D7-DBD14ED53706}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P45" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{E1C9BA7F-CA9B-C28D-CDFC-F17719A0EBB2}">
+  <xltc:threadedComment ref="P45" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{CA531C19-FD45-25C9-0D70-197E1279C769}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P46" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{057F447F-84A0-FE01-54A6-E5B1957E058E}">
+  <xltc:threadedComment ref="P46" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{8774F1F6-5214-2114-2D61-8456D5360289}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P47" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{8FF56FC9-DE0E-E4F8-D33E-05FC6B5D72A5}">
+  <xltc:threadedComment ref="P47" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{30902EAC-5720-96A7-8284-3D2CCAB7443B}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P48" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{9C8A34A8-8CB0-CB37-B659-2765B7286F51}">
+  <xltc:threadedComment ref="P48" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{0CB4A533-3016-5908-0FCF-23076D4239A8}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P49" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{A52F21B2-F7F1-89FB-088A-6B573542A95A}">
+  <xltc:threadedComment ref="P49" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{E740C3D1-D9F7-5D7D-AFF3-68BEEEF5AFB6}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 118
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P50" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{B3D29C51-43CA-18B8-F661-9AC7B04E76C2}">
+  <xltc:threadedComment ref="P50" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{F69FF8B4-C804-AEE4-CB67-276CB58FECC3}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P51" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{895E733F-9450-F643-A586-C9778BCFEF53}">
+  <xltc:threadedComment ref="P51" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{C43B89C3-9376-EAD3-76C9-17647D15CCF5}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P52" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{E6634DA4-21AA-05EC-F06D-B9D5A9029DF0}">
+  <xltc:threadedComment ref="P52" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{E454CB3F-C1C8-45BE-B525-60EFF4CDE1A6}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P53" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{41664D94-9B65-23EB-6D48-DE9DB5D48E7E}">
+  <xltc:threadedComment ref="P53" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{676951D3-752E-15EF-F207-A9C4AD907FBD}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-STF</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P54" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{D8706B28-69B3-9F03-9DD7-886259DD8C69}">
+  <xltc:threadedComment ref="P54" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{B43928D3-C753-0831-5261-410F7BBF0732}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P55" dT="2026-08-14T20:48:54.6" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{D4F74F82-BBBB-6122-E9FE-F14DAE37B14A}">
+  <xltc:threadedComment ref="P55" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{7AEC7DF7-C2FC-5FD1-43E7-E31427E0CB4D}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P56" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{67A80EB2-6450-F365-0B53-F66EF759A5B2}">
+  <xltc:threadedComment ref="P56" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{483F7CB9-A550-4C88-F30A-79F3465B8236}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 18
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P57" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{63BE2D86-BC91-9099-14D4-20CA68378DC7}">
+  <xltc:threadedComment ref="P57" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{57E4D7D6-EAC9-3255-FC08-228D23302E84}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P58" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{DE361AF7-1C5C-532F-D7E1-1E40636E490B}">
+  <xltc:threadedComment ref="P58" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{63285F2A-DBA1-0A5B-0BD2-5CF8872592B7}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P59" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{0E8348F2-AC6D-4391-024E-2BB4B1396566}">
+  <xltc:threadedComment ref="P59" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{5E490997-C386-5F07-4415-3BF718F6583D}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P60" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{5297095B-D43A-8FE6-6F7E-CD5A9B27EA97}">
+  <xltc:threadedComment ref="P60" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{530EEE62-CA06-D2AD-47F5-B427C42F71A7}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P61" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{DA505CEF-AD44-D5D1-9EBC-8FBF8727A618}">
+  <xltc:threadedComment ref="P61" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{D3192F1B-D4AE-761E-78F3-B7200E4D78DD}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P62" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{D310B17F-864A-65D6-C23B-18D651A1BCA9}">
+  <xltc:threadedComment ref="P62" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{5ECB39A3-6CD9-BC08-DE2C-8BC987C1390A}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P63" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{99302A77-FD55-DE9E-B462-BC716BFA9BB5}">
+  <xltc:threadedComment ref="P63" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{83C028C4-B49A-845A-F950-45971513DB9D}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P64" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{E66C77C3-9DB9-77B6-0264-53B6C1B54F2D}">
+  <xltc:threadedComment ref="P64" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{14DD0686-1E74-4983-CD5F-91C8010BF879}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P65" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{DC9B3809-0C62-C255-8FE9-E64A74085043}">
+  <xltc:threadedComment ref="P65" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{42144CB2-40A1-FE82-EC8C-D7B918D43B31}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 311
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P66" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{2B3B55AF-EB7A-60A7-0288-A2A428FD6C08}">
+  <xltc:threadedComment ref="P66" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{175AC13F-5A05-534D-C6C5-368C220513B3}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P67" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{276AFF59-0B12-12D0-1431-5C76483864FF}">
+  <xltc:threadedComment ref="P67" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{98B1FE03-8508-60EB-FB28-AC6EB4FF17EC}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P68" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{D0D0533F-41FA-AB3B-9E96-F9659D12551B}">
+  <xltc:threadedComment ref="P68" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{CA1C4C92-831F-ADC4-1168-DE41412AB513}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 141
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P69" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{CA5C3F8B-3FB1-F256-BF7C-CF6073C0018C}">
+  <xltc:threadedComment ref="P69" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{66D08A53-A46F-B39D-BF8B-2F91FA5544EC}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P70" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{323181B4-321D-C42A-1A18-A4AEC9952C57}">
+  <xltc:threadedComment ref="P70" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{8253EE86-7926-8F10-8D36-CD8E983846E3}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P71" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{4CF5C5D2-52D9-A3C3-9A30-81F574BE209A}">
+  <xltc:threadedComment ref="P71" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{63C5B54E-3382-3032-03BC-A4D566E81015}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 33
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P72" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{3E520E3F-3E8D-0F95-D221-C87981A69FF7}">
+  <xltc:threadedComment ref="P72" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{19946973-1CB9-F97A-932A-4CDC93DA4076}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P73" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{F7DB273B-83BD-C7BB-95C1-735B3AF1B205}">
+  <xltc:threadedComment ref="P73" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{502F2BD0-069C-A1CB-BE2A-316524EA0FE7}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P74" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{22866379-A890-E2D9-0B92-FACDCC7AB0BC}">
+  <xltc:threadedComment ref="P74" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{8D3E5E07-996C-6FA2-B7D2-F0A38B3ECA78}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 21
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P75" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{6D8065DD-C4EF-A377-7BFD-3DEDCF918431}">
+  <xltc:threadedComment ref="P75" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{8E3F859E-A8E6-CD0C-796D-3ABA463D042C}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P76" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{A39373E7-D5D7-F8D4-9E1F-40821AB51A56}">
+  <xltc:threadedComment ref="P76" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{7598B2B6-A8FF-7FC1-B339-88714951EF7C}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P77" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{0A44F521-9201-C9A1-7C6D-695551F24ABE}">
+  <xltc:threadedComment ref="P77" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{C5D97150-6CE8-0ED7-9C73-F66D04986243}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 19
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P78" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{786A3C30-A168-1FE7-0EF4-AFE4E8F47993}">
+  <xltc:threadedComment ref="P78" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{18CF715D-516E-7251-B463-8CC3AF4028CF}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 43
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P79" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{68A7284C-A659-0183-CDD3-AEE90897FAAE}">
+  <xltc:threadedComment ref="P79" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{75B47754-69C2-3985-00C8-8438A73DE06D}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 44
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P80" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{E10ADEC7-AB15-EC53-EDE8-D3A26CA60955}">
+  <xltc:threadedComment ref="P80" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{F799C9D6-E29B-DA0B-A2F7-63ADB832072B}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 40
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P81" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{42F3A693-983F-A53F-D994-965ABBF672D0}">
+  <xltc:threadedComment ref="P81" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{2387B878-7100-9F16-32DA-86297144DD8C}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P82" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{40E2782A-C3CC-2E07-7DE1-DB388D05A7A8}">
+  <xltc:threadedComment ref="P82" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{059C83C8-6D8C-66EA-6ABF-D9624BFBCF3A}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P83" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{E50522DB-6CC5-0301-2314-72EC58FE6953}">
+  <xltc:threadedComment ref="P83" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{63C2F3AB-4FB1-6250-E0A7-BE401E20C4CB}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 16
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P84" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{58739544-7137-FB67-590F-28D001FB2D1D}">
+  <xltc:threadedComment ref="P84" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{162FEE63-E7EE-3E1C-C9D1-370CE352712E}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P85" dT="2026-08-14T20:48:54.601" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{AD0E6454-9F8B-B5E0-95B7-AFEDC038B461}">
+  <xltc:threadedComment ref="P85" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{E1DE05A5-76A2-0262-A273-87EDC9B8395D}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P86" dT="2026-08-14T20:48:54.602" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{1C8AD75C-462E-DBCB-8E4B-37D4695C94F8}">
+  <xltc:threadedComment ref="P86" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{EEA21B70-769F-D42F-BB3B-483AAC8DA47C}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 21
 Available: 2026-02-25
@@ -2765,64 +2765,64 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="J5" dT="2026-08-14T20:48:55.323" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{2E8BB02A-3139-CD3C-5D0E-AC88CA8F2019}">
+  <xltc:threadedComment ref="J5" dT="2026-08-15T06:47:05.762" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{84E13648-C7F0-652B-D6D1-50FB9ABCAD46}">
     <xltc:text>Official source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J6" dT="2026-08-14T20:48:55.329" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{3DDB81FF-15FD-E60F-489B-1575646D8469}">
+  <xltc:threadedComment ref="J6" dT="2026-08-15T06:47:05.764" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{BAE23548-9F72-6653-9CCE-AB5D6CE12D22}">
     <xltc:text>Official source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J7" dT="2026-08-14T20:48:55.335" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{0B5932A0-8591-84E1-4B70-F63B49F3453B}">
+  <xltc:threadedComment ref="J7" dT="2026-08-15T06:47:05.766" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{7F7FC2C5-35C0-7E18-21CF-E7ABD151C178}">
     <xltc:text>Official source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J8" dT="2026-08-14T20:48:55.34" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{85C98FD3-C693-02C5-3332-CF1177B551E1}">
+  <xltc:threadedComment ref="J8" dT="2026-08-15T06:47:05.768" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{1C87D2BD-002E-EFEC-6449-F4CC621DAF19}">
     <xltc:text>Official source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J9" dT="2026-08-14T20:48:55.346" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{AF6C3FB9-AED5-75A6-14A0-709E8AB91D48}">
+  <xltc:threadedComment ref="J9" dT="2026-08-15T06:47:05.771" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{D82E1942-60FB-A94F-1231-55C186DFE77A}">
     <xltc:text>Official source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J10" dT="2026-08-14T20:48:55.35" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{4772060B-833A-E9E9-3AFE-49A8716C7E71}">
+  <xltc:threadedComment ref="J10" dT="2026-08-15T06:47:05.774" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{8C7CBC23-095B-389F-1CE9-66A020ED5F65}">
     <xltc:text>Official source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J11" dT="2026-08-14T20:48:55.355" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{463A4A0F-682B-B1D6-D77A-560A23DBEFDF}">
+  <xltc:threadedComment ref="J11" dT="2026-08-15T06:47:05.776" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{FE08B92E-A8FF-1755-3A77-7296DB082B8F}">
     <xltc:text>Official source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J12" dT="2026-08-14T20:48:55.359" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{01F27E2A-6725-0C5C-B670-5509C805B925}">
+  <xltc:threadedComment ref="J12" dT="2026-08-15T06:47:05.778" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{17E4C51A-99FC-A26E-FA58-241D1896C185}">
     <xltc:text>Official source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J13" dT="2026-08-14T20:48:55.363" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{D34C2E48-D415-F647-028A-2040DCF81395}">
+  <xltc:threadedComment ref="J13" dT="2026-08-15T06:47:05.779" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{EB6DCDB8-08F5-2F6B-58D9-D67FEBC4BF08}">
     <xltc:text>Official source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J14" dT="2026-08-14T20:48:55.368" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{DF49BA02-A9B1-2100-E76D-0280662C0C24}">
+  <xltc:threadedComment ref="J14" dT="2026-08-15T06:47:05.782" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{D1283C43-349C-5B77-B9BC-15E4F74CDBF7}">
     <xltc:text>Official source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J15" dT="2026-08-14T20:48:55.372" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{887B564B-6DF2-1A16-A87D-1690562134E3}">
+  <xltc:threadedComment ref="J15" dT="2026-08-15T06:47:05.784" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{22CEF8D1-497B-0746-E712-0902C2295F03}">
     <xltc:text>Official source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J16" dT="2026-08-14T20:48:55.377" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{A9408D64-360A-F652-AEBE-EA30854B6D47}">
+  <xltc:threadedComment ref="J16" dT="2026-08-15T06:47:05.786" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{80D5AC2B-9FE7-A4E9-D58C-4B8B483C5C5C}">
     <xltc:text>Official source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J17" dT="2026-08-14T20:48:55.38" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{CFA78485-73F2-87C3-2112-AECA95F2BC16}">
+  <xltc:threadedComment ref="J17" dT="2026-08-15T06:47:05.787" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{335B0CFE-336B-8BFF-E374-338B849103E5}">
     <xltc:text>Official source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J18" dT="2026-08-14T20:48:55.384" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{ACDF2784-4668-8932-E7E5-FED5F88FC129}">
+  <xltc:threadedComment ref="J18" dT="2026-08-15T06:47:05.79" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{1A55DFCA-C281-6722-8F99-5EBA993935F7}">
     <xltc:text>Official source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J19" dT="2026-08-14T20:48:55.39" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{8E8819F0-B3BC-BADA-0386-C459F25795B7}">
+  <xltc:threadedComment ref="J19" dT="2026-08-15T06:47:05.795" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{ED05C87E-0A75-049A-05E7-96420E3A1BAD}">
     <xltc:text>Official source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J20" dT="2026-08-14T20:48:55.393" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{6AEB76BF-D747-D827-DA1F-1DFFC2C9ABE1}">
+  <xltc:threadedComment ref="J20" dT="2026-08-15T06:47:05.797" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{5CCA1910-7668-C27B-F4A8-D382B08AB157}">
     <xltc:text>Official source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J21" dT="2026-08-14T20:48:55.397" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{42395BE8-EFDC-96FB-9DDC-BBE06E46377B}">
+  <xltc:threadedComment ref="J21" dT="2026-08-15T06:47:05.798" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{66930877-5ABE-EA1E-A91D-1E239C1A010D}">
     <xltc:text>Official source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J22" dT="2026-08-14T20:48:55.4" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{BAC90213-71EA-9619-CF8B-747A266CC1BE}">
+  <xltc:threadedComment ref="J22" dT="2026-08-15T06:47:05.8" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{BA48A1C2-E567-A40A-25BB-8868A2F95826}">
     <xltc:text>Official source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J23" dT="2026-08-14T20:48:55.403" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{6832C9B6-023D-39E0-35B5-084E38F583BC}">
+  <xltc:threadedComment ref="J23" dT="2026-08-15T06:47:05.801" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{5362AA48-E0BF-4B27-6BFF-54D0DEDB7AE8}">
     <xltc:text>Official source: https://www.aspenpharma.com/download/annual-financial-statements-2/</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J24" dT="2026-08-14T20:48:55.406" personId="{98806F8D-1B23-42E5-B5EC-41B17E56C056}" id="{7993912D-A7F7-7C1A-88A0-D39B35A8B006}">
+  <xltc:threadedComment ref="J24" dT="2026-08-15T06:47:05.803" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{3831B5BD-3244-FA9B-D90E-2023EACB683C}">
     <xltc:text>Official source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -3877,7 +3877,7 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R197aeb9524e2433e"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f43e8fb0cb14fa4"/>
 </x:worksheet>
 </file>
 
@@ -8611,7 +8611,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R528b73a12e734350"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc977ac405e143db"/>
 </x:worksheet>
 </file>
 
@@ -9671,7 +9671,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d2884a664a446d2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb88cdafbb43b432f"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Finalize V3.2.0 release artifacts
</commit_message>
<xml_diff>
--- a/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
+++ b/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Ra1182a63c5894c67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R448d143ca02b418c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="R4fa6f96291d74d3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Raf050af4020f48df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="Rc1ad0475627043e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R4ae43fe769874c98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Rb31cfb05154f48eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="R72998ff4388441f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R9c4233326ec74bde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="Rd4f648fe156f49b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R380f9c27d3944774"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="Rfffcb405ec464c1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="R48c193a887c4416e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Rd66998ed3cc04402"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R49c40c130e0d45ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R631bd8a5e6674ca9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Rde69964a6bf84944"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="R858c58fbb73144bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="Rf02af7084cc44489"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R85030ef8203c4a51"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,88 +19,88 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={D7179BD9-5380-A2BE-37A2-542620D11FD6}</x:author>
-    <x:author>tc={F5D5EA40-9C27-8916-42CA-9F80A998B239}</x:author>
-    <x:author>tc={F4A30194-1A72-1C1B-D3D1-88F0876A8B1C}</x:author>
-    <x:author>tc={058CC015-9E61-4F60-3707-3AA969865D33}</x:author>
-    <x:author>tc={0EA9266E-93A4-B7F3-00BA-8A7A79DFC82B}</x:author>
-    <x:author>tc={E0C25A1B-6CEF-EF90-AC34-65B59EB516C3}</x:author>
-    <x:author>tc={D3577678-9795-3AEE-F6E6-5B7E42106D9E}</x:author>
-    <x:author>tc={741168DD-C778-7C15-2B65-17B7C07ED33D}</x:author>
-    <x:author>tc={95736628-F1F7-FE17-043B-CA174AE01EDE}</x:author>
-    <x:author>tc={829B1B69-69D1-E6CE-9B21-D90E9F236E79}</x:author>
-    <x:author>tc={E10C328C-B958-A22D-795B-86894E174992}</x:author>
-    <x:author>tc={275B946E-B475-F338-1312-E8A66EEE3FB6}</x:author>
-    <x:author>tc={25671AA7-6F50-28BD-184D-157B185AC6A1}</x:author>
-    <x:author>tc={7A90692C-D081-3F82-41F4-9D743B5AB740}</x:author>
-    <x:author>tc={4027D3F6-5103-811E-9867-0F88B7313B4E}</x:author>
-    <x:author>tc={5452B241-D82F-7E23-08FB-0FF6597AF014}</x:author>
-    <x:author>tc={846887CC-6779-2558-F219-69B7F4C9101A}</x:author>
-    <x:author>tc={4F0D7BAC-731A-10AB-17F0-CF67BEA1E0C5}</x:author>
-    <x:author>tc={71806FB6-0323-8EF2-734E-695EBE8E5C19}</x:author>
-    <x:author>tc={8C6DD087-476A-4C57-960D-E2895732691A}</x:author>
-    <x:author>tc={B47EBC4F-9B31-E559-6ED9-AAC1C334946A}</x:author>
-    <x:author>tc={58727869-8ACA-389D-CD7D-8FBA1F5DE493}</x:author>
-    <x:author>tc={62B5311B-9855-6101-F68A-04824B833B3D}</x:author>
-    <x:author>tc={BBE37CF9-417B-8492-B4BC-F67A0FB38F22}</x:author>
-    <x:author>tc={11CAB389-76D8-7602-E738-77CB6C823411}</x:author>
-    <x:author>tc={53C4CB1B-0E8D-3634-8EB7-DFF2141C14F3}</x:author>
-    <x:author>tc={52C4F871-DAB1-FC43-B689-E83208D5BDC2}</x:author>
-    <x:author>tc={5A8F28C0-DCAF-9B4F-60C2-B5519288078D}</x:author>
-    <x:author>tc={BC440591-751F-ADDA-3E20-D28B53716826}</x:author>
-    <x:author>tc={129D4D19-7FD2-1FAB-C3F2-3D85C2143407}</x:author>
-    <x:author>tc={C00BE146-1A1C-DE84-6CEC-66E28A34FB62}</x:author>
-    <x:author>tc={B2453065-6EF2-25EE-C743-1AF12D44A7E2}</x:author>
-    <x:author>tc={42F5722C-BA58-306D-7716-E7DB46B06E1C}</x:author>
-    <x:author>tc={308E1DA8-4C3B-C720-C61A-B4FD5B863D5A}</x:author>
-    <x:author>tc={575A735C-1490-C525-7FDA-D0D6CC2167F3}</x:author>
-    <x:author>tc={F04ECB4C-E296-D7B7-16F0-976919B7E452}</x:author>
-    <x:author>tc={890C7111-93D9-523E-D457-71A4254BA046}</x:author>
-    <x:author>tc={73A6DDDE-3DDB-F0A0-8427-697A1F7CA9D6}</x:author>
-    <x:author>tc={F8EC0B12-3474-AF0F-5A97-A40007A76C72}</x:author>
-    <x:author>tc={835BEA1E-53F0-17E6-E7D7-DBD14ED53706}</x:author>
-    <x:author>tc={CA531C19-FD45-25C9-0D70-197E1279C769}</x:author>
-    <x:author>tc={8774F1F6-5214-2114-2D61-8456D5360289}</x:author>
-    <x:author>tc={30902EAC-5720-96A7-8284-3D2CCAB7443B}</x:author>
-    <x:author>tc={0CB4A533-3016-5908-0FCF-23076D4239A8}</x:author>
-    <x:author>tc={E740C3D1-D9F7-5D7D-AFF3-68BEEEF5AFB6}</x:author>
-    <x:author>tc={F69FF8B4-C804-AEE4-CB67-276CB58FECC3}</x:author>
-    <x:author>tc={C43B89C3-9376-EAD3-76C9-17647D15CCF5}</x:author>
-    <x:author>tc={E454CB3F-C1C8-45BE-B525-60EFF4CDE1A6}</x:author>
-    <x:author>tc={676951D3-752E-15EF-F207-A9C4AD907FBD}</x:author>
-    <x:author>tc={B43928D3-C753-0831-5261-410F7BBF0732}</x:author>
-    <x:author>tc={7AEC7DF7-C2FC-5FD1-43E7-E31427E0CB4D}</x:author>
-    <x:author>tc={483F7CB9-A550-4C88-F30A-79F3465B8236}</x:author>
-    <x:author>tc={57E4D7D6-EAC9-3255-FC08-228D23302E84}</x:author>
-    <x:author>tc={63285F2A-DBA1-0A5B-0BD2-5CF8872592B7}</x:author>
-    <x:author>tc={5E490997-C386-5F07-4415-3BF718F6583D}</x:author>
-    <x:author>tc={530EEE62-CA06-D2AD-47F5-B427C42F71A7}</x:author>
-    <x:author>tc={D3192F1B-D4AE-761E-78F3-B7200E4D78DD}</x:author>
-    <x:author>tc={5ECB39A3-6CD9-BC08-DE2C-8BC987C1390A}</x:author>
-    <x:author>tc={83C028C4-B49A-845A-F950-45971513DB9D}</x:author>
-    <x:author>tc={14DD0686-1E74-4983-CD5F-91C8010BF879}</x:author>
-    <x:author>tc={42144CB2-40A1-FE82-EC8C-D7B918D43B31}</x:author>
-    <x:author>tc={175AC13F-5A05-534D-C6C5-368C220513B3}</x:author>
-    <x:author>tc={98B1FE03-8508-60EB-FB28-AC6EB4FF17EC}</x:author>
-    <x:author>tc={CA1C4C92-831F-ADC4-1168-DE41412AB513}</x:author>
-    <x:author>tc={66D08A53-A46F-B39D-BF8B-2F91FA5544EC}</x:author>
-    <x:author>tc={8253EE86-7926-8F10-8D36-CD8E983846E3}</x:author>
-    <x:author>tc={63C5B54E-3382-3032-03BC-A4D566E81015}</x:author>
-    <x:author>tc={19946973-1CB9-F97A-932A-4CDC93DA4076}</x:author>
-    <x:author>tc={502F2BD0-069C-A1CB-BE2A-316524EA0FE7}</x:author>
-    <x:author>tc={8D3E5E07-996C-6FA2-B7D2-F0A38B3ECA78}</x:author>
-    <x:author>tc={8E3F859E-A8E6-CD0C-796D-3ABA463D042C}</x:author>
-    <x:author>tc={7598B2B6-A8FF-7FC1-B339-88714951EF7C}</x:author>
-    <x:author>tc={C5D97150-6CE8-0ED7-9C73-F66D04986243}</x:author>
-    <x:author>tc={18CF715D-516E-7251-B463-8CC3AF4028CF}</x:author>
-    <x:author>tc={75B47754-69C2-3985-00C8-8438A73DE06D}</x:author>
-    <x:author>tc={F799C9D6-E29B-DA0B-A2F7-63ADB832072B}</x:author>
-    <x:author>tc={2387B878-7100-9F16-32DA-86297144DD8C}</x:author>
-    <x:author>tc={059C83C8-6D8C-66EA-6ABF-D9624BFBCF3A}</x:author>
-    <x:author>tc={63C2F3AB-4FB1-6250-E0A7-BE401E20C4CB}</x:author>
-    <x:author>tc={162FEE63-E7EE-3E1C-C9D1-370CE352712E}</x:author>
-    <x:author>tc={E1DE05A5-76A2-0262-A273-87EDC9B8395D}</x:author>
-    <x:author>tc={EEA21B70-769F-D42F-BB3B-483AAC8DA47C}</x:author>
+    <x:author>tc={0AF4FEDA-AC03-3F9A-4677-E614750C0BE6}</x:author>
+    <x:author>tc={7B13601B-A686-D1F6-E2C3-2DEAACC41826}</x:author>
+    <x:author>tc={10B9DE82-DAAF-597E-4424-E67283E9A4F8}</x:author>
+    <x:author>tc={9DDF9D19-AAB7-35C6-6EAB-ADE447886907}</x:author>
+    <x:author>tc={CEC6EDDA-4333-DE39-19A1-CD6C28B0071E}</x:author>
+    <x:author>tc={9E0A3C03-F7F7-40B8-594C-1134A321AF12}</x:author>
+    <x:author>tc={6A469CC5-9E84-42E7-A4A2-5046B5EB797A}</x:author>
+    <x:author>tc={49F38930-D4FC-9148-B4AB-7B8868A6B1C4}</x:author>
+    <x:author>tc={6AE471B8-00A6-D8CA-E30E-F2F43B242CB2}</x:author>
+    <x:author>tc={070A3F26-F4D3-3501-5B26-B76E24181EE6}</x:author>
+    <x:author>tc={DB4AA7DC-83F7-AA9C-6650-AC0FBB081C37}</x:author>
+    <x:author>tc={E8A6B8CE-ACDD-0EA3-3036-3FEA4BE387E5}</x:author>
+    <x:author>tc={F5132FA4-62BD-C63C-B25A-A7E1FE946B04}</x:author>
+    <x:author>tc={924A75EC-79F9-BE2D-03E1-123D59F3BF71}</x:author>
+    <x:author>tc={7DFAAAEE-9F37-70B4-1295-82F48891DA0C}</x:author>
+    <x:author>tc={E2EA446D-49CF-67B3-25D3-448163193339}</x:author>
+    <x:author>tc={130AC7D8-E99A-FB9E-EC90-C0CC209F65EE}</x:author>
+    <x:author>tc={DFEDA6A7-98B9-D90B-F8E4-87463C1ABE71}</x:author>
+    <x:author>tc={F908D626-E856-7A2E-B578-6FFFAF10A067}</x:author>
+    <x:author>tc={4691BC9F-FA65-4FBB-BE88-C3485B37BF5B}</x:author>
+    <x:author>tc={54D1659D-A9A9-797D-09FE-9CCD3046EB3B}</x:author>
+    <x:author>tc={32021335-239B-D7CF-C593-02492073755E}</x:author>
+    <x:author>tc={2D4C52F2-DF0E-98A8-DBAD-465EFEA6430C}</x:author>
+    <x:author>tc={4F673CEB-0DB2-16EC-1BF9-E9916FC0D89C}</x:author>
+    <x:author>tc={8C766CE4-DCA4-0227-2719-EC43FBE4EB3E}</x:author>
+    <x:author>tc={030B07FB-3D16-4698-B4D5-9BFD808ED081}</x:author>
+    <x:author>tc={BB835A0A-AC15-BD40-37D2-BB2D5D7D1A29}</x:author>
+    <x:author>tc={ACE1C8E0-F10B-F24B-C4C3-09990BA1EAF5}</x:author>
+    <x:author>tc={89E2F11B-ECCC-3429-226F-74770117AB92}</x:author>
+    <x:author>tc={FE94A6DE-84F6-0201-3EFF-69B3D6B7D622}</x:author>
+    <x:author>tc={5FADB78B-442A-2857-7CCC-D525C440BCCF}</x:author>
+    <x:author>tc={33238565-3127-12AD-ACAF-5A83E4E3101E}</x:author>
+    <x:author>tc={DBA819E1-2CFB-40C0-8E60-4EBBB4963742}</x:author>
+    <x:author>tc={831BC617-DC59-E847-0D3A-95946FD8D988}</x:author>
+    <x:author>tc={9625D7E8-9A23-1EEE-66C1-3D1F41528532}</x:author>
+    <x:author>tc={36A13555-305E-B2C5-2B7A-87476C5BA766}</x:author>
+    <x:author>tc={69541CEA-6E11-BC48-6898-36AE3D548AB4}</x:author>
+    <x:author>tc={12AFE746-FDD9-963F-DCFD-DC968D22FFA6}</x:author>
+    <x:author>tc={425C83BD-D4DC-BDED-071D-487523F8AC3F}</x:author>
+    <x:author>tc={2D72A011-0216-7D35-09A3-D704E88BAEE3}</x:author>
+    <x:author>tc={86FBCAB8-88A0-F97B-4FA1-13C4BEAA369D}</x:author>
+    <x:author>tc={9185AC7C-5FA5-8BAE-5D74-F86F31883FC5}</x:author>
+    <x:author>tc={8F348568-9728-931E-D9B2-061F382ED13A}</x:author>
+    <x:author>tc={E5746BEC-90A8-ABA0-16B5-A6A9F11A2C96}</x:author>
+    <x:author>tc={4B1E6C62-4809-1469-5784-9EA7A65F2E2D}</x:author>
+    <x:author>tc={271EEFA8-492B-5EC5-67E3-8B28D1AE9871}</x:author>
+    <x:author>tc={3430FD27-2DAA-4633-A322-0688F2FCD467}</x:author>
+    <x:author>tc={8D7DF3C9-36A9-2E8C-6160-11B116238A97}</x:author>
+    <x:author>tc={31933AFB-CA47-471A-E7EB-D7E5B693D87A}</x:author>
+    <x:author>tc={CEB8E96A-F9CE-D6E4-1345-25BEA6D4853C}</x:author>
+    <x:author>tc={CE8B63E6-EC70-4885-EBBF-C61B84B9BD02}</x:author>
+    <x:author>tc={1236AB2A-50DD-58C5-F0CF-0A77396ECCB9}</x:author>
+    <x:author>tc={23B809AB-666E-3843-AA8B-2E06C9D6735C}</x:author>
+    <x:author>tc={F9218197-D7D7-96FC-5DEE-19E1B89C6668}</x:author>
+    <x:author>tc={49C564EF-C6E1-AA3E-BAE6-F9B6B7DAF702}</x:author>
+    <x:author>tc={6A34B57F-09E3-5DA4-9CDF-BDD9AFC15C62}</x:author>
+    <x:author>tc={EA67CC0C-3B7B-6001-4E9C-C907CB9A2E41}</x:author>
+    <x:author>tc={2C705125-9621-DC7B-9356-1AFFFB014183}</x:author>
+    <x:author>tc={4127462E-7049-10C8-6E6D-2726FCAFA040}</x:author>
+    <x:author>tc={DDC7860C-4BF8-FE8E-AB94-BF36F51E4742}</x:author>
+    <x:author>tc={355CD349-BEF2-1F91-3717-B7779FC267B7}</x:author>
+    <x:author>tc={BE707954-D4F8-3036-E784-0F6EF373E3B1}</x:author>
+    <x:author>tc={30C17E09-F415-E5D5-1412-983D6592AE59}</x:author>
+    <x:author>tc={946D1FE7-F4AA-6563-A358-3F55219C3AED}</x:author>
+    <x:author>tc={FF9DEADC-5F2B-2C71-0EDD-31A65A1DAC80}</x:author>
+    <x:author>tc={99FA21E2-86C5-2A76-2880-8215954AA3D4}</x:author>
+    <x:author>tc={901E21A1-49DD-A0DA-0A10-1EDE8076C1B3}</x:author>
+    <x:author>tc={FCB3C38E-B0AF-A412-700D-4D9A9D2C2741}</x:author>
+    <x:author>tc={9382A565-2A1D-550E-54B1-678F98943EC6}</x:author>
+    <x:author>tc={40576489-4A24-6AA0-06F2-24F75770098B}</x:author>
+    <x:author>tc={D80EF366-6BBD-D5AC-E71F-5666ED857ED8}</x:author>
+    <x:author>tc={8E28E375-5E9B-B43C-02D8-1D69B6DBCCB7}</x:author>
+    <x:author>tc={C52D303F-E26F-AEB2-82AD-C196257D053A}</x:author>
+    <x:author>tc={AD3CBF1C-654B-022F-1CCE-E3B6B02846E3}</x:author>
+    <x:author>tc={2EEF0622-B8D5-960E-069D-57BC28C46AE4}</x:author>
+    <x:author>tc={C7A17400-8C3D-04F3-BB45-75623A8D8379}</x:author>
+    <x:author>tc={9CB15BCB-A81F-4C51-B6D7-CA70F830A75F}</x:author>
+    <x:author>tc={9CDE5188-52E3-BEBE-AC4D-8F98AC717AA6}</x:author>
+    <x:author>tc={96D773F7-6FC9-4DF1-46BC-3C5A65EBE44A}</x:author>
+    <x:author>tc={69BF4FC0-9856-F2BC-F517-9DC02348AB96}</x:author>
+    <x:author>tc={EF1A8A33-3E41-8002-8157-23C7596AF4CA}</x:author>
+    <x:author>tc={CBA415B4-31A9-6F43-882D-D511ADAA6836}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="P5" authorId="0">
@@ -1176,26 +1176,26 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={84E13648-C7F0-652B-D6D1-50FB9ABCAD46}</x:author>
-    <x:author>tc={BAE23548-9F72-6653-9CCE-AB5D6CE12D22}</x:author>
-    <x:author>tc={7F7FC2C5-35C0-7E18-21CF-E7ABD151C178}</x:author>
-    <x:author>tc={1C87D2BD-002E-EFEC-6449-F4CC621DAF19}</x:author>
-    <x:author>tc={D82E1942-60FB-A94F-1231-55C186DFE77A}</x:author>
-    <x:author>tc={8C7CBC23-095B-389F-1CE9-66A020ED5F65}</x:author>
-    <x:author>tc={FE08B92E-A8FF-1755-3A77-7296DB082B8F}</x:author>
-    <x:author>tc={17E4C51A-99FC-A26E-FA58-241D1896C185}</x:author>
-    <x:author>tc={EB6DCDB8-08F5-2F6B-58D9-D67FEBC4BF08}</x:author>
-    <x:author>tc={D1283C43-349C-5B77-B9BC-15E4F74CDBF7}</x:author>
-    <x:author>tc={22CEF8D1-497B-0746-E712-0902C2295F03}</x:author>
-    <x:author>tc={80D5AC2B-9FE7-A4E9-D58C-4B8B483C5C5C}</x:author>
-    <x:author>tc={335B0CFE-336B-8BFF-E374-338B849103E5}</x:author>
-    <x:author>tc={1A55DFCA-C281-6722-8F99-5EBA993935F7}</x:author>
-    <x:author>tc={ED05C87E-0A75-049A-05E7-96420E3A1BAD}</x:author>
-    <x:author>tc={5CCA1910-7668-C27B-F4A8-D382B08AB157}</x:author>
-    <x:author>tc={66930877-5ABE-EA1E-A91D-1E239C1A010D}</x:author>
-    <x:author>tc={BA48A1C2-E567-A40A-25BB-8868A2F95826}</x:author>
-    <x:author>tc={5362AA48-E0BF-4B27-6BFF-54D0DEDB7AE8}</x:author>
-    <x:author>tc={3831B5BD-3244-FA9B-D90E-2023EACB683C}</x:author>
+    <x:author>tc={B01406AF-5C54-1385-E93F-8BC31DCEF046}</x:author>
+    <x:author>tc={6DD7D282-4D5B-6CEA-034D-91D0362B1489}</x:author>
+    <x:author>tc={B744CA31-60A8-7C0A-67C6-4F7042734E04}</x:author>
+    <x:author>tc={2CBFDB07-DAC4-1F7C-80B7-A9AE350E67F7}</x:author>
+    <x:author>tc={C6FFBF76-75E5-A885-90FC-7A4822669D85}</x:author>
+    <x:author>tc={48B6FC78-C54C-A341-9A8A-BAE4F532FF12}</x:author>
+    <x:author>tc={40834F88-B44F-30F0-0C1E-7A7EA53D4250}</x:author>
+    <x:author>tc={8C86F84D-BA29-E3DB-77BF-71A0444405B8}</x:author>
+    <x:author>tc={E119E111-72FF-3D54-C250-0ADC5886F9C3}</x:author>
+    <x:author>tc={82842CDD-4566-2F54-CBEE-B39CF6B61B97}</x:author>
+    <x:author>tc={87E8F4DE-0F6B-C100-170D-96C85EA2694F}</x:author>
+    <x:author>tc={327772B5-06F7-BF98-168C-1F90F7D50CBB}</x:author>
+    <x:author>tc={36BE7540-24E4-876F-B0E7-5753CB3F9B1F}</x:author>
+    <x:author>tc={3977E859-D6B3-767C-5E5F-B7BC8DA6835F}</x:author>
+    <x:author>tc={0EEA68E2-7763-CC47-F71C-8F260986727F}</x:author>
+    <x:author>tc={2E5078F9-9194-8A06-23A5-2ACD828EBE10}</x:author>
+    <x:author>tc={7D7BDFB5-CE3D-259A-6186-A2557641EECC}</x:author>
+    <x:author>tc={E14E0F78-126D-771B-A1F2-85F72686862D}</x:author>
+    <x:author>tc={9669977D-6EF4-2826-924E-2C0BB9D74365}</x:author>
+    <x:author>tc={0D86104F-0064-7B27-F768-D1C5A87ABBBB}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="J5" authorId="0">
@@ -2060,7 +2060,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb2a91248ccaa4d79"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9c3b9377a8c64228"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2071,7 +2071,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}"/>
+  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}"/>
 </xltc:personList>
 </file>
 
@@ -2268,493 +2268,493 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="P5" dT="2026-08-15T06:47:05.396" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{D7179BD9-5380-A2BE-37A2-542620D11FD6}">
+  <xltc:threadedComment ref="P5" dT="2026-08-15T06:51:35.606" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{0AF4FEDA-AC03-3F9A-4677-E614750C0BE6}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P6" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{F5D5EA40-9C27-8916-42CA-9F80A998B239}">
+  <xltc:threadedComment ref="P6" dT="2026-08-15T06:51:35.608" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{7B13601B-A686-D1F6-E2C3-2DEAACC41826}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P7" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{F4A30194-1A72-1C1B-D3D1-88F0876A8B1C}">
+  <xltc:threadedComment ref="P7" dT="2026-08-15T06:51:35.608" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{10B9DE82-DAAF-597E-4424-E67283E9A4F8}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P8" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{058CC015-9E61-4F60-3707-3AA969865D33}">
+  <xltc:threadedComment ref="P8" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9DDF9D19-AAB7-35C6-6EAB-ADE447886907}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P9" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{0EA9266E-93A4-B7F3-00BA-8A7A79DFC82B}">
+  <xltc:threadedComment ref="P9" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{CEC6EDDA-4333-DE39-19A1-CD6C28B0071E}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P10" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{E0C25A1B-6CEF-EF90-AC34-65B59EB516C3}">
+  <xltc:threadedComment ref="P10" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9E0A3C03-F7F7-40B8-594C-1134A321AF12}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 119
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P11" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{D3577678-9795-3AEE-F6E6-5B7E42106D9E}">
+  <xltc:threadedComment ref="P11" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{6A469CC5-9E84-42E7-A4A2-5046B5EB797A}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 160
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P12" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{741168DD-C778-7C15-2B65-17B7C07ED33D}">
+  <xltc:threadedComment ref="P12" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{49F38930-D4FC-9148-B4AB-7B8868A6B1C4}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P13" dT="2026-08-15T06:47:05.399" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{95736628-F1F7-FE17-043B-CA174AE01EDE}">
+  <xltc:threadedComment ref="P13" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{6AE471B8-00A6-D8CA-E30E-F2F43B242CB2}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P14" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{829B1B69-69D1-E6CE-9B21-D90E9F236E79}">
+  <xltc:threadedComment ref="P14" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{070A3F26-F4D3-3501-5B26-B76E24181EE6}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P15" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{E10C328C-B958-A22D-795B-86894E174992}">
+  <xltc:threadedComment ref="P15" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{DB4AA7DC-83F7-AA9C-6650-AC0FBB081C37}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P16" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{275B946E-B475-F338-1312-E8A66EEE3FB6}">
+  <xltc:threadedComment ref="P16" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{E8A6B8CE-ACDD-0EA3-3036-3FEA4BE387E5}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P17" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{25671AA7-6F50-28BD-184D-157B185AC6A1}">
+  <xltc:threadedComment ref="P17" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{F5132FA4-62BD-C63C-B25A-A7E1FE946B04}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P18" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{7A90692C-D081-3F82-41F4-9D743B5AB740}">
+  <xltc:threadedComment ref="P18" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{924A75EC-79F9-BE2D-03E1-123D59F3BF71}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P19" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{4027D3F6-5103-811E-9867-0F88B7313B4E}">
+  <xltc:threadedComment ref="P19" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{7DFAAAEE-9F37-70B4-1295-82F48891DA0C}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P20" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{5452B241-D82F-7E23-08FB-0FF6597AF014}">
+  <xltc:threadedComment ref="P20" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{E2EA446D-49CF-67B3-25D3-448163193339}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 138
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P21" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{846887CC-6779-2558-F219-69B7F4C9101A}">
+  <xltc:threadedComment ref="P21" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{130AC7D8-E99A-FB9E-EC90-C0CC209F65EE}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 212
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P22" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{4F0D7BAC-731A-10AB-17F0-CF67BEA1E0C5}">
+  <xltc:threadedComment ref="P22" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{DFEDA6A7-98B9-D90B-F8E4-87463C1ABE71}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P23" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{71806FB6-0323-8EF2-734E-695EBE8E5C19}">
+  <xltc:threadedComment ref="P23" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{F908D626-E856-7A2E-B578-6FFFAF10A067}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P24" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{8C6DD087-476A-4C57-960D-E2895732691A}">
+  <xltc:threadedComment ref="P24" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{4691BC9F-FA65-4FBB-BE88-C3485B37BF5B}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P25" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{B47EBC4F-9B31-E559-6ED9-AAC1C334946A}">
+  <xltc:threadedComment ref="P25" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{54D1659D-A9A9-797D-09FE-9CCD3046EB3B}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P26" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{58727869-8ACA-389D-CD7D-8FBA1F5DE493}">
+  <xltc:threadedComment ref="P26" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{32021335-239B-D7CF-C593-02492073755E}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P27" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{62B5311B-9855-6101-F68A-04824B833B3D}">
+  <xltc:threadedComment ref="P27" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2D4C52F2-DF0E-98A8-DBAD-465EFEA6430C}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 272
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P28" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{BBE37CF9-417B-8492-B4BC-F67A0FB38F22}">
+  <xltc:threadedComment ref="P28" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{4F673CEB-0DB2-16EC-1BF9-E9916FC0D89C}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P29" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{11CAB389-76D8-7602-E738-77CB6C823411}">
+  <xltc:threadedComment ref="P29" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{8C766CE4-DCA4-0227-2719-EC43FBE4EB3E}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P30" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{53C4CB1B-0E8D-3634-8EB7-DFF2141C14F3}">
+  <xltc:threadedComment ref="P30" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{030B07FB-3D16-4698-B4D5-9BFD808ED081}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 158
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P31" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{52C4F871-DAB1-FC43-B689-E83208D5BDC2}">
+  <xltc:threadedComment ref="P31" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{BB835A0A-AC15-BD40-37D2-BB2D5D7D1A29}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P32" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{5A8F28C0-DCAF-9B4F-60C2-B5519288078D}">
+  <xltc:threadedComment ref="P32" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{ACE1C8E0-F10B-F24B-C4C3-09990BA1EAF5}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P33" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{BC440591-751F-ADDA-3E20-D28B53716826}">
+  <xltc:threadedComment ref="P33" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{89E2F11B-ECCC-3429-226F-74770117AB92}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 72
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P34" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{129D4D19-7FD2-1FAB-C3F2-3D85C2143407}">
+  <xltc:threadedComment ref="P34" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{FE94A6DE-84F6-0201-3EFF-69B3D6B7D622}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P35" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{C00BE146-1A1C-DE84-6CEC-66E28A34FB62}">
+  <xltc:threadedComment ref="P35" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{5FADB78B-442A-2857-7CCC-D525C440BCCF}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P36" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{B2453065-6EF2-25EE-C743-1AF12D44A7E2}">
+  <xltc:threadedComment ref="P36" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{33238565-3127-12AD-ACAF-5A83E4E3101E}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 24
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P37" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{42F5722C-BA58-306D-7716-E7DB46B06E1C}">
+  <xltc:threadedComment ref="P37" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{DBA819E1-2CFB-40C0-8E60-4EBBB4963742}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P38" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{308E1DA8-4C3B-C720-C61A-B4FD5B863D5A}">
+  <xltc:threadedComment ref="P38" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{831BC617-DC59-E847-0D3A-95946FD8D988}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P39" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{575A735C-1490-C525-7FDA-D0D6CC2167F3}">
+  <xltc:threadedComment ref="P39" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9625D7E8-9A23-1EEE-66C1-3D1F41528532}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 19
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P40" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{F04ECB4C-E296-D7B7-16F0-976919B7E452}">
+  <xltc:threadedComment ref="P40" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{36A13555-305E-B2C5-2B7A-87476C5BA766}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P41" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{890C7111-93D9-523E-D457-71A4254BA046}">
+  <xltc:threadedComment ref="P41" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{69541CEA-6E11-BC48-6898-36AE3D548AB4}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P42" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{73A6DDDE-3DDB-F0A0-8427-697A1F7CA9D6}">
+  <xltc:threadedComment ref="P42" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{12AFE746-FDD9-963F-DCFD-DC968D22FFA6}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P43" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{F8EC0B12-3474-AF0F-5A97-A40007A76C72}">
+  <xltc:threadedComment ref="P43" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{425C83BD-D4DC-BDED-071D-487523F8AC3F}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P44" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{835BEA1E-53F0-17E6-E7D7-DBD14ED53706}">
+  <xltc:threadedComment ref="P44" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2D72A011-0216-7D35-09A3-D704E88BAEE3}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P45" dT="2026-08-15T06:47:05.4" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{CA531C19-FD45-25C9-0D70-197E1279C769}">
+  <xltc:threadedComment ref="P45" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{86FBCAB8-88A0-F97B-4FA1-13C4BEAA369D}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P46" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{8774F1F6-5214-2114-2D61-8456D5360289}">
+  <xltc:threadedComment ref="P46" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9185AC7C-5FA5-8BAE-5D74-F86F31883FC5}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P47" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{30902EAC-5720-96A7-8284-3D2CCAB7443B}">
+  <xltc:threadedComment ref="P47" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{8F348568-9728-931E-D9B2-061F382ED13A}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P48" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{0CB4A533-3016-5908-0FCF-23076D4239A8}">
+  <xltc:threadedComment ref="P48" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{E5746BEC-90A8-ABA0-16B5-A6A9F11A2C96}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P49" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{E740C3D1-D9F7-5D7D-AFF3-68BEEEF5AFB6}">
+  <xltc:threadedComment ref="P49" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{4B1E6C62-4809-1469-5784-9EA7A65F2E2D}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 118
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P50" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{F69FF8B4-C804-AEE4-CB67-276CB58FECC3}">
+  <xltc:threadedComment ref="P50" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{271EEFA8-492B-5EC5-67E3-8B28D1AE9871}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P51" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{C43B89C3-9376-EAD3-76C9-17647D15CCF5}">
+  <xltc:threadedComment ref="P51" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{3430FD27-2DAA-4633-A322-0688F2FCD467}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P52" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{E454CB3F-C1C8-45BE-B525-60EFF4CDE1A6}">
+  <xltc:threadedComment ref="P52" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{8D7DF3C9-36A9-2E8C-6160-11B116238A97}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P53" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{676951D3-752E-15EF-F207-A9C4AD907FBD}">
+  <xltc:threadedComment ref="P53" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{31933AFB-CA47-471A-E7EB-D7E5B693D87A}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-STF</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P54" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{B43928D3-C753-0831-5261-410F7BBF0732}">
+  <xltc:threadedComment ref="P54" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{CEB8E96A-F9CE-D6E4-1345-25BEA6D4853C}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P55" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{7AEC7DF7-C2FC-5FD1-43E7-E31427E0CB4D}">
+  <xltc:threadedComment ref="P55" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{CE8B63E6-EC70-4885-EBBF-C61B84B9BD02}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P56" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{483F7CB9-A550-4C88-F30A-79F3465B8236}">
+  <xltc:threadedComment ref="P56" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{1236AB2A-50DD-58C5-F0CF-0A77396ECCB9}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 18
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P57" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{57E4D7D6-EAC9-3255-FC08-228D23302E84}">
+  <xltc:threadedComment ref="P57" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{23B809AB-666E-3843-AA8B-2E06C9D6735C}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P58" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{63285F2A-DBA1-0A5B-0BD2-5CF8872592B7}">
+  <xltc:threadedComment ref="P58" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{F9218197-D7D7-96FC-5DEE-19E1B89C6668}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P59" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{5E490997-C386-5F07-4415-3BF718F6583D}">
+  <xltc:threadedComment ref="P59" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{49C564EF-C6E1-AA3E-BAE6-F9B6B7DAF702}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P60" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{530EEE62-CA06-D2AD-47F5-B427C42F71A7}">
+  <xltc:threadedComment ref="P60" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{6A34B57F-09E3-5DA4-9CDF-BDD9AFC15C62}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P61" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{D3192F1B-D4AE-761E-78F3-B7200E4D78DD}">
+  <xltc:threadedComment ref="P61" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{EA67CC0C-3B7B-6001-4E9C-C907CB9A2E41}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P62" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{5ECB39A3-6CD9-BC08-DE2C-8BC987C1390A}">
+  <xltc:threadedComment ref="P62" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2C705125-9621-DC7B-9356-1AFFFB014183}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P63" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{83C028C4-B49A-845A-F950-45971513DB9D}">
+  <xltc:threadedComment ref="P63" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{4127462E-7049-10C8-6E6D-2726FCAFA040}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P64" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{14DD0686-1E74-4983-CD5F-91C8010BF879}">
+  <xltc:threadedComment ref="P64" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{DDC7860C-4BF8-FE8E-AB94-BF36F51E4742}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P65" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{42144CB2-40A1-FE82-EC8C-D7B918D43B31}">
+  <xltc:threadedComment ref="P65" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{355CD349-BEF2-1F91-3717-B7779FC267B7}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 311
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P66" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{175AC13F-5A05-534D-C6C5-368C220513B3}">
+  <xltc:threadedComment ref="P66" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{BE707954-D4F8-3036-E784-0F6EF373E3B1}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P67" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{98B1FE03-8508-60EB-FB28-AC6EB4FF17EC}">
+  <xltc:threadedComment ref="P67" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{30C17E09-F415-E5D5-1412-983D6592AE59}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P68" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{CA1C4C92-831F-ADC4-1168-DE41412AB513}">
+  <xltc:threadedComment ref="P68" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{946D1FE7-F4AA-6563-A358-3F55219C3AED}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 141
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P69" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{66D08A53-A46F-B39D-BF8B-2F91FA5544EC}">
+  <xltc:threadedComment ref="P69" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{FF9DEADC-5F2B-2C71-0EDD-31A65A1DAC80}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P70" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{8253EE86-7926-8F10-8D36-CD8E983846E3}">
+  <xltc:threadedComment ref="P70" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{99FA21E2-86C5-2A76-2880-8215954AA3D4}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P71" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{63C5B54E-3382-3032-03BC-A4D566E81015}">
+  <xltc:threadedComment ref="P71" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{901E21A1-49DD-A0DA-0A10-1EDE8076C1B3}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 33
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P72" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{19946973-1CB9-F97A-932A-4CDC93DA4076}">
+  <xltc:threadedComment ref="P72" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{FCB3C38E-B0AF-A412-700D-4D9A9D2C2741}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P73" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{502F2BD0-069C-A1CB-BE2A-316524EA0FE7}">
+  <xltc:threadedComment ref="P73" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9382A565-2A1D-550E-54B1-678F98943EC6}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P74" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{8D3E5E07-996C-6FA2-B7D2-F0A38B3ECA78}">
+  <xltc:threadedComment ref="P74" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{40576489-4A24-6AA0-06F2-24F75770098B}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 21
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P75" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{8E3F859E-A8E6-CD0C-796D-3ABA463D042C}">
+  <xltc:threadedComment ref="P75" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{D80EF366-6BBD-D5AC-E71F-5666ED857ED8}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P76" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{7598B2B6-A8FF-7FC1-B339-88714951EF7C}">
+  <xltc:threadedComment ref="P76" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{8E28E375-5E9B-B43C-02D8-1D69B6DBCCB7}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P77" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{C5D97150-6CE8-0ED7-9C73-F66D04986243}">
+  <xltc:threadedComment ref="P77" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{C52D303F-E26F-AEB2-82AD-C196257D053A}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 19
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P78" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{18CF715D-516E-7251-B463-8CC3AF4028CF}">
+  <xltc:threadedComment ref="P78" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{AD3CBF1C-654B-022F-1CCE-E3B6B02846E3}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 43
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P79" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{75B47754-69C2-3985-00C8-8438A73DE06D}">
+  <xltc:threadedComment ref="P79" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2EEF0622-B8D5-960E-069D-57BC28C46AE4}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 44
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P80" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{F799C9D6-E29B-DA0B-A2F7-63ADB832072B}">
+  <xltc:threadedComment ref="P80" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{C7A17400-8C3D-04F3-BB45-75623A8D8379}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 40
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P81" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{2387B878-7100-9F16-32DA-86297144DD8C}">
+  <xltc:threadedComment ref="P81" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9CB15BCB-A81F-4C51-B6D7-CA70F830A75F}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P82" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{059C83C8-6D8C-66EA-6ABF-D9624BFBCF3A}">
+  <xltc:threadedComment ref="P82" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9CDE5188-52E3-BEBE-AC4D-8F98AC717AA6}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P83" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{63C2F3AB-4FB1-6250-E0A7-BE401E20C4CB}">
+  <xltc:threadedComment ref="P83" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{96D773F7-6FC9-4DF1-46BC-3C5A65EBE44A}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 16
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P84" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{162FEE63-E7EE-3E1C-C9D1-370CE352712E}">
+  <xltc:threadedComment ref="P84" dT="2026-08-15T06:51:35.612" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{69BF4FC0-9856-F2BC-F517-9DC02348AB96}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P85" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{E1DE05A5-76A2-0262-A273-87EDC9B8395D}">
+  <xltc:threadedComment ref="P85" dT="2026-08-15T06:51:35.612" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{EF1A8A33-3E41-8002-8157-23C7596AF4CA}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P86" dT="2026-08-15T06:47:05.401" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{EEA21B70-769F-D42F-BB3B-483AAC8DA47C}">
+  <xltc:threadedComment ref="P86" dT="2026-08-15T06:51:35.612" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{CBA415B4-31A9-6F43-882D-D511ADAA6836}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 21
 Available: 2026-02-25
@@ -2765,64 +2765,64 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="J5" dT="2026-08-15T06:47:05.762" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{84E13648-C7F0-652B-D6D1-50FB9ABCAD46}">
+  <xltc:threadedComment ref="J5" dT="2026-08-15T06:51:36.013" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{B01406AF-5C54-1385-E93F-8BC31DCEF046}">
     <xltc:text>Official source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J6" dT="2026-08-15T06:47:05.764" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{BAE23548-9F72-6653-9CCE-AB5D6CE12D22}">
+  <xltc:threadedComment ref="J6" dT="2026-08-15T06:51:36.015" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{6DD7D282-4D5B-6CEA-034D-91D0362B1489}">
     <xltc:text>Official source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J7" dT="2026-08-15T06:47:05.766" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{7F7FC2C5-35C0-7E18-21CF-E7ABD151C178}">
+  <xltc:threadedComment ref="J7" dT="2026-08-15T06:51:36.019" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{B744CA31-60A8-7C0A-67C6-4F7042734E04}">
     <xltc:text>Official source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J8" dT="2026-08-15T06:47:05.768" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{1C87D2BD-002E-EFEC-6449-F4CC621DAF19}">
+  <xltc:threadedComment ref="J8" dT="2026-08-15T06:51:36.022" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2CBFDB07-DAC4-1F7C-80B7-A9AE350E67F7}">
     <xltc:text>Official source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J9" dT="2026-08-15T06:47:05.771" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{D82E1942-60FB-A94F-1231-55C186DFE77A}">
+  <xltc:threadedComment ref="J9" dT="2026-08-15T06:51:36.025" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{C6FFBF76-75E5-A885-90FC-7A4822669D85}">
     <xltc:text>Official source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J10" dT="2026-08-15T06:47:05.774" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{8C7CBC23-095B-389F-1CE9-66A020ED5F65}">
+  <xltc:threadedComment ref="J10" dT="2026-08-15T06:51:36.029" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{48B6FC78-C54C-A341-9A8A-BAE4F532FF12}">
     <xltc:text>Official source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J11" dT="2026-08-15T06:47:05.776" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{FE08B92E-A8FF-1755-3A77-7296DB082B8F}">
+  <xltc:threadedComment ref="J11" dT="2026-08-15T06:51:36.031" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{40834F88-B44F-30F0-0C1E-7A7EA53D4250}">
     <xltc:text>Official source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J12" dT="2026-08-15T06:47:05.778" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{17E4C51A-99FC-A26E-FA58-241D1896C185}">
+  <xltc:threadedComment ref="J12" dT="2026-08-15T06:51:36.033" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{8C86F84D-BA29-E3DB-77BF-71A0444405B8}">
     <xltc:text>Official source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J13" dT="2026-08-15T06:47:05.779" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{EB6DCDB8-08F5-2F6B-58D9-D67FEBC4BF08}">
+  <xltc:threadedComment ref="J13" dT="2026-08-15T06:51:36.035" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{E119E111-72FF-3D54-C250-0ADC5886F9C3}">
     <xltc:text>Official source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J14" dT="2026-08-15T06:47:05.782" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{D1283C43-349C-5B77-B9BC-15E4F74CDBF7}">
+  <xltc:threadedComment ref="J14" dT="2026-08-15T06:51:36.038" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{82842CDD-4566-2F54-CBEE-B39CF6B61B97}">
     <xltc:text>Official source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J15" dT="2026-08-15T06:47:05.784" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{22CEF8D1-497B-0746-E712-0902C2295F03}">
+  <xltc:threadedComment ref="J15" dT="2026-08-15T06:51:36.041" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{87E8F4DE-0F6B-C100-170D-96C85EA2694F}">
     <xltc:text>Official source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J16" dT="2026-08-15T06:47:05.786" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{80D5AC2B-9FE7-A4E9-D58C-4B8B483C5C5C}">
+  <xltc:threadedComment ref="J16" dT="2026-08-15T06:51:36.043" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{327772B5-06F7-BF98-168C-1F90F7D50CBB}">
     <xltc:text>Official source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J17" dT="2026-08-15T06:47:05.787" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{335B0CFE-336B-8BFF-E374-338B849103E5}">
+  <xltc:threadedComment ref="J17" dT="2026-08-15T06:51:36.045" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{36BE7540-24E4-876F-B0E7-5753CB3F9B1F}">
     <xltc:text>Official source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J18" dT="2026-08-15T06:47:05.79" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{1A55DFCA-C281-6722-8F99-5EBA993935F7}">
+  <xltc:threadedComment ref="J18" dT="2026-08-15T06:51:36.047" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{3977E859-D6B3-767C-5E5F-B7BC8DA6835F}">
     <xltc:text>Official source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J19" dT="2026-08-15T06:47:05.795" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{ED05C87E-0A75-049A-05E7-96420E3A1BAD}">
+  <xltc:threadedComment ref="J19" dT="2026-08-15T06:51:36.048" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{0EEA68E2-7763-CC47-F71C-8F260986727F}">
     <xltc:text>Official source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J20" dT="2026-08-15T06:47:05.797" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{5CCA1910-7668-C27B-F4A8-D382B08AB157}">
+  <xltc:threadedComment ref="J20" dT="2026-08-15T06:51:36.054" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2E5078F9-9194-8A06-23A5-2ACD828EBE10}">
     <xltc:text>Official source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J21" dT="2026-08-15T06:47:05.798" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{66930877-5ABE-EA1E-A91D-1E239C1A010D}">
+  <xltc:threadedComment ref="J21" dT="2026-08-15T06:51:36.057" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{7D7BDFB5-CE3D-259A-6186-A2557641EECC}">
     <xltc:text>Official source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J22" dT="2026-08-15T06:47:05.8" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{BA48A1C2-E567-A40A-25BB-8868A2F95826}">
+  <xltc:threadedComment ref="J22" dT="2026-08-15T06:51:36.059" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{E14E0F78-126D-771B-A1F2-85F72686862D}">
     <xltc:text>Official source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J23" dT="2026-08-15T06:47:05.801" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{5362AA48-E0BF-4B27-6BFF-54D0DEDB7AE8}">
+  <xltc:threadedComment ref="J23" dT="2026-08-15T06:51:36.061" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9669977D-6EF4-2826-924E-2C0BB9D74365}">
     <xltc:text>Official source: https://www.aspenpharma.com/download/annual-financial-statements-2/</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J24" dT="2026-08-15T06:47:05.803" personId="{1DABF6B7-B550-4FBD-B0D4-EE8D5BF268BF}" id="{3831B5BD-3244-FA9B-D90E-2023EACB683C}">
+  <xltc:threadedComment ref="J24" dT="2026-08-15T06:51:36.063" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{0D86104F-0064-7B27-F768-D1C5A87ABBBB}">
     <xltc:text>Official source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -3877,7 +3877,7 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f43e8fb0cb14fa4"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c7810c6b47b416f"/>
 </x:worksheet>
 </file>
 
@@ -8611,7 +8611,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc977ac405e143db"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc12e983b47534b1a"/>
 </x:worksheet>
 </file>
 
@@ -9671,7 +9671,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb88cdafbb43b432f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R458cac95bef44c85"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Refresh V3.2 judging artifacts
</commit_message>
<xml_diff>
--- a/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
+++ b/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R380f9c27d3944774"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="Rfffcb405ec464c1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="R48c193a887c4416e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Rd66998ed3cc04402"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R49c40c130e0d45ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R631bd8a5e6674ca9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Rde69964a6bf84944"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="R858c58fbb73144bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="Rf02af7084cc44489"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R85030ef8203c4a51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rcb2c4e1a55b942b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R1862c38eec4f4fd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="Rff96f59aa3c04679"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="R1583a0a66d6b4d3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R892f299ff0ed4564"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="Rb12c3646ad1d4600"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Re458eca1bce74f85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="Rfded105b212a4b17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R2f52fd7a8ac94db2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R97807c487b9a4e4b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,88 +19,88 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={0AF4FEDA-AC03-3F9A-4677-E614750C0BE6}</x:author>
-    <x:author>tc={7B13601B-A686-D1F6-E2C3-2DEAACC41826}</x:author>
-    <x:author>tc={10B9DE82-DAAF-597E-4424-E67283E9A4F8}</x:author>
-    <x:author>tc={9DDF9D19-AAB7-35C6-6EAB-ADE447886907}</x:author>
-    <x:author>tc={CEC6EDDA-4333-DE39-19A1-CD6C28B0071E}</x:author>
-    <x:author>tc={9E0A3C03-F7F7-40B8-594C-1134A321AF12}</x:author>
-    <x:author>tc={6A469CC5-9E84-42E7-A4A2-5046B5EB797A}</x:author>
-    <x:author>tc={49F38930-D4FC-9148-B4AB-7B8868A6B1C4}</x:author>
-    <x:author>tc={6AE471B8-00A6-D8CA-E30E-F2F43B242CB2}</x:author>
-    <x:author>tc={070A3F26-F4D3-3501-5B26-B76E24181EE6}</x:author>
-    <x:author>tc={DB4AA7DC-83F7-AA9C-6650-AC0FBB081C37}</x:author>
-    <x:author>tc={E8A6B8CE-ACDD-0EA3-3036-3FEA4BE387E5}</x:author>
-    <x:author>tc={F5132FA4-62BD-C63C-B25A-A7E1FE946B04}</x:author>
-    <x:author>tc={924A75EC-79F9-BE2D-03E1-123D59F3BF71}</x:author>
-    <x:author>tc={7DFAAAEE-9F37-70B4-1295-82F48891DA0C}</x:author>
-    <x:author>tc={E2EA446D-49CF-67B3-25D3-448163193339}</x:author>
-    <x:author>tc={130AC7D8-E99A-FB9E-EC90-C0CC209F65EE}</x:author>
-    <x:author>tc={DFEDA6A7-98B9-D90B-F8E4-87463C1ABE71}</x:author>
-    <x:author>tc={F908D626-E856-7A2E-B578-6FFFAF10A067}</x:author>
-    <x:author>tc={4691BC9F-FA65-4FBB-BE88-C3485B37BF5B}</x:author>
-    <x:author>tc={54D1659D-A9A9-797D-09FE-9CCD3046EB3B}</x:author>
-    <x:author>tc={32021335-239B-D7CF-C593-02492073755E}</x:author>
-    <x:author>tc={2D4C52F2-DF0E-98A8-DBAD-465EFEA6430C}</x:author>
-    <x:author>tc={4F673CEB-0DB2-16EC-1BF9-E9916FC0D89C}</x:author>
-    <x:author>tc={8C766CE4-DCA4-0227-2719-EC43FBE4EB3E}</x:author>
-    <x:author>tc={030B07FB-3D16-4698-B4D5-9BFD808ED081}</x:author>
-    <x:author>tc={BB835A0A-AC15-BD40-37D2-BB2D5D7D1A29}</x:author>
-    <x:author>tc={ACE1C8E0-F10B-F24B-C4C3-09990BA1EAF5}</x:author>
-    <x:author>tc={89E2F11B-ECCC-3429-226F-74770117AB92}</x:author>
-    <x:author>tc={FE94A6DE-84F6-0201-3EFF-69B3D6B7D622}</x:author>
-    <x:author>tc={5FADB78B-442A-2857-7CCC-D525C440BCCF}</x:author>
-    <x:author>tc={33238565-3127-12AD-ACAF-5A83E4E3101E}</x:author>
-    <x:author>tc={DBA819E1-2CFB-40C0-8E60-4EBBB4963742}</x:author>
-    <x:author>tc={831BC617-DC59-E847-0D3A-95946FD8D988}</x:author>
-    <x:author>tc={9625D7E8-9A23-1EEE-66C1-3D1F41528532}</x:author>
-    <x:author>tc={36A13555-305E-B2C5-2B7A-87476C5BA766}</x:author>
-    <x:author>tc={69541CEA-6E11-BC48-6898-36AE3D548AB4}</x:author>
-    <x:author>tc={12AFE746-FDD9-963F-DCFD-DC968D22FFA6}</x:author>
-    <x:author>tc={425C83BD-D4DC-BDED-071D-487523F8AC3F}</x:author>
-    <x:author>tc={2D72A011-0216-7D35-09A3-D704E88BAEE3}</x:author>
-    <x:author>tc={86FBCAB8-88A0-F97B-4FA1-13C4BEAA369D}</x:author>
-    <x:author>tc={9185AC7C-5FA5-8BAE-5D74-F86F31883FC5}</x:author>
-    <x:author>tc={8F348568-9728-931E-D9B2-061F382ED13A}</x:author>
-    <x:author>tc={E5746BEC-90A8-ABA0-16B5-A6A9F11A2C96}</x:author>
-    <x:author>tc={4B1E6C62-4809-1469-5784-9EA7A65F2E2D}</x:author>
-    <x:author>tc={271EEFA8-492B-5EC5-67E3-8B28D1AE9871}</x:author>
-    <x:author>tc={3430FD27-2DAA-4633-A322-0688F2FCD467}</x:author>
-    <x:author>tc={8D7DF3C9-36A9-2E8C-6160-11B116238A97}</x:author>
-    <x:author>tc={31933AFB-CA47-471A-E7EB-D7E5B693D87A}</x:author>
-    <x:author>tc={CEB8E96A-F9CE-D6E4-1345-25BEA6D4853C}</x:author>
-    <x:author>tc={CE8B63E6-EC70-4885-EBBF-C61B84B9BD02}</x:author>
-    <x:author>tc={1236AB2A-50DD-58C5-F0CF-0A77396ECCB9}</x:author>
-    <x:author>tc={23B809AB-666E-3843-AA8B-2E06C9D6735C}</x:author>
-    <x:author>tc={F9218197-D7D7-96FC-5DEE-19E1B89C6668}</x:author>
-    <x:author>tc={49C564EF-C6E1-AA3E-BAE6-F9B6B7DAF702}</x:author>
-    <x:author>tc={6A34B57F-09E3-5DA4-9CDF-BDD9AFC15C62}</x:author>
-    <x:author>tc={EA67CC0C-3B7B-6001-4E9C-C907CB9A2E41}</x:author>
-    <x:author>tc={2C705125-9621-DC7B-9356-1AFFFB014183}</x:author>
-    <x:author>tc={4127462E-7049-10C8-6E6D-2726FCAFA040}</x:author>
-    <x:author>tc={DDC7860C-4BF8-FE8E-AB94-BF36F51E4742}</x:author>
-    <x:author>tc={355CD349-BEF2-1F91-3717-B7779FC267B7}</x:author>
-    <x:author>tc={BE707954-D4F8-3036-E784-0F6EF373E3B1}</x:author>
-    <x:author>tc={30C17E09-F415-E5D5-1412-983D6592AE59}</x:author>
-    <x:author>tc={946D1FE7-F4AA-6563-A358-3F55219C3AED}</x:author>
-    <x:author>tc={FF9DEADC-5F2B-2C71-0EDD-31A65A1DAC80}</x:author>
-    <x:author>tc={99FA21E2-86C5-2A76-2880-8215954AA3D4}</x:author>
-    <x:author>tc={901E21A1-49DD-A0DA-0A10-1EDE8076C1B3}</x:author>
-    <x:author>tc={FCB3C38E-B0AF-A412-700D-4D9A9D2C2741}</x:author>
-    <x:author>tc={9382A565-2A1D-550E-54B1-678F98943EC6}</x:author>
-    <x:author>tc={40576489-4A24-6AA0-06F2-24F75770098B}</x:author>
-    <x:author>tc={D80EF366-6BBD-D5AC-E71F-5666ED857ED8}</x:author>
-    <x:author>tc={8E28E375-5E9B-B43C-02D8-1D69B6DBCCB7}</x:author>
-    <x:author>tc={C52D303F-E26F-AEB2-82AD-C196257D053A}</x:author>
-    <x:author>tc={AD3CBF1C-654B-022F-1CCE-E3B6B02846E3}</x:author>
-    <x:author>tc={2EEF0622-B8D5-960E-069D-57BC28C46AE4}</x:author>
-    <x:author>tc={C7A17400-8C3D-04F3-BB45-75623A8D8379}</x:author>
-    <x:author>tc={9CB15BCB-A81F-4C51-B6D7-CA70F830A75F}</x:author>
-    <x:author>tc={9CDE5188-52E3-BEBE-AC4D-8F98AC717AA6}</x:author>
-    <x:author>tc={96D773F7-6FC9-4DF1-46BC-3C5A65EBE44A}</x:author>
-    <x:author>tc={69BF4FC0-9856-F2BC-F517-9DC02348AB96}</x:author>
-    <x:author>tc={EF1A8A33-3E41-8002-8157-23C7596AF4CA}</x:author>
-    <x:author>tc={CBA415B4-31A9-6F43-882D-D511ADAA6836}</x:author>
+    <x:author>tc={B010C51E-1279-1014-33BC-2602466A0653}</x:author>
+    <x:author>tc={C1FCCBE0-DA45-F004-62DE-931492BB7B55}</x:author>
+    <x:author>tc={AC4872FE-E925-0F71-A1A0-B51C3BE471D4}</x:author>
+    <x:author>tc={78456A9C-33CF-DC3E-ACC9-771E9401AB46}</x:author>
+    <x:author>tc={A3652911-0C8B-2C28-FADE-73D328A5BF26}</x:author>
+    <x:author>tc={6F2EBCD8-23F2-D22F-38CC-ED40EFF8AEC8}</x:author>
+    <x:author>tc={92F20AFD-1D39-B8DE-5BD9-BC3E03CB8C0F}</x:author>
+    <x:author>tc={CA2CD762-5110-A555-E40D-9C5F0FB6D9CC}</x:author>
+    <x:author>tc={9DAD665B-4B78-CB05-6BFF-8A259A25099D}</x:author>
+    <x:author>tc={B404A4C9-0C5D-FB04-5F38-B466A0729AB3}</x:author>
+    <x:author>tc={A778AC8E-E3EE-EF95-340F-71DE58C4379A}</x:author>
+    <x:author>tc={CF9789CE-401E-9368-3823-F3D6EB9FB0AE}</x:author>
+    <x:author>tc={E0F7EB04-9E7A-C956-F66F-04924C0BBF6B}</x:author>
+    <x:author>tc={432D59DF-0456-250E-3705-7E52A846CC07}</x:author>
+    <x:author>tc={8E40EC39-F650-2BB9-AA8A-B164C8F0D6DB}</x:author>
+    <x:author>tc={06B31F52-AE05-C750-E2E4-8BE8C077E3ED}</x:author>
+    <x:author>tc={C4AB3B82-976E-0559-3794-2F2F9216C552}</x:author>
+    <x:author>tc={3AAB5A1B-8E7D-C179-2DC1-E2DBD2705DB9}</x:author>
+    <x:author>tc={7D66F2E6-7D62-9517-832E-57FFAA140850}</x:author>
+    <x:author>tc={01EA68F6-A6AF-EEF9-FC79-C83DFF706D5F}</x:author>
+    <x:author>tc={7EBEBBB5-1D36-3EC8-8615-2492FBE68CC4}</x:author>
+    <x:author>tc={67EA088D-22B9-ECEE-A157-D88A9B7AAFA9}</x:author>
+    <x:author>tc={A2333FE9-49D5-C016-953E-7E0B47F95EF5}</x:author>
+    <x:author>tc={93C06E00-D895-402F-7E27-987889902425}</x:author>
+    <x:author>tc={AEE536DF-8184-66AA-DD13-2B4E3E8B93C2}</x:author>
+    <x:author>tc={5997CBC9-B8DA-7AF8-6285-53F3711B14B9}</x:author>
+    <x:author>tc={626792A5-658D-324B-98D1-7D4E6DE536BD}</x:author>
+    <x:author>tc={8D7BFCFD-3E48-D195-6EB4-5521380E05C9}</x:author>
+    <x:author>tc={E15B3E52-7A06-CC45-DE2B-41A9C12FF48D}</x:author>
+    <x:author>tc={B960910A-8477-2846-1613-88C2913E5C85}</x:author>
+    <x:author>tc={3F019C8B-A8FF-A1C1-F480-A723F813C270}</x:author>
+    <x:author>tc={8B0451A6-6D51-3B85-B608-44D73A90BE00}</x:author>
+    <x:author>tc={6E34B664-AA4F-7D25-5EB4-CAE4F78D331D}</x:author>
+    <x:author>tc={B2D6B7C4-FB9F-7569-768C-9F19B0EDBA9D}</x:author>
+    <x:author>tc={F2C939C5-67DD-99B6-503C-636AE1C76D8C}</x:author>
+    <x:author>tc={091770E0-D8A8-A17E-211F-BF39D2DE3D21}</x:author>
+    <x:author>tc={C81BBC94-53F4-9708-39C3-5CB664703880}</x:author>
+    <x:author>tc={A06A1A63-4CF5-E445-56FC-BD4A588968F1}</x:author>
+    <x:author>tc={CF996379-C6D9-0FBB-656E-63B1D66BAFC8}</x:author>
+    <x:author>tc={B957E27C-1147-FAF3-74E7-EA8EC5908CC6}</x:author>
+    <x:author>tc={420E6EE9-F0FD-3EE6-7002-0F87931DE2C3}</x:author>
+    <x:author>tc={72E4C9A4-FDB4-C94D-DCDC-B2D8F3FC1E58}</x:author>
+    <x:author>tc={1CB140F6-0570-D58E-D0A8-4551FD74BA90}</x:author>
+    <x:author>tc={4C23F7C6-D3C7-A4BE-F36C-2F5E0923875B}</x:author>
+    <x:author>tc={A18D8527-4F44-6611-303D-A0E50FC512E3}</x:author>
+    <x:author>tc={DCF389D3-4242-623B-AE66-3E44891929C8}</x:author>
+    <x:author>tc={942E9BB5-C21B-6000-23BC-C0925210FA48}</x:author>
+    <x:author>tc={B8533D65-8426-863A-B312-F367AD0B4444}</x:author>
+    <x:author>tc={0886CFC9-D7DE-1471-513A-71A37582BE87}</x:author>
+    <x:author>tc={BCB573C2-22CD-DDD1-A5ED-1DC2F5CE50B5}</x:author>
+    <x:author>tc={E9D0B5CE-5209-E0BE-3237-DB8B632D7235}</x:author>
+    <x:author>tc={B704E177-02B4-47FB-A7F9-206D3C4F097F}</x:author>
+    <x:author>tc={6F3A1B45-FF5A-DF64-19ED-AA0695469814}</x:author>
+    <x:author>tc={ACCA67AD-3C83-ACC1-2D98-C4C6D0AFD638}</x:author>
+    <x:author>tc={B238E13A-91E5-5386-8C34-F67463D45FB1}</x:author>
+    <x:author>tc={C0BA2EF8-C1B1-64BE-3EA0-F77C4E23AD4C}</x:author>
+    <x:author>tc={9E7079E2-8399-4258-574A-B9F9C79E592C}</x:author>
+    <x:author>tc={4D4A8E67-5958-A3C1-70C2-33CB58A773FF}</x:author>
+    <x:author>tc={0CA8FE98-EDDA-A7FC-8A90-7852EAD6A4FF}</x:author>
+    <x:author>tc={C13917A4-524D-2A26-A42D-6D16A66166CA}</x:author>
+    <x:author>tc={C4039E66-57C0-F444-53E6-FCCF8A6DA3E9}</x:author>
+    <x:author>tc={03D96BF4-9AE3-9DF8-CC14-62B6DA87E1BA}</x:author>
+    <x:author>tc={68867B5D-2E79-11B5-AD2B-6426A7112DA5}</x:author>
+    <x:author>tc={54A9DCF0-8852-0B11-508D-950C7B9284A4}</x:author>
+    <x:author>tc={22D8A23D-9682-E3ED-C9FB-E779AA2720B1}</x:author>
+    <x:author>tc={91E699CE-9A06-219F-5833-E4E864BED089}</x:author>
+    <x:author>tc={F8EB5DB1-1D5C-47D0-D1DD-184B283C0C6C}</x:author>
+    <x:author>tc={6EF67E32-E7EC-94F6-3F4E-584F0BE95656}</x:author>
+    <x:author>tc={99F57B06-4D37-016A-C483-B1735DED682F}</x:author>
+    <x:author>tc={5D7317F8-C323-677A-8020-3361BEEEB812}</x:author>
+    <x:author>tc={513B22C5-53D5-D9FA-E2B0-84DC9C63BD75}</x:author>
+    <x:author>tc={C676EC9E-9A20-A1B2-3E1F-20A28A26A61A}</x:author>
+    <x:author>tc={BD7320DD-EB8C-3619-ABDC-27A23A838BFD}</x:author>
+    <x:author>tc={DCCE526A-71D7-E02C-4253-8778B920726E}</x:author>
+    <x:author>tc={33C6E653-4ECD-66D3-31ED-37F8D530BBCA}</x:author>
+    <x:author>tc={2D51D488-F2CD-1656-7FC5-C0BE0926F124}</x:author>
+    <x:author>tc={620305EA-1DAC-09F1-F096-0BEF7B4B8CA1}</x:author>
+    <x:author>tc={E5082642-40DD-D305-F257-8AEF1B0F3468}</x:author>
+    <x:author>tc={A227902C-BE3D-E28E-3D70-D78E36E76664}</x:author>
+    <x:author>tc={8DC1750F-5595-5639-B653-027050CAA390}</x:author>
+    <x:author>tc={DD3E8D93-9C02-6410-C382-7C25C24F3F42}</x:author>
+    <x:author>tc={83154AE6-98B5-8AE9-06F0-2B1446B9C581}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="P5" authorId="0">
@@ -1176,26 +1176,26 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={B01406AF-5C54-1385-E93F-8BC31DCEF046}</x:author>
-    <x:author>tc={6DD7D282-4D5B-6CEA-034D-91D0362B1489}</x:author>
-    <x:author>tc={B744CA31-60A8-7C0A-67C6-4F7042734E04}</x:author>
-    <x:author>tc={2CBFDB07-DAC4-1F7C-80B7-A9AE350E67F7}</x:author>
-    <x:author>tc={C6FFBF76-75E5-A885-90FC-7A4822669D85}</x:author>
-    <x:author>tc={48B6FC78-C54C-A341-9A8A-BAE4F532FF12}</x:author>
-    <x:author>tc={40834F88-B44F-30F0-0C1E-7A7EA53D4250}</x:author>
-    <x:author>tc={8C86F84D-BA29-E3DB-77BF-71A0444405B8}</x:author>
-    <x:author>tc={E119E111-72FF-3D54-C250-0ADC5886F9C3}</x:author>
-    <x:author>tc={82842CDD-4566-2F54-CBEE-B39CF6B61B97}</x:author>
-    <x:author>tc={87E8F4DE-0F6B-C100-170D-96C85EA2694F}</x:author>
-    <x:author>tc={327772B5-06F7-BF98-168C-1F90F7D50CBB}</x:author>
-    <x:author>tc={36BE7540-24E4-876F-B0E7-5753CB3F9B1F}</x:author>
-    <x:author>tc={3977E859-D6B3-767C-5E5F-B7BC8DA6835F}</x:author>
-    <x:author>tc={0EEA68E2-7763-CC47-F71C-8F260986727F}</x:author>
-    <x:author>tc={2E5078F9-9194-8A06-23A5-2ACD828EBE10}</x:author>
-    <x:author>tc={7D7BDFB5-CE3D-259A-6186-A2557641EECC}</x:author>
-    <x:author>tc={E14E0F78-126D-771B-A1F2-85F72686862D}</x:author>
-    <x:author>tc={9669977D-6EF4-2826-924E-2C0BB9D74365}</x:author>
-    <x:author>tc={0D86104F-0064-7B27-F768-D1C5A87ABBBB}</x:author>
+    <x:author>tc={98531AC1-4941-7A52-E013-EE7B6AE34866}</x:author>
+    <x:author>tc={D157483F-6BDA-7F1C-DCCF-23C8E64A35F7}</x:author>
+    <x:author>tc={552A1BEC-EA87-5403-5908-968977F501D8}</x:author>
+    <x:author>tc={A3DA3D31-7AAA-72A0-4EF5-95EFCC71CD2B}</x:author>
+    <x:author>tc={76E3920F-E519-3C1E-3E0D-4BD1A2A66133}</x:author>
+    <x:author>tc={5E262495-50B1-C8A9-AA8E-A574EC7E8A3D}</x:author>
+    <x:author>tc={7EB79C36-B5A2-F049-7BDF-9F3B596F6820}</x:author>
+    <x:author>tc={22CB9419-E586-D4C1-50B9-A021EC148AC5}</x:author>
+    <x:author>tc={620B1091-CEB4-C37C-3382-EE621929B02A}</x:author>
+    <x:author>tc={1405AEF0-4174-F4F3-F1A4-C31A5255643D}</x:author>
+    <x:author>tc={B66A228C-307C-CC5B-C01D-0898704EE8A3}</x:author>
+    <x:author>tc={AA3B7332-904E-A09B-2432-C36A1595C35A}</x:author>
+    <x:author>tc={58E0E191-E399-7CE9-F247-C1CFF9615D23}</x:author>
+    <x:author>tc={E1D11912-9D5F-2807-3A5F-26545A058958}</x:author>
+    <x:author>tc={8C849A78-52FB-4F6A-C60B-5C3DD9A318B8}</x:author>
+    <x:author>tc={A8EB206C-B5DF-647E-1A30-B65652F54204}</x:author>
+    <x:author>tc={A281D42C-43AC-B97E-892E-1520D6E7A5F3}</x:author>
+    <x:author>tc={AD9FEFBE-F579-CDA9-FC02-DD01D955F713}</x:author>
+    <x:author>tc={28D2157A-9BBF-4F6E-79EF-FA7ECA05A5C8}</x:author>
+    <x:author>tc={3DE68A57-0B2F-A77D-77DF-55430FAAA6F7}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="J5" authorId="0">
@@ -2060,7 +2060,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9c3b9377a8c64228"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Reda8774676904c7c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2071,7 +2071,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}"/>
+  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}"/>
 </xltc:personList>
 </file>
 
@@ -2268,493 +2268,493 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="P5" dT="2026-08-15T06:51:35.606" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{0AF4FEDA-AC03-3F9A-4677-E614750C0BE6}">
+  <xltc:threadedComment ref="P5" dT="2026-08-15T14:19:02.132" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B010C51E-1279-1014-33BC-2602466A0653}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P6" dT="2026-08-15T06:51:35.608" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{7B13601B-A686-D1F6-E2C3-2DEAACC41826}">
+  <xltc:threadedComment ref="P6" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{C1FCCBE0-DA45-F004-62DE-931492BB7B55}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P7" dT="2026-08-15T06:51:35.608" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{10B9DE82-DAAF-597E-4424-E67283E9A4F8}">
+  <xltc:threadedComment ref="P7" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{AC4872FE-E925-0F71-A1A0-B51C3BE471D4}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P8" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9DDF9D19-AAB7-35C6-6EAB-ADE447886907}">
+  <xltc:threadedComment ref="P8" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{78456A9C-33CF-DC3E-ACC9-771E9401AB46}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P9" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{CEC6EDDA-4333-DE39-19A1-CD6C28B0071E}">
+  <xltc:threadedComment ref="P9" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A3652911-0C8B-2C28-FADE-73D328A5BF26}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P10" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9E0A3C03-F7F7-40B8-594C-1134A321AF12}">
+  <xltc:threadedComment ref="P10" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{6F2EBCD8-23F2-D22F-38CC-ED40EFF8AEC8}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 119
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P11" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{6A469CC5-9E84-42E7-A4A2-5046B5EB797A}">
+  <xltc:threadedComment ref="P11" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{92F20AFD-1D39-B8DE-5BD9-BC3E03CB8C0F}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 160
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P12" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{49F38930-D4FC-9148-B4AB-7B8868A6B1C4}">
+  <xltc:threadedComment ref="P12" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{CA2CD762-5110-A555-E40D-9C5F0FB6D9CC}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P13" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{6AE471B8-00A6-D8CA-E30E-F2F43B242CB2}">
+  <xltc:threadedComment ref="P13" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{9DAD665B-4B78-CB05-6BFF-8A259A25099D}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P14" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{070A3F26-F4D3-3501-5B26-B76E24181EE6}">
+  <xltc:threadedComment ref="P14" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B404A4C9-0C5D-FB04-5F38-B466A0729AB3}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P15" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{DB4AA7DC-83F7-AA9C-6650-AC0FBB081C37}">
+  <xltc:threadedComment ref="P15" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A778AC8E-E3EE-EF95-340F-71DE58C4379A}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P16" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{E8A6B8CE-ACDD-0EA3-3036-3FEA4BE387E5}">
+  <xltc:threadedComment ref="P16" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{CF9789CE-401E-9368-3823-F3D6EB9FB0AE}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P17" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{F5132FA4-62BD-C63C-B25A-A7E1FE946B04}">
+  <xltc:threadedComment ref="P17" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{E0F7EB04-9E7A-C956-F66F-04924C0BBF6B}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P18" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{924A75EC-79F9-BE2D-03E1-123D59F3BF71}">
+  <xltc:threadedComment ref="P18" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{432D59DF-0456-250E-3705-7E52A846CC07}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P19" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{7DFAAAEE-9F37-70B4-1295-82F48891DA0C}">
+  <xltc:threadedComment ref="P19" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{8E40EC39-F650-2BB9-AA8A-B164C8F0D6DB}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P20" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{E2EA446D-49CF-67B3-25D3-448163193339}">
+  <xltc:threadedComment ref="P20" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{06B31F52-AE05-C750-E2E4-8BE8C077E3ED}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 138
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P21" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{130AC7D8-E99A-FB9E-EC90-C0CC209F65EE}">
+  <xltc:threadedComment ref="P21" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{C4AB3B82-976E-0559-3794-2F2F9216C552}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 212
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P22" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{DFEDA6A7-98B9-D90B-F8E4-87463C1ABE71}">
+  <xltc:threadedComment ref="P22" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{3AAB5A1B-8E7D-C179-2DC1-E2DBD2705DB9}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P23" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{F908D626-E856-7A2E-B578-6FFFAF10A067}">
+  <xltc:threadedComment ref="P23" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{7D66F2E6-7D62-9517-832E-57FFAA140850}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P24" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{4691BC9F-FA65-4FBB-BE88-C3485B37BF5B}">
+  <xltc:threadedComment ref="P24" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{01EA68F6-A6AF-EEF9-FC79-C83DFF706D5F}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P25" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{54D1659D-A9A9-797D-09FE-9CCD3046EB3B}">
+  <xltc:threadedComment ref="P25" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{7EBEBBB5-1D36-3EC8-8615-2492FBE68CC4}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P26" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{32021335-239B-D7CF-C593-02492073755E}">
+  <xltc:threadedComment ref="P26" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{67EA088D-22B9-ECEE-A157-D88A9B7AAFA9}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P27" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2D4C52F2-DF0E-98A8-DBAD-465EFEA6430C}">
+  <xltc:threadedComment ref="P27" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A2333FE9-49D5-C016-953E-7E0B47F95EF5}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 272
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P28" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{4F673CEB-0DB2-16EC-1BF9-E9916FC0D89C}">
+  <xltc:threadedComment ref="P28" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{93C06E00-D895-402F-7E27-987889902425}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P29" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{8C766CE4-DCA4-0227-2719-EC43FBE4EB3E}">
+  <xltc:threadedComment ref="P29" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{AEE536DF-8184-66AA-DD13-2B4E3E8B93C2}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P30" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{030B07FB-3D16-4698-B4D5-9BFD808ED081}">
+  <xltc:threadedComment ref="P30" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{5997CBC9-B8DA-7AF8-6285-53F3711B14B9}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 158
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P31" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{BB835A0A-AC15-BD40-37D2-BB2D5D7D1A29}">
+  <xltc:threadedComment ref="P31" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{626792A5-658D-324B-98D1-7D4E6DE536BD}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P32" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{ACE1C8E0-F10B-F24B-C4C3-09990BA1EAF5}">
+  <xltc:threadedComment ref="P32" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{8D7BFCFD-3E48-D195-6EB4-5521380E05C9}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P33" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{89E2F11B-ECCC-3429-226F-74770117AB92}">
+  <xltc:threadedComment ref="P33" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{E15B3E52-7A06-CC45-DE2B-41A9C12FF48D}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 72
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P34" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{FE94A6DE-84F6-0201-3EFF-69B3D6B7D622}">
+  <xltc:threadedComment ref="P34" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B960910A-8477-2846-1613-88C2913E5C85}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P35" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{5FADB78B-442A-2857-7CCC-D525C440BCCF}">
+  <xltc:threadedComment ref="P35" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{3F019C8B-A8FF-A1C1-F480-A723F813C270}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P36" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{33238565-3127-12AD-ACAF-5A83E4E3101E}">
+  <xltc:threadedComment ref="P36" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{8B0451A6-6D51-3B85-B608-44D73A90BE00}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 24
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P37" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{DBA819E1-2CFB-40C0-8E60-4EBBB4963742}">
+  <xltc:threadedComment ref="P37" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{6E34B664-AA4F-7D25-5EB4-CAE4F78D331D}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P38" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{831BC617-DC59-E847-0D3A-95946FD8D988}">
+  <xltc:threadedComment ref="P38" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B2D6B7C4-FB9F-7569-768C-9F19B0EDBA9D}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P39" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9625D7E8-9A23-1EEE-66C1-3D1F41528532}">
+  <xltc:threadedComment ref="P39" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{F2C939C5-67DD-99B6-503C-636AE1C76D8C}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 19
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P40" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{36A13555-305E-B2C5-2B7A-87476C5BA766}">
+  <xltc:threadedComment ref="P40" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{091770E0-D8A8-A17E-211F-BF39D2DE3D21}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P41" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{69541CEA-6E11-BC48-6898-36AE3D548AB4}">
+  <xltc:threadedComment ref="P41" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{C81BBC94-53F4-9708-39C3-5CB664703880}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P42" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{12AFE746-FDD9-963F-DCFD-DC968D22FFA6}">
+  <xltc:threadedComment ref="P42" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A06A1A63-4CF5-E445-56FC-BD4A588968F1}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P43" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{425C83BD-D4DC-BDED-071D-487523F8AC3F}">
+  <xltc:threadedComment ref="P43" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{CF996379-C6D9-0FBB-656E-63B1D66BAFC8}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P44" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2D72A011-0216-7D35-09A3-D704E88BAEE3}">
+  <xltc:threadedComment ref="P44" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B957E27C-1147-FAF3-74E7-EA8EC5908CC6}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P45" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{86FBCAB8-88A0-F97B-4FA1-13C4BEAA369D}">
+  <xltc:threadedComment ref="P45" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{420E6EE9-F0FD-3EE6-7002-0F87931DE2C3}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P46" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9185AC7C-5FA5-8BAE-5D74-F86F31883FC5}">
+  <xltc:threadedComment ref="P46" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{72E4C9A4-FDB4-C94D-DCDC-B2D8F3FC1E58}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P47" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{8F348568-9728-931E-D9B2-061F382ED13A}">
+  <xltc:threadedComment ref="P47" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{1CB140F6-0570-D58E-D0A8-4551FD74BA90}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P48" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{E5746BEC-90A8-ABA0-16B5-A6A9F11A2C96}">
+  <xltc:threadedComment ref="P48" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{4C23F7C6-D3C7-A4BE-F36C-2F5E0923875B}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P49" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{4B1E6C62-4809-1469-5784-9EA7A65F2E2D}">
+  <xltc:threadedComment ref="P49" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A18D8527-4F44-6611-303D-A0E50FC512E3}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 118
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P50" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{271EEFA8-492B-5EC5-67E3-8B28D1AE9871}">
+  <xltc:threadedComment ref="P50" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{DCF389D3-4242-623B-AE66-3E44891929C8}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P51" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{3430FD27-2DAA-4633-A322-0688F2FCD467}">
+  <xltc:threadedComment ref="P51" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{942E9BB5-C21B-6000-23BC-C0925210FA48}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P52" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{8D7DF3C9-36A9-2E8C-6160-11B116238A97}">
+  <xltc:threadedComment ref="P52" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B8533D65-8426-863A-B312-F367AD0B4444}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P53" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{31933AFB-CA47-471A-E7EB-D7E5B693D87A}">
+  <xltc:threadedComment ref="P53" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{0886CFC9-D7DE-1471-513A-71A37582BE87}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-STF</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P54" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{CEB8E96A-F9CE-D6E4-1345-25BEA6D4853C}">
+  <xltc:threadedComment ref="P54" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{BCB573C2-22CD-DDD1-A5ED-1DC2F5CE50B5}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P55" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{CE8B63E6-EC70-4885-EBBF-C61B84B9BD02}">
+  <xltc:threadedComment ref="P55" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{E9D0B5CE-5209-E0BE-3237-DB8B632D7235}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P56" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{1236AB2A-50DD-58C5-F0CF-0A77396ECCB9}">
+  <xltc:threadedComment ref="P56" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B704E177-02B4-47FB-A7F9-206D3C4F097F}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 18
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P57" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{23B809AB-666E-3843-AA8B-2E06C9D6735C}">
+  <xltc:threadedComment ref="P57" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{6F3A1B45-FF5A-DF64-19ED-AA0695469814}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P58" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{F9218197-D7D7-96FC-5DEE-19E1B89C6668}">
+  <xltc:threadedComment ref="P58" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{ACCA67AD-3C83-ACC1-2D98-C4C6D0AFD638}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P59" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{49C564EF-C6E1-AA3E-BAE6-F9B6B7DAF702}">
+  <xltc:threadedComment ref="P59" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B238E13A-91E5-5386-8C34-F67463D45FB1}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P60" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{6A34B57F-09E3-5DA4-9CDF-BDD9AFC15C62}">
+  <xltc:threadedComment ref="P60" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{C0BA2EF8-C1B1-64BE-3EA0-F77C4E23AD4C}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P61" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{EA67CC0C-3B7B-6001-4E9C-C907CB9A2E41}">
+  <xltc:threadedComment ref="P61" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{9E7079E2-8399-4258-574A-B9F9C79E592C}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P62" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2C705125-9621-DC7B-9356-1AFFFB014183}">
+  <xltc:threadedComment ref="P62" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{4D4A8E67-5958-A3C1-70C2-33CB58A773FF}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P63" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{4127462E-7049-10C8-6E6D-2726FCAFA040}">
+  <xltc:threadedComment ref="P63" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{0CA8FE98-EDDA-A7FC-8A90-7852EAD6A4FF}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P64" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{DDC7860C-4BF8-FE8E-AB94-BF36F51E4742}">
+  <xltc:threadedComment ref="P64" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{C13917A4-524D-2A26-A42D-6D16A66166CA}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P65" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{355CD349-BEF2-1F91-3717-B7779FC267B7}">
+  <xltc:threadedComment ref="P65" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{C4039E66-57C0-F444-53E6-FCCF8A6DA3E9}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 311
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P66" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{BE707954-D4F8-3036-E784-0F6EF373E3B1}">
+  <xltc:threadedComment ref="P66" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{03D96BF4-9AE3-9DF8-CC14-62B6DA87E1BA}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P67" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{30C17E09-F415-E5D5-1412-983D6592AE59}">
+  <xltc:threadedComment ref="P67" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{68867B5D-2E79-11B5-AD2B-6426A7112DA5}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P68" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{946D1FE7-F4AA-6563-A358-3F55219C3AED}">
+  <xltc:threadedComment ref="P68" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{54A9DCF0-8852-0B11-508D-950C7B9284A4}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 141
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P69" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{FF9DEADC-5F2B-2C71-0EDD-31A65A1DAC80}">
+  <xltc:threadedComment ref="P69" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{22D8A23D-9682-E3ED-C9FB-E779AA2720B1}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P70" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{99FA21E2-86C5-2A76-2880-8215954AA3D4}">
+  <xltc:threadedComment ref="P70" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{91E699CE-9A06-219F-5833-E4E864BED089}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P71" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{901E21A1-49DD-A0DA-0A10-1EDE8076C1B3}">
+  <xltc:threadedComment ref="P71" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{F8EB5DB1-1D5C-47D0-D1DD-184B283C0C6C}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 33
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P72" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{FCB3C38E-B0AF-A412-700D-4D9A9D2C2741}">
+  <xltc:threadedComment ref="P72" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{6EF67E32-E7EC-94F6-3F4E-584F0BE95656}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P73" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9382A565-2A1D-550E-54B1-678F98943EC6}">
+  <xltc:threadedComment ref="P73" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{99F57B06-4D37-016A-C483-B1735DED682F}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P74" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{40576489-4A24-6AA0-06F2-24F75770098B}">
+  <xltc:threadedComment ref="P74" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{5D7317F8-C323-677A-8020-3361BEEEB812}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 21
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P75" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{D80EF366-6BBD-D5AC-E71F-5666ED857ED8}">
+  <xltc:threadedComment ref="P75" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{513B22C5-53D5-D9FA-E2B0-84DC9C63BD75}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P76" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{8E28E375-5E9B-B43C-02D8-1D69B6DBCCB7}">
+  <xltc:threadedComment ref="P76" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{C676EC9E-9A20-A1B2-3E1F-20A28A26A61A}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P77" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{C52D303F-E26F-AEB2-82AD-C196257D053A}">
+  <xltc:threadedComment ref="P77" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{BD7320DD-EB8C-3619-ABDC-27A23A838BFD}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 19
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P78" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{AD3CBF1C-654B-022F-1CCE-E3B6B02846E3}">
+  <xltc:threadedComment ref="P78" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{DCCE526A-71D7-E02C-4253-8778B920726E}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 43
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P79" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2EEF0622-B8D5-960E-069D-57BC28C46AE4}">
+  <xltc:threadedComment ref="P79" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{33C6E653-4ECD-66D3-31ED-37F8D530BBCA}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 44
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P80" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{C7A17400-8C3D-04F3-BB45-75623A8D8379}">
+  <xltc:threadedComment ref="P80" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{2D51D488-F2CD-1656-7FC5-C0BE0926F124}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 40
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P81" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9CB15BCB-A81F-4C51-B6D7-CA70F830A75F}">
+  <xltc:threadedComment ref="P81" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{620305EA-1DAC-09F1-F096-0BEF7B4B8CA1}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P82" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9CDE5188-52E3-BEBE-AC4D-8F98AC717AA6}">
+  <xltc:threadedComment ref="P82" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{E5082642-40DD-D305-F257-8AEF1B0F3468}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P83" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{96D773F7-6FC9-4DF1-46BC-3C5A65EBE44A}">
+  <xltc:threadedComment ref="P83" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A227902C-BE3D-E28E-3D70-D78E36E76664}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 16
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P84" dT="2026-08-15T06:51:35.612" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{69BF4FC0-9856-F2BC-F517-9DC02348AB96}">
+  <xltc:threadedComment ref="P84" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{8DC1750F-5595-5639-B653-027050CAA390}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P85" dT="2026-08-15T06:51:35.612" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{EF1A8A33-3E41-8002-8157-23C7596AF4CA}">
+  <xltc:threadedComment ref="P85" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{DD3E8D93-9C02-6410-C382-7C25C24F3F42}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P86" dT="2026-08-15T06:51:35.612" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{CBA415B4-31A9-6F43-882D-D511ADAA6836}">
+  <xltc:threadedComment ref="P86" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{83154AE6-98B5-8AE9-06F0-2B1446B9C581}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 21
 Available: 2026-02-25
@@ -2765,64 +2765,64 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="J5" dT="2026-08-15T06:51:36.013" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{B01406AF-5C54-1385-E93F-8BC31DCEF046}">
+  <xltc:threadedComment ref="J5" dT="2026-08-15T14:19:02.445" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{98531AC1-4941-7A52-E013-EE7B6AE34866}">
     <xltc:text>Official source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J6" dT="2026-08-15T06:51:36.015" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{6DD7D282-4D5B-6CEA-034D-91D0362B1489}">
+  <xltc:threadedComment ref="J6" dT="2026-08-15T14:19:02.447" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{D157483F-6BDA-7F1C-DCCF-23C8E64A35F7}">
     <xltc:text>Official source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J7" dT="2026-08-15T06:51:36.019" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{B744CA31-60A8-7C0A-67C6-4F7042734E04}">
+  <xltc:threadedComment ref="J7" dT="2026-08-15T14:19:02.451" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{552A1BEC-EA87-5403-5908-968977F501D8}">
     <xltc:text>Official source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J8" dT="2026-08-15T06:51:36.022" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2CBFDB07-DAC4-1F7C-80B7-A9AE350E67F7}">
+  <xltc:threadedComment ref="J8" dT="2026-08-15T14:19:02.453" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A3DA3D31-7AAA-72A0-4EF5-95EFCC71CD2B}">
     <xltc:text>Official source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J9" dT="2026-08-15T06:51:36.025" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{C6FFBF76-75E5-A885-90FC-7A4822669D85}">
+  <xltc:threadedComment ref="J9" dT="2026-08-15T14:19:02.456" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{76E3920F-E519-3C1E-3E0D-4BD1A2A66133}">
     <xltc:text>Official source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J10" dT="2026-08-15T06:51:36.029" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{48B6FC78-C54C-A341-9A8A-BAE4F532FF12}">
+  <xltc:threadedComment ref="J10" dT="2026-08-15T14:19:02.458" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{5E262495-50B1-C8A9-AA8E-A574EC7E8A3D}">
     <xltc:text>Official source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J11" dT="2026-08-15T06:51:36.031" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{40834F88-B44F-30F0-0C1E-7A7EA53D4250}">
+  <xltc:threadedComment ref="J11" dT="2026-08-15T14:19:02.46" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{7EB79C36-B5A2-F049-7BDF-9F3B596F6820}">
     <xltc:text>Official source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J12" dT="2026-08-15T06:51:36.033" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{8C86F84D-BA29-E3DB-77BF-71A0444405B8}">
+  <xltc:threadedComment ref="J12" dT="2026-08-15T14:19:02.463" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{22CB9419-E586-D4C1-50B9-A021EC148AC5}">
     <xltc:text>Official source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J13" dT="2026-08-15T06:51:36.035" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{E119E111-72FF-3D54-C250-0ADC5886F9C3}">
+  <xltc:threadedComment ref="J13" dT="2026-08-15T14:19:02.466" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{620B1091-CEB4-C37C-3382-EE621929B02A}">
     <xltc:text>Official source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J14" dT="2026-08-15T06:51:36.038" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{82842CDD-4566-2F54-CBEE-B39CF6B61B97}">
+  <xltc:threadedComment ref="J14" dT="2026-08-15T14:19:02.47" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{1405AEF0-4174-F4F3-F1A4-C31A5255643D}">
     <xltc:text>Official source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J15" dT="2026-08-15T06:51:36.041" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{87E8F4DE-0F6B-C100-170D-96C85EA2694F}">
+  <xltc:threadedComment ref="J15" dT="2026-08-15T14:19:02.472" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B66A228C-307C-CC5B-C01D-0898704EE8A3}">
     <xltc:text>Official source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J16" dT="2026-08-15T06:51:36.043" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{327772B5-06F7-BF98-168C-1F90F7D50CBB}">
+  <xltc:threadedComment ref="J16" dT="2026-08-15T14:19:02.476" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{AA3B7332-904E-A09B-2432-C36A1595C35A}">
     <xltc:text>Official source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J17" dT="2026-08-15T06:51:36.045" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{36BE7540-24E4-876F-B0E7-5753CB3F9B1F}">
+  <xltc:threadedComment ref="J17" dT="2026-08-15T14:19:02.477" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{58E0E191-E399-7CE9-F247-C1CFF9615D23}">
     <xltc:text>Official source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J18" dT="2026-08-15T06:51:36.047" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{3977E859-D6B3-767C-5E5F-B7BC8DA6835F}">
+  <xltc:threadedComment ref="J18" dT="2026-08-15T14:19:02.479" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{E1D11912-9D5F-2807-3A5F-26545A058958}">
     <xltc:text>Official source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J19" dT="2026-08-15T06:51:36.048" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{0EEA68E2-7763-CC47-F71C-8F260986727F}">
+  <xltc:threadedComment ref="J19" dT="2026-08-15T14:19:02.481" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{8C849A78-52FB-4F6A-C60B-5C3DD9A318B8}">
     <xltc:text>Official source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J20" dT="2026-08-15T06:51:36.054" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2E5078F9-9194-8A06-23A5-2ACD828EBE10}">
+  <xltc:threadedComment ref="J20" dT="2026-08-15T14:19:02.484" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A8EB206C-B5DF-647E-1A30-B65652F54204}">
     <xltc:text>Official source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J21" dT="2026-08-15T06:51:36.057" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{7D7BDFB5-CE3D-259A-6186-A2557641EECC}">
+  <xltc:threadedComment ref="J21" dT="2026-08-15T14:19:02.486" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A281D42C-43AC-B97E-892E-1520D6E7A5F3}">
     <xltc:text>Official source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J22" dT="2026-08-15T06:51:36.059" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{E14E0F78-126D-771B-A1F2-85F72686862D}">
+  <xltc:threadedComment ref="J22" dT="2026-08-15T14:19:02.487" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{AD9FEFBE-F579-CDA9-FC02-DD01D955F713}">
     <xltc:text>Official source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J23" dT="2026-08-15T06:51:36.061" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9669977D-6EF4-2826-924E-2C0BB9D74365}">
+  <xltc:threadedComment ref="J23" dT="2026-08-15T14:19:02.489" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{28D2157A-9BBF-4F6E-79EF-FA7ECA05A5C8}">
     <xltc:text>Official source: https://www.aspenpharma.com/download/annual-financial-statements-2/</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J24" dT="2026-08-15T06:51:36.063" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{0D86104F-0064-7B27-F768-D1C5A87ABBBB}">
+  <xltc:threadedComment ref="J24" dT="2026-08-15T14:19:02.491" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{3DE68A57-0B2F-A77D-77DF-55430FAAA6F7}">
     <xltc:text>Official source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -3877,7 +3877,7 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c7810c6b47b416f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f41b2e2cafc4af8"/>
 </x:worksheet>
 </file>
 
@@ -8611,7 +8611,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc12e983b47534b1a"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c0baf671f3c4ecb"/>
 </x:worksheet>
 </file>
 
@@ -9671,7 +9671,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R458cac95bef44c85"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb56dd16d91fa437d"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Bind V3.2 artifacts to final status authority
</commit_message>
<xml_diff>
--- a/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
+++ b/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rcb2c4e1a55b942b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R1862c38eec4f4fd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="Rff96f59aa3c04679"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="R1583a0a66d6b4d3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R892f299ff0ed4564"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="Rb12c3646ad1d4600"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Re458eca1bce74f85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="Rfded105b212a4b17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R2f52fd7a8ac94db2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R97807c487b9a4e4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R886ca569ce0f4ff3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R8a98d8abaa2d444f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="R20915aa5a6a045f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Ra739eb80933c41b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R06c7793f53ca43ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R629ff89fcfc14280"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R3695fa6daf0b4fa2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="R13ff4ef65ee04163"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R800728acfd374c23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R37349b6bb9a4454e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,88 +19,88 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={B010C51E-1279-1014-33BC-2602466A0653}</x:author>
-    <x:author>tc={C1FCCBE0-DA45-F004-62DE-931492BB7B55}</x:author>
-    <x:author>tc={AC4872FE-E925-0F71-A1A0-B51C3BE471D4}</x:author>
-    <x:author>tc={78456A9C-33CF-DC3E-ACC9-771E9401AB46}</x:author>
-    <x:author>tc={A3652911-0C8B-2C28-FADE-73D328A5BF26}</x:author>
-    <x:author>tc={6F2EBCD8-23F2-D22F-38CC-ED40EFF8AEC8}</x:author>
-    <x:author>tc={92F20AFD-1D39-B8DE-5BD9-BC3E03CB8C0F}</x:author>
-    <x:author>tc={CA2CD762-5110-A555-E40D-9C5F0FB6D9CC}</x:author>
-    <x:author>tc={9DAD665B-4B78-CB05-6BFF-8A259A25099D}</x:author>
-    <x:author>tc={B404A4C9-0C5D-FB04-5F38-B466A0729AB3}</x:author>
-    <x:author>tc={A778AC8E-E3EE-EF95-340F-71DE58C4379A}</x:author>
-    <x:author>tc={CF9789CE-401E-9368-3823-F3D6EB9FB0AE}</x:author>
-    <x:author>tc={E0F7EB04-9E7A-C956-F66F-04924C0BBF6B}</x:author>
-    <x:author>tc={432D59DF-0456-250E-3705-7E52A846CC07}</x:author>
-    <x:author>tc={8E40EC39-F650-2BB9-AA8A-B164C8F0D6DB}</x:author>
-    <x:author>tc={06B31F52-AE05-C750-E2E4-8BE8C077E3ED}</x:author>
-    <x:author>tc={C4AB3B82-976E-0559-3794-2F2F9216C552}</x:author>
-    <x:author>tc={3AAB5A1B-8E7D-C179-2DC1-E2DBD2705DB9}</x:author>
-    <x:author>tc={7D66F2E6-7D62-9517-832E-57FFAA140850}</x:author>
-    <x:author>tc={01EA68F6-A6AF-EEF9-FC79-C83DFF706D5F}</x:author>
-    <x:author>tc={7EBEBBB5-1D36-3EC8-8615-2492FBE68CC4}</x:author>
-    <x:author>tc={67EA088D-22B9-ECEE-A157-D88A9B7AAFA9}</x:author>
-    <x:author>tc={A2333FE9-49D5-C016-953E-7E0B47F95EF5}</x:author>
-    <x:author>tc={93C06E00-D895-402F-7E27-987889902425}</x:author>
-    <x:author>tc={AEE536DF-8184-66AA-DD13-2B4E3E8B93C2}</x:author>
-    <x:author>tc={5997CBC9-B8DA-7AF8-6285-53F3711B14B9}</x:author>
-    <x:author>tc={626792A5-658D-324B-98D1-7D4E6DE536BD}</x:author>
-    <x:author>tc={8D7BFCFD-3E48-D195-6EB4-5521380E05C9}</x:author>
-    <x:author>tc={E15B3E52-7A06-CC45-DE2B-41A9C12FF48D}</x:author>
-    <x:author>tc={B960910A-8477-2846-1613-88C2913E5C85}</x:author>
-    <x:author>tc={3F019C8B-A8FF-A1C1-F480-A723F813C270}</x:author>
-    <x:author>tc={8B0451A6-6D51-3B85-B608-44D73A90BE00}</x:author>
-    <x:author>tc={6E34B664-AA4F-7D25-5EB4-CAE4F78D331D}</x:author>
-    <x:author>tc={B2D6B7C4-FB9F-7569-768C-9F19B0EDBA9D}</x:author>
-    <x:author>tc={F2C939C5-67DD-99B6-503C-636AE1C76D8C}</x:author>
-    <x:author>tc={091770E0-D8A8-A17E-211F-BF39D2DE3D21}</x:author>
-    <x:author>tc={C81BBC94-53F4-9708-39C3-5CB664703880}</x:author>
-    <x:author>tc={A06A1A63-4CF5-E445-56FC-BD4A588968F1}</x:author>
-    <x:author>tc={CF996379-C6D9-0FBB-656E-63B1D66BAFC8}</x:author>
-    <x:author>tc={B957E27C-1147-FAF3-74E7-EA8EC5908CC6}</x:author>
-    <x:author>tc={420E6EE9-F0FD-3EE6-7002-0F87931DE2C3}</x:author>
-    <x:author>tc={72E4C9A4-FDB4-C94D-DCDC-B2D8F3FC1E58}</x:author>
-    <x:author>tc={1CB140F6-0570-D58E-D0A8-4551FD74BA90}</x:author>
-    <x:author>tc={4C23F7C6-D3C7-A4BE-F36C-2F5E0923875B}</x:author>
-    <x:author>tc={A18D8527-4F44-6611-303D-A0E50FC512E3}</x:author>
-    <x:author>tc={DCF389D3-4242-623B-AE66-3E44891929C8}</x:author>
-    <x:author>tc={942E9BB5-C21B-6000-23BC-C0925210FA48}</x:author>
-    <x:author>tc={B8533D65-8426-863A-B312-F367AD0B4444}</x:author>
-    <x:author>tc={0886CFC9-D7DE-1471-513A-71A37582BE87}</x:author>
-    <x:author>tc={BCB573C2-22CD-DDD1-A5ED-1DC2F5CE50B5}</x:author>
-    <x:author>tc={E9D0B5CE-5209-E0BE-3237-DB8B632D7235}</x:author>
-    <x:author>tc={B704E177-02B4-47FB-A7F9-206D3C4F097F}</x:author>
-    <x:author>tc={6F3A1B45-FF5A-DF64-19ED-AA0695469814}</x:author>
-    <x:author>tc={ACCA67AD-3C83-ACC1-2D98-C4C6D0AFD638}</x:author>
-    <x:author>tc={B238E13A-91E5-5386-8C34-F67463D45FB1}</x:author>
-    <x:author>tc={C0BA2EF8-C1B1-64BE-3EA0-F77C4E23AD4C}</x:author>
-    <x:author>tc={9E7079E2-8399-4258-574A-B9F9C79E592C}</x:author>
-    <x:author>tc={4D4A8E67-5958-A3C1-70C2-33CB58A773FF}</x:author>
-    <x:author>tc={0CA8FE98-EDDA-A7FC-8A90-7852EAD6A4FF}</x:author>
-    <x:author>tc={C13917A4-524D-2A26-A42D-6D16A66166CA}</x:author>
-    <x:author>tc={C4039E66-57C0-F444-53E6-FCCF8A6DA3E9}</x:author>
-    <x:author>tc={03D96BF4-9AE3-9DF8-CC14-62B6DA87E1BA}</x:author>
-    <x:author>tc={68867B5D-2E79-11B5-AD2B-6426A7112DA5}</x:author>
-    <x:author>tc={54A9DCF0-8852-0B11-508D-950C7B9284A4}</x:author>
-    <x:author>tc={22D8A23D-9682-E3ED-C9FB-E779AA2720B1}</x:author>
-    <x:author>tc={91E699CE-9A06-219F-5833-E4E864BED089}</x:author>
-    <x:author>tc={F8EB5DB1-1D5C-47D0-D1DD-184B283C0C6C}</x:author>
-    <x:author>tc={6EF67E32-E7EC-94F6-3F4E-584F0BE95656}</x:author>
-    <x:author>tc={99F57B06-4D37-016A-C483-B1735DED682F}</x:author>
-    <x:author>tc={5D7317F8-C323-677A-8020-3361BEEEB812}</x:author>
-    <x:author>tc={513B22C5-53D5-D9FA-E2B0-84DC9C63BD75}</x:author>
-    <x:author>tc={C676EC9E-9A20-A1B2-3E1F-20A28A26A61A}</x:author>
-    <x:author>tc={BD7320DD-EB8C-3619-ABDC-27A23A838BFD}</x:author>
-    <x:author>tc={DCCE526A-71D7-E02C-4253-8778B920726E}</x:author>
-    <x:author>tc={33C6E653-4ECD-66D3-31ED-37F8D530BBCA}</x:author>
-    <x:author>tc={2D51D488-F2CD-1656-7FC5-C0BE0926F124}</x:author>
-    <x:author>tc={620305EA-1DAC-09F1-F096-0BEF7B4B8CA1}</x:author>
-    <x:author>tc={E5082642-40DD-D305-F257-8AEF1B0F3468}</x:author>
-    <x:author>tc={A227902C-BE3D-E28E-3D70-D78E36E76664}</x:author>
-    <x:author>tc={8DC1750F-5595-5639-B653-027050CAA390}</x:author>
-    <x:author>tc={DD3E8D93-9C02-6410-C382-7C25C24F3F42}</x:author>
-    <x:author>tc={83154AE6-98B5-8AE9-06F0-2B1446B9C581}</x:author>
+    <x:author>tc={19394B01-E00F-53AA-5F9F-DAAE5B249735}</x:author>
+    <x:author>tc={1D42977D-73AE-7F9C-73B4-25926AE6C8A1}</x:author>
+    <x:author>tc={140AC83F-8B13-BB91-21C7-92173351B7FD}</x:author>
+    <x:author>tc={A84656BA-F870-0843-455C-366684097531}</x:author>
+    <x:author>tc={BA677552-5189-E26A-5201-2CAD593114D5}</x:author>
+    <x:author>tc={0D3AC6A7-2087-6C91-F3FC-49238524123A}</x:author>
+    <x:author>tc={E8B2DFAC-DBDB-1D70-FB96-A57BB882E591}</x:author>
+    <x:author>tc={BBEB777E-28A0-34D9-C7CE-3E0C0793382D}</x:author>
+    <x:author>tc={ADC69843-37EC-D20B-3201-7C998E761773}</x:author>
+    <x:author>tc={BDBE4742-2E5F-F5FF-5F4B-89143E394265}</x:author>
+    <x:author>tc={28186EC5-DD20-8D1B-177E-611D02905D17}</x:author>
+    <x:author>tc={BAC8BFD3-8437-83A1-ADAA-3C6FF249CBC5}</x:author>
+    <x:author>tc={AD89F10E-24F9-800C-BA8F-E4D4E60E2600}</x:author>
+    <x:author>tc={09A3F634-8B76-FDEA-01DA-76BD9B40C5DC}</x:author>
+    <x:author>tc={3C08E262-2F52-00E7-DFDC-875B7B0D6EB2}</x:author>
+    <x:author>tc={DBE49284-42F5-EA4C-4BD7-F83AA247DE86}</x:author>
+    <x:author>tc={AB326A0C-B59B-FD02-5084-BB0536D0FFF8}</x:author>
+    <x:author>tc={0E7E0B0F-050B-01DE-68E9-AB117F4B736F}</x:author>
+    <x:author>tc={B9AB9439-79A4-44E8-233A-BDC4B20B2561}</x:author>
+    <x:author>tc={E7A35A0C-1940-0A0A-66B2-28D3BAD76624}</x:author>
+    <x:author>tc={331D7CA0-CA52-FE29-30A6-EF44576A4681}</x:author>
+    <x:author>tc={4BA54249-5798-912A-B087-6931A573E9B2}</x:author>
+    <x:author>tc={F269CB9E-DAD7-377C-B6AE-46737C2B1FF1}</x:author>
+    <x:author>tc={D489D1BF-740A-033D-7501-81175165C33D}</x:author>
+    <x:author>tc={69054F3D-B908-030A-11FC-898D2FC0C7D0}</x:author>
+    <x:author>tc={9AB7B4F9-820A-DC76-6A9D-F632F3D10365}</x:author>
+    <x:author>tc={232896F9-7500-E0D3-F70A-6EE4CE5F563B}</x:author>
+    <x:author>tc={2444243E-848D-6DAA-B664-ECFC23B3EF1C}</x:author>
+    <x:author>tc={0DD6D8EF-35DB-0CF2-E74A-E012E6E1A9FB}</x:author>
+    <x:author>tc={72304EE7-ED25-9CD4-678B-EB502A085A57}</x:author>
+    <x:author>tc={AACC62A3-0F19-9957-7145-4DAB6497B294}</x:author>
+    <x:author>tc={E3249311-112C-5A89-889A-DDF8E4F2FE53}</x:author>
+    <x:author>tc={A1538091-C1CC-DD54-5406-206EC7D07274}</x:author>
+    <x:author>tc={35CF49BE-ABF2-3F42-5FCD-91DFBC78DD13}</x:author>
+    <x:author>tc={95CA0DC2-6586-FC1C-2C42-C17AF3387EFC}</x:author>
+    <x:author>tc={B020CB65-337E-C3E8-BDF2-537D485963B9}</x:author>
+    <x:author>tc={3CE09352-BDFF-41B3-5C7D-17838504BAD6}</x:author>
+    <x:author>tc={010FF20E-4C5A-31F9-FD05-17751B865D53}</x:author>
+    <x:author>tc={6FFA3CA4-6C2E-A91A-BE12-A7CEB29C5EF9}</x:author>
+    <x:author>tc={4E125750-51DA-850B-CD1B-D0D473F001F6}</x:author>
+    <x:author>tc={DB7B7D09-45E4-8974-B566-9C42E8A66070}</x:author>
+    <x:author>tc={DFA5C51F-06D5-BA4F-608D-865B6B3F0E8D}</x:author>
+    <x:author>tc={E14B8F74-ABA3-1B58-B20D-5F43358ACADA}</x:author>
+    <x:author>tc={94123791-288B-7DEE-DBEE-A50EAF2CEF3A}</x:author>
+    <x:author>tc={60F2A683-77E6-217F-085F-8010A834277D}</x:author>
+    <x:author>tc={5C75B7BD-F355-6365-F6A6-7F035F95D631}</x:author>
+    <x:author>tc={8B485069-42C9-BCF7-2564-CF877FB3332C}</x:author>
+    <x:author>tc={30F59ABA-66A2-F07B-EA84-2F9EC8DC22D6}</x:author>
+    <x:author>tc={4E18A03C-4BA4-7217-8027-9B09EB09244A}</x:author>
+    <x:author>tc={83C78788-EEEE-C237-020B-AE43B435EC46}</x:author>
+    <x:author>tc={55E4FEE1-9B5B-E551-7070-77A55CA1826E}</x:author>
+    <x:author>tc={77B71704-FA27-C535-F961-039BDB63EC0E}</x:author>
+    <x:author>tc={CD5687F0-0DDF-839C-1C45-7E3BB7495273}</x:author>
+    <x:author>tc={AEC31414-5E16-DD3D-89F8-40EE87A1C59D}</x:author>
+    <x:author>tc={6864D662-D838-948E-F2EF-F5F5FB71DE9B}</x:author>
+    <x:author>tc={3C9BE7BE-F9BA-CFAE-C694-1568251BE342}</x:author>
+    <x:author>tc={3C7B18CA-C167-B6B3-E28B-BA081E641EA3}</x:author>
+    <x:author>tc={A0F88A35-48DA-EE36-C7D1-AA9702B6245E}</x:author>
+    <x:author>tc={96C28C0B-4897-01F2-1C3C-EC1BD1A4C594}</x:author>
+    <x:author>tc={4EBD50A2-D0F8-C104-9A27-FDB811B9F2F1}</x:author>
+    <x:author>tc={2BAE9845-5089-4FB2-9155-03120E278CD5}</x:author>
+    <x:author>tc={0DBB817D-C9F7-F450-6447-4B61420F33C6}</x:author>
+    <x:author>tc={0C8DE577-8367-42EE-9B4B-A13AD3846F90}</x:author>
+    <x:author>tc={8A1603E1-6F97-4B78-AF27-CFDF20B95D58}</x:author>
+    <x:author>tc={BA6A8336-F4DF-E87C-DF14-F79812F1411D}</x:author>
+    <x:author>tc={6EE3B779-CB9D-65F9-3D25-66C174840379}</x:author>
+    <x:author>tc={EF88ABD5-BC27-CCC3-B3CA-7FC32267D4AF}</x:author>
+    <x:author>tc={F33C65C3-F551-D2AC-D628-FB5B78181AA7}</x:author>
+    <x:author>tc={AFDB57BC-1227-DC20-5E62-FEE3E8445830}</x:author>
+    <x:author>tc={F48AC48A-7628-95B7-FD95-B1B568391ACE}</x:author>
+    <x:author>tc={AE9CAB17-F322-2981-065F-C74301AD1B41}</x:author>
+    <x:author>tc={0F39D044-4F3C-9712-7B3C-A13B1A8FD36C}</x:author>
+    <x:author>tc={B7C788FE-7A08-37E9-F12A-9DA325EF5877}</x:author>
+    <x:author>tc={D60815FD-2FC4-EDF0-84D3-3A5E4E44F184}</x:author>
+    <x:author>tc={205EB334-F928-87C4-D82E-FEA9BA425AC5}</x:author>
+    <x:author>tc={F78CFAC1-E06B-9C87-763A-B4860DBAB1B8}</x:author>
+    <x:author>tc={0472304C-FEC5-1785-6CC1-52C96690EE46}</x:author>
+    <x:author>tc={4207741A-DE03-1BE3-B143-1BA6BF02C297}</x:author>
+    <x:author>tc={CAE4E73D-84BC-45FB-7B6A-FF3CC4C999F3}</x:author>
+    <x:author>tc={7F3E3A0C-214E-A648-AB74-D12724638463}</x:author>
+    <x:author>tc={8FB32A91-0D5B-4485-EE74-CB324EAF6F28}</x:author>
+    <x:author>tc={50FD3967-A051-5A71-20A1-A86789127CCB}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="P5" authorId="0">
@@ -1176,26 +1176,26 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={98531AC1-4941-7A52-E013-EE7B6AE34866}</x:author>
-    <x:author>tc={D157483F-6BDA-7F1C-DCCF-23C8E64A35F7}</x:author>
-    <x:author>tc={552A1BEC-EA87-5403-5908-968977F501D8}</x:author>
-    <x:author>tc={A3DA3D31-7AAA-72A0-4EF5-95EFCC71CD2B}</x:author>
-    <x:author>tc={76E3920F-E519-3C1E-3E0D-4BD1A2A66133}</x:author>
-    <x:author>tc={5E262495-50B1-C8A9-AA8E-A574EC7E8A3D}</x:author>
-    <x:author>tc={7EB79C36-B5A2-F049-7BDF-9F3B596F6820}</x:author>
-    <x:author>tc={22CB9419-E586-D4C1-50B9-A021EC148AC5}</x:author>
-    <x:author>tc={620B1091-CEB4-C37C-3382-EE621929B02A}</x:author>
-    <x:author>tc={1405AEF0-4174-F4F3-F1A4-C31A5255643D}</x:author>
-    <x:author>tc={B66A228C-307C-CC5B-C01D-0898704EE8A3}</x:author>
-    <x:author>tc={AA3B7332-904E-A09B-2432-C36A1595C35A}</x:author>
-    <x:author>tc={58E0E191-E399-7CE9-F247-C1CFF9615D23}</x:author>
-    <x:author>tc={E1D11912-9D5F-2807-3A5F-26545A058958}</x:author>
-    <x:author>tc={8C849A78-52FB-4F6A-C60B-5C3DD9A318B8}</x:author>
-    <x:author>tc={A8EB206C-B5DF-647E-1A30-B65652F54204}</x:author>
-    <x:author>tc={A281D42C-43AC-B97E-892E-1520D6E7A5F3}</x:author>
-    <x:author>tc={AD9FEFBE-F579-CDA9-FC02-DD01D955F713}</x:author>
-    <x:author>tc={28D2157A-9BBF-4F6E-79EF-FA7ECA05A5C8}</x:author>
-    <x:author>tc={3DE68A57-0B2F-A77D-77DF-55430FAAA6F7}</x:author>
+    <x:author>tc={F1DDF034-E12A-7BB5-8B27-8E0A77990B7F}</x:author>
+    <x:author>tc={A27FE3CE-58EE-9146-F293-955465F0CB1F}</x:author>
+    <x:author>tc={6A50C978-5309-D064-EBC6-23A94A3EE4D1}</x:author>
+    <x:author>tc={A3E41E1D-2961-84E0-42EC-35FFFE6CA772}</x:author>
+    <x:author>tc={82EEAB1F-45E5-5945-F994-799D5FCA8249}</x:author>
+    <x:author>tc={EA451E30-939F-5824-3AD2-283825979700}</x:author>
+    <x:author>tc={3D4150B1-DB11-5A7D-AE29-0347DFB19553}</x:author>
+    <x:author>tc={179A041E-8A29-CDE7-B9A2-A6340557FF6D}</x:author>
+    <x:author>tc={6414D9D1-981F-0106-FC22-A83B835227BF}</x:author>
+    <x:author>tc={003A8738-F53E-F29A-4836-83CD88CBD5D3}</x:author>
+    <x:author>tc={52A80459-605E-DE47-A560-B5294919DA3A}</x:author>
+    <x:author>tc={EA49137A-B2C3-1699-19C1-386362AAD204}</x:author>
+    <x:author>tc={A743B0C9-B331-3FE6-5A9C-7368C8C621E3}</x:author>
+    <x:author>tc={B9A0315D-4AA7-FF04-062A-23F5A3A8C057}</x:author>
+    <x:author>tc={58F44AC5-131C-E73F-2EF9-0F03167CE636}</x:author>
+    <x:author>tc={03872F08-FCC4-073E-DCF7-71462B38E10F}</x:author>
+    <x:author>tc={53B86A32-AD64-73D4-6684-A35D7850F2AB}</x:author>
+    <x:author>tc={EDD1FBE0-9C7B-8E26-0237-3229A3282A1E}</x:author>
+    <x:author>tc={7F8E6C93-4097-9C02-87A3-623D41D62A58}</x:author>
+    <x:author>tc={12A5D7D5-7F54-1EE0-1CAD-41DE6B533C67}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="J5" authorId="0">
@@ -2060,7 +2060,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Reda8774676904c7c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdf59ed672d7e48ea"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2071,7 +2071,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}"/>
+  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}"/>
 </xltc:personList>
 </file>
 
@@ -2268,493 +2268,493 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="P5" dT="2026-08-15T14:19:02.132" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B010C51E-1279-1014-33BC-2602466A0653}">
+  <xltc:threadedComment ref="P5" dT="2026-08-15T14:25:31.982" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{19394B01-E00F-53AA-5F9F-DAAE5B249735}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P6" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{C1FCCBE0-DA45-F004-62DE-931492BB7B55}">
+  <xltc:threadedComment ref="P6" dT="2026-08-15T14:25:31.984" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{1D42977D-73AE-7F9C-73B4-25926AE6C8A1}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P7" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{AC4872FE-E925-0F71-A1A0-B51C3BE471D4}">
+  <xltc:threadedComment ref="P7" dT="2026-08-15T14:25:31.984" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{140AC83F-8B13-BB91-21C7-92173351B7FD}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P8" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{78456A9C-33CF-DC3E-ACC9-771E9401AB46}">
+  <xltc:threadedComment ref="P8" dT="2026-08-15T14:25:31.984" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{A84656BA-F870-0843-455C-366684097531}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P9" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A3652911-0C8B-2C28-FADE-73D328A5BF26}">
+  <xltc:threadedComment ref="P9" dT="2026-08-15T14:25:31.984" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{BA677552-5189-E26A-5201-2CAD593114D5}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P10" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{6F2EBCD8-23F2-D22F-38CC-ED40EFF8AEC8}">
+  <xltc:threadedComment ref="P10" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{0D3AC6A7-2087-6C91-F3FC-49238524123A}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 119
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P11" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{92F20AFD-1D39-B8DE-5BD9-BC3E03CB8C0F}">
+  <xltc:threadedComment ref="P11" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{E8B2DFAC-DBDB-1D70-FB96-A57BB882E591}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 160
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P12" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{CA2CD762-5110-A555-E40D-9C5F0FB6D9CC}">
+  <xltc:threadedComment ref="P12" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{BBEB777E-28A0-34D9-C7CE-3E0C0793382D}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P13" dT="2026-08-15T14:19:02.134" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{9DAD665B-4B78-CB05-6BFF-8A259A25099D}">
+  <xltc:threadedComment ref="P13" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{ADC69843-37EC-D20B-3201-7C998E761773}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P14" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B404A4C9-0C5D-FB04-5F38-B466A0729AB3}">
+  <xltc:threadedComment ref="P14" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{BDBE4742-2E5F-F5FF-5F4B-89143E394265}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P15" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A778AC8E-E3EE-EF95-340F-71DE58C4379A}">
+  <xltc:threadedComment ref="P15" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{28186EC5-DD20-8D1B-177E-611D02905D17}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P16" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{CF9789CE-401E-9368-3823-F3D6EB9FB0AE}">
+  <xltc:threadedComment ref="P16" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{BAC8BFD3-8437-83A1-ADAA-3C6FF249CBC5}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P17" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{E0F7EB04-9E7A-C956-F66F-04924C0BBF6B}">
+  <xltc:threadedComment ref="P17" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{AD89F10E-24F9-800C-BA8F-E4D4E60E2600}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P18" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{432D59DF-0456-250E-3705-7E52A846CC07}">
+  <xltc:threadedComment ref="P18" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{09A3F634-8B76-FDEA-01DA-76BD9B40C5DC}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P19" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{8E40EC39-F650-2BB9-AA8A-B164C8F0D6DB}">
+  <xltc:threadedComment ref="P19" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{3C08E262-2F52-00E7-DFDC-875B7B0D6EB2}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P20" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{06B31F52-AE05-C750-E2E4-8BE8C077E3ED}">
+  <xltc:threadedComment ref="P20" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{DBE49284-42F5-EA4C-4BD7-F83AA247DE86}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 138
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P21" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{C4AB3B82-976E-0559-3794-2F2F9216C552}">
+  <xltc:threadedComment ref="P21" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{AB326A0C-B59B-FD02-5084-BB0536D0FFF8}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 212
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P22" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{3AAB5A1B-8E7D-C179-2DC1-E2DBD2705DB9}">
+  <xltc:threadedComment ref="P22" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{0E7E0B0F-050B-01DE-68E9-AB117F4B736F}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P23" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{7D66F2E6-7D62-9517-832E-57FFAA140850}">
+  <xltc:threadedComment ref="P23" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{B9AB9439-79A4-44E8-233A-BDC4B20B2561}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P24" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{01EA68F6-A6AF-EEF9-FC79-C83DFF706D5F}">
+  <xltc:threadedComment ref="P24" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{E7A35A0C-1940-0A0A-66B2-28D3BAD76624}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P25" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{7EBEBBB5-1D36-3EC8-8615-2492FBE68CC4}">
+  <xltc:threadedComment ref="P25" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{331D7CA0-CA52-FE29-30A6-EF44576A4681}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P26" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{67EA088D-22B9-ECEE-A157-D88A9B7AAFA9}">
+  <xltc:threadedComment ref="P26" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{4BA54249-5798-912A-B087-6931A573E9B2}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P27" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A2333FE9-49D5-C016-953E-7E0B47F95EF5}">
+  <xltc:threadedComment ref="P27" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{F269CB9E-DAD7-377C-B6AE-46737C2B1FF1}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 272
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P28" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{93C06E00-D895-402F-7E27-987889902425}">
+  <xltc:threadedComment ref="P28" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{D489D1BF-740A-033D-7501-81175165C33D}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P29" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{AEE536DF-8184-66AA-DD13-2B4E3E8B93C2}">
+  <xltc:threadedComment ref="P29" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{69054F3D-B908-030A-11FC-898D2FC0C7D0}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P30" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{5997CBC9-B8DA-7AF8-6285-53F3711B14B9}">
+  <xltc:threadedComment ref="P30" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{9AB7B4F9-820A-DC76-6A9D-F632F3D10365}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 158
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P31" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{626792A5-658D-324B-98D1-7D4E6DE536BD}">
+  <xltc:threadedComment ref="P31" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{232896F9-7500-E0D3-F70A-6EE4CE5F563B}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P32" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{8D7BFCFD-3E48-D195-6EB4-5521380E05C9}">
+  <xltc:threadedComment ref="P32" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{2444243E-848D-6DAA-B664-ECFC23B3EF1C}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P33" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{E15B3E52-7A06-CC45-DE2B-41A9C12FF48D}">
+  <xltc:threadedComment ref="P33" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{0DD6D8EF-35DB-0CF2-E74A-E012E6E1A9FB}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 72
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P34" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B960910A-8477-2846-1613-88C2913E5C85}">
+  <xltc:threadedComment ref="P34" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{72304EE7-ED25-9CD4-678B-EB502A085A57}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P35" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{3F019C8B-A8FF-A1C1-F480-A723F813C270}">
+  <xltc:threadedComment ref="P35" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{AACC62A3-0F19-9957-7145-4DAB6497B294}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P36" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{8B0451A6-6D51-3B85-B608-44D73A90BE00}">
+  <xltc:threadedComment ref="P36" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{E3249311-112C-5A89-889A-DDF8E4F2FE53}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 24
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P37" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{6E34B664-AA4F-7D25-5EB4-CAE4F78D331D}">
+  <xltc:threadedComment ref="P37" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{A1538091-C1CC-DD54-5406-206EC7D07274}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P38" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B2D6B7C4-FB9F-7569-768C-9F19B0EDBA9D}">
+  <xltc:threadedComment ref="P38" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{35CF49BE-ABF2-3F42-5FCD-91DFBC78DD13}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P39" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{F2C939C5-67DD-99B6-503C-636AE1C76D8C}">
+  <xltc:threadedComment ref="P39" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{95CA0DC2-6586-FC1C-2C42-C17AF3387EFC}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 19
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P40" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{091770E0-D8A8-A17E-211F-BF39D2DE3D21}">
+  <xltc:threadedComment ref="P40" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{B020CB65-337E-C3E8-BDF2-537D485963B9}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P41" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{C81BBC94-53F4-9708-39C3-5CB664703880}">
+  <xltc:threadedComment ref="P41" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{3CE09352-BDFF-41B3-5C7D-17838504BAD6}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P42" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A06A1A63-4CF5-E445-56FC-BD4A588968F1}">
+  <xltc:threadedComment ref="P42" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{010FF20E-4C5A-31F9-FD05-17751B865D53}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P43" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{CF996379-C6D9-0FBB-656E-63B1D66BAFC8}">
+  <xltc:threadedComment ref="P43" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{6FFA3CA4-6C2E-A91A-BE12-A7CEB29C5EF9}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P44" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B957E27C-1147-FAF3-74E7-EA8EC5908CC6}">
+  <xltc:threadedComment ref="P44" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{4E125750-51DA-850B-CD1B-D0D473F001F6}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P45" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{420E6EE9-F0FD-3EE6-7002-0F87931DE2C3}">
+  <xltc:threadedComment ref="P45" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{DB7B7D09-45E4-8974-B566-9C42E8A66070}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P46" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{72E4C9A4-FDB4-C94D-DCDC-B2D8F3FC1E58}">
+  <xltc:threadedComment ref="P46" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{DFA5C51F-06D5-BA4F-608D-865B6B3F0E8D}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P47" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{1CB140F6-0570-D58E-D0A8-4551FD74BA90}">
+  <xltc:threadedComment ref="P47" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{E14B8F74-ABA3-1B58-B20D-5F43358ACADA}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P48" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{4C23F7C6-D3C7-A4BE-F36C-2F5E0923875B}">
+  <xltc:threadedComment ref="P48" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{94123791-288B-7DEE-DBEE-A50EAF2CEF3A}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P49" dT="2026-08-15T14:19:02.135" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A18D8527-4F44-6611-303D-A0E50FC512E3}">
+  <xltc:threadedComment ref="P49" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{60F2A683-77E6-217F-085F-8010A834277D}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 118
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P50" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{DCF389D3-4242-623B-AE66-3E44891929C8}">
+  <xltc:threadedComment ref="P50" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{5C75B7BD-F355-6365-F6A6-7F035F95D631}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P51" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{942E9BB5-C21B-6000-23BC-C0925210FA48}">
+  <xltc:threadedComment ref="P51" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{8B485069-42C9-BCF7-2564-CF877FB3332C}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P52" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B8533D65-8426-863A-B312-F367AD0B4444}">
+  <xltc:threadedComment ref="P52" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{30F59ABA-66A2-F07B-EA84-2F9EC8DC22D6}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P53" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{0886CFC9-D7DE-1471-513A-71A37582BE87}">
+  <xltc:threadedComment ref="P53" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{4E18A03C-4BA4-7217-8027-9B09EB09244A}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-STF</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P54" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{BCB573C2-22CD-DDD1-A5ED-1DC2F5CE50B5}">
+  <xltc:threadedComment ref="P54" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{83C78788-EEEE-C237-020B-AE43B435EC46}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P55" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{E9D0B5CE-5209-E0BE-3237-DB8B632D7235}">
+  <xltc:threadedComment ref="P55" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{55E4FEE1-9B5B-E551-7070-77A55CA1826E}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P56" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B704E177-02B4-47FB-A7F9-206D3C4F097F}">
+  <xltc:threadedComment ref="P56" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{77B71704-FA27-C535-F961-039BDB63EC0E}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 18
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P57" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{6F3A1B45-FF5A-DF64-19ED-AA0695469814}">
+  <xltc:threadedComment ref="P57" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{CD5687F0-0DDF-839C-1C45-7E3BB7495273}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P58" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{ACCA67AD-3C83-ACC1-2D98-C4C6D0AFD638}">
+  <xltc:threadedComment ref="P58" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{AEC31414-5E16-DD3D-89F8-40EE87A1C59D}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P59" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B238E13A-91E5-5386-8C34-F67463D45FB1}">
+  <xltc:threadedComment ref="P59" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{6864D662-D838-948E-F2EF-F5F5FB71DE9B}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P60" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{C0BA2EF8-C1B1-64BE-3EA0-F77C4E23AD4C}">
+  <xltc:threadedComment ref="P60" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{3C9BE7BE-F9BA-CFAE-C694-1568251BE342}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P61" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{9E7079E2-8399-4258-574A-B9F9C79E592C}">
+  <xltc:threadedComment ref="P61" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{3C7B18CA-C167-B6B3-E28B-BA081E641EA3}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P62" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{4D4A8E67-5958-A3C1-70C2-33CB58A773FF}">
+  <xltc:threadedComment ref="P62" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{A0F88A35-48DA-EE36-C7D1-AA9702B6245E}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P63" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{0CA8FE98-EDDA-A7FC-8A90-7852EAD6A4FF}">
+  <xltc:threadedComment ref="P63" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{96C28C0B-4897-01F2-1C3C-EC1BD1A4C594}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P64" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{C13917A4-524D-2A26-A42D-6D16A66166CA}">
+  <xltc:threadedComment ref="P64" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{4EBD50A2-D0F8-C104-9A27-FDB811B9F2F1}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P65" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{C4039E66-57C0-F444-53E6-FCCF8A6DA3E9}">
+  <xltc:threadedComment ref="P65" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{2BAE9845-5089-4FB2-9155-03120E278CD5}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 311
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P66" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{03D96BF4-9AE3-9DF8-CC14-62B6DA87E1BA}">
+  <xltc:threadedComment ref="P66" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{0DBB817D-C9F7-F450-6447-4B61420F33C6}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P67" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{68867B5D-2E79-11B5-AD2B-6426A7112DA5}">
+  <xltc:threadedComment ref="P67" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{0C8DE577-8367-42EE-9B4B-A13AD3846F90}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P68" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{54A9DCF0-8852-0B11-508D-950C7B9284A4}">
+  <xltc:threadedComment ref="P68" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{8A1603E1-6F97-4B78-AF27-CFDF20B95D58}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 141
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P69" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{22D8A23D-9682-E3ED-C9FB-E779AA2720B1}">
+  <xltc:threadedComment ref="P69" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{BA6A8336-F4DF-E87C-DF14-F79812F1411D}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P70" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{91E699CE-9A06-219F-5833-E4E864BED089}">
+  <xltc:threadedComment ref="P70" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{6EE3B779-CB9D-65F9-3D25-66C174840379}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P71" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{F8EB5DB1-1D5C-47D0-D1DD-184B283C0C6C}">
+  <xltc:threadedComment ref="P71" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{EF88ABD5-BC27-CCC3-B3CA-7FC32267D4AF}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 33
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P72" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{6EF67E32-E7EC-94F6-3F4E-584F0BE95656}">
+  <xltc:threadedComment ref="P72" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{F33C65C3-F551-D2AC-D628-FB5B78181AA7}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P73" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{99F57B06-4D37-016A-C483-B1735DED682F}">
+  <xltc:threadedComment ref="P73" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{AFDB57BC-1227-DC20-5E62-FEE3E8445830}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P74" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{5D7317F8-C323-677A-8020-3361BEEEB812}">
+  <xltc:threadedComment ref="P74" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{F48AC48A-7628-95B7-FD95-B1B568391ACE}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 21
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P75" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{513B22C5-53D5-D9FA-E2B0-84DC9C63BD75}">
+  <xltc:threadedComment ref="P75" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{AE9CAB17-F322-2981-065F-C74301AD1B41}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P76" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{C676EC9E-9A20-A1B2-3E1F-20A28A26A61A}">
+  <xltc:threadedComment ref="P76" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{0F39D044-4F3C-9712-7B3C-A13B1A8FD36C}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P77" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{BD7320DD-EB8C-3619-ABDC-27A23A838BFD}">
+  <xltc:threadedComment ref="P77" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{B7C788FE-7A08-37E9-F12A-9DA325EF5877}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 19
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P78" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{DCCE526A-71D7-E02C-4253-8778B920726E}">
+  <xltc:threadedComment ref="P78" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{D60815FD-2FC4-EDF0-84D3-3A5E4E44F184}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 43
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P79" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{33C6E653-4ECD-66D3-31ED-37F8D530BBCA}">
+  <xltc:threadedComment ref="P79" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{205EB334-F928-87C4-D82E-FEA9BA425AC5}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 44
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P80" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{2D51D488-F2CD-1656-7FC5-C0BE0926F124}">
+  <xltc:threadedComment ref="P80" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{F78CFAC1-E06B-9C87-763A-B4860DBAB1B8}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 40
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P81" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{620305EA-1DAC-09F1-F096-0BEF7B4B8CA1}">
+  <xltc:threadedComment ref="P81" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{0472304C-FEC5-1785-6CC1-52C96690EE46}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P82" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{E5082642-40DD-D305-F257-8AEF1B0F3468}">
+  <xltc:threadedComment ref="P82" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{4207741A-DE03-1BE3-B143-1BA6BF02C297}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P83" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A227902C-BE3D-E28E-3D70-D78E36E76664}">
+  <xltc:threadedComment ref="P83" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{CAE4E73D-84BC-45FB-7B6A-FF3CC4C999F3}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 16
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P84" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{8DC1750F-5595-5639-B653-027050CAA390}">
+  <xltc:threadedComment ref="P84" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{7F3E3A0C-214E-A648-AB74-D12724638463}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P85" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{DD3E8D93-9C02-6410-C382-7C25C24F3F42}">
+  <xltc:threadedComment ref="P85" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{8FB32A91-0D5B-4485-EE74-CB324EAF6F28}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P86" dT="2026-08-15T14:19:02.136" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{83154AE6-98B5-8AE9-06F0-2B1446B9C581}">
+  <xltc:threadedComment ref="P86" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{50FD3967-A051-5A71-20A1-A86789127CCB}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 21
 Available: 2026-02-25
@@ -2765,64 +2765,64 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="J5" dT="2026-08-15T14:19:02.445" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{98531AC1-4941-7A52-E013-EE7B6AE34866}">
+  <xltc:threadedComment ref="J5" dT="2026-08-15T14:25:32.296" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{F1DDF034-E12A-7BB5-8B27-8E0A77990B7F}">
     <xltc:text>Official source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J6" dT="2026-08-15T14:19:02.447" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{D157483F-6BDA-7F1C-DCCF-23C8E64A35F7}">
+  <xltc:threadedComment ref="J6" dT="2026-08-15T14:25:32.298" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{A27FE3CE-58EE-9146-F293-955465F0CB1F}">
     <xltc:text>Official source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J7" dT="2026-08-15T14:19:02.451" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{552A1BEC-EA87-5403-5908-968977F501D8}">
+  <xltc:threadedComment ref="J7" dT="2026-08-15T14:25:32.302" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{6A50C978-5309-D064-EBC6-23A94A3EE4D1}">
     <xltc:text>Official source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J8" dT="2026-08-15T14:19:02.453" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A3DA3D31-7AAA-72A0-4EF5-95EFCC71CD2B}">
+  <xltc:threadedComment ref="J8" dT="2026-08-15T14:25:32.304" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{A3E41E1D-2961-84E0-42EC-35FFFE6CA772}">
     <xltc:text>Official source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J9" dT="2026-08-15T14:19:02.456" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{76E3920F-E519-3C1E-3E0D-4BD1A2A66133}">
+  <xltc:threadedComment ref="J9" dT="2026-08-15T14:25:32.307" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{82EEAB1F-45E5-5945-F994-799D5FCA8249}">
     <xltc:text>Official source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J10" dT="2026-08-15T14:19:02.458" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{5E262495-50B1-C8A9-AA8E-A574EC7E8A3D}">
+  <xltc:threadedComment ref="J10" dT="2026-08-15T14:25:32.309" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{EA451E30-939F-5824-3AD2-283825979700}">
     <xltc:text>Official source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J11" dT="2026-08-15T14:19:02.46" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{7EB79C36-B5A2-F049-7BDF-9F3B596F6820}">
+  <xltc:threadedComment ref="J11" dT="2026-08-15T14:25:32.311" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{3D4150B1-DB11-5A7D-AE29-0347DFB19553}">
     <xltc:text>Official source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J12" dT="2026-08-15T14:19:02.463" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{22CB9419-E586-D4C1-50B9-A021EC148AC5}">
+  <xltc:threadedComment ref="J12" dT="2026-08-15T14:25:32.313" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{179A041E-8A29-CDE7-B9A2-A6340557FF6D}">
     <xltc:text>Official source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J13" dT="2026-08-15T14:19:02.466" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{620B1091-CEB4-C37C-3382-EE621929B02A}">
+  <xltc:threadedComment ref="J13" dT="2026-08-15T14:25:32.314" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{6414D9D1-981F-0106-FC22-A83B835227BF}">
     <xltc:text>Official source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J14" dT="2026-08-15T14:19:02.47" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{1405AEF0-4174-F4F3-F1A4-C31A5255643D}">
+  <xltc:threadedComment ref="J14" dT="2026-08-15T14:25:32.316" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{003A8738-F53E-F29A-4836-83CD88CBD5D3}">
     <xltc:text>Official source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J15" dT="2026-08-15T14:19:02.472" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{B66A228C-307C-CC5B-C01D-0898704EE8A3}">
+  <xltc:threadedComment ref="J15" dT="2026-08-15T14:25:32.317" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{52A80459-605E-DE47-A560-B5294919DA3A}">
     <xltc:text>Official source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J16" dT="2026-08-15T14:19:02.476" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{AA3B7332-904E-A09B-2432-C36A1595C35A}">
+  <xltc:threadedComment ref="J16" dT="2026-08-15T14:25:32.319" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{EA49137A-B2C3-1699-19C1-386362AAD204}">
     <xltc:text>Official source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J17" dT="2026-08-15T14:19:02.477" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{58E0E191-E399-7CE9-F247-C1CFF9615D23}">
+  <xltc:threadedComment ref="J17" dT="2026-08-15T14:25:32.321" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{A743B0C9-B331-3FE6-5A9C-7368C8C621E3}">
     <xltc:text>Official source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J18" dT="2026-08-15T14:19:02.479" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{E1D11912-9D5F-2807-3A5F-26545A058958}">
+  <xltc:threadedComment ref="J18" dT="2026-08-15T14:25:32.324" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{B9A0315D-4AA7-FF04-062A-23F5A3A8C057}">
     <xltc:text>Official source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J19" dT="2026-08-15T14:19:02.481" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{8C849A78-52FB-4F6A-C60B-5C3DD9A318B8}">
+  <xltc:threadedComment ref="J19" dT="2026-08-15T14:25:32.326" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{58F44AC5-131C-E73F-2EF9-0F03167CE636}">
     <xltc:text>Official source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J20" dT="2026-08-15T14:19:02.484" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A8EB206C-B5DF-647E-1A30-B65652F54204}">
+  <xltc:threadedComment ref="J20" dT="2026-08-15T14:25:32.328" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{03872F08-FCC4-073E-DCF7-71462B38E10F}">
     <xltc:text>Official source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J21" dT="2026-08-15T14:19:02.486" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{A281D42C-43AC-B97E-892E-1520D6E7A5F3}">
+  <xltc:threadedComment ref="J21" dT="2026-08-15T14:25:32.33" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{53B86A32-AD64-73D4-6684-A35D7850F2AB}">
     <xltc:text>Official source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J22" dT="2026-08-15T14:19:02.487" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{AD9FEFBE-F579-CDA9-FC02-DD01D955F713}">
+  <xltc:threadedComment ref="J22" dT="2026-08-15T14:25:32.331" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{EDD1FBE0-9C7B-8E26-0237-3229A3282A1E}">
     <xltc:text>Official source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J23" dT="2026-08-15T14:19:02.489" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{28D2157A-9BBF-4F6E-79EF-FA7ECA05A5C8}">
+  <xltc:threadedComment ref="J23" dT="2026-08-15T14:25:32.333" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{7F8E6C93-4097-9C02-87A3-623D41D62A58}">
     <xltc:text>Official source: https://www.aspenpharma.com/download/annual-financial-statements-2/</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J24" dT="2026-08-15T14:19:02.491" personId="{BDE9FFFE-8BC2-4317-A3B7-E3281AEF22D2}" id="{3DE68A57-0B2F-A77D-77DF-55430FAAA6F7}">
+  <xltc:threadedComment ref="J24" dT="2026-08-15T14:25:32.335" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{12A5D7D5-7F54-1EE0-1CAD-41DE6B533C67}">
     <xltc:text>Official source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -3877,7 +3877,7 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f41b2e2cafc4af8"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52d299b37d534f47"/>
 </x:worksheet>
 </file>
 
@@ -8611,7 +8611,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c0baf671f3c4ecb"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61e4ea28e4d94631"/>
 </x:worksheet>
 </file>
 
@@ -9671,7 +9671,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb56dd16d91fa437d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d3b1e7973b34151"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Normalize cross-platform presentation provenance
</commit_message>
<xml_diff>
--- a/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
+++ b/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R886ca569ce0f4ff3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R8a98d8abaa2d444f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="R20915aa5a6a045f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Ra739eb80933c41b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R06c7793f53ca43ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R629ff89fcfc14280"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R3695fa6daf0b4fa2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="R13ff4ef65ee04163"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R800728acfd374c23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R37349b6bb9a4454e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R5ac3e9ad10e94c46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="Re405443f102a4561"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="R9d2f9c0d3f9d4b07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="R40205d2538e34e8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R0798a282546d40f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R70493432f9204b35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R211da85b2f5441fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="Rd8f1816cfdfc445d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R9e3ddb93ccef4256"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R6e3252a1afe044be"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,88 +19,88 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={19394B01-E00F-53AA-5F9F-DAAE5B249735}</x:author>
-    <x:author>tc={1D42977D-73AE-7F9C-73B4-25926AE6C8A1}</x:author>
-    <x:author>tc={140AC83F-8B13-BB91-21C7-92173351B7FD}</x:author>
-    <x:author>tc={A84656BA-F870-0843-455C-366684097531}</x:author>
-    <x:author>tc={BA677552-5189-E26A-5201-2CAD593114D5}</x:author>
-    <x:author>tc={0D3AC6A7-2087-6C91-F3FC-49238524123A}</x:author>
-    <x:author>tc={E8B2DFAC-DBDB-1D70-FB96-A57BB882E591}</x:author>
-    <x:author>tc={BBEB777E-28A0-34D9-C7CE-3E0C0793382D}</x:author>
-    <x:author>tc={ADC69843-37EC-D20B-3201-7C998E761773}</x:author>
-    <x:author>tc={BDBE4742-2E5F-F5FF-5F4B-89143E394265}</x:author>
-    <x:author>tc={28186EC5-DD20-8D1B-177E-611D02905D17}</x:author>
-    <x:author>tc={BAC8BFD3-8437-83A1-ADAA-3C6FF249CBC5}</x:author>
-    <x:author>tc={AD89F10E-24F9-800C-BA8F-E4D4E60E2600}</x:author>
-    <x:author>tc={09A3F634-8B76-FDEA-01DA-76BD9B40C5DC}</x:author>
-    <x:author>tc={3C08E262-2F52-00E7-DFDC-875B7B0D6EB2}</x:author>
-    <x:author>tc={DBE49284-42F5-EA4C-4BD7-F83AA247DE86}</x:author>
-    <x:author>tc={AB326A0C-B59B-FD02-5084-BB0536D0FFF8}</x:author>
-    <x:author>tc={0E7E0B0F-050B-01DE-68E9-AB117F4B736F}</x:author>
-    <x:author>tc={B9AB9439-79A4-44E8-233A-BDC4B20B2561}</x:author>
-    <x:author>tc={E7A35A0C-1940-0A0A-66B2-28D3BAD76624}</x:author>
-    <x:author>tc={331D7CA0-CA52-FE29-30A6-EF44576A4681}</x:author>
-    <x:author>tc={4BA54249-5798-912A-B087-6931A573E9B2}</x:author>
-    <x:author>tc={F269CB9E-DAD7-377C-B6AE-46737C2B1FF1}</x:author>
-    <x:author>tc={D489D1BF-740A-033D-7501-81175165C33D}</x:author>
-    <x:author>tc={69054F3D-B908-030A-11FC-898D2FC0C7D0}</x:author>
-    <x:author>tc={9AB7B4F9-820A-DC76-6A9D-F632F3D10365}</x:author>
-    <x:author>tc={232896F9-7500-E0D3-F70A-6EE4CE5F563B}</x:author>
-    <x:author>tc={2444243E-848D-6DAA-B664-ECFC23B3EF1C}</x:author>
-    <x:author>tc={0DD6D8EF-35DB-0CF2-E74A-E012E6E1A9FB}</x:author>
-    <x:author>tc={72304EE7-ED25-9CD4-678B-EB502A085A57}</x:author>
-    <x:author>tc={AACC62A3-0F19-9957-7145-4DAB6497B294}</x:author>
-    <x:author>tc={E3249311-112C-5A89-889A-DDF8E4F2FE53}</x:author>
-    <x:author>tc={A1538091-C1CC-DD54-5406-206EC7D07274}</x:author>
-    <x:author>tc={35CF49BE-ABF2-3F42-5FCD-91DFBC78DD13}</x:author>
-    <x:author>tc={95CA0DC2-6586-FC1C-2C42-C17AF3387EFC}</x:author>
-    <x:author>tc={B020CB65-337E-C3E8-BDF2-537D485963B9}</x:author>
-    <x:author>tc={3CE09352-BDFF-41B3-5C7D-17838504BAD6}</x:author>
-    <x:author>tc={010FF20E-4C5A-31F9-FD05-17751B865D53}</x:author>
-    <x:author>tc={6FFA3CA4-6C2E-A91A-BE12-A7CEB29C5EF9}</x:author>
-    <x:author>tc={4E125750-51DA-850B-CD1B-D0D473F001F6}</x:author>
-    <x:author>tc={DB7B7D09-45E4-8974-B566-9C42E8A66070}</x:author>
-    <x:author>tc={DFA5C51F-06D5-BA4F-608D-865B6B3F0E8D}</x:author>
-    <x:author>tc={E14B8F74-ABA3-1B58-B20D-5F43358ACADA}</x:author>
-    <x:author>tc={94123791-288B-7DEE-DBEE-A50EAF2CEF3A}</x:author>
-    <x:author>tc={60F2A683-77E6-217F-085F-8010A834277D}</x:author>
-    <x:author>tc={5C75B7BD-F355-6365-F6A6-7F035F95D631}</x:author>
-    <x:author>tc={8B485069-42C9-BCF7-2564-CF877FB3332C}</x:author>
-    <x:author>tc={30F59ABA-66A2-F07B-EA84-2F9EC8DC22D6}</x:author>
-    <x:author>tc={4E18A03C-4BA4-7217-8027-9B09EB09244A}</x:author>
-    <x:author>tc={83C78788-EEEE-C237-020B-AE43B435EC46}</x:author>
-    <x:author>tc={55E4FEE1-9B5B-E551-7070-77A55CA1826E}</x:author>
-    <x:author>tc={77B71704-FA27-C535-F961-039BDB63EC0E}</x:author>
-    <x:author>tc={CD5687F0-0DDF-839C-1C45-7E3BB7495273}</x:author>
-    <x:author>tc={AEC31414-5E16-DD3D-89F8-40EE87A1C59D}</x:author>
-    <x:author>tc={6864D662-D838-948E-F2EF-F5F5FB71DE9B}</x:author>
-    <x:author>tc={3C9BE7BE-F9BA-CFAE-C694-1568251BE342}</x:author>
-    <x:author>tc={3C7B18CA-C167-B6B3-E28B-BA081E641EA3}</x:author>
-    <x:author>tc={A0F88A35-48DA-EE36-C7D1-AA9702B6245E}</x:author>
-    <x:author>tc={96C28C0B-4897-01F2-1C3C-EC1BD1A4C594}</x:author>
-    <x:author>tc={4EBD50A2-D0F8-C104-9A27-FDB811B9F2F1}</x:author>
-    <x:author>tc={2BAE9845-5089-4FB2-9155-03120E278CD5}</x:author>
-    <x:author>tc={0DBB817D-C9F7-F450-6447-4B61420F33C6}</x:author>
-    <x:author>tc={0C8DE577-8367-42EE-9B4B-A13AD3846F90}</x:author>
-    <x:author>tc={8A1603E1-6F97-4B78-AF27-CFDF20B95D58}</x:author>
-    <x:author>tc={BA6A8336-F4DF-E87C-DF14-F79812F1411D}</x:author>
-    <x:author>tc={6EE3B779-CB9D-65F9-3D25-66C174840379}</x:author>
-    <x:author>tc={EF88ABD5-BC27-CCC3-B3CA-7FC32267D4AF}</x:author>
-    <x:author>tc={F33C65C3-F551-D2AC-D628-FB5B78181AA7}</x:author>
-    <x:author>tc={AFDB57BC-1227-DC20-5E62-FEE3E8445830}</x:author>
-    <x:author>tc={F48AC48A-7628-95B7-FD95-B1B568391ACE}</x:author>
-    <x:author>tc={AE9CAB17-F322-2981-065F-C74301AD1B41}</x:author>
-    <x:author>tc={0F39D044-4F3C-9712-7B3C-A13B1A8FD36C}</x:author>
-    <x:author>tc={B7C788FE-7A08-37E9-F12A-9DA325EF5877}</x:author>
-    <x:author>tc={D60815FD-2FC4-EDF0-84D3-3A5E4E44F184}</x:author>
-    <x:author>tc={205EB334-F928-87C4-D82E-FEA9BA425AC5}</x:author>
-    <x:author>tc={F78CFAC1-E06B-9C87-763A-B4860DBAB1B8}</x:author>
-    <x:author>tc={0472304C-FEC5-1785-6CC1-52C96690EE46}</x:author>
-    <x:author>tc={4207741A-DE03-1BE3-B143-1BA6BF02C297}</x:author>
-    <x:author>tc={CAE4E73D-84BC-45FB-7B6A-FF3CC4C999F3}</x:author>
-    <x:author>tc={7F3E3A0C-214E-A648-AB74-D12724638463}</x:author>
-    <x:author>tc={8FB32A91-0D5B-4485-EE74-CB324EAF6F28}</x:author>
-    <x:author>tc={50FD3967-A051-5A71-20A1-A86789127CCB}</x:author>
+    <x:author>tc={1D3C2439-FC74-878C-F5CC-58746046E7DD}</x:author>
+    <x:author>tc={4F7AA636-1509-2E5C-DE28-B75201399C36}</x:author>
+    <x:author>tc={A0CD7F65-E81E-117D-3010-1A3C4FC7E806}</x:author>
+    <x:author>tc={2BC4F4CE-3028-E376-38C4-A45C077178D6}</x:author>
+    <x:author>tc={76EA9DBC-445A-F6C9-149B-948379B25610}</x:author>
+    <x:author>tc={0E403EE3-E209-12D7-8BE8-BE38EA659A20}</x:author>
+    <x:author>tc={77871C4C-9F32-FF56-76D1-50A3CE47932D}</x:author>
+    <x:author>tc={09EF5B64-315D-CAEF-D3B6-A613340519E8}</x:author>
+    <x:author>tc={F3076964-832D-6FBD-D1F9-7564B56EBCE0}</x:author>
+    <x:author>tc={18C726D0-AA21-F490-84A5-71DB293A0C81}</x:author>
+    <x:author>tc={00894FF3-35F3-A1B1-9AA8-919CE49171F6}</x:author>
+    <x:author>tc={B353F4D8-5FFA-1545-40A6-FC8A27BB12AD}</x:author>
+    <x:author>tc={0B0729F6-5064-5F9D-2C55-23A49C0C3BDF}</x:author>
+    <x:author>tc={561A2902-D66D-F16E-E875-B7F800F6DE67}</x:author>
+    <x:author>tc={04513763-CC95-6FB5-A722-817CEE7F4448}</x:author>
+    <x:author>tc={5EF56C96-5B69-E27F-A7E1-39D4A3249AF6}</x:author>
+    <x:author>tc={7B1AE671-4D9A-C858-A69E-ED2AFA642A73}</x:author>
+    <x:author>tc={AC0117BC-E1F4-E1AA-B76E-94A004DD9A2B}</x:author>
+    <x:author>tc={7D56B634-D6AE-7A54-E4E4-59751F9EFFA4}</x:author>
+    <x:author>tc={3D509607-46DB-7367-3162-1CF1E4AC14E5}</x:author>
+    <x:author>tc={7273B247-70AB-04AF-C8F5-2CECE0DB2154}</x:author>
+    <x:author>tc={51C26273-DA34-381A-AAA1-1ECF5361C5E3}</x:author>
+    <x:author>tc={872C1AB3-1D16-04B8-606E-94AD13555A92}</x:author>
+    <x:author>tc={E79D887C-4BBA-0E20-9459-5A62A87E70F1}</x:author>
+    <x:author>tc={7046CB68-34C3-4D68-4F2E-C72388D9B45C}</x:author>
+    <x:author>tc={17B572EE-F697-8A66-04F7-87A62EA99760}</x:author>
+    <x:author>tc={C3E6A717-103F-8456-AC9B-C1175D5A8D47}</x:author>
+    <x:author>tc={FAEDA356-D777-0F8D-E232-2190C749AB82}</x:author>
+    <x:author>tc={BDAA3432-17AD-9F84-A992-3486F4D0812C}</x:author>
+    <x:author>tc={7096F403-3B9B-74B0-DDAC-4627E2727349}</x:author>
+    <x:author>tc={88122F83-F833-65D9-2D99-C170BFF1392E}</x:author>
+    <x:author>tc={27F15BE4-3771-AFF2-BF41-321B1E49DE21}</x:author>
+    <x:author>tc={2E6D83D0-C451-4B7D-2947-32079232326B}</x:author>
+    <x:author>tc={DE1C6661-BA06-94A6-774C-502B82A55C16}</x:author>
+    <x:author>tc={5382E1A5-60EF-6617-E10A-2C7E2B01057A}</x:author>
+    <x:author>tc={AE187217-C536-9ACE-B5BD-4ED40B01AF40}</x:author>
+    <x:author>tc={3DCAEE3E-C8CC-9B34-BA33-5ED9926790F1}</x:author>
+    <x:author>tc={029C4BF4-C621-DCAF-AA85-04C011CBCBEF}</x:author>
+    <x:author>tc={8DCE8E91-9F14-EFA4-2258-38657ACF07D6}</x:author>
+    <x:author>tc={244F49B3-5E2A-EFF5-741E-4212B12BEFD8}</x:author>
+    <x:author>tc={08875AF0-1E94-BD18-36F2-7FD2B7B8CDC3}</x:author>
+    <x:author>tc={454D49F2-E141-4C9B-8888-AF85F24D5231}</x:author>
+    <x:author>tc={99D865B6-8236-D481-618A-183EED9AD1C6}</x:author>
+    <x:author>tc={32F6D986-C933-3A46-379A-2E7F9DA41503}</x:author>
+    <x:author>tc={C36D4AF8-6A63-ECEE-4C92-630427FD9946}</x:author>
+    <x:author>tc={A65E46BB-285D-2221-F52B-39DD2024B265}</x:author>
+    <x:author>tc={9FDF306B-B63B-0B4A-D97E-4E8BF3989E3C}</x:author>
+    <x:author>tc={0DE09241-7611-CE47-83C3-C6E2A7213D83}</x:author>
+    <x:author>tc={15FAE1BB-C7E1-0F2E-87B6-517512B3FAE7}</x:author>
+    <x:author>tc={16D0131A-22BB-5957-7DBE-4B3D4AC9E90F}</x:author>
+    <x:author>tc={AF3C113F-B419-4CAA-8AAC-97EB9E101504}</x:author>
+    <x:author>tc={12838B92-4969-AF76-89D2-09087AE8BE65}</x:author>
+    <x:author>tc={13D8AF17-1334-372C-540D-57229F735583}</x:author>
+    <x:author>tc={6F2114EA-4845-2E1A-D087-9257AA50DFD9}</x:author>
+    <x:author>tc={286E08B1-D255-CC53-FE49-22D8F3030644}</x:author>
+    <x:author>tc={D14CF8CC-BDEA-A800-CDE3-48664676FEE7}</x:author>
+    <x:author>tc={D6BDBFE5-356C-B17F-F44F-DAA01D856D02}</x:author>
+    <x:author>tc={24905B2F-F9AE-274F-72BA-8F54DCE7E670}</x:author>
+    <x:author>tc={0732FFA9-94E7-87B5-4F7F-4AEAC96F7BD4}</x:author>
+    <x:author>tc={D2768598-BCCC-945F-3081-2DDA076AC7B5}</x:author>
+    <x:author>tc={D01A5B5D-1357-61AA-D4A2-AD9A45DD0A29}</x:author>
+    <x:author>tc={306D1132-835F-2461-847B-25DE4DB9FAEA}</x:author>
+    <x:author>tc={33464B4C-C331-D9FA-3DD2-CF201C835D67}</x:author>
+    <x:author>tc={D5279CD2-E00F-B95B-4DC2-7BAC89393443}</x:author>
+    <x:author>tc={FA50F35F-1B8C-76C5-ABC3-5AE659E19D2A}</x:author>
+    <x:author>tc={8CED9D41-7A2D-379A-125F-22DCA8021657}</x:author>
+    <x:author>tc={D8B5ED89-4462-4852-E22E-220F763A0477}</x:author>
+    <x:author>tc={EC330868-4883-AA27-0953-CD4A48E1ADF3}</x:author>
+    <x:author>tc={B12A67A1-C569-A860-97FB-BC8182C6D95E}</x:author>
+    <x:author>tc={D35606E1-B3C6-654B-C080-751905F8D3EF}</x:author>
+    <x:author>tc={A67054DF-4000-C49A-6A04-26F573EFEE52}</x:author>
+    <x:author>tc={09A5EB70-BF1F-34F1-64B2-5817DC85674B}</x:author>
+    <x:author>tc={323B98CD-2990-3DDC-6A40-15D2694A87DB}</x:author>
+    <x:author>tc={E094BE2E-BB68-693E-C1B2-B5B9891A05F1}</x:author>
+    <x:author>tc={17C77E87-BB03-92C5-C663-BF9FF11590A3}</x:author>
+    <x:author>tc={9C93F06B-74ED-F293-5E3E-FCB1407B9776}</x:author>
+    <x:author>tc={645E15D3-D9E0-480F-F123-03CDE49AABA9}</x:author>
+    <x:author>tc={ADF298A1-1553-FA00-3AE9-13140404D18D}</x:author>
+    <x:author>tc={145948C2-1781-1C6D-AD20-AD2A4E75E6CA}</x:author>
+    <x:author>tc={68C23CBB-2408-CE14-3F39-48E9043543CB}</x:author>
+    <x:author>tc={105C36BC-F67F-B935-902B-87430FB850C8}</x:author>
+    <x:author>tc={74A4F098-CABD-0354-4F0F-EBA77AA25914}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="P5" authorId="0">
@@ -1176,26 +1176,26 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={F1DDF034-E12A-7BB5-8B27-8E0A77990B7F}</x:author>
-    <x:author>tc={A27FE3CE-58EE-9146-F293-955465F0CB1F}</x:author>
-    <x:author>tc={6A50C978-5309-D064-EBC6-23A94A3EE4D1}</x:author>
-    <x:author>tc={A3E41E1D-2961-84E0-42EC-35FFFE6CA772}</x:author>
-    <x:author>tc={82EEAB1F-45E5-5945-F994-799D5FCA8249}</x:author>
-    <x:author>tc={EA451E30-939F-5824-3AD2-283825979700}</x:author>
-    <x:author>tc={3D4150B1-DB11-5A7D-AE29-0347DFB19553}</x:author>
-    <x:author>tc={179A041E-8A29-CDE7-B9A2-A6340557FF6D}</x:author>
-    <x:author>tc={6414D9D1-981F-0106-FC22-A83B835227BF}</x:author>
-    <x:author>tc={003A8738-F53E-F29A-4836-83CD88CBD5D3}</x:author>
-    <x:author>tc={52A80459-605E-DE47-A560-B5294919DA3A}</x:author>
-    <x:author>tc={EA49137A-B2C3-1699-19C1-386362AAD204}</x:author>
-    <x:author>tc={A743B0C9-B331-3FE6-5A9C-7368C8C621E3}</x:author>
-    <x:author>tc={B9A0315D-4AA7-FF04-062A-23F5A3A8C057}</x:author>
-    <x:author>tc={58F44AC5-131C-E73F-2EF9-0F03167CE636}</x:author>
-    <x:author>tc={03872F08-FCC4-073E-DCF7-71462B38E10F}</x:author>
-    <x:author>tc={53B86A32-AD64-73D4-6684-A35D7850F2AB}</x:author>
-    <x:author>tc={EDD1FBE0-9C7B-8E26-0237-3229A3282A1E}</x:author>
-    <x:author>tc={7F8E6C93-4097-9C02-87A3-623D41D62A58}</x:author>
-    <x:author>tc={12A5D7D5-7F54-1EE0-1CAD-41DE6B533C67}</x:author>
+    <x:author>tc={AB31FEAC-03E5-043B-780A-F44BF9CFCDDC}</x:author>
+    <x:author>tc={3C765B3E-DC35-B78B-4560-DAE01F8E8ACF}</x:author>
+    <x:author>tc={738792AE-B315-B455-AC29-E0F5DEF15EF3}</x:author>
+    <x:author>tc={F9AA18FF-ED7E-EB19-1A17-EDE8BB0A3971}</x:author>
+    <x:author>tc={9D8C46A8-2E04-7410-B846-E598134DD49F}</x:author>
+    <x:author>tc={04899C4D-F36B-69C9-B05A-3A58E5C22D85}</x:author>
+    <x:author>tc={B617AA04-5E42-5027-7162-06FCD4C146B9}</x:author>
+    <x:author>tc={3D900691-7755-ED89-AF3D-7A5806073765}</x:author>
+    <x:author>tc={F31C6032-2C92-F67E-09D0-3FE50F942BB7}</x:author>
+    <x:author>tc={7E3FFAD7-7692-8F3C-2AB1-915769C955C0}</x:author>
+    <x:author>tc={8D5E7050-80F6-3EDC-2079-F9038B8A87EF}</x:author>
+    <x:author>tc={9D79E362-9CBF-4382-59AB-0315583DE075}</x:author>
+    <x:author>tc={455FD18B-489F-850A-7F0C-21B99A925DFA}</x:author>
+    <x:author>tc={AC06C054-4207-3DDD-FB06-3F98FF6BE164}</x:author>
+    <x:author>tc={2BAEA3A0-B5A7-A503-3B40-8AB4A8357D2A}</x:author>
+    <x:author>tc={2697D796-9F9D-599D-00B2-9D7190A65914}</x:author>
+    <x:author>tc={D7C6A2D1-718C-3256-F2D5-7BC1FBA3B70A}</x:author>
+    <x:author>tc={656BFEF9-7580-14C9-A19D-4F50DA72122B}</x:author>
+    <x:author>tc={A0063F0A-EF17-7408-1570-B2A312DA1035}</x:author>
+    <x:author>tc={47404D22-6ACB-012B-2A94-989A531B023D}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="J5" authorId="0">
@@ -2060,7 +2060,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdf59ed672d7e48ea"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2edd2dab42be4a13"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2071,7 +2071,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}"/>
+  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}"/>
 </xltc:personList>
 </file>
 
@@ -2268,493 +2268,493 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="P5" dT="2026-08-15T14:25:31.982" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{19394B01-E00F-53AA-5F9F-DAAE5B249735}">
+  <xltc:threadedComment ref="P5" dT="2026-08-15T14:31:01.523" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{1D3C2439-FC74-878C-F5CC-58746046E7DD}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P6" dT="2026-08-15T14:25:31.984" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{1D42977D-73AE-7F9C-73B4-25926AE6C8A1}">
+  <xltc:threadedComment ref="P6" dT="2026-08-15T14:31:01.525" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{4F7AA636-1509-2E5C-DE28-B75201399C36}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P7" dT="2026-08-15T14:25:31.984" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{140AC83F-8B13-BB91-21C7-92173351B7FD}">
+  <xltc:threadedComment ref="P7" dT="2026-08-15T14:31:01.525" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{A0CD7F65-E81E-117D-3010-1A3C4FC7E806}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P8" dT="2026-08-15T14:25:31.984" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{A84656BA-F870-0843-455C-366684097531}">
+  <xltc:threadedComment ref="P8" dT="2026-08-15T14:31:01.525" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{2BC4F4CE-3028-E376-38C4-A45C077178D6}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P9" dT="2026-08-15T14:25:31.984" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{BA677552-5189-E26A-5201-2CAD593114D5}">
+  <xltc:threadedComment ref="P9" dT="2026-08-15T14:31:01.525" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{76EA9DBC-445A-F6C9-149B-948379B25610}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P10" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{0D3AC6A7-2087-6C91-F3FC-49238524123A}">
+  <xltc:threadedComment ref="P10" dT="2026-08-15T14:31:01.525" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{0E403EE3-E209-12D7-8BE8-BE38EA659A20}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 119
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P11" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{E8B2DFAC-DBDB-1D70-FB96-A57BB882E591}">
+  <xltc:threadedComment ref="P11" dT="2026-08-15T14:31:01.525" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{77871C4C-9F32-FF56-76D1-50A3CE47932D}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 160
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P12" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{BBEB777E-28A0-34D9-C7CE-3E0C0793382D}">
+  <xltc:threadedComment ref="P12" dT="2026-08-15T14:31:01.525" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{09EF5B64-315D-CAEF-D3B6-A613340519E8}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P13" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{ADC69843-37EC-D20B-3201-7C998E761773}">
+  <xltc:threadedComment ref="P13" dT="2026-08-15T14:31:01.526" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{F3076964-832D-6FBD-D1F9-7564B56EBCE0}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P14" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{BDBE4742-2E5F-F5FF-5F4B-89143E394265}">
+  <xltc:threadedComment ref="P14" dT="2026-08-15T14:31:01.526" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{18C726D0-AA21-F490-84A5-71DB293A0C81}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P15" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{28186EC5-DD20-8D1B-177E-611D02905D17}">
+  <xltc:threadedComment ref="P15" dT="2026-08-15T14:31:01.526" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{00894FF3-35F3-A1B1-9AA8-919CE49171F6}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P16" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{BAC8BFD3-8437-83A1-ADAA-3C6FF249CBC5}">
+  <xltc:threadedComment ref="P16" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{B353F4D8-5FFA-1545-40A6-FC8A27BB12AD}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P17" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{AD89F10E-24F9-800C-BA8F-E4D4E60E2600}">
+  <xltc:threadedComment ref="P17" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{0B0729F6-5064-5F9D-2C55-23A49C0C3BDF}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P18" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{09A3F634-8B76-FDEA-01DA-76BD9B40C5DC}">
+  <xltc:threadedComment ref="P18" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{561A2902-D66D-F16E-E875-B7F800F6DE67}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P19" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{3C08E262-2F52-00E7-DFDC-875B7B0D6EB2}">
+  <xltc:threadedComment ref="P19" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{04513763-CC95-6FB5-A722-817CEE7F4448}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P20" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{DBE49284-42F5-EA4C-4BD7-F83AA247DE86}">
+  <xltc:threadedComment ref="P20" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{5EF56C96-5B69-E27F-A7E1-39D4A3249AF6}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 138
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P21" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{AB326A0C-B59B-FD02-5084-BB0536D0FFF8}">
+  <xltc:threadedComment ref="P21" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{7B1AE671-4D9A-C858-A69E-ED2AFA642A73}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 212
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P22" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{0E7E0B0F-050B-01DE-68E9-AB117F4B736F}">
+  <xltc:threadedComment ref="P22" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{AC0117BC-E1F4-E1AA-B76E-94A004DD9A2B}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P23" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{B9AB9439-79A4-44E8-233A-BDC4B20B2561}">
+  <xltc:threadedComment ref="P23" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{7D56B634-D6AE-7A54-E4E4-59751F9EFFA4}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P24" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{E7A35A0C-1940-0A0A-66B2-28D3BAD76624}">
+  <xltc:threadedComment ref="P24" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{3D509607-46DB-7367-3162-1CF1E4AC14E5}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P25" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{331D7CA0-CA52-FE29-30A6-EF44576A4681}">
+  <xltc:threadedComment ref="P25" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{7273B247-70AB-04AF-C8F5-2CECE0DB2154}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P26" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{4BA54249-5798-912A-B087-6931A573E9B2}">
+  <xltc:threadedComment ref="P26" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{51C26273-DA34-381A-AAA1-1ECF5361C5E3}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P27" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{F269CB9E-DAD7-377C-B6AE-46737C2B1FF1}">
+  <xltc:threadedComment ref="P27" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{872C1AB3-1D16-04B8-606E-94AD13555A92}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 272
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P28" dT="2026-08-15T14:25:31.985" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{D489D1BF-740A-033D-7501-81175165C33D}">
+  <xltc:threadedComment ref="P28" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{E79D887C-4BBA-0E20-9459-5A62A87E70F1}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P29" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{69054F3D-B908-030A-11FC-898D2FC0C7D0}">
+  <xltc:threadedComment ref="P29" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{7046CB68-34C3-4D68-4F2E-C72388D9B45C}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P30" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{9AB7B4F9-820A-DC76-6A9D-F632F3D10365}">
+  <xltc:threadedComment ref="P30" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{17B572EE-F697-8A66-04F7-87A62EA99760}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 158
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P31" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{232896F9-7500-E0D3-F70A-6EE4CE5F563B}">
+  <xltc:threadedComment ref="P31" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{C3E6A717-103F-8456-AC9B-C1175D5A8D47}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P32" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{2444243E-848D-6DAA-B664-ECFC23B3EF1C}">
+  <xltc:threadedComment ref="P32" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{FAEDA356-D777-0F8D-E232-2190C749AB82}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P33" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{0DD6D8EF-35DB-0CF2-E74A-E012E6E1A9FB}">
+  <xltc:threadedComment ref="P33" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{BDAA3432-17AD-9F84-A992-3486F4D0812C}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 72
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P34" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{72304EE7-ED25-9CD4-678B-EB502A085A57}">
+  <xltc:threadedComment ref="P34" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{7096F403-3B9B-74B0-DDAC-4627E2727349}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P35" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{AACC62A3-0F19-9957-7145-4DAB6497B294}">
+  <xltc:threadedComment ref="P35" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{88122F83-F833-65D9-2D99-C170BFF1392E}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P36" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{E3249311-112C-5A89-889A-DDF8E4F2FE53}">
+  <xltc:threadedComment ref="P36" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{27F15BE4-3771-AFF2-BF41-321B1E49DE21}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 24
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P37" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{A1538091-C1CC-DD54-5406-206EC7D07274}">
+  <xltc:threadedComment ref="P37" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{2E6D83D0-C451-4B7D-2947-32079232326B}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P38" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{35CF49BE-ABF2-3F42-5FCD-91DFBC78DD13}">
+  <xltc:threadedComment ref="P38" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{DE1C6661-BA06-94A6-774C-502B82A55C16}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P39" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{95CA0DC2-6586-FC1C-2C42-C17AF3387EFC}">
+  <xltc:threadedComment ref="P39" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{5382E1A5-60EF-6617-E10A-2C7E2B01057A}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 19
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P40" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{B020CB65-337E-C3E8-BDF2-537D485963B9}">
+  <xltc:threadedComment ref="P40" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{AE187217-C536-9ACE-B5BD-4ED40B01AF40}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P41" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{3CE09352-BDFF-41B3-5C7D-17838504BAD6}">
+  <xltc:threadedComment ref="P41" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{3DCAEE3E-C8CC-9B34-BA33-5ED9926790F1}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P42" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{010FF20E-4C5A-31F9-FD05-17751B865D53}">
+  <xltc:threadedComment ref="P42" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{029C4BF4-C621-DCAF-AA85-04C011CBCBEF}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P43" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{6FFA3CA4-6C2E-A91A-BE12-A7CEB29C5EF9}">
+  <xltc:threadedComment ref="P43" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{8DCE8E91-9F14-EFA4-2258-38657ACF07D6}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P44" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{4E125750-51DA-850B-CD1B-D0D473F001F6}">
+  <xltc:threadedComment ref="P44" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{244F49B3-5E2A-EFF5-741E-4212B12BEFD8}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P45" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{DB7B7D09-45E4-8974-B566-9C42E8A66070}">
+  <xltc:threadedComment ref="P45" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{08875AF0-1E94-BD18-36F2-7FD2B7B8CDC3}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P46" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{DFA5C51F-06D5-BA4F-608D-865B6B3F0E8D}">
+  <xltc:threadedComment ref="P46" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{454D49F2-E141-4C9B-8888-AF85F24D5231}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P47" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{E14B8F74-ABA3-1B58-B20D-5F43358ACADA}">
+  <xltc:threadedComment ref="P47" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{99D865B6-8236-D481-618A-183EED9AD1C6}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P48" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{94123791-288B-7DEE-DBEE-A50EAF2CEF3A}">
+  <xltc:threadedComment ref="P48" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{32F6D986-C933-3A46-379A-2E7F9DA41503}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P49" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{60F2A683-77E6-217F-085F-8010A834277D}">
+  <xltc:threadedComment ref="P49" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{C36D4AF8-6A63-ECEE-4C92-630427FD9946}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 118
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P50" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{5C75B7BD-F355-6365-F6A6-7F035F95D631}">
+  <xltc:threadedComment ref="P50" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{A65E46BB-285D-2221-F52B-39DD2024B265}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P51" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{8B485069-42C9-BCF7-2564-CF877FB3332C}">
+  <xltc:threadedComment ref="P51" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{9FDF306B-B63B-0B4A-D97E-4E8BF3989E3C}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P52" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{30F59ABA-66A2-F07B-EA84-2F9EC8DC22D6}">
+  <xltc:threadedComment ref="P52" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{0DE09241-7611-CE47-83C3-C6E2A7213D83}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P53" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{4E18A03C-4BA4-7217-8027-9B09EB09244A}">
+  <xltc:threadedComment ref="P53" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{15FAE1BB-C7E1-0F2E-87B6-517512B3FAE7}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-STF</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P54" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{83C78788-EEEE-C237-020B-AE43B435EC46}">
+  <xltc:threadedComment ref="P54" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{16D0131A-22BB-5957-7DBE-4B3D4AC9E90F}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P55" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{55E4FEE1-9B5B-E551-7070-77A55CA1826E}">
+  <xltc:threadedComment ref="P55" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{AF3C113F-B419-4CAA-8AAC-97EB9E101504}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P56" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{77B71704-FA27-C535-F961-039BDB63EC0E}">
+  <xltc:threadedComment ref="P56" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{12838B92-4969-AF76-89D2-09087AE8BE65}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 18
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P57" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{CD5687F0-0DDF-839C-1C45-7E3BB7495273}">
+  <xltc:threadedComment ref="P57" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{13D8AF17-1334-372C-540D-57229F735583}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P58" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{AEC31414-5E16-DD3D-89F8-40EE87A1C59D}">
+  <xltc:threadedComment ref="P58" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{6F2114EA-4845-2E1A-D087-9257AA50DFD9}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P59" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{6864D662-D838-948E-F2EF-F5F5FB71DE9B}">
+  <xltc:threadedComment ref="P59" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{286E08B1-D255-CC53-FE49-22D8F3030644}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P60" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{3C9BE7BE-F9BA-CFAE-C694-1568251BE342}">
+  <xltc:threadedComment ref="P60" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D14CF8CC-BDEA-A800-CDE3-48664676FEE7}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P61" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{3C7B18CA-C167-B6B3-E28B-BA081E641EA3}">
+  <xltc:threadedComment ref="P61" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D6BDBFE5-356C-B17F-F44F-DAA01D856D02}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P62" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{A0F88A35-48DA-EE36-C7D1-AA9702B6245E}">
+  <xltc:threadedComment ref="P62" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{24905B2F-F9AE-274F-72BA-8F54DCE7E670}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P63" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{96C28C0B-4897-01F2-1C3C-EC1BD1A4C594}">
+  <xltc:threadedComment ref="P63" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{0732FFA9-94E7-87B5-4F7F-4AEAC96F7BD4}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P64" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{4EBD50A2-D0F8-C104-9A27-FDB811B9F2F1}">
+  <xltc:threadedComment ref="P64" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D2768598-BCCC-945F-3081-2DDA076AC7B5}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P65" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{2BAE9845-5089-4FB2-9155-03120E278CD5}">
+  <xltc:threadedComment ref="P65" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D01A5B5D-1357-61AA-D4A2-AD9A45DD0A29}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 311
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P66" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{0DBB817D-C9F7-F450-6447-4B61420F33C6}">
+  <xltc:threadedComment ref="P66" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{306D1132-835F-2461-847B-25DE4DB9FAEA}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P67" dT="2026-08-15T14:25:31.986" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{0C8DE577-8367-42EE-9B4B-A13AD3846F90}">
+  <xltc:threadedComment ref="P67" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{33464B4C-C331-D9FA-3DD2-CF201C835D67}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P68" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{8A1603E1-6F97-4B78-AF27-CFDF20B95D58}">
+  <xltc:threadedComment ref="P68" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D5279CD2-E00F-B95B-4DC2-7BAC89393443}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 141
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P69" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{BA6A8336-F4DF-E87C-DF14-F79812F1411D}">
+  <xltc:threadedComment ref="P69" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{FA50F35F-1B8C-76C5-ABC3-5AE659E19D2A}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P70" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{6EE3B779-CB9D-65F9-3D25-66C174840379}">
+  <xltc:threadedComment ref="P70" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{8CED9D41-7A2D-379A-125F-22DCA8021657}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P71" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{EF88ABD5-BC27-CCC3-B3CA-7FC32267D4AF}">
+  <xltc:threadedComment ref="P71" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D8B5ED89-4462-4852-E22E-220F763A0477}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 33
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P72" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{F33C65C3-F551-D2AC-D628-FB5B78181AA7}">
+  <xltc:threadedComment ref="P72" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{EC330868-4883-AA27-0953-CD4A48E1ADF3}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P73" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{AFDB57BC-1227-DC20-5E62-FEE3E8445830}">
+  <xltc:threadedComment ref="P73" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{B12A67A1-C569-A860-97FB-BC8182C6D95E}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P74" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{F48AC48A-7628-95B7-FD95-B1B568391ACE}">
+  <xltc:threadedComment ref="P74" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D35606E1-B3C6-654B-C080-751905F8D3EF}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 21
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P75" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{AE9CAB17-F322-2981-065F-C74301AD1B41}">
+  <xltc:threadedComment ref="P75" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{A67054DF-4000-C49A-6A04-26F573EFEE52}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P76" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{0F39D044-4F3C-9712-7B3C-A13B1A8FD36C}">
+  <xltc:threadedComment ref="P76" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{09A5EB70-BF1F-34F1-64B2-5817DC85674B}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P77" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{B7C788FE-7A08-37E9-F12A-9DA325EF5877}">
+  <xltc:threadedComment ref="P77" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{323B98CD-2990-3DDC-6A40-15D2694A87DB}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 19
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P78" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{D60815FD-2FC4-EDF0-84D3-3A5E4E44F184}">
+  <xltc:threadedComment ref="P78" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{E094BE2E-BB68-693E-C1B2-B5B9891A05F1}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 43
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P79" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{205EB334-F928-87C4-D82E-FEA9BA425AC5}">
+  <xltc:threadedComment ref="P79" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{17C77E87-BB03-92C5-C663-BF9FF11590A3}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 44
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P80" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{F78CFAC1-E06B-9C87-763A-B4860DBAB1B8}">
+  <xltc:threadedComment ref="P80" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{9C93F06B-74ED-F293-5E3E-FCB1407B9776}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 40
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P81" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{0472304C-FEC5-1785-6CC1-52C96690EE46}">
+  <xltc:threadedComment ref="P81" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{645E15D3-D9E0-480F-F123-03CDE49AABA9}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P82" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{4207741A-DE03-1BE3-B143-1BA6BF02C297}">
+  <xltc:threadedComment ref="P82" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{ADF298A1-1553-FA00-3AE9-13140404D18D}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P83" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{CAE4E73D-84BC-45FB-7B6A-FF3CC4C999F3}">
+  <xltc:threadedComment ref="P83" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{145948C2-1781-1C6D-AD20-AD2A4E75E6CA}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 16
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P84" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{7F3E3A0C-214E-A648-AB74-D12724638463}">
+  <xltc:threadedComment ref="P84" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{68C23CBB-2408-CE14-3F39-48E9043543CB}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P85" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{8FB32A91-0D5B-4485-EE74-CB324EAF6F28}">
+  <xltc:threadedComment ref="P85" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{105C36BC-F67F-B935-902B-87430FB850C8}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P86" dT="2026-08-15T14:25:31.987" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{50FD3967-A051-5A71-20A1-A86789127CCB}">
+  <xltc:threadedComment ref="P86" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{74A4F098-CABD-0354-4F0F-EBA77AA25914}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 21
 Available: 2026-02-25
@@ -2765,64 +2765,64 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="J5" dT="2026-08-15T14:25:32.296" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{F1DDF034-E12A-7BB5-8B27-8E0A77990B7F}">
+  <xltc:threadedComment ref="J5" dT="2026-08-15T14:31:01.789" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{AB31FEAC-03E5-043B-780A-F44BF9CFCDDC}">
     <xltc:text>Official source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J6" dT="2026-08-15T14:25:32.298" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{A27FE3CE-58EE-9146-F293-955465F0CB1F}">
+  <xltc:threadedComment ref="J6" dT="2026-08-15T14:31:01.791" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{3C765B3E-DC35-B78B-4560-DAE01F8E8ACF}">
     <xltc:text>Official source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J7" dT="2026-08-15T14:25:32.302" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{6A50C978-5309-D064-EBC6-23A94A3EE4D1}">
+  <xltc:threadedComment ref="J7" dT="2026-08-15T14:31:01.793" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{738792AE-B315-B455-AC29-E0F5DEF15EF3}">
     <xltc:text>Official source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J8" dT="2026-08-15T14:25:32.304" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{A3E41E1D-2961-84E0-42EC-35FFFE6CA772}">
+  <xltc:threadedComment ref="J8" dT="2026-08-15T14:31:01.795" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{F9AA18FF-ED7E-EB19-1A17-EDE8BB0A3971}">
     <xltc:text>Official source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J9" dT="2026-08-15T14:25:32.307" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{82EEAB1F-45E5-5945-F994-799D5FCA8249}">
+  <xltc:threadedComment ref="J9" dT="2026-08-15T14:31:01.797" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{9D8C46A8-2E04-7410-B846-E598134DD49F}">
     <xltc:text>Official source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J10" dT="2026-08-15T14:25:32.309" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{EA451E30-939F-5824-3AD2-283825979700}">
+  <xltc:threadedComment ref="J10" dT="2026-08-15T14:31:01.798" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{04899C4D-F36B-69C9-B05A-3A58E5C22D85}">
     <xltc:text>Official source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J11" dT="2026-08-15T14:25:32.311" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{3D4150B1-DB11-5A7D-AE29-0347DFB19553}">
+  <xltc:threadedComment ref="J11" dT="2026-08-15T14:31:01.8" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{B617AA04-5E42-5027-7162-06FCD4C146B9}">
     <xltc:text>Official source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J12" dT="2026-08-15T14:25:32.313" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{179A041E-8A29-CDE7-B9A2-A6340557FF6D}">
+  <xltc:threadedComment ref="J12" dT="2026-08-15T14:31:01.801" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{3D900691-7755-ED89-AF3D-7A5806073765}">
     <xltc:text>Official source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J13" dT="2026-08-15T14:25:32.314" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{6414D9D1-981F-0106-FC22-A83B835227BF}">
+  <xltc:threadedComment ref="J13" dT="2026-08-15T14:31:01.802" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{F31C6032-2C92-F67E-09D0-3FE50F942BB7}">
     <xltc:text>Official source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J14" dT="2026-08-15T14:25:32.316" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{003A8738-F53E-F29A-4836-83CD88CBD5D3}">
+  <xltc:threadedComment ref="J14" dT="2026-08-15T14:31:01.804" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{7E3FFAD7-7692-8F3C-2AB1-915769C955C0}">
     <xltc:text>Official source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J15" dT="2026-08-15T14:25:32.317" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{52A80459-605E-DE47-A560-B5294919DA3A}">
+  <xltc:threadedComment ref="J15" dT="2026-08-15T14:31:01.805" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{8D5E7050-80F6-3EDC-2079-F9038B8A87EF}">
     <xltc:text>Official source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J16" dT="2026-08-15T14:25:32.319" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{EA49137A-B2C3-1699-19C1-386362AAD204}">
+  <xltc:threadedComment ref="J16" dT="2026-08-15T14:31:01.807" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{9D79E362-9CBF-4382-59AB-0315583DE075}">
     <xltc:text>Official source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J17" dT="2026-08-15T14:25:32.321" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{A743B0C9-B331-3FE6-5A9C-7368C8C621E3}">
+  <xltc:threadedComment ref="J17" dT="2026-08-15T14:31:01.81" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{455FD18B-489F-850A-7F0C-21B99A925DFA}">
     <xltc:text>Official source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J18" dT="2026-08-15T14:25:32.324" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{B9A0315D-4AA7-FF04-062A-23F5A3A8C057}">
+  <xltc:threadedComment ref="J18" dT="2026-08-15T14:31:01.813" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{AC06C054-4207-3DDD-FB06-3F98FF6BE164}">
     <xltc:text>Official source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J19" dT="2026-08-15T14:25:32.326" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{58F44AC5-131C-E73F-2EF9-0F03167CE636}">
+  <xltc:threadedComment ref="J19" dT="2026-08-15T14:31:01.814" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{2BAEA3A0-B5A7-A503-3B40-8AB4A8357D2A}">
     <xltc:text>Official source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J20" dT="2026-08-15T14:25:32.328" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{03872F08-FCC4-073E-DCF7-71462B38E10F}">
+  <xltc:threadedComment ref="J20" dT="2026-08-15T14:31:01.816" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{2697D796-9F9D-599D-00B2-9D7190A65914}">
     <xltc:text>Official source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J21" dT="2026-08-15T14:25:32.33" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{53B86A32-AD64-73D4-6684-A35D7850F2AB}">
+  <xltc:threadedComment ref="J21" dT="2026-08-15T14:31:01.817" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D7C6A2D1-718C-3256-F2D5-7BC1FBA3B70A}">
     <xltc:text>Official source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J22" dT="2026-08-15T14:25:32.331" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{EDD1FBE0-9C7B-8E26-0237-3229A3282A1E}">
+  <xltc:threadedComment ref="J22" dT="2026-08-15T14:31:01.818" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{656BFEF9-7580-14C9-A19D-4F50DA72122B}">
     <xltc:text>Official source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J23" dT="2026-08-15T14:25:32.333" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{7F8E6C93-4097-9C02-87A3-623D41D62A58}">
+  <xltc:threadedComment ref="J23" dT="2026-08-15T14:31:01.82" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{A0063F0A-EF17-7408-1570-B2A312DA1035}">
     <xltc:text>Official source: https://www.aspenpharma.com/download/annual-financial-statements-2/</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J24" dT="2026-08-15T14:25:32.335" personId="{35B736B1-6FA6-4720-9337-F0E5DDF28B8D}" id="{12A5D7D5-7F54-1EE0-1CAD-41DE6B533C67}">
+  <xltc:threadedComment ref="J24" dT="2026-08-15T14:31:01.821" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{47404D22-6ACB-012B-2A94-989A531B023D}">
     <xltc:text>Official source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -3877,7 +3877,7 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52d299b37d534f47"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07c4c9558b554740"/>
 </x:worksheet>
 </file>
 
@@ -8611,7 +8611,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61e4ea28e4d94631"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R103f07e236234cab"/>
 </x:worksheet>
 </file>
 
@@ -9671,7 +9671,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d3b1e7973b34151"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref1935d300ad4ec0"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Use content-based submission drift checks
</commit_message>
<xml_diff>
--- a/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
+++ b/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R5ac3e9ad10e94c46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="Re405443f102a4561"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="R9d2f9c0d3f9d4b07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="R40205d2538e34e8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R0798a282546d40f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R70493432f9204b35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R211da85b2f5441fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="Rd8f1816cfdfc445d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R9e3ddb93ccef4256"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R6e3252a1afe044be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rda1e709cb03d4f06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R438ec5c348d64d3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="Rc623ca943c7e4a52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Rada818a4ce454957"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R3be6021be7bf49a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R0bc589a5e8014c52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R8d9d6c0ca74642c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="Raedf4a8f4bcb4142"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R5f9e04f8f6094ff8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="Re2dab5b911f24a01"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,88 +19,88 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={1D3C2439-FC74-878C-F5CC-58746046E7DD}</x:author>
-    <x:author>tc={4F7AA636-1509-2E5C-DE28-B75201399C36}</x:author>
-    <x:author>tc={A0CD7F65-E81E-117D-3010-1A3C4FC7E806}</x:author>
-    <x:author>tc={2BC4F4CE-3028-E376-38C4-A45C077178D6}</x:author>
-    <x:author>tc={76EA9DBC-445A-F6C9-149B-948379B25610}</x:author>
-    <x:author>tc={0E403EE3-E209-12D7-8BE8-BE38EA659A20}</x:author>
-    <x:author>tc={77871C4C-9F32-FF56-76D1-50A3CE47932D}</x:author>
-    <x:author>tc={09EF5B64-315D-CAEF-D3B6-A613340519E8}</x:author>
-    <x:author>tc={F3076964-832D-6FBD-D1F9-7564B56EBCE0}</x:author>
-    <x:author>tc={18C726D0-AA21-F490-84A5-71DB293A0C81}</x:author>
-    <x:author>tc={00894FF3-35F3-A1B1-9AA8-919CE49171F6}</x:author>
-    <x:author>tc={B353F4D8-5FFA-1545-40A6-FC8A27BB12AD}</x:author>
-    <x:author>tc={0B0729F6-5064-5F9D-2C55-23A49C0C3BDF}</x:author>
-    <x:author>tc={561A2902-D66D-F16E-E875-B7F800F6DE67}</x:author>
-    <x:author>tc={04513763-CC95-6FB5-A722-817CEE7F4448}</x:author>
-    <x:author>tc={5EF56C96-5B69-E27F-A7E1-39D4A3249AF6}</x:author>
-    <x:author>tc={7B1AE671-4D9A-C858-A69E-ED2AFA642A73}</x:author>
-    <x:author>tc={AC0117BC-E1F4-E1AA-B76E-94A004DD9A2B}</x:author>
-    <x:author>tc={7D56B634-D6AE-7A54-E4E4-59751F9EFFA4}</x:author>
-    <x:author>tc={3D509607-46DB-7367-3162-1CF1E4AC14E5}</x:author>
-    <x:author>tc={7273B247-70AB-04AF-C8F5-2CECE0DB2154}</x:author>
-    <x:author>tc={51C26273-DA34-381A-AAA1-1ECF5361C5E3}</x:author>
-    <x:author>tc={872C1AB3-1D16-04B8-606E-94AD13555A92}</x:author>
-    <x:author>tc={E79D887C-4BBA-0E20-9459-5A62A87E70F1}</x:author>
-    <x:author>tc={7046CB68-34C3-4D68-4F2E-C72388D9B45C}</x:author>
-    <x:author>tc={17B572EE-F697-8A66-04F7-87A62EA99760}</x:author>
-    <x:author>tc={C3E6A717-103F-8456-AC9B-C1175D5A8D47}</x:author>
-    <x:author>tc={FAEDA356-D777-0F8D-E232-2190C749AB82}</x:author>
-    <x:author>tc={BDAA3432-17AD-9F84-A992-3486F4D0812C}</x:author>
-    <x:author>tc={7096F403-3B9B-74B0-DDAC-4627E2727349}</x:author>
-    <x:author>tc={88122F83-F833-65D9-2D99-C170BFF1392E}</x:author>
-    <x:author>tc={27F15BE4-3771-AFF2-BF41-321B1E49DE21}</x:author>
-    <x:author>tc={2E6D83D0-C451-4B7D-2947-32079232326B}</x:author>
-    <x:author>tc={DE1C6661-BA06-94A6-774C-502B82A55C16}</x:author>
-    <x:author>tc={5382E1A5-60EF-6617-E10A-2C7E2B01057A}</x:author>
-    <x:author>tc={AE187217-C536-9ACE-B5BD-4ED40B01AF40}</x:author>
-    <x:author>tc={3DCAEE3E-C8CC-9B34-BA33-5ED9926790F1}</x:author>
-    <x:author>tc={029C4BF4-C621-DCAF-AA85-04C011CBCBEF}</x:author>
-    <x:author>tc={8DCE8E91-9F14-EFA4-2258-38657ACF07D6}</x:author>
-    <x:author>tc={244F49B3-5E2A-EFF5-741E-4212B12BEFD8}</x:author>
-    <x:author>tc={08875AF0-1E94-BD18-36F2-7FD2B7B8CDC3}</x:author>
-    <x:author>tc={454D49F2-E141-4C9B-8888-AF85F24D5231}</x:author>
-    <x:author>tc={99D865B6-8236-D481-618A-183EED9AD1C6}</x:author>
-    <x:author>tc={32F6D986-C933-3A46-379A-2E7F9DA41503}</x:author>
-    <x:author>tc={C36D4AF8-6A63-ECEE-4C92-630427FD9946}</x:author>
-    <x:author>tc={A65E46BB-285D-2221-F52B-39DD2024B265}</x:author>
-    <x:author>tc={9FDF306B-B63B-0B4A-D97E-4E8BF3989E3C}</x:author>
-    <x:author>tc={0DE09241-7611-CE47-83C3-C6E2A7213D83}</x:author>
-    <x:author>tc={15FAE1BB-C7E1-0F2E-87B6-517512B3FAE7}</x:author>
-    <x:author>tc={16D0131A-22BB-5957-7DBE-4B3D4AC9E90F}</x:author>
-    <x:author>tc={AF3C113F-B419-4CAA-8AAC-97EB9E101504}</x:author>
-    <x:author>tc={12838B92-4969-AF76-89D2-09087AE8BE65}</x:author>
-    <x:author>tc={13D8AF17-1334-372C-540D-57229F735583}</x:author>
-    <x:author>tc={6F2114EA-4845-2E1A-D087-9257AA50DFD9}</x:author>
-    <x:author>tc={286E08B1-D255-CC53-FE49-22D8F3030644}</x:author>
-    <x:author>tc={D14CF8CC-BDEA-A800-CDE3-48664676FEE7}</x:author>
-    <x:author>tc={D6BDBFE5-356C-B17F-F44F-DAA01D856D02}</x:author>
-    <x:author>tc={24905B2F-F9AE-274F-72BA-8F54DCE7E670}</x:author>
-    <x:author>tc={0732FFA9-94E7-87B5-4F7F-4AEAC96F7BD4}</x:author>
-    <x:author>tc={D2768598-BCCC-945F-3081-2DDA076AC7B5}</x:author>
-    <x:author>tc={D01A5B5D-1357-61AA-D4A2-AD9A45DD0A29}</x:author>
-    <x:author>tc={306D1132-835F-2461-847B-25DE4DB9FAEA}</x:author>
-    <x:author>tc={33464B4C-C331-D9FA-3DD2-CF201C835D67}</x:author>
-    <x:author>tc={D5279CD2-E00F-B95B-4DC2-7BAC89393443}</x:author>
-    <x:author>tc={FA50F35F-1B8C-76C5-ABC3-5AE659E19D2A}</x:author>
-    <x:author>tc={8CED9D41-7A2D-379A-125F-22DCA8021657}</x:author>
-    <x:author>tc={D8B5ED89-4462-4852-E22E-220F763A0477}</x:author>
-    <x:author>tc={EC330868-4883-AA27-0953-CD4A48E1ADF3}</x:author>
-    <x:author>tc={B12A67A1-C569-A860-97FB-BC8182C6D95E}</x:author>
-    <x:author>tc={D35606E1-B3C6-654B-C080-751905F8D3EF}</x:author>
-    <x:author>tc={A67054DF-4000-C49A-6A04-26F573EFEE52}</x:author>
-    <x:author>tc={09A5EB70-BF1F-34F1-64B2-5817DC85674B}</x:author>
-    <x:author>tc={323B98CD-2990-3DDC-6A40-15D2694A87DB}</x:author>
-    <x:author>tc={E094BE2E-BB68-693E-C1B2-B5B9891A05F1}</x:author>
-    <x:author>tc={17C77E87-BB03-92C5-C663-BF9FF11590A3}</x:author>
-    <x:author>tc={9C93F06B-74ED-F293-5E3E-FCB1407B9776}</x:author>
-    <x:author>tc={645E15D3-D9E0-480F-F123-03CDE49AABA9}</x:author>
-    <x:author>tc={ADF298A1-1553-FA00-3AE9-13140404D18D}</x:author>
-    <x:author>tc={145948C2-1781-1C6D-AD20-AD2A4E75E6CA}</x:author>
-    <x:author>tc={68C23CBB-2408-CE14-3F39-48E9043543CB}</x:author>
-    <x:author>tc={105C36BC-F67F-B935-902B-87430FB850C8}</x:author>
-    <x:author>tc={74A4F098-CABD-0354-4F0F-EBA77AA25914}</x:author>
+    <x:author>tc={173C717C-6858-7160-C636-C83BB42F4532}</x:author>
+    <x:author>tc={63B2970C-3788-C112-A8CB-3B3F13ACBE33}</x:author>
+    <x:author>tc={1004044F-FE88-537F-AC06-F229E6AF84A6}</x:author>
+    <x:author>tc={1E2BDBA3-BE2D-AA43-6606-B5993279A758}</x:author>
+    <x:author>tc={3F9E6F84-FE0D-36B7-9ADD-24B5BCFA51E6}</x:author>
+    <x:author>tc={52AA49C5-8E9B-AE59-8B98-6545B28EE15B}</x:author>
+    <x:author>tc={B1891568-FC99-A969-F70D-CDEE8457BEFC}</x:author>
+    <x:author>tc={082D8A79-A0D4-C019-F864-DBE641EEAB38}</x:author>
+    <x:author>tc={BDC1023A-5DD2-F2EB-A432-D3B36A50FE54}</x:author>
+    <x:author>tc={51E90830-4873-6DFE-41AE-2C910C9EEC9A}</x:author>
+    <x:author>tc={3ED164EE-A0A3-1A42-DA4E-68B6CC7260DF}</x:author>
+    <x:author>tc={CD8DF9C8-1E20-61D4-7F1C-891F953050CD}</x:author>
+    <x:author>tc={E95BF887-32D2-04EB-A1EE-98E9C196D9F3}</x:author>
+    <x:author>tc={CFB45910-E24C-077D-186B-932BFADA7BB1}</x:author>
+    <x:author>tc={47009490-050D-D2C8-1D90-48664025D854}</x:author>
+    <x:author>tc={06CB3692-098C-5306-68AC-91CCFF18BE8F}</x:author>
+    <x:author>tc={F26F73B4-C89E-B0B5-6F81-517E9959514E}</x:author>
+    <x:author>tc={8C7801E9-DFAA-9CEC-1604-7E8730022DCD}</x:author>
+    <x:author>tc={2E910827-D22C-F652-E278-F78E32BB95D1}</x:author>
+    <x:author>tc={F8058C0F-D0E2-3A18-9FD0-3A84595B81D3}</x:author>
+    <x:author>tc={4E7D4B04-0DB5-1B68-B26D-A0513C7909AE}</x:author>
+    <x:author>tc={A5421185-8955-0192-1B5D-5FA24B4854CE}</x:author>
+    <x:author>tc={0EA2A1B3-BE69-7BC7-D93B-5925841F1A59}</x:author>
+    <x:author>tc={12584A4C-4517-9B31-E395-34E738042FAA}</x:author>
+    <x:author>tc={6441A2AC-3623-5BD9-B536-033F6323D5EE}</x:author>
+    <x:author>tc={AB84A56E-9609-E927-6600-C0AC02186EA5}</x:author>
+    <x:author>tc={86FA8428-52FC-537E-D895-7C577F1B0D25}</x:author>
+    <x:author>tc={14FB8611-E78E-C75D-EC48-3871F4AEFC06}</x:author>
+    <x:author>tc={99635604-65F2-307E-FADC-135187FF0D1F}</x:author>
+    <x:author>tc={B27FFCF3-F14E-0235-2C1A-8E7397E20E00}</x:author>
+    <x:author>tc={25CD3762-ABE2-6CD8-5ECA-882CFCFDFB28}</x:author>
+    <x:author>tc={7482A080-D14E-D33F-31C2-3D2B683AEEDB}</x:author>
+    <x:author>tc={05D0B2B8-7D76-EC43-30FD-ADED4B860D66}</x:author>
+    <x:author>tc={BE7F4BA9-DA30-4C28-6BE5-4A368E0CA4D9}</x:author>
+    <x:author>tc={D8D08379-B543-B20B-C166-5B2F5E58674D}</x:author>
+    <x:author>tc={2514B5B4-895E-E9D1-0755-E6B42562A8B6}</x:author>
+    <x:author>tc={43E6F669-33EA-0919-B765-BB8AC1041BB1}</x:author>
+    <x:author>tc={8336B492-3FF6-8AC2-E3A6-5F44649A0793}</x:author>
+    <x:author>tc={0CE2DDAB-726A-1C7D-E5A5-092266E6B8A7}</x:author>
+    <x:author>tc={B1C20038-E535-B4B6-8559-C261A73A67A1}</x:author>
+    <x:author>tc={57536159-910E-5D86-FB2B-73B577D12D3E}</x:author>
+    <x:author>tc={D8BAA6FE-5711-436E-F6EA-EC4A4D479D92}</x:author>
+    <x:author>tc={F5755A1F-8854-9435-2022-0AAB87F7C037}</x:author>
+    <x:author>tc={44FD8D82-299B-AD44-7B33-5F8860959C9B}</x:author>
+    <x:author>tc={B44CBE08-D433-F425-B76C-F08D9E356FFC}</x:author>
+    <x:author>tc={6D90F121-6572-2506-1058-7D5A9144D000}</x:author>
+    <x:author>tc={0CA59E25-F025-10EF-9141-692AEF3B8F83}</x:author>
+    <x:author>tc={D9640E49-A5C7-B65F-9A0D-65D7DB24EEBB}</x:author>
+    <x:author>tc={3BCB9DCC-576A-8A6F-A65E-71776E316C77}</x:author>
+    <x:author>tc={054F0263-F06E-2F91-A378-2F9A307D6D3D}</x:author>
+    <x:author>tc={F3A816E8-0428-7682-BDE7-835E8A07F037}</x:author>
+    <x:author>tc={0FBC7355-F891-4C26-0974-184BF3E0A490}</x:author>
+    <x:author>tc={5379010D-20B2-3559-7434-AC60A3BF9149}</x:author>
+    <x:author>tc={51ED7905-5FC0-2EFA-FCDE-ECB06F341B85}</x:author>
+    <x:author>tc={460F10D2-05CC-CAD6-9D7B-42E804103D60}</x:author>
+    <x:author>tc={B0D2CF89-A5D6-BB93-1A21-2092A154CDEB}</x:author>
+    <x:author>tc={0FF99E4B-1649-B79E-6846-BAB0B145BE40}</x:author>
+    <x:author>tc={474588F9-4D2F-A36A-DCA6-06FE18FC9D3F}</x:author>
+    <x:author>tc={8F95FF9A-75EB-FA03-9D2C-BA0BD80069C7}</x:author>
+    <x:author>tc={4FA8524D-4B33-0F1D-CFB8-A4A4B3CF6D22}</x:author>
+    <x:author>tc={6A13DB9F-7B8D-7945-B42B-55E9B525BE4D}</x:author>
+    <x:author>tc={C0FFAB0F-E235-51E1-F5A7-702EBE41B4BC}</x:author>
+    <x:author>tc={558F1A80-BA34-1373-D92E-130F76E0C9DE}</x:author>
+    <x:author>tc={7D0D67D7-EDCA-0883-5925-8C9CA41D3ED5}</x:author>
+    <x:author>tc={26B419AF-C3DC-BC5C-BB92-7C27A26EAA95}</x:author>
+    <x:author>tc={B229E44D-B4F8-845C-BDF5-06F06E4AC987}</x:author>
+    <x:author>tc={3E3301DB-5DB0-34EC-8884-441067EF8773}</x:author>
+    <x:author>tc={8DB03130-4013-2315-00A4-399BAEAA7F88}</x:author>
+    <x:author>tc={986C3E99-675F-B218-0291-236382FB05A2}</x:author>
+    <x:author>tc={CC7C148B-B643-114F-7100-4F32E1A7D46E}</x:author>
+    <x:author>tc={FD756AED-3359-1847-B024-B000A9F62B6D}</x:author>
+    <x:author>tc={D002F702-8EF9-9DAA-6B83-D18075632BAD}</x:author>
+    <x:author>tc={847AF31F-15DC-F58D-7348-44272FF30608}</x:author>
+    <x:author>tc={C96A5CA6-0B02-6230-71B6-16D0BEAF2C32}</x:author>
+    <x:author>tc={003727CF-D765-0E72-39DF-F489DF2AB89F}</x:author>
+    <x:author>tc={94C07DE9-2411-7BFD-D930-FDAE7DE86182}</x:author>
+    <x:author>tc={15E2FF33-AEF0-4F29-0077-E9841AB6D1F2}</x:author>
+    <x:author>tc={94BDFAEF-248A-4ECF-AF7B-95B24E03AEF6}</x:author>
+    <x:author>tc={66C2F9EA-58E2-8003-9F91-275B9AD1AE85}</x:author>
+    <x:author>tc={C2F46B24-2450-5E98-6D52-DF86BB7667DC}</x:author>
+    <x:author>tc={8FAC92D9-1FE1-F845-F816-AAEEFE3656BE}</x:author>
+    <x:author>tc={1686F699-B0D7-C1A8-9524-B59E2785A701}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="P5" authorId="0">
@@ -1176,26 +1176,26 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={AB31FEAC-03E5-043B-780A-F44BF9CFCDDC}</x:author>
-    <x:author>tc={3C765B3E-DC35-B78B-4560-DAE01F8E8ACF}</x:author>
-    <x:author>tc={738792AE-B315-B455-AC29-E0F5DEF15EF3}</x:author>
-    <x:author>tc={F9AA18FF-ED7E-EB19-1A17-EDE8BB0A3971}</x:author>
-    <x:author>tc={9D8C46A8-2E04-7410-B846-E598134DD49F}</x:author>
-    <x:author>tc={04899C4D-F36B-69C9-B05A-3A58E5C22D85}</x:author>
-    <x:author>tc={B617AA04-5E42-5027-7162-06FCD4C146B9}</x:author>
-    <x:author>tc={3D900691-7755-ED89-AF3D-7A5806073765}</x:author>
-    <x:author>tc={F31C6032-2C92-F67E-09D0-3FE50F942BB7}</x:author>
-    <x:author>tc={7E3FFAD7-7692-8F3C-2AB1-915769C955C0}</x:author>
-    <x:author>tc={8D5E7050-80F6-3EDC-2079-F9038B8A87EF}</x:author>
-    <x:author>tc={9D79E362-9CBF-4382-59AB-0315583DE075}</x:author>
-    <x:author>tc={455FD18B-489F-850A-7F0C-21B99A925DFA}</x:author>
-    <x:author>tc={AC06C054-4207-3DDD-FB06-3F98FF6BE164}</x:author>
-    <x:author>tc={2BAEA3A0-B5A7-A503-3B40-8AB4A8357D2A}</x:author>
-    <x:author>tc={2697D796-9F9D-599D-00B2-9D7190A65914}</x:author>
-    <x:author>tc={D7C6A2D1-718C-3256-F2D5-7BC1FBA3B70A}</x:author>
-    <x:author>tc={656BFEF9-7580-14C9-A19D-4F50DA72122B}</x:author>
-    <x:author>tc={A0063F0A-EF17-7408-1570-B2A312DA1035}</x:author>
-    <x:author>tc={47404D22-6ACB-012B-2A94-989A531B023D}</x:author>
+    <x:author>tc={1AC6FA9D-6EAF-4D3D-C375-CE877C69E260}</x:author>
+    <x:author>tc={3326CE3D-BC56-94A6-EE75-9FF44A04FBF9}</x:author>
+    <x:author>tc={A198EC00-C1E3-A8A8-AC4A-67A8B8F010BB}</x:author>
+    <x:author>tc={776DE28D-8AC0-2C7A-9807-00F5444D703D}</x:author>
+    <x:author>tc={6796EA78-A81F-DDBF-7E66-30157FC65830}</x:author>
+    <x:author>tc={CACFC29D-1990-F2B4-3C09-1DA8A69188E8}</x:author>
+    <x:author>tc={4190D384-F5E8-3DFD-D3CD-FF286FB9D4A6}</x:author>
+    <x:author>tc={DAFC6F34-CDF1-903C-10A6-184187A22E45}</x:author>
+    <x:author>tc={70F2FEBE-C8AF-EC53-9654-05E07CEE7755}</x:author>
+    <x:author>tc={67293E1B-F0C0-D9F1-5F84-C1B0961128F9}</x:author>
+    <x:author>tc={8F554A60-1949-E8A2-381C-F75948BE7625}</x:author>
+    <x:author>tc={098ED24E-3E3F-B884-77A6-1F1588D94C89}</x:author>
+    <x:author>tc={F1CE5709-A240-337C-D02D-CA48439B5DE4}</x:author>
+    <x:author>tc={14AF2B76-3471-DAB3-580D-D5C33A1454D9}</x:author>
+    <x:author>tc={7EF3A7A6-3D3F-E608-1ADE-2C7F9793F446}</x:author>
+    <x:author>tc={36D05D5C-837A-8195-8F78-0276FD04F15A}</x:author>
+    <x:author>tc={4A543F82-A7AD-EAD9-AE30-DA0D3AE12465}</x:author>
+    <x:author>tc={DA604E42-7C6E-CBE1-A6DC-5AC2EE98E227}</x:author>
+    <x:author>tc={3D7D7B80-DA40-ABB3-0828-1BEACC3AC788}</x:author>
+    <x:author>tc={FD461D61-E8E0-FF46-FCCC-F572C22C9E49}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="J5" authorId="0">
@@ -2060,7 +2060,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2edd2dab42be4a13"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7ee2500d485f42f8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2071,7 +2071,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}"/>
+  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}"/>
 </xltc:personList>
 </file>
 
@@ -2268,493 +2268,493 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="P5" dT="2026-08-15T14:31:01.523" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{1D3C2439-FC74-878C-F5CC-58746046E7DD}">
+  <xltc:threadedComment ref="P5" dT="2026-08-15T14:36:30.107" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{173C717C-6858-7160-C636-C83BB42F4532}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P6" dT="2026-08-15T14:31:01.525" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{4F7AA636-1509-2E5C-DE28-B75201399C36}">
+  <xltc:threadedComment ref="P6" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{63B2970C-3788-C112-A8CB-3B3F13ACBE33}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P7" dT="2026-08-15T14:31:01.525" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{A0CD7F65-E81E-117D-3010-1A3C4FC7E806}">
+  <xltc:threadedComment ref="P7" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{1004044F-FE88-537F-AC06-F229E6AF84A6}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P8" dT="2026-08-15T14:31:01.525" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{2BC4F4CE-3028-E376-38C4-A45C077178D6}">
+  <xltc:threadedComment ref="P8" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{1E2BDBA3-BE2D-AA43-6606-B5993279A758}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P9" dT="2026-08-15T14:31:01.525" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{76EA9DBC-445A-F6C9-149B-948379B25610}">
+  <xltc:threadedComment ref="P9" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{3F9E6F84-FE0D-36B7-9ADD-24B5BCFA51E6}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P10" dT="2026-08-15T14:31:01.525" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{0E403EE3-E209-12D7-8BE8-BE38EA659A20}">
+  <xltc:threadedComment ref="P10" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{52AA49C5-8E9B-AE59-8B98-6545B28EE15B}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 119
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P11" dT="2026-08-15T14:31:01.525" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{77871C4C-9F32-FF56-76D1-50A3CE47932D}">
+  <xltc:threadedComment ref="P11" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{B1891568-FC99-A969-F70D-CDEE8457BEFC}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 160
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P12" dT="2026-08-15T14:31:01.525" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{09EF5B64-315D-CAEF-D3B6-A613340519E8}">
+  <xltc:threadedComment ref="P12" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{082D8A79-A0D4-C019-F864-DBE641EEAB38}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P13" dT="2026-08-15T14:31:01.526" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{F3076964-832D-6FBD-D1F9-7564B56EBCE0}">
+  <xltc:threadedComment ref="P13" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{BDC1023A-5DD2-F2EB-A432-D3B36A50FE54}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P14" dT="2026-08-15T14:31:01.526" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{18C726D0-AA21-F490-84A5-71DB293A0C81}">
+  <xltc:threadedComment ref="P14" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{51E90830-4873-6DFE-41AE-2C910C9EEC9A}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P15" dT="2026-08-15T14:31:01.526" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{00894FF3-35F3-A1B1-9AA8-919CE49171F6}">
+  <xltc:threadedComment ref="P15" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{3ED164EE-A0A3-1A42-DA4E-68B6CC7260DF}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P16" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{B353F4D8-5FFA-1545-40A6-FC8A27BB12AD}">
+  <xltc:threadedComment ref="P16" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{CD8DF9C8-1E20-61D4-7F1C-891F953050CD}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P17" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{0B0729F6-5064-5F9D-2C55-23A49C0C3BDF}">
+  <xltc:threadedComment ref="P17" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{E95BF887-32D2-04EB-A1EE-98E9C196D9F3}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P18" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{561A2902-D66D-F16E-E875-B7F800F6DE67}">
+  <xltc:threadedComment ref="P18" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{CFB45910-E24C-077D-186B-932BFADA7BB1}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P19" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{04513763-CC95-6FB5-A722-817CEE7F4448}">
+  <xltc:threadedComment ref="P19" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{47009490-050D-D2C8-1D90-48664025D854}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P20" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{5EF56C96-5B69-E27F-A7E1-39D4A3249AF6}">
+  <xltc:threadedComment ref="P20" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{06CB3692-098C-5306-68AC-91CCFF18BE8F}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 138
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P21" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{7B1AE671-4D9A-C858-A69E-ED2AFA642A73}">
+  <xltc:threadedComment ref="P21" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{F26F73B4-C89E-B0B5-6F81-517E9959514E}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 212
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P22" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{AC0117BC-E1F4-E1AA-B76E-94A004DD9A2B}">
+  <xltc:threadedComment ref="P22" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{8C7801E9-DFAA-9CEC-1604-7E8730022DCD}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P23" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{7D56B634-D6AE-7A54-E4E4-59751F9EFFA4}">
+  <xltc:threadedComment ref="P23" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{2E910827-D22C-F652-E278-F78E32BB95D1}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P24" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{3D509607-46DB-7367-3162-1CF1E4AC14E5}">
+  <xltc:threadedComment ref="P24" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{F8058C0F-D0E2-3A18-9FD0-3A84595B81D3}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P25" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{7273B247-70AB-04AF-C8F5-2CECE0DB2154}">
+  <xltc:threadedComment ref="P25" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{4E7D4B04-0DB5-1B68-B26D-A0513C7909AE}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P26" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{51C26273-DA34-381A-AAA1-1ECF5361C5E3}">
+  <xltc:threadedComment ref="P26" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{A5421185-8955-0192-1B5D-5FA24B4854CE}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P27" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{872C1AB3-1D16-04B8-606E-94AD13555A92}">
+  <xltc:threadedComment ref="P27" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{0EA2A1B3-BE69-7BC7-D93B-5925841F1A59}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 272
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P28" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{E79D887C-4BBA-0E20-9459-5A62A87E70F1}">
+  <xltc:threadedComment ref="P28" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{12584A4C-4517-9B31-E395-34E738042FAA}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P29" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{7046CB68-34C3-4D68-4F2E-C72388D9B45C}">
+  <xltc:threadedComment ref="P29" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{6441A2AC-3623-5BD9-B536-033F6323D5EE}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P30" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{17B572EE-F697-8A66-04F7-87A62EA99760}">
+  <xltc:threadedComment ref="P30" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{AB84A56E-9609-E927-6600-C0AC02186EA5}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 158
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P31" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{C3E6A717-103F-8456-AC9B-C1175D5A8D47}">
+  <xltc:threadedComment ref="P31" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{86FA8428-52FC-537E-D895-7C577F1B0D25}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P32" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{FAEDA356-D777-0F8D-E232-2190C749AB82}">
+  <xltc:threadedComment ref="P32" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{14FB8611-E78E-C75D-EC48-3871F4AEFC06}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P33" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{BDAA3432-17AD-9F84-A992-3486F4D0812C}">
+  <xltc:threadedComment ref="P33" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{99635604-65F2-307E-FADC-135187FF0D1F}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 72
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P34" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{7096F403-3B9B-74B0-DDAC-4627E2727349}">
+  <xltc:threadedComment ref="P34" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{B27FFCF3-F14E-0235-2C1A-8E7397E20E00}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P35" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{88122F83-F833-65D9-2D99-C170BFF1392E}">
+  <xltc:threadedComment ref="P35" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{25CD3762-ABE2-6CD8-5ECA-882CFCFDFB28}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P36" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{27F15BE4-3771-AFF2-BF41-321B1E49DE21}">
+  <xltc:threadedComment ref="P36" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{7482A080-D14E-D33F-31C2-3D2B683AEEDB}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 24
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P37" dT="2026-08-15T14:31:01.527" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{2E6D83D0-C451-4B7D-2947-32079232326B}">
+  <xltc:threadedComment ref="P37" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{05D0B2B8-7D76-EC43-30FD-ADED4B860D66}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P38" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{DE1C6661-BA06-94A6-774C-502B82A55C16}">
+  <xltc:threadedComment ref="P38" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{BE7F4BA9-DA30-4C28-6BE5-4A368E0CA4D9}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P39" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{5382E1A5-60EF-6617-E10A-2C7E2B01057A}">
+  <xltc:threadedComment ref="P39" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{D8D08379-B543-B20B-C166-5B2F5E58674D}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 19
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P40" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{AE187217-C536-9ACE-B5BD-4ED40B01AF40}">
+  <xltc:threadedComment ref="P40" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{2514B5B4-895E-E9D1-0755-E6B42562A8B6}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P41" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{3DCAEE3E-C8CC-9B34-BA33-5ED9926790F1}">
+  <xltc:threadedComment ref="P41" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{43E6F669-33EA-0919-B765-BB8AC1041BB1}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P42" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{029C4BF4-C621-DCAF-AA85-04C011CBCBEF}">
+  <xltc:threadedComment ref="P42" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{8336B492-3FF6-8AC2-E3A6-5F44649A0793}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P43" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{8DCE8E91-9F14-EFA4-2258-38657ACF07D6}">
+  <xltc:threadedComment ref="P43" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{0CE2DDAB-726A-1C7D-E5A5-092266E6B8A7}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P44" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{244F49B3-5E2A-EFF5-741E-4212B12BEFD8}">
+  <xltc:threadedComment ref="P44" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{B1C20038-E535-B4B6-8559-C261A73A67A1}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P45" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{08875AF0-1E94-BD18-36F2-7FD2B7B8CDC3}">
+  <xltc:threadedComment ref="P45" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{57536159-910E-5D86-FB2B-73B577D12D3E}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P46" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{454D49F2-E141-4C9B-8888-AF85F24D5231}">
+  <xltc:threadedComment ref="P46" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{D8BAA6FE-5711-436E-F6EA-EC4A4D479D92}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P47" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{99D865B6-8236-D481-618A-183EED9AD1C6}">
+  <xltc:threadedComment ref="P47" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{F5755A1F-8854-9435-2022-0AAB87F7C037}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P48" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{32F6D986-C933-3A46-379A-2E7F9DA41503}">
+  <xltc:threadedComment ref="P48" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{44FD8D82-299B-AD44-7B33-5F8860959C9B}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P49" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{C36D4AF8-6A63-ECEE-4C92-630427FD9946}">
+  <xltc:threadedComment ref="P49" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{B44CBE08-D433-F425-B76C-F08D9E356FFC}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 118
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P50" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{A65E46BB-285D-2221-F52B-39DD2024B265}">
+  <xltc:threadedComment ref="P50" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{6D90F121-6572-2506-1058-7D5A9144D000}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P51" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{9FDF306B-B63B-0B4A-D97E-4E8BF3989E3C}">
+  <xltc:threadedComment ref="P51" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{0CA59E25-F025-10EF-9141-692AEF3B8F83}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P52" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{0DE09241-7611-CE47-83C3-C6E2A7213D83}">
+  <xltc:threadedComment ref="P52" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{D9640E49-A5C7-B65F-9A0D-65D7DB24EEBB}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P53" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{15FAE1BB-C7E1-0F2E-87B6-517512B3FAE7}">
+  <xltc:threadedComment ref="P53" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{3BCB9DCC-576A-8A6F-A65E-71776E316C77}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-STF</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P54" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{16D0131A-22BB-5957-7DBE-4B3D4AC9E90F}">
+  <xltc:threadedComment ref="P54" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{054F0263-F06E-2F91-A378-2F9A307D6D3D}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P55" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{AF3C113F-B419-4CAA-8AAC-97EB9E101504}">
+  <xltc:threadedComment ref="P55" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{F3A816E8-0428-7682-BDE7-835E8A07F037}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P56" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{12838B92-4969-AF76-89D2-09087AE8BE65}">
+  <xltc:threadedComment ref="P56" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{0FBC7355-F891-4C26-0974-184BF3E0A490}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 18
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P57" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{13D8AF17-1334-372C-540D-57229F735583}">
+  <xltc:threadedComment ref="P57" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{5379010D-20B2-3559-7434-AC60A3BF9149}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P58" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{6F2114EA-4845-2E1A-D087-9257AA50DFD9}">
+  <xltc:threadedComment ref="P58" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{51ED7905-5FC0-2EFA-FCDE-ECB06F341B85}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P59" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{286E08B1-D255-CC53-FE49-22D8F3030644}">
+  <xltc:threadedComment ref="P59" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{460F10D2-05CC-CAD6-9D7B-42E804103D60}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P60" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D14CF8CC-BDEA-A800-CDE3-48664676FEE7}">
+  <xltc:threadedComment ref="P60" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{B0D2CF89-A5D6-BB93-1A21-2092A154CDEB}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P61" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D6BDBFE5-356C-B17F-F44F-DAA01D856D02}">
+  <xltc:threadedComment ref="P61" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{0FF99E4B-1649-B79E-6846-BAB0B145BE40}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P62" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{24905B2F-F9AE-274F-72BA-8F54DCE7E670}">
+  <xltc:threadedComment ref="P62" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{474588F9-4D2F-A36A-DCA6-06FE18FC9D3F}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P63" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{0732FFA9-94E7-87B5-4F7F-4AEAC96F7BD4}">
+  <xltc:threadedComment ref="P63" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{8F95FF9A-75EB-FA03-9D2C-BA0BD80069C7}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P64" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D2768598-BCCC-945F-3081-2DDA076AC7B5}">
+  <xltc:threadedComment ref="P64" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{4FA8524D-4B33-0F1D-CFB8-A4A4B3CF6D22}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P65" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D01A5B5D-1357-61AA-D4A2-AD9A45DD0A29}">
+  <xltc:threadedComment ref="P65" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{6A13DB9F-7B8D-7945-B42B-55E9B525BE4D}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 311
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P66" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{306D1132-835F-2461-847B-25DE4DB9FAEA}">
+  <xltc:threadedComment ref="P66" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{C0FFAB0F-E235-51E1-F5A7-702EBE41B4BC}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P67" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{33464B4C-C331-D9FA-3DD2-CF201C835D67}">
+  <xltc:threadedComment ref="P67" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{558F1A80-BA34-1373-D92E-130F76E0C9DE}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P68" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D5279CD2-E00F-B95B-4DC2-7BAC89393443}">
+  <xltc:threadedComment ref="P68" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{7D0D67D7-EDCA-0883-5925-8C9CA41D3ED5}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 141
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P69" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{FA50F35F-1B8C-76C5-ABC3-5AE659E19D2A}">
+  <xltc:threadedComment ref="P69" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{26B419AF-C3DC-BC5C-BB92-7C27A26EAA95}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P70" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{8CED9D41-7A2D-379A-125F-22DCA8021657}">
+  <xltc:threadedComment ref="P70" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{B229E44D-B4F8-845C-BDF5-06F06E4AC987}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P71" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D8B5ED89-4462-4852-E22E-220F763A0477}">
+  <xltc:threadedComment ref="P71" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{3E3301DB-5DB0-34EC-8884-441067EF8773}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 33
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P72" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{EC330868-4883-AA27-0953-CD4A48E1ADF3}">
+  <xltc:threadedComment ref="P72" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{8DB03130-4013-2315-00A4-399BAEAA7F88}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P73" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{B12A67A1-C569-A860-97FB-BC8182C6D95E}">
+  <xltc:threadedComment ref="P73" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{986C3E99-675F-B218-0291-236382FB05A2}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P74" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D35606E1-B3C6-654B-C080-751905F8D3EF}">
+  <xltc:threadedComment ref="P74" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{CC7C148B-B643-114F-7100-4F32E1A7D46E}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 21
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P75" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{A67054DF-4000-C49A-6A04-26F573EFEE52}">
+  <xltc:threadedComment ref="P75" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{FD756AED-3359-1847-B024-B000A9F62B6D}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P76" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{09A5EB70-BF1F-34F1-64B2-5817DC85674B}">
+  <xltc:threadedComment ref="P76" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{D002F702-8EF9-9DAA-6B83-D18075632BAD}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P77" dT="2026-08-15T14:31:01.528" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{323B98CD-2990-3DDC-6A40-15D2694A87DB}">
+  <xltc:threadedComment ref="P77" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{847AF31F-15DC-F58D-7348-44272FF30608}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 19
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P78" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{E094BE2E-BB68-693E-C1B2-B5B9891A05F1}">
+  <xltc:threadedComment ref="P78" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{C96A5CA6-0B02-6230-71B6-16D0BEAF2C32}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 43
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P79" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{17C77E87-BB03-92C5-C663-BF9FF11590A3}">
+  <xltc:threadedComment ref="P79" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{003727CF-D765-0E72-39DF-F489DF2AB89F}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 44
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P80" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{9C93F06B-74ED-F293-5E3E-FCB1407B9776}">
+  <xltc:threadedComment ref="P80" dT="2026-08-15T14:36:30.114" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{94C07DE9-2411-7BFD-D930-FDAE7DE86182}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 40
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P81" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{645E15D3-D9E0-480F-F123-03CDE49AABA9}">
+  <xltc:threadedComment ref="P81" dT="2026-08-15T14:36:30.114" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{15E2FF33-AEF0-4F29-0077-E9841AB6D1F2}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P82" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{ADF298A1-1553-FA00-3AE9-13140404D18D}">
+  <xltc:threadedComment ref="P82" dT="2026-08-15T14:36:30.114" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{94BDFAEF-248A-4ECF-AF7B-95B24E03AEF6}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P83" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{145948C2-1781-1C6D-AD20-AD2A4E75E6CA}">
+  <xltc:threadedComment ref="P83" dT="2026-08-15T14:36:30.114" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{66C2F9EA-58E2-8003-9F91-275B9AD1AE85}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 16
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P84" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{68C23CBB-2408-CE14-3F39-48E9043543CB}">
+  <xltc:threadedComment ref="P84" dT="2026-08-15T14:36:30.114" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{C2F46B24-2450-5E98-6D52-DF86BB7667DC}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P85" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{105C36BC-F67F-B935-902B-87430FB850C8}">
+  <xltc:threadedComment ref="P85" dT="2026-08-15T14:36:30.114" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{8FAC92D9-1FE1-F845-F816-AAEEFE3656BE}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P86" dT="2026-08-15T14:31:01.529" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{74A4F098-CABD-0354-4F0F-EBA77AA25914}">
+  <xltc:threadedComment ref="P86" dT="2026-08-15T14:36:30.114" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{1686F699-B0D7-C1A8-9524-B59E2785A701}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 21
 Available: 2026-02-25
@@ -2765,64 +2765,64 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="J5" dT="2026-08-15T14:31:01.789" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{AB31FEAC-03E5-043B-780A-F44BF9CFCDDC}">
+  <xltc:threadedComment ref="J5" dT="2026-08-15T14:36:30.456" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{1AC6FA9D-6EAF-4D3D-C375-CE877C69E260}">
     <xltc:text>Official source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J6" dT="2026-08-15T14:31:01.791" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{3C765B3E-DC35-B78B-4560-DAE01F8E8ACF}">
+  <xltc:threadedComment ref="J6" dT="2026-08-15T14:36:30.459" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{3326CE3D-BC56-94A6-EE75-9FF44A04FBF9}">
     <xltc:text>Official source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J7" dT="2026-08-15T14:31:01.793" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{738792AE-B315-B455-AC29-E0F5DEF15EF3}">
+  <xltc:threadedComment ref="J7" dT="2026-08-15T14:36:30.462" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{A198EC00-C1E3-A8A8-AC4A-67A8B8F010BB}">
     <xltc:text>Official source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J8" dT="2026-08-15T14:31:01.795" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{F9AA18FF-ED7E-EB19-1A17-EDE8BB0A3971}">
+  <xltc:threadedComment ref="J8" dT="2026-08-15T14:36:30.465" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{776DE28D-8AC0-2C7A-9807-00F5444D703D}">
     <xltc:text>Official source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J9" dT="2026-08-15T14:31:01.797" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{9D8C46A8-2E04-7410-B846-E598134DD49F}">
+  <xltc:threadedComment ref="J9" dT="2026-08-15T14:36:30.466" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{6796EA78-A81F-DDBF-7E66-30157FC65830}">
     <xltc:text>Official source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J10" dT="2026-08-15T14:31:01.798" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{04899C4D-F36B-69C9-B05A-3A58E5C22D85}">
+  <xltc:threadedComment ref="J10" dT="2026-08-15T14:36:30.469" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{CACFC29D-1990-F2B4-3C09-1DA8A69188E8}">
     <xltc:text>Official source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J11" dT="2026-08-15T14:31:01.8" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{B617AA04-5E42-5027-7162-06FCD4C146B9}">
+  <xltc:threadedComment ref="J11" dT="2026-08-15T14:36:30.471" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{4190D384-F5E8-3DFD-D3CD-FF286FB9D4A6}">
     <xltc:text>Official source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J12" dT="2026-08-15T14:31:01.801" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{3D900691-7755-ED89-AF3D-7A5806073765}">
+  <xltc:threadedComment ref="J12" dT="2026-08-15T14:36:30.473" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{DAFC6F34-CDF1-903C-10A6-184187A22E45}">
     <xltc:text>Official source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J13" dT="2026-08-15T14:31:01.802" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{F31C6032-2C92-F67E-09D0-3FE50F942BB7}">
+  <xltc:threadedComment ref="J13" dT="2026-08-15T14:36:30.475" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{70F2FEBE-C8AF-EC53-9654-05E07CEE7755}">
     <xltc:text>Official source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J14" dT="2026-08-15T14:31:01.804" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{7E3FFAD7-7692-8F3C-2AB1-915769C955C0}">
+  <xltc:threadedComment ref="J14" dT="2026-08-15T14:36:30.478" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{67293E1B-F0C0-D9F1-5F84-C1B0961128F9}">
     <xltc:text>Official source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J15" dT="2026-08-15T14:31:01.805" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{8D5E7050-80F6-3EDC-2079-F9038B8A87EF}">
+  <xltc:threadedComment ref="J15" dT="2026-08-15T14:36:30.48" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{8F554A60-1949-E8A2-381C-F75948BE7625}">
     <xltc:text>Official source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J16" dT="2026-08-15T14:31:01.807" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{9D79E362-9CBF-4382-59AB-0315583DE075}">
+  <xltc:threadedComment ref="J16" dT="2026-08-15T14:36:30.481" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{098ED24E-3E3F-B884-77A6-1F1588D94C89}">
     <xltc:text>Official source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J17" dT="2026-08-15T14:31:01.81" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{455FD18B-489F-850A-7F0C-21B99A925DFA}">
+  <xltc:threadedComment ref="J17" dT="2026-08-15T14:36:30.483" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{F1CE5709-A240-337C-D02D-CA48439B5DE4}">
     <xltc:text>Official source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J18" dT="2026-08-15T14:31:01.813" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{AC06C054-4207-3DDD-FB06-3F98FF6BE164}">
+  <xltc:threadedComment ref="J18" dT="2026-08-15T14:36:30.484" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{14AF2B76-3471-DAB3-580D-D5C33A1454D9}">
     <xltc:text>Official source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J19" dT="2026-08-15T14:31:01.814" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{2BAEA3A0-B5A7-A503-3B40-8AB4A8357D2A}">
+  <xltc:threadedComment ref="J19" dT="2026-08-15T14:36:30.488" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{7EF3A7A6-3D3F-E608-1ADE-2C7F9793F446}">
     <xltc:text>Official source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J20" dT="2026-08-15T14:31:01.816" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{2697D796-9F9D-599D-00B2-9D7190A65914}">
+  <xltc:threadedComment ref="J20" dT="2026-08-15T14:36:30.49" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{36D05D5C-837A-8195-8F78-0276FD04F15A}">
     <xltc:text>Official source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J21" dT="2026-08-15T14:31:01.817" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{D7C6A2D1-718C-3256-F2D5-7BC1FBA3B70A}">
+  <xltc:threadedComment ref="J21" dT="2026-08-15T14:36:30.491" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{4A543F82-A7AD-EAD9-AE30-DA0D3AE12465}">
     <xltc:text>Official source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J22" dT="2026-08-15T14:31:01.818" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{656BFEF9-7580-14C9-A19D-4F50DA72122B}">
+  <xltc:threadedComment ref="J22" dT="2026-08-15T14:36:30.493" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{DA604E42-7C6E-CBE1-A6DC-5AC2EE98E227}">
     <xltc:text>Official source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J23" dT="2026-08-15T14:31:01.82" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{A0063F0A-EF17-7408-1570-B2A312DA1035}">
+  <xltc:threadedComment ref="J23" dT="2026-08-15T14:36:30.495" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{3D7D7B80-DA40-ABB3-0828-1BEACC3AC788}">
     <xltc:text>Official source: https://www.aspenpharma.com/download/annual-financial-statements-2/</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J24" dT="2026-08-15T14:31:01.821" personId="{B5FB5AAB-58AF-4551-BCC5-E77322CCD9A7}" id="{47404D22-6ACB-012B-2A94-989A531B023D}">
+  <xltc:threadedComment ref="J24" dT="2026-08-15T14:36:30.496" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{FD461D61-E8E0-FF46-FCCC-F572C22C9E49}">
     <xltc:text>Official source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -3877,7 +3877,7 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07c4c9558b554740"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R817a88bcb3fc44b6"/>
 </x:worksheet>
 </file>
 
@@ -8611,7 +8611,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R103f07e236234cab"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb15147641d114dca"/>
 </x:worksheet>
 </file>
 
@@ -9671,7 +9671,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref1935d300ad4ec0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc20f38d184d94b29"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Stamp final V3.2 submission artifacts
</commit_message>
<xml_diff>
--- a/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
+++ b/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rda1e709cb03d4f06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R438ec5c348d64d3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="Rc623ca943c7e4a52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Rada818a4ce454957"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R3be6021be7bf49a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R0bc589a5e8014c52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R8d9d6c0ca74642c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="Raedf4a8f4bcb4142"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R5f9e04f8f6094ff8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="Re2dab5b911f24a01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R5ded0f81741d4f65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R4a49f1ac8efb40a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="R70d09ac268784577"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="R809eb01ba2d54f08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R14e4144764b449e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="Ra942e43c5fb24b49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Rfa974438e19e4dbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="Re2c2af9be93b49af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R500b0e8dc2794605"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="Radbea52237a3498b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,88 +19,88 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={173C717C-6858-7160-C636-C83BB42F4532}</x:author>
-    <x:author>tc={63B2970C-3788-C112-A8CB-3B3F13ACBE33}</x:author>
-    <x:author>tc={1004044F-FE88-537F-AC06-F229E6AF84A6}</x:author>
-    <x:author>tc={1E2BDBA3-BE2D-AA43-6606-B5993279A758}</x:author>
-    <x:author>tc={3F9E6F84-FE0D-36B7-9ADD-24B5BCFA51E6}</x:author>
-    <x:author>tc={52AA49C5-8E9B-AE59-8B98-6545B28EE15B}</x:author>
-    <x:author>tc={B1891568-FC99-A969-F70D-CDEE8457BEFC}</x:author>
-    <x:author>tc={082D8A79-A0D4-C019-F864-DBE641EEAB38}</x:author>
-    <x:author>tc={BDC1023A-5DD2-F2EB-A432-D3B36A50FE54}</x:author>
-    <x:author>tc={51E90830-4873-6DFE-41AE-2C910C9EEC9A}</x:author>
-    <x:author>tc={3ED164EE-A0A3-1A42-DA4E-68B6CC7260DF}</x:author>
-    <x:author>tc={CD8DF9C8-1E20-61D4-7F1C-891F953050CD}</x:author>
-    <x:author>tc={E95BF887-32D2-04EB-A1EE-98E9C196D9F3}</x:author>
-    <x:author>tc={CFB45910-E24C-077D-186B-932BFADA7BB1}</x:author>
-    <x:author>tc={47009490-050D-D2C8-1D90-48664025D854}</x:author>
-    <x:author>tc={06CB3692-098C-5306-68AC-91CCFF18BE8F}</x:author>
-    <x:author>tc={F26F73B4-C89E-B0B5-6F81-517E9959514E}</x:author>
-    <x:author>tc={8C7801E9-DFAA-9CEC-1604-7E8730022DCD}</x:author>
-    <x:author>tc={2E910827-D22C-F652-E278-F78E32BB95D1}</x:author>
-    <x:author>tc={F8058C0F-D0E2-3A18-9FD0-3A84595B81D3}</x:author>
-    <x:author>tc={4E7D4B04-0DB5-1B68-B26D-A0513C7909AE}</x:author>
-    <x:author>tc={A5421185-8955-0192-1B5D-5FA24B4854CE}</x:author>
-    <x:author>tc={0EA2A1B3-BE69-7BC7-D93B-5925841F1A59}</x:author>
-    <x:author>tc={12584A4C-4517-9B31-E395-34E738042FAA}</x:author>
-    <x:author>tc={6441A2AC-3623-5BD9-B536-033F6323D5EE}</x:author>
-    <x:author>tc={AB84A56E-9609-E927-6600-C0AC02186EA5}</x:author>
-    <x:author>tc={86FA8428-52FC-537E-D895-7C577F1B0D25}</x:author>
-    <x:author>tc={14FB8611-E78E-C75D-EC48-3871F4AEFC06}</x:author>
-    <x:author>tc={99635604-65F2-307E-FADC-135187FF0D1F}</x:author>
-    <x:author>tc={B27FFCF3-F14E-0235-2C1A-8E7397E20E00}</x:author>
-    <x:author>tc={25CD3762-ABE2-6CD8-5ECA-882CFCFDFB28}</x:author>
-    <x:author>tc={7482A080-D14E-D33F-31C2-3D2B683AEEDB}</x:author>
-    <x:author>tc={05D0B2B8-7D76-EC43-30FD-ADED4B860D66}</x:author>
-    <x:author>tc={BE7F4BA9-DA30-4C28-6BE5-4A368E0CA4D9}</x:author>
-    <x:author>tc={D8D08379-B543-B20B-C166-5B2F5E58674D}</x:author>
-    <x:author>tc={2514B5B4-895E-E9D1-0755-E6B42562A8B6}</x:author>
-    <x:author>tc={43E6F669-33EA-0919-B765-BB8AC1041BB1}</x:author>
-    <x:author>tc={8336B492-3FF6-8AC2-E3A6-5F44649A0793}</x:author>
-    <x:author>tc={0CE2DDAB-726A-1C7D-E5A5-092266E6B8A7}</x:author>
-    <x:author>tc={B1C20038-E535-B4B6-8559-C261A73A67A1}</x:author>
-    <x:author>tc={57536159-910E-5D86-FB2B-73B577D12D3E}</x:author>
-    <x:author>tc={D8BAA6FE-5711-436E-F6EA-EC4A4D479D92}</x:author>
-    <x:author>tc={F5755A1F-8854-9435-2022-0AAB87F7C037}</x:author>
-    <x:author>tc={44FD8D82-299B-AD44-7B33-5F8860959C9B}</x:author>
-    <x:author>tc={B44CBE08-D433-F425-B76C-F08D9E356FFC}</x:author>
-    <x:author>tc={6D90F121-6572-2506-1058-7D5A9144D000}</x:author>
-    <x:author>tc={0CA59E25-F025-10EF-9141-692AEF3B8F83}</x:author>
-    <x:author>tc={D9640E49-A5C7-B65F-9A0D-65D7DB24EEBB}</x:author>
-    <x:author>tc={3BCB9DCC-576A-8A6F-A65E-71776E316C77}</x:author>
-    <x:author>tc={054F0263-F06E-2F91-A378-2F9A307D6D3D}</x:author>
-    <x:author>tc={F3A816E8-0428-7682-BDE7-835E8A07F037}</x:author>
-    <x:author>tc={0FBC7355-F891-4C26-0974-184BF3E0A490}</x:author>
-    <x:author>tc={5379010D-20B2-3559-7434-AC60A3BF9149}</x:author>
-    <x:author>tc={51ED7905-5FC0-2EFA-FCDE-ECB06F341B85}</x:author>
-    <x:author>tc={460F10D2-05CC-CAD6-9D7B-42E804103D60}</x:author>
-    <x:author>tc={B0D2CF89-A5D6-BB93-1A21-2092A154CDEB}</x:author>
-    <x:author>tc={0FF99E4B-1649-B79E-6846-BAB0B145BE40}</x:author>
-    <x:author>tc={474588F9-4D2F-A36A-DCA6-06FE18FC9D3F}</x:author>
-    <x:author>tc={8F95FF9A-75EB-FA03-9D2C-BA0BD80069C7}</x:author>
-    <x:author>tc={4FA8524D-4B33-0F1D-CFB8-A4A4B3CF6D22}</x:author>
-    <x:author>tc={6A13DB9F-7B8D-7945-B42B-55E9B525BE4D}</x:author>
-    <x:author>tc={C0FFAB0F-E235-51E1-F5A7-702EBE41B4BC}</x:author>
-    <x:author>tc={558F1A80-BA34-1373-D92E-130F76E0C9DE}</x:author>
-    <x:author>tc={7D0D67D7-EDCA-0883-5925-8C9CA41D3ED5}</x:author>
-    <x:author>tc={26B419AF-C3DC-BC5C-BB92-7C27A26EAA95}</x:author>
-    <x:author>tc={B229E44D-B4F8-845C-BDF5-06F06E4AC987}</x:author>
-    <x:author>tc={3E3301DB-5DB0-34EC-8884-441067EF8773}</x:author>
-    <x:author>tc={8DB03130-4013-2315-00A4-399BAEAA7F88}</x:author>
-    <x:author>tc={986C3E99-675F-B218-0291-236382FB05A2}</x:author>
-    <x:author>tc={CC7C148B-B643-114F-7100-4F32E1A7D46E}</x:author>
-    <x:author>tc={FD756AED-3359-1847-B024-B000A9F62B6D}</x:author>
-    <x:author>tc={D002F702-8EF9-9DAA-6B83-D18075632BAD}</x:author>
-    <x:author>tc={847AF31F-15DC-F58D-7348-44272FF30608}</x:author>
-    <x:author>tc={C96A5CA6-0B02-6230-71B6-16D0BEAF2C32}</x:author>
-    <x:author>tc={003727CF-D765-0E72-39DF-F489DF2AB89F}</x:author>
-    <x:author>tc={94C07DE9-2411-7BFD-D930-FDAE7DE86182}</x:author>
-    <x:author>tc={15E2FF33-AEF0-4F29-0077-E9841AB6D1F2}</x:author>
-    <x:author>tc={94BDFAEF-248A-4ECF-AF7B-95B24E03AEF6}</x:author>
-    <x:author>tc={66C2F9EA-58E2-8003-9F91-275B9AD1AE85}</x:author>
-    <x:author>tc={C2F46B24-2450-5E98-6D52-DF86BB7667DC}</x:author>
-    <x:author>tc={8FAC92D9-1FE1-F845-F816-AAEEFE3656BE}</x:author>
-    <x:author>tc={1686F699-B0D7-C1A8-9524-B59E2785A701}</x:author>
+    <x:author>tc={27470C1F-3E86-8AB5-8DB2-4196211928B4}</x:author>
+    <x:author>tc={43B9B88D-1E17-4E9D-74E8-79D88964076A}</x:author>
+    <x:author>tc={09C81470-7D1E-7221-B2D8-AA6FD4872EA8}</x:author>
+    <x:author>tc={B59682A6-6FDF-C9D6-870D-7DFF71907310}</x:author>
+    <x:author>tc={A878EB5D-8AA5-15D0-1FA1-02C44890B262}</x:author>
+    <x:author>tc={95008EB4-3C0F-98C5-23B3-F71424269E1D}</x:author>
+    <x:author>tc={6B501EBC-3B59-1C5A-6193-2997D84A5FBB}</x:author>
+    <x:author>tc={11DFB307-4A3F-3FDB-1070-4151518E0AEE}</x:author>
+    <x:author>tc={17A3383E-26CF-FF32-8293-53AA83273718}</x:author>
+    <x:author>tc={0895042D-2EC8-4E8E-011C-BD30B2542F82}</x:author>
+    <x:author>tc={DE321951-CF60-2B51-28A6-7C21ECDC92A6}</x:author>
+    <x:author>tc={C5BB0CCC-B25B-84F6-9375-86524FB267AC}</x:author>
+    <x:author>tc={6412D127-5C7A-8179-ACAD-A754CB27998E}</x:author>
+    <x:author>tc={D1907D5E-7F3C-9668-216D-2F5A5682EBA9}</x:author>
+    <x:author>tc={8468B24A-1F34-D920-1D08-3C2BCB9FBF9C}</x:author>
+    <x:author>tc={EE993572-ECCA-649C-B5F1-BEB76AC2CEAB}</x:author>
+    <x:author>tc={66E75104-6D85-7D8A-3B72-FE434D67D1E9}</x:author>
+    <x:author>tc={B7BFF56B-7F7A-1E49-543F-E2938CD11F48}</x:author>
+    <x:author>tc={F131E133-4295-35BA-8C5E-AED07532BAFE}</x:author>
+    <x:author>tc={5DD49923-5E31-F51D-F964-B00D6B7355DC}</x:author>
+    <x:author>tc={2ACC0BB8-7789-7C2D-2CFB-67C3CF3FD4F3}</x:author>
+    <x:author>tc={B53DB07E-4BFC-B3DE-D0FF-6B25A369037B}</x:author>
+    <x:author>tc={65F3C94E-0D3D-417F-90E4-49B726CC0C03}</x:author>
+    <x:author>tc={4B0328F8-ED35-E3C0-9FF9-3FCDCA19A578}</x:author>
+    <x:author>tc={AEB20C69-FF92-1059-3CB3-67FB80E83B25}</x:author>
+    <x:author>tc={CC51BCE6-9571-9338-4887-DFB1DDBE7CFE}</x:author>
+    <x:author>tc={57BF8223-B24F-CB96-C67D-FE3778AB7A98}</x:author>
+    <x:author>tc={9DB71CD8-5F5A-D445-BA69-7431FF07F420}</x:author>
+    <x:author>tc={BC682973-4495-F651-1E6B-5D638F213481}</x:author>
+    <x:author>tc={B29A439B-5573-E40C-A3F2-47DC01C114CA}</x:author>
+    <x:author>tc={27FB8DDD-912C-1E7A-7752-AC2705E606D1}</x:author>
+    <x:author>tc={D64CC503-5D80-D76D-2203-9D94BA4D1DD6}</x:author>
+    <x:author>tc={2D48482E-942F-70F1-9A1F-3042DF18F561}</x:author>
+    <x:author>tc={C6B6AE69-95AE-3428-95C7-F692D3F5D5E7}</x:author>
+    <x:author>tc={8B99EECA-E1B0-BB8C-FDE3-12304B6E8837}</x:author>
+    <x:author>tc={F0E086AD-557A-9367-4ADE-1174F432B4B0}</x:author>
+    <x:author>tc={67850FFA-4D8D-12EF-F53E-9156F80A11A3}</x:author>
+    <x:author>tc={042B242A-E4E4-1CEA-BC47-62C535AD710E}</x:author>
+    <x:author>tc={C18243BE-FBA2-E2DB-596C-F13761AAE732}</x:author>
+    <x:author>tc={48E8FE26-4F2B-76EF-9633-0159BA519100}</x:author>
+    <x:author>tc={587E4A9F-063E-97FE-91A7-D7AA3D4C7D0C}</x:author>
+    <x:author>tc={DD15F858-A966-B3D7-AE9F-F7E782BCF67F}</x:author>
+    <x:author>tc={698148F6-A858-A2E4-43B4-090624731F08}</x:author>
+    <x:author>tc={3C42F2E9-5177-361F-C391-72A553BBDCFD}</x:author>
+    <x:author>tc={615871BF-6F97-376B-4041-7D4A2BE913E4}</x:author>
+    <x:author>tc={29076D46-81AC-3DA1-E553-FB2CF9C5DB53}</x:author>
+    <x:author>tc={640CFE87-0AB4-B553-BD22-210F6ED666FE}</x:author>
+    <x:author>tc={FF2EA90D-4615-E514-5382-8D7E2A36F5C8}</x:author>
+    <x:author>tc={26168C5B-79CB-D690-B1F7-4645EDB98430}</x:author>
+    <x:author>tc={B7520A70-7331-EEF2-D384-8DA397742486}</x:author>
+    <x:author>tc={4A348036-AB29-AC77-7331-B011B8134AE2}</x:author>
+    <x:author>tc={4042F39D-46F4-EEDE-CCC8-9BBA2F58914E}</x:author>
+    <x:author>tc={0AB46C1E-AB8F-81EA-04D0-66352A0116C5}</x:author>
+    <x:author>tc={D210A386-4279-382A-0842-A075EAF7050A}</x:author>
+    <x:author>tc={D8EB7CCD-07F5-1D6D-9311-D9670A2252D0}</x:author>
+    <x:author>tc={208C58C9-AD84-A1B7-1B1D-5E8F708B725B}</x:author>
+    <x:author>tc={CDB5BC5C-C7CE-B2C9-6BC5-729C2FE78534}</x:author>
+    <x:author>tc={B82F8D3D-4FA3-34A2-007F-93F66166FCE9}</x:author>
+    <x:author>tc={355858EA-94D6-A5F1-5963-0D4B997DA6C7}</x:author>
+    <x:author>tc={0A6E155D-B6F7-4B90-E2F6-8434C38B6F32}</x:author>
+    <x:author>tc={8D39E17F-76E1-A06B-2B06-E442780A77FA}</x:author>
+    <x:author>tc={CB4D955D-631A-8D96-DA59-2A911C6CB46F}</x:author>
+    <x:author>tc={1945AC02-CDAF-71E1-C7DC-047DA0EF251B}</x:author>
+    <x:author>tc={DFA5B975-6AB1-8691-97D2-36BCCCC8EDC8}</x:author>
+    <x:author>tc={56DC07E0-8BA3-3FE7-E501-566B57DA91F2}</x:author>
+    <x:author>tc={6B070A3A-232C-704C-5690-A92B4F27B006}</x:author>
+    <x:author>tc={915CDFF3-212A-29C2-9707-BF1B51CEEF46}</x:author>
+    <x:author>tc={B63BE17A-0F55-CC42-213E-DA710F640E8E}</x:author>
+    <x:author>tc={47566A22-B4FC-24A0-4A33-5499E94221F3}</x:author>
+    <x:author>tc={94F3B43E-34AA-D7D0-4C98-A0704157CD3B}</x:author>
+    <x:author>tc={3746D14E-7E36-4093-679A-03CB636182CB}</x:author>
+    <x:author>tc={07D3A048-4A5B-9511-5E96-DA82AC82981A}</x:author>
+    <x:author>tc={955769CA-F12C-6DE2-267A-2F9FA6FA447D}</x:author>
+    <x:author>tc={8B151F4C-CDFE-87DA-66A2-3019B71A46CA}</x:author>
+    <x:author>tc={E7294CE3-02B5-FE19-12E8-574930490330}</x:author>
+    <x:author>tc={351C48BB-DDEC-1F7B-E62E-199377745A55}</x:author>
+    <x:author>tc={7B935A8A-05BF-F039-71E6-6CC5A47A6FF7}</x:author>
+    <x:author>tc={C98FDE63-8E41-FCB8-46F4-EB23F118E951}</x:author>
+    <x:author>tc={B386906A-8267-D740-4904-2411DA5BE461}</x:author>
+    <x:author>tc={86940D5A-A9E3-91D3-D186-E09042CF5A01}</x:author>
+    <x:author>tc={F97DBEE1-5872-FF44-12BC-64BD321E1FD5}</x:author>
+    <x:author>tc={D60FA9C1-54B0-8F3B-C9BB-6E08D839AC43}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="P5" authorId="0">
@@ -1176,26 +1176,26 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={1AC6FA9D-6EAF-4D3D-C375-CE877C69E260}</x:author>
-    <x:author>tc={3326CE3D-BC56-94A6-EE75-9FF44A04FBF9}</x:author>
-    <x:author>tc={A198EC00-C1E3-A8A8-AC4A-67A8B8F010BB}</x:author>
-    <x:author>tc={776DE28D-8AC0-2C7A-9807-00F5444D703D}</x:author>
-    <x:author>tc={6796EA78-A81F-DDBF-7E66-30157FC65830}</x:author>
-    <x:author>tc={CACFC29D-1990-F2B4-3C09-1DA8A69188E8}</x:author>
-    <x:author>tc={4190D384-F5E8-3DFD-D3CD-FF286FB9D4A6}</x:author>
-    <x:author>tc={DAFC6F34-CDF1-903C-10A6-184187A22E45}</x:author>
-    <x:author>tc={70F2FEBE-C8AF-EC53-9654-05E07CEE7755}</x:author>
-    <x:author>tc={67293E1B-F0C0-D9F1-5F84-C1B0961128F9}</x:author>
-    <x:author>tc={8F554A60-1949-E8A2-381C-F75948BE7625}</x:author>
-    <x:author>tc={098ED24E-3E3F-B884-77A6-1F1588D94C89}</x:author>
-    <x:author>tc={F1CE5709-A240-337C-D02D-CA48439B5DE4}</x:author>
-    <x:author>tc={14AF2B76-3471-DAB3-580D-D5C33A1454D9}</x:author>
-    <x:author>tc={7EF3A7A6-3D3F-E608-1ADE-2C7F9793F446}</x:author>
-    <x:author>tc={36D05D5C-837A-8195-8F78-0276FD04F15A}</x:author>
-    <x:author>tc={4A543F82-A7AD-EAD9-AE30-DA0D3AE12465}</x:author>
-    <x:author>tc={DA604E42-7C6E-CBE1-A6DC-5AC2EE98E227}</x:author>
-    <x:author>tc={3D7D7B80-DA40-ABB3-0828-1BEACC3AC788}</x:author>
-    <x:author>tc={FD461D61-E8E0-FF46-FCCC-F572C22C9E49}</x:author>
+    <x:author>tc={FF8E5068-65B0-98F7-06E8-04DF16836F9E}</x:author>
+    <x:author>tc={7F2D520E-EEB8-9B5B-A5FA-AC8684943CFC}</x:author>
+    <x:author>tc={99E54B8E-9A24-1D9B-D18D-A99CEE3073A9}</x:author>
+    <x:author>tc={E2408B08-DC23-E00C-ABC8-F8B0509D3010}</x:author>
+    <x:author>tc={04258BAD-A27F-91D5-78C7-2A8BA5B7C41F}</x:author>
+    <x:author>tc={ED6A5C66-C750-3738-9A68-F382389FA981}</x:author>
+    <x:author>tc={F9AF018B-7EE4-8405-B37E-D109D51BFAFF}</x:author>
+    <x:author>tc={51269B21-4255-FF54-E2AF-8E4098E64A3F}</x:author>
+    <x:author>tc={649E091F-A36A-D779-650E-6BBCA18ACD93}</x:author>
+    <x:author>tc={4E7BBEF9-CE9F-16C6-EDE8-5E5C7A9D23BD}</x:author>
+    <x:author>tc={1C2DA460-DAAE-BC6C-6F6F-B3EDEE0A4861}</x:author>
+    <x:author>tc={20437B8E-9FE6-66D8-BB72-40C14527F354}</x:author>
+    <x:author>tc={D749FECF-1A2E-3C4C-80B3-998EA745BA3E}</x:author>
+    <x:author>tc={E25AF189-AEEE-2810-9414-A95677204CDA}</x:author>
+    <x:author>tc={2525E799-85EE-FA6A-EE32-F00FF4E0A7B5}</x:author>
+    <x:author>tc={FFC2E545-B41D-A496-7326-AEAA054FC0A0}</x:author>
+    <x:author>tc={9CA82BEE-D657-5811-0AE1-EA4678C0CB1B}</x:author>
+    <x:author>tc={E71B444B-6DC1-88D6-1590-4082B5507BF4}</x:author>
+    <x:author>tc={AB5B8F92-786E-326A-1D64-8D139AAECF36}</x:author>
+    <x:author>tc={9AA7456A-20BE-E4F2-DA0E-556803D2059F}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="J5" authorId="0">
@@ -2060,7 +2060,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7ee2500d485f42f8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdfcace26e8534658"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2071,7 +2071,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}"/>
+  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{574C0617-F997-4DBE-9033-40879B9F29D3}"/>
 </xltc:personList>
 </file>
 
@@ -2268,493 +2268,493 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="P5" dT="2026-08-15T14:36:30.107" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{173C717C-6858-7160-C636-C83BB42F4532}">
+  <xltc:threadedComment ref="P5" dT="2026-08-15T14:42:13.3" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{27470C1F-3E86-8AB5-8DB2-4196211928B4}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P6" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{63B2970C-3788-C112-A8CB-3B3F13ACBE33}">
+  <xltc:threadedComment ref="P6" dT="2026-08-15T14:42:13.304" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{43B9B88D-1E17-4E9D-74E8-79D88964076A}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P7" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{1004044F-FE88-537F-AC06-F229E6AF84A6}">
+  <xltc:threadedComment ref="P7" dT="2026-08-15T14:42:13.304" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{09C81470-7D1E-7221-B2D8-AA6FD4872EA8}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P8" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{1E2BDBA3-BE2D-AA43-6606-B5993279A758}">
+  <xltc:threadedComment ref="P8" dT="2026-08-15T14:42:13.304" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B59682A6-6FDF-C9D6-870D-7DFF71907310}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P9" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{3F9E6F84-FE0D-36B7-9ADD-24B5BCFA51E6}">
+  <xltc:threadedComment ref="P9" dT="2026-08-15T14:42:13.304" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{A878EB5D-8AA5-15D0-1FA1-02C44890B262}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P10" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{52AA49C5-8E9B-AE59-8B98-6545B28EE15B}">
+  <xltc:threadedComment ref="P10" dT="2026-08-15T14:42:13.304" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{95008EB4-3C0F-98C5-23B3-F71424269E1D}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 119
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P11" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{B1891568-FC99-A969-F70D-CDEE8457BEFC}">
+  <xltc:threadedComment ref="P11" dT="2026-08-15T14:42:13.304" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{6B501EBC-3B59-1C5A-6193-2997D84A5FBB}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 160
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P12" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{082D8A79-A0D4-C019-F864-DBE641EEAB38}">
+  <xltc:threadedComment ref="P12" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{11DFB307-4A3F-3FDB-1070-4151518E0AEE}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P13" dT="2026-08-15T14:36:30.11" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{BDC1023A-5DD2-F2EB-A432-D3B36A50FE54}">
+  <xltc:threadedComment ref="P13" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{17A3383E-26CF-FF32-8293-53AA83273718}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P14" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{51E90830-4873-6DFE-41AE-2C910C9EEC9A}">
+  <xltc:threadedComment ref="P14" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{0895042D-2EC8-4E8E-011C-BD30B2542F82}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P15" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{3ED164EE-A0A3-1A42-DA4E-68B6CC7260DF}">
+  <xltc:threadedComment ref="P15" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{DE321951-CF60-2B51-28A6-7C21ECDC92A6}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P16" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{CD8DF9C8-1E20-61D4-7F1C-891F953050CD}">
+  <xltc:threadedComment ref="P16" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{C5BB0CCC-B25B-84F6-9375-86524FB267AC}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P17" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{E95BF887-32D2-04EB-A1EE-98E9C196D9F3}">
+  <xltc:threadedComment ref="P17" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{6412D127-5C7A-8179-ACAD-A754CB27998E}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P18" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{CFB45910-E24C-077D-186B-932BFADA7BB1}">
+  <xltc:threadedComment ref="P18" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{D1907D5E-7F3C-9668-216D-2F5A5682EBA9}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P19" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{47009490-050D-D2C8-1D90-48664025D854}">
+  <xltc:threadedComment ref="P19" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{8468B24A-1F34-D920-1D08-3C2BCB9FBF9C}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P20" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{06CB3692-098C-5306-68AC-91CCFF18BE8F}">
+  <xltc:threadedComment ref="P20" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{EE993572-ECCA-649C-B5F1-BEB76AC2CEAB}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 138
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P21" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{F26F73B4-C89E-B0B5-6F81-517E9959514E}">
+  <xltc:threadedComment ref="P21" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{66E75104-6D85-7D8A-3B72-FE434D67D1E9}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 212
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P22" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{8C7801E9-DFAA-9CEC-1604-7E8730022DCD}">
+  <xltc:threadedComment ref="P22" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B7BFF56B-7F7A-1E49-543F-E2938CD11F48}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P23" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{2E910827-D22C-F652-E278-F78E32BB95D1}">
+  <xltc:threadedComment ref="P23" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{F131E133-4295-35BA-8C5E-AED07532BAFE}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P24" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{F8058C0F-D0E2-3A18-9FD0-3A84595B81D3}">
+  <xltc:threadedComment ref="P24" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{5DD49923-5E31-F51D-F964-B00D6B7355DC}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P25" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{4E7D4B04-0DB5-1B68-B26D-A0513C7909AE}">
+  <xltc:threadedComment ref="P25" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{2ACC0BB8-7789-7C2D-2CFB-67C3CF3FD4F3}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P26" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{A5421185-8955-0192-1B5D-5FA24B4854CE}">
+  <xltc:threadedComment ref="P26" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B53DB07E-4BFC-B3DE-D0FF-6B25A369037B}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P27" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{0EA2A1B3-BE69-7BC7-D93B-5925841F1A59}">
+  <xltc:threadedComment ref="P27" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{65F3C94E-0D3D-417F-90E4-49B726CC0C03}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 272
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P28" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{12584A4C-4517-9B31-E395-34E738042FAA}">
+  <xltc:threadedComment ref="P28" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{4B0328F8-ED35-E3C0-9FF9-3FCDCA19A578}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P29" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{6441A2AC-3623-5BD9-B536-033F6323D5EE}">
+  <xltc:threadedComment ref="P29" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{AEB20C69-FF92-1059-3CB3-67FB80E83B25}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P30" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{AB84A56E-9609-E927-6600-C0AC02186EA5}">
+  <xltc:threadedComment ref="P30" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{CC51BCE6-9571-9338-4887-DFB1DDBE7CFE}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 158
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P31" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{86FA8428-52FC-537E-D895-7C577F1B0D25}">
+  <xltc:threadedComment ref="P31" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{57BF8223-B24F-CB96-C67D-FE3778AB7A98}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P32" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{14FB8611-E78E-C75D-EC48-3871F4AEFC06}">
+  <xltc:threadedComment ref="P32" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{9DB71CD8-5F5A-D445-BA69-7431FF07F420}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P33" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{99635604-65F2-307E-FADC-135187FF0D1F}">
+  <xltc:threadedComment ref="P33" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{BC682973-4495-F651-1E6B-5D638F213481}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 72
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P34" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{B27FFCF3-F14E-0235-2C1A-8E7397E20E00}">
+  <xltc:threadedComment ref="P34" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B29A439B-5573-E40C-A3F2-47DC01C114CA}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P35" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{25CD3762-ABE2-6CD8-5ECA-882CFCFDFB28}">
+  <xltc:threadedComment ref="P35" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{27FB8DDD-912C-1E7A-7752-AC2705E606D1}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P36" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{7482A080-D14E-D33F-31C2-3D2B683AEEDB}">
+  <xltc:threadedComment ref="P36" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{D64CC503-5D80-D76D-2203-9D94BA4D1DD6}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 24
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P37" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{05D0B2B8-7D76-EC43-30FD-ADED4B860D66}">
+  <xltc:threadedComment ref="P37" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{2D48482E-942F-70F1-9A1F-3042DF18F561}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P38" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{BE7F4BA9-DA30-4C28-6BE5-4A368E0CA4D9}">
+  <xltc:threadedComment ref="P38" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{C6B6AE69-95AE-3428-95C7-F692D3F5D5E7}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P39" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{D8D08379-B543-B20B-C166-5B2F5E58674D}">
+  <xltc:threadedComment ref="P39" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{8B99EECA-E1B0-BB8C-FDE3-12304B6E8837}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 19
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P40" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{2514B5B4-895E-E9D1-0755-E6B42562A8B6}">
+  <xltc:threadedComment ref="P40" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{F0E086AD-557A-9367-4ADE-1174F432B4B0}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P41" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{43E6F669-33EA-0919-B765-BB8AC1041BB1}">
+  <xltc:threadedComment ref="P41" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{67850FFA-4D8D-12EF-F53E-9156F80A11A3}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P42" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{8336B492-3FF6-8AC2-E3A6-5F44649A0793}">
+  <xltc:threadedComment ref="P42" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{042B242A-E4E4-1CEA-BC47-62C535AD710E}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P43" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{0CE2DDAB-726A-1C7D-E5A5-092266E6B8A7}">
+  <xltc:threadedComment ref="P43" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{C18243BE-FBA2-E2DB-596C-F13761AAE732}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P44" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{B1C20038-E535-B4B6-8559-C261A73A67A1}">
+  <xltc:threadedComment ref="P44" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{48E8FE26-4F2B-76EF-9633-0159BA519100}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P45" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{57536159-910E-5D86-FB2B-73B577D12D3E}">
+  <xltc:threadedComment ref="P45" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{587E4A9F-063E-97FE-91A7-D7AA3D4C7D0C}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P46" dT="2026-08-15T14:36:30.111" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{D8BAA6FE-5711-436E-F6EA-EC4A4D479D92}">
+  <xltc:threadedComment ref="P46" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{DD15F858-A966-B3D7-AE9F-F7E782BCF67F}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P47" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{F5755A1F-8854-9435-2022-0AAB87F7C037}">
+  <xltc:threadedComment ref="P47" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{698148F6-A858-A2E4-43B4-090624731F08}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P48" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{44FD8D82-299B-AD44-7B33-5F8860959C9B}">
+  <xltc:threadedComment ref="P48" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{3C42F2E9-5177-361F-C391-72A553BBDCFD}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P49" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{B44CBE08-D433-F425-B76C-F08D9E356FFC}">
+  <xltc:threadedComment ref="P49" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{615871BF-6F97-376B-4041-7D4A2BE913E4}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 118
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P50" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{6D90F121-6572-2506-1058-7D5A9144D000}">
+  <xltc:threadedComment ref="P50" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{29076D46-81AC-3DA1-E553-FB2CF9C5DB53}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P51" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{0CA59E25-F025-10EF-9141-692AEF3B8F83}">
+  <xltc:threadedComment ref="P51" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{640CFE87-0AB4-B553-BD22-210F6ED666FE}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P52" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{D9640E49-A5C7-B65F-9A0D-65D7DB24EEBB}">
+  <xltc:threadedComment ref="P52" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{FF2EA90D-4615-E514-5382-8D7E2A36F5C8}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P53" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{3BCB9DCC-576A-8A6F-A65E-71776E316C77}">
+  <xltc:threadedComment ref="P53" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{26168C5B-79CB-D690-B1F7-4645EDB98430}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-STF</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P54" dT="2026-08-15T14:36:30.112" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{054F0263-F06E-2F91-A378-2F9A307D6D3D}">
+  <xltc:threadedComment ref="P54" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B7520A70-7331-EEF2-D384-8DA397742486}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P55" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{F3A816E8-0428-7682-BDE7-835E8A07F037}">
+  <xltc:threadedComment ref="P55" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{4A348036-AB29-AC77-7331-B011B8134AE2}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P56" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{0FBC7355-F891-4C26-0974-184BF3E0A490}">
+  <xltc:threadedComment ref="P56" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{4042F39D-46F4-EEDE-CCC8-9BBA2F58914E}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 18
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P57" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{5379010D-20B2-3559-7434-AC60A3BF9149}">
+  <xltc:threadedComment ref="P57" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{0AB46C1E-AB8F-81EA-04D0-66352A0116C5}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P58" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{51ED7905-5FC0-2EFA-FCDE-ECB06F341B85}">
+  <xltc:threadedComment ref="P58" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{D210A386-4279-382A-0842-A075EAF7050A}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P59" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{460F10D2-05CC-CAD6-9D7B-42E804103D60}">
+  <xltc:threadedComment ref="P59" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{D8EB7CCD-07F5-1D6D-9311-D9670A2252D0}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P60" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{B0D2CF89-A5D6-BB93-1A21-2092A154CDEB}">
+  <xltc:threadedComment ref="P60" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{208C58C9-AD84-A1B7-1B1D-5E8F708B725B}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P61" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{0FF99E4B-1649-B79E-6846-BAB0B145BE40}">
+  <xltc:threadedComment ref="P61" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{CDB5BC5C-C7CE-B2C9-6BC5-729C2FE78534}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P62" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{474588F9-4D2F-A36A-DCA6-06FE18FC9D3F}">
+  <xltc:threadedComment ref="P62" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B82F8D3D-4FA3-34A2-007F-93F66166FCE9}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P63" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{8F95FF9A-75EB-FA03-9D2C-BA0BD80069C7}">
+  <xltc:threadedComment ref="P63" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{355858EA-94D6-A5F1-5963-0D4B997DA6C7}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P64" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{4FA8524D-4B33-0F1D-CFB8-A4A4B3CF6D22}">
+  <xltc:threadedComment ref="P64" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{0A6E155D-B6F7-4B90-E2F6-8434C38B6F32}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P65" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{6A13DB9F-7B8D-7945-B42B-55E9B525BE4D}">
+  <xltc:threadedComment ref="P65" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{8D39E17F-76E1-A06B-2B06-E442780A77FA}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 311
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P66" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{C0FFAB0F-E235-51E1-F5A7-702EBE41B4BC}">
+  <xltc:threadedComment ref="P66" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{CB4D955D-631A-8D96-DA59-2A911C6CB46F}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P67" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{558F1A80-BA34-1373-D92E-130F76E0C9DE}">
+  <xltc:threadedComment ref="P67" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{1945AC02-CDAF-71E1-C7DC-047DA0EF251B}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P68" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{7D0D67D7-EDCA-0883-5925-8C9CA41D3ED5}">
+  <xltc:threadedComment ref="P68" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{DFA5B975-6AB1-8691-97D2-36BCCCC8EDC8}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 141
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P69" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{26B419AF-C3DC-BC5C-BB92-7C27A26EAA95}">
+  <xltc:threadedComment ref="P69" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{56DC07E0-8BA3-3FE7-E501-566B57DA91F2}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P70" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{B229E44D-B4F8-845C-BDF5-06F06E4AC987}">
+  <xltc:threadedComment ref="P70" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{6B070A3A-232C-704C-5690-A92B4F27B006}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P71" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{3E3301DB-5DB0-34EC-8884-441067EF8773}">
+  <xltc:threadedComment ref="P71" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{915CDFF3-212A-29C2-9707-BF1B51CEEF46}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 33
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P72" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{8DB03130-4013-2315-00A4-399BAEAA7F88}">
+  <xltc:threadedComment ref="P72" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B63BE17A-0F55-CC42-213E-DA710F640E8E}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P73" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{986C3E99-675F-B218-0291-236382FB05A2}">
+  <xltc:threadedComment ref="P73" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{47566A22-B4FC-24A0-4A33-5499E94221F3}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P74" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{CC7C148B-B643-114F-7100-4F32E1A7D46E}">
+  <xltc:threadedComment ref="P74" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{94F3B43E-34AA-D7D0-4C98-A0704157CD3B}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 21
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P75" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{FD756AED-3359-1847-B024-B000A9F62B6D}">
+  <xltc:threadedComment ref="P75" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{3746D14E-7E36-4093-679A-03CB636182CB}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P76" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{D002F702-8EF9-9DAA-6B83-D18075632BAD}">
+  <xltc:threadedComment ref="P76" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{07D3A048-4A5B-9511-5E96-DA82AC82981A}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P77" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{847AF31F-15DC-F58D-7348-44272FF30608}">
+  <xltc:threadedComment ref="P77" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{955769CA-F12C-6DE2-267A-2F9FA6FA447D}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 19
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P78" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{C96A5CA6-0B02-6230-71B6-16D0BEAF2C32}">
+  <xltc:threadedComment ref="P78" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{8B151F4C-CDFE-87DA-66A2-3019B71A46CA}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 43
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P79" dT="2026-08-15T14:36:30.113" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{003727CF-D765-0E72-39DF-F489DF2AB89F}">
+  <xltc:threadedComment ref="P79" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{E7294CE3-02B5-FE19-12E8-574930490330}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 44
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P80" dT="2026-08-15T14:36:30.114" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{94C07DE9-2411-7BFD-D930-FDAE7DE86182}">
+  <xltc:threadedComment ref="P80" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{351C48BB-DDEC-1F7B-E62E-199377745A55}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 40
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P81" dT="2026-08-15T14:36:30.114" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{15E2FF33-AEF0-4F29-0077-E9841AB6D1F2}">
+  <xltc:threadedComment ref="P81" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{7B935A8A-05BF-F039-71E6-6CC5A47A6FF7}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P82" dT="2026-08-15T14:36:30.114" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{94BDFAEF-248A-4ECF-AF7B-95B24E03AEF6}">
+  <xltc:threadedComment ref="P82" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{C98FDE63-8E41-FCB8-46F4-EB23F118E951}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P83" dT="2026-08-15T14:36:30.114" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{66C2F9EA-58E2-8003-9F91-275B9AD1AE85}">
+  <xltc:threadedComment ref="P83" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B386906A-8267-D740-4904-2411DA5BE461}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 16
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P84" dT="2026-08-15T14:36:30.114" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{C2F46B24-2450-5E98-6D52-DF86BB7667DC}">
+  <xltc:threadedComment ref="P84" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{86940D5A-A9E3-91D3-D186-E09042CF5A01}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P85" dT="2026-08-15T14:36:30.114" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{8FAC92D9-1FE1-F845-F816-AAEEFE3656BE}">
+  <xltc:threadedComment ref="P85" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{F97DBEE1-5872-FF44-12BC-64BD321E1FD5}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P86" dT="2026-08-15T14:36:30.114" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{1686F699-B0D7-C1A8-9524-B59E2785A701}">
+  <xltc:threadedComment ref="P86" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{D60FA9C1-54B0-8F3B-C9BB-6E08D839AC43}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 21
 Available: 2026-02-25
@@ -2765,64 +2765,64 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="J5" dT="2026-08-15T14:36:30.456" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{1AC6FA9D-6EAF-4D3D-C375-CE877C69E260}">
+  <xltc:threadedComment ref="J5" dT="2026-08-15T14:42:13.65" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{FF8E5068-65B0-98F7-06E8-04DF16836F9E}">
     <xltc:text>Official source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J6" dT="2026-08-15T14:36:30.459" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{3326CE3D-BC56-94A6-EE75-9FF44A04FBF9}">
+  <xltc:threadedComment ref="J6" dT="2026-08-15T14:42:13.652" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{7F2D520E-EEB8-9B5B-A5FA-AC8684943CFC}">
     <xltc:text>Official source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J7" dT="2026-08-15T14:36:30.462" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{A198EC00-C1E3-A8A8-AC4A-67A8B8F010BB}">
+  <xltc:threadedComment ref="J7" dT="2026-08-15T14:42:13.654" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{99E54B8E-9A24-1D9B-D18D-A99CEE3073A9}">
     <xltc:text>Official source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J8" dT="2026-08-15T14:36:30.465" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{776DE28D-8AC0-2C7A-9807-00F5444D703D}">
+  <xltc:threadedComment ref="J8" dT="2026-08-15T14:42:13.656" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{E2408B08-DC23-E00C-ABC8-F8B0509D3010}">
     <xltc:text>Official source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J9" dT="2026-08-15T14:36:30.466" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{6796EA78-A81F-DDBF-7E66-30157FC65830}">
+  <xltc:threadedComment ref="J9" dT="2026-08-15T14:42:13.658" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{04258BAD-A27F-91D5-78C7-2A8BA5B7C41F}">
     <xltc:text>Official source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J10" dT="2026-08-15T14:36:30.469" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{CACFC29D-1990-F2B4-3C09-1DA8A69188E8}">
+  <xltc:threadedComment ref="J10" dT="2026-08-15T14:42:13.661" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{ED6A5C66-C750-3738-9A68-F382389FA981}">
     <xltc:text>Official source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J11" dT="2026-08-15T14:36:30.471" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{4190D384-F5E8-3DFD-D3CD-FF286FB9D4A6}">
+  <xltc:threadedComment ref="J11" dT="2026-08-15T14:42:13.663" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{F9AF018B-7EE4-8405-B37E-D109D51BFAFF}">
     <xltc:text>Official source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J12" dT="2026-08-15T14:36:30.473" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{DAFC6F34-CDF1-903C-10A6-184187A22E45}">
+  <xltc:threadedComment ref="J12" dT="2026-08-15T14:42:13.664" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{51269B21-4255-FF54-E2AF-8E4098E64A3F}">
     <xltc:text>Official source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J13" dT="2026-08-15T14:36:30.475" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{70F2FEBE-C8AF-EC53-9654-05E07CEE7755}">
+  <xltc:threadedComment ref="J13" dT="2026-08-15T14:42:13.666" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{649E091F-A36A-D779-650E-6BBCA18ACD93}">
     <xltc:text>Official source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J14" dT="2026-08-15T14:36:30.478" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{67293E1B-F0C0-D9F1-5F84-C1B0961128F9}">
+  <xltc:threadedComment ref="J14" dT="2026-08-15T14:42:13.667" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{4E7BBEF9-CE9F-16C6-EDE8-5E5C7A9D23BD}">
     <xltc:text>Official source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J15" dT="2026-08-15T14:36:30.48" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{8F554A60-1949-E8A2-381C-F75948BE7625}">
+  <xltc:threadedComment ref="J15" dT="2026-08-15T14:42:13.669" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{1C2DA460-DAAE-BC6C-6F6F-B3EDEE0A4861}">
     <xltc:text>Official source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J16" dT="2026-08-15T14:36:30.481" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{098ED24E-3E3F-B884-77A6-1F1588D94C89}">
+  <xltc:threadedComment ref="J16" dT="2026-08-15T14:42:13.673" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{20437B8E-9FE6-66D8-BB72-40C14527F354}">
     <xltc:text>Official source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J17" dT="2026-08-15T14:36:30.483" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{F1CE5709-A240-337C-D02D-CA48439B5DE4}">
+  <xltc:threadedComment ref="J17" dT="2026-08-15T14:42:13.674" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{D749FECF-1A2E-3C4C-80B3-998EA745BA3E}">
     <xltc:text>Official source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J18" dT="2026-08-15T14:36:30.484" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{14AF2B76-3471-DAB3-580D-D5C33A1454D9}">
+  <xltc:threadedComment ref="J18" dT="2026-08-15T14:42:13.677" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{E25AF189-AEEE-2810-9414-A95677204CDA}">
     <xltc:text>Official source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J19" dT="2026-08-15T14:36:30.488" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{7EF3A7A6-3D3F-E608-1ADE-2C7F9793F446}">
+  <xltc:threadedComment ref="J19" dT="2026-08-15T14:42:13.679" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{2525E799-85EE-FA6A-EE32-F00FF4E0A7B5}">
     <xltc:text>Official source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J20" dT="2026-08-15T14:36:30.49" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{36D05D5C-837A-8195-8F78-0276FD04F15A}">
+  <xltc:threadedComment ref="J20" dT="2026-08-15T14:42:13.68" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{FFC2E545-B41D-A496-7326-AEAA054FC0A0}">
     <xltc:text>Official source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J21" dT="2026-08-15T14:36:30.491" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{4A543F82-A7AD-EAD9-AE30-DA0D3AE12465}">
+  <xltc:threadedComment ref="J21" dT="2026-08-15T14:42:13.682" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{9CA82BEE-D657-5811-0AE1-EA4678C0CB1B}">
     <xltc:text>Official source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J22" dT="2026-08-15T14:36:30.493" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{DA604E42-7C6E-CBE1-A6DC-5AC2EE98E227}">
+  <xltc:threadedComment ref="J22" dT="2026-08-15T14:42:13.684" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{E71B444B-6DC1-88D6-1590-4082B5507BF4}">
     <xltc:text>Official source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J23" dT="2026-08-15T14:36:30.495" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{3D7D7B80-DA40-ABB3-0828-1BEACC3AC788}">
+  <xltc:threadedComment ref="J23" dT="2026-08-15T14:42:13.685" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{AB5B8F92-786E-326A-1D64-8D139AAECF36}">
     <xltc:text>Official source: https://www.aspenpharma.com/download/annual-financial-statements-2/</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J24" dT="2026-08-15T14:36:30.496" personId="{8BFD9CA2-AF75-4211-B7A8-BCBD38BD78C3}" id="{FD461D61-E8E0-FF46-FCCC-F572C22C9E49}">
+  <xltc:threadedComment ref="J24" dT="2026-08-15T14:42:13.687" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{9AA7456A-20BE-E4F2-DA0E-556803D2059F}">
     <xltc:text>Official source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -3877,7 +3877,7 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R817a88bcb3fc44b6"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5057e7e7dc734e7a"/>
 </x:worksheet>
 </file>
 
@@ -8611,7 +8611,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb15147641d114dca"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80794ba59efd42e3"/>
 </x:worksheet>
 </file>
 
@@ -9671,7 +9671,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc20f38d184d94b29"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re696f294952b47c0"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Restamp V3.2 artifacts after portable hash fix
</commit_message>
<xml_diff>
--- a/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
+++ b/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R5ded0f81741d4f65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R4a49f1ac8efb40a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="R70d09ac268784577"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="R809eb01ba2d54f08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R14e4144764b449e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="Ra942e43c5fb24b49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Rfa974438e19e4dbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="Re2c2af9be93b49af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R500b0e8dc2794605"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="Radbea52237a3498b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Refa4995be3d04ee7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R8af1eebdbf8d4e62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="R7f50b9fc52bc4285"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="R8e7a6f998fc742c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R6d10c4373f9a45d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="Ra17269f826874465"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Rd5f4997859c94c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="Rf21410be4c814f8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="Rc712395c96ae4d64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="Rb1d41ec840144a46"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,88 +19,88 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={27470C1F-3E86-8AB5-8DB2-4196211928B4}</x:author>
-    <x:author>tc={43B9B88D-1E17-4E9D-74E8-79D88964076A}</x:author>
-    <x:author>tc={09C81470-7D1E-7221-B2D8-AA6FD4872EA8}</x:author>
-    <x:author>tc={B59682A6-6FDF-C9D6-870D-7DFF71907310}</x:author>
-    <x:author>tc={A878EB5D-8AA5-15D0-1FA1-02C44890B262}</x:author>
-    <x:author>tc={95008EB4-3C0F-98C5-23B3-F71424269E1D}</x:author>
-    <x:author>tc={6B501EBC-3B59-1C5A-6193-2997D84A5FBB}</x:author>
-    <x:author>tc={11DFB307-4A3F-3FDB-1070-4151518E0AEE}</x:author>
-    <x:author>tc={17A3383E-26CF-FF32-8293-53AA83273718}</x:author>
-    <x:author>tc={0895042D-2EC8-4E8E-011C-BD30B2542F82}</x:author>
-    <x:author>tc={DE321951-CF60-2B51-28A6-7C21ECDC92A6}</x:author>
-    <x:author>tc={C5BB0CCC-B25B-84F6-9375-86524FB267AC}</x:author>
-    <x:author>tc={6412D127-5C7A-8179-ACAD-A754CB27998E}</x:author>
-    <x:author>tc={D1907D5E-7F3C-9668-216D-2F5A5682EBA9}</x:author>
-    <x:author>tc={8468B24A-1F34-D920-1D08-3C2BCB9FBF9C}</x:author>
-    <x:author>tc={EE993572-ECCA-649C-B5F1-BEB76AC2CEAB}</x:author>
-    <x:author>tc={66E75104-6D85-7D8A-3B72-FE434D67D1E9}</x:author>
-    <x:author>tc={B7BFF56B-7F7A-1E49-543F-E2938CD11F48}</x:author>
-    <x:author>tc={F131E133-4295-35BA-8C5E-AED07532BAFE}</x:author>
-    <x:author>tc={5DD49923-5E31-F51D-F964-B00D6B7355DC}</x:author>
-    <x:author>tc={2ACC0BB8-7789-7C2D-2CFB-67C3CF3FD4F3}</x:author>
-    <x:author>tc={B53DB07E-4BFC-B3DE-D0FF-6B25A369037B}</x:author>
-    <x:author>tc={65F3C94E-0D3D-417F-90E4-49B726CC0C03}</x:author>
-    <x:author>tc={4B0328F8-ED35-E3C0-9FF9-3FCDCA19A578}</x:author>
-    <x:author>tc={AEB20C69-FF92-1059-3CB3-67FB80E83B25}</x:author>
-    <x:author>tc={CC51BCE6-9571-9338-4887-DFB1DDBE7CFE}</x:author>
-    <x:author>tc={57BF8223-B24F-CB96-C67D-FE3778AB7A98}</x:author>
-    <x:author>tc={9DB71CD8-5F5A-D445-BA69-7431FF07F420}</x:author>
-    <x:author>tc={BC682973-4495-F651-1E6B-5D638F213481}</x:author>
-    <x:author>tc={B29A439B-5573-E40C-A3F2-47DC01C114CA}</x:author>
-    <x:author>tc={27FB8DDD-912C-1E7A-7752-AC2705E606D1}</x:author>
-    <x:author>tc={D64CC503-5D80-D76D-2203-9D94BA4D1DD6}</x:author>
-    <x:author>tc={2D48482E-942F-70F1-9A1F-3042DF18F561}</x:author>
-    <x:author>tc={C6B6AE69-95AE-3428-95C7-F692D3F5D5E7}</x:author>
-    <x:author>tc={8B99EECA-E1B0-BB8C-FDE3-12304B6E8837}</x:author>
-    <x:author>tc={F0E086AD-557A-9367-4ADE-1174F432B4B0}</x:author>
-    <x:author>tc={67850FFA-4D8D-12EF-F53E-9156F80A11A3}</x:author>
-    <x:author>tc={042B242A-E4E4-1CEA-BC47-62C535AD710E}</x:author>
-    <x:author>tc={C18243BE-FBA2-E2DB-596C-F13761AAE732}</x:author>
-    <x:author>tc={48E8FE26-4F2B-76EF-9633-0159BA519100}</x:author>
-    <x:author>tc={587E4A9F-063E-97FE-91A7-D7AA3D4C7D0C}</x:author>
-    <x:author>tc={DD15F858-A966-B3D7-AE9F-F7E782BCF67F}</x:author>
-    <x:author>tc={698148F6-A858-A2E4-43B4-090624731F08}</x:author>
-    <x:author>tc={3C42F2E9-5177-361F-C391-72A553BBDCFD}</x:author>
-    <x:author>tc={615871BF-6F97-376B-4041-7D4A2BE913E4}</x:author>
-    <x:author>tc={29076D46-81AC-3DA1-E553-FB2CF9C5DB53}</x:author>
-    <x:author>tc={640CFE87-0AB4-B553-BD22-210F6ED666FE}</x:author>
-    <x:author>tc={FF2EA90D-4615-E514-5382-8D7E2A36F5C8}</x:author>
-    <x:author>tc={26168C5B-79CB-D690-B1F7-4645EDB98430}</x:author>
-    <x:author>tc={B7520A70-7331-EEF2-D384-8DA397742486}</x:author>
-    <x:author>tc={4A348036-AB29-AC77-7331-B011B8134AE2}</x:author>
-    <x:author>tc={4042F39D-46F4-EEDE-CCC8-9BBA2F58914E}</x:author>
-    <x:author>tc={0AB46C1E-AB8F-81EA-04D0-66352A0116C5}</x:author>
-    <x:author>tc={D210A386-4279-382A-0842-A075EAF7050A}</x:author>
-    <x:author>tc={D8EB7CCD-07F5-1D6D-9311-D9670A2252D0}</x:author>
-    <x:author>tc={208C58C9-AD84-A1B7-1B1D-5E8F708B725B}</x:author>
-    <x:author>tc={CDB5BC5C-C7CE-B2C9-6BC5-729C2FE78534}</x:author>
-    <x:author>tc={B82F8D3D-4FA3-34A2-007F-93F66166FCE9}</x:author>
-    <x:author>tc={355858EA-94D6-A5F1-5963-0D4B997DA6C7}</x:author>
-    <x:author>tc={0A6E155D-B6F7-4B90-E2F6-8434C38B6F32}</x:author>
-    <x:author>tc={8D39E17F-76E1-A06B-2B06-E442780A77FA}</x:author>
-    <x:author>tc={CB4D955D-631A-8D96-DA59-2A911C6CB46F}</x:author>
-    <x:author>tc={1945AC02-CDAF-71E1-C7DC-047DA0EF251B}</x:author>
-    <x:author>tc={DFA5B975-6AB1-8691-97D2-36BCCCC8EDC8}</x:author>
-    <x:author>tc={56DC07E0-8BA3-3FE7-E501-566B57DA91F2}</x:author>
-    <x:author>tc={6B070A3A-232C-704C-5690-A92B4F27B006}</x:author>
-    <x:author>tc={915CDFF3-212A-29C2-9707-BF1B51CEEF46}</x:author>
-    <x:author>tc={B63BE17A-0F55-CC42-213E-DA710F640E8E}</x:author>
-    <x:author>tc={47566A22-B4FC-24A0-4A33-5499E94221F3}</x:author>
-    <x:author>tc={94F3B43E-34AA-D7D0-4C98-A0704157CD3B}</x:author>
-    <x:author>tc={3746D14E-7E36-4093-679A-03CB636182CB}</x:author>
-    <x:author>tc={07D3A048-4A5B-9511-5E96-DA82AC82981A}</x:author>
-    <x:author>tc={955769CA-F12C-6DE2-267A-2F9FA6FA447D}</x:author>
-    <x:author>tc={8B151F4C-CDFE-87DA-66A2-3019B71A46CA}</x:author>
-    <x:author>tc={E7294CE3-02B5-FE19-12E8-574930490330}</x:author>
-    <x:author>tc={351C48BB-DDEC-1F7B-E62E-199377745A55}</x:author>
-    <x:author>tc={7B935A8A-05BF-F039-71E6-6CC5A47A6FF7}</x:author>
-    <x:author>tc={C98FDE63-8E41-FCB8-46F4-EB23F118E951}</x:author>
-    <x:author>tc={B386906A-8267-D740-4904-2411DA5BE461}</x:author>
-    <x:author>tc={86940D5A-A9E3-91D3-D186-E09042CF5A01}</x:author>
-    <x:author>tc={F97DBEE1-5872-FF44-12BC-64BD321E1FD5}</x:author>
-    <x:author>tc={D60FA9C1-54B0-8F3B-C9BB-6E08D839AC43}</x:author>
+    <x:author>tc={4DBD6BF6-10DC-C9AB-9CD1-709939978DBA}</x:author>
+    <x:author>tc={BBA7CF7E-AC28-261A-8B13-2F207C1218A0}</x:author>
+    <x:author>tc={72A601D1-876A-91CE-FFAD-4372EAC3B044}</x:author>
+    <x:author>tc={63AEFE69-E87F-CB50-C251-F53F91B5BC7D}</x:author>
+    <x:author>tc={34BD6919-CEFF-A072-C07C-DF821615DC08}</x:author>
+    <x:author>tc={06E212B9-C215-9B55-79D0-3DCC68FDC5F2}</x:author>
+    <x:author>tc={B3B2D943-46C7-7159-C4D2-5A2561471484}</x:author>
+    <x:author>tc={B7F42A5F-C7FD-3C66-478C-F3F30EC65E76}</x:author>
+    <x:author>tc={A4597E1D-F181-CFE5-0579-CB8E395D5F43}</x:author>
+    <x:author>tc={15C385B1-3102-7CB9-2CC5-9E1619C28EFF}</x:author>
+    <x:author>tc={71943B6E-65A7-8FB9-D610-7EAAF042FB72}</x:author>
+    <x:author>tc={9C0C8A6E-1868-2889-498E-623A34106926}</x:author>
+    <x:author>tc={334D3079-E2A2-64EF-8548-37B4110F83CB}</x:author>
+    <x:author>tc={E3828EA9-DCD7-589A-8909-33C5D206AAAB}</x:author>
+    <x:author>tc={7FDAF406-68E0-40BF-FF2E-810ED1C6B3AE}</x:author>
+    <x:author>tc={923B38B5-CB1F-C29F-3341-278DDD42C0D1}</x:author>
+    <x:author>tc={1A013CBB-E706-00DF-8726-CF619CEB3A04}</x:author>
+    <x:author>tc={EAC196E9-9494-9C63-D76F-35D9C8B67077}</x:author>
+    <x:author>tc={10D40289-30D1-453D-67F2-D072A488FDF3}</x:author>
+    <x:author>tc={52EC0200-BA64-4464-226D-17C81EC16731}</x:author>
+    <x:author>tc={9CC16C61-D3B8-BFC6-1D65-26993EA95662}</x:author>
+    <x:author>tc={87792696-2512-1D5F-88FE-607EFE850C91}</x:author>
+    <x:author>tc={4D963CBD-121C-D231-C8E6-271C69C09FBC}</x:author>
+    <x:author>tc={7C7A7265-25A8-9CD8-BDFF-10D4C242D312}</x:author>
+    <x:author>tc={42EE7233-7324-8500-FA56-AE3756E9E833}</x:author>
+    <x:author>tc={4B348341-5383-CFE2-3931-37A2FB3A6796}</x:author>
+    <x:author>tc={1A3E9420-C80E-612F-6856-03663BE6B961}</x:author>
+    <x:author>tc={AA18FF0C-0609-3DC9-E3CB-79DB6840A473}</x:author>
+    <x:author>tc={A69C99CA-A057-D8BB-284B-25BDF9CCEC33}</x:author>
+    <x:author>tc={D50807E6-8164-064B-B075-38383003CD54}</x:author>
+    <x:author>tc={BE002E50-346C-2ED1-02B3-A8794F3AB605}</x:author>
+    <x:author>tc={B098C298-69AE-EEB7-D1C2-F7BC866E55B9}</x:author>
+    <x:author>tc={F3A4232B-B2F0-E38E-C4CD-27D2A497F98F}</x:author>
+    <x:author>tc={501C0B3C-E9F4-5518-C3B8-8CD0B037469A}</x:author>
+    <x:author>tc={BC165DAF-BA11-F405-6CBF-79578886B019}</x:author>
+    <x:author>tc={580C07C1-9FAB-9F69-74D0-3B9278C97DDA}</x:author>
+    <x:author>tc={8CD97F42-50C5-7B2D-C42C-71A1179025FC}</x:author>
+    <x:author>tc={6C0F0126-E58B-902E-A8E6-295BFBA74E7B}</x:author>
+    <x:author>tc={D63E76FC-0272-8768-DE65-B5AF8778D0B0}</x:author>
+    <x:author>tc={B09B5ACD-368E-1E68-6052-475ECD03C5BF}</x:author>
+    <x:author>tc={522883C0-51F3-52B3-5700-E265E06929EF}</x:author>
+    <x:author>tc={54087D2A-D6F4-3D3A-D693-CAD90133167F}</x:author>
+    <x:author>tc={5F18F3D5-8D17-8C4C-2D06-CDD09EA4D216}</x:author>
+    <x:author>tc={13740A3D-A1FC-15E2-13DB-4FFB05B462BF}</x:author>
+    <x:author>tc={847A4145-4A0C-DA46-C37F-6096CA91F67D}</x:author>
+    <x:author>tc={D6864198-192F-5FD4-B268-3D436B7AC010}</x:author>
+    <x:author>tc={EBFCBED8-6CFC-ECB3-8C0A-7C4E9AD344F5}</x:author>
+    <x:author>tc={9AD77AC5-C741-5D2F-DBAB-2B74EE25C270}</x:author>
+    <x:author>tc={ED12DAB1-3AFE-11C4-196F-7EE762522CAC}</x:author>
+    <x:author>tc={02AE57B2-7B9E-C2C4-B082-B19B326B3377}</x:author>
+    <x:author>tc={675B19DD-8D0C-3276-6CE4-66346F83A194}</x:author>
+    <x:author>tc={762EADA7-A8B4-889D-2C9B-B45528872477}</x:author>
+    <x:author>tc={EE508AFA-CBC9-9D04-C56A-ADE149A617D2}</x:author>
+    <x:author>tc={7C3918C2-74FE-3B30-0011-76B90C31220D}</x:author>
+    <x:author>tc={B0FB2B0B-0E15-0FE4-7CE3-AD5EA4809E58}</x:author>
+    <x:author>tc={D23A2CFB-B4DA-68EC-FAF4-DF302B3BF193}</x:author>
+    <x:author>tc={7AD41A11-0701-521D-0569-2ED6CDD82249}</x:author>
+    <x:author>tc={BCAC211D-B580-F9C0-E665-E57993EB833C}</x:author>
+    <x:author>tc={F6DDB6CD-A478-A288-D046-D50AE0A2F4F6}</x:author>
+    <x:author>tc={AB6399B6-CEFB-A3AE-273C-3B6F7674686D}</x:author>
+    <x:author>tc={9194F186-D8EE-E399-BA03-2D260FE5AAA6}</x:author>
+    <x:author>tc={6FF53E52-37D4-CC19-3305-7182C053444B}</x:author>
+    <x:author>tc={7C97B6C7-01FC-A9B4-6016-4EF64AFF88BA}</x:author>
+    <x:author>tc={B2345AD4-1F0A-8132-33EE-B7AB8CFFBC6B}</x:author>
+    <x:author>tc={8E4DE5D3-82C1-B07F-9C4A-9689FB42A15A}</x:author>
+    <x:author>tc={3F4FFDE4-26EA-E657-F41C-D27365F25776}</x:author>
+    <x:author>tc={971388A1-D191-476F-30E3-CAF0BDF52814}</x:author>
+    <x:author>tc={87E9E59C-24D1-4B9B-2AAB-86BED77B3F37}</x:author>
+    <x:author>tc={4976AFE0-5E10-3595-15C3-A927BCBB7717}</x:author>
+    <x:author>tc={1D183FA9-A787-A694-E39D-E98D2922412B}</x:author>
+    <x:author>tc={58AF00BE-79AC-4743-650E-E7324330A1BA}</x:author>
+    <x:author>tc={D0EF5D59-18D7-6229-0688-54F1699A15EF}</x:author>
+    <x:author>tc={111F6C62-CBBA-BE4F-FF75-9BBDF71AE371}</x:author>
+    <x:author>tc={EC36B2E5-7EB6-7E1B-F633-1386EF2A8501}</x:author>
+    <x:author>tc={94020BB4-4F25-D013-B6E5-BB7F36D27B62}</x:author>
+    <x:author>tc={FEF6468A-A138-F925-C425-925FC389C735}</x:author>
+    <x:author>tc={256ED2F9-711C-D379-9CF7-0C33127AB323}</x:author>
+    <x:author>tc={7FB9D626-25E8-1DBD-4F9B-E1D2D52EE7B2}</x:author>
+    <x:author>tc={6A9B9A15-4C5F-9E87-6014-3970EF50A532}</x:author>
+    <x:author>tc={BA8AB825-F19D-0BB0-BBFA-A0876A1836D0}</x:author>
+    <x:author>tc={AC1C627A-2A35-C925-6C42-AE55C1F90C62}</x:author>
+    <x:author>tc={2E768F64-774D-1D28-E9F7-5D8185ADD575}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="P5" authorId="0">
@@ -1176,26 +1176,26 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={FF8E5068-65B0-98F7-06E8-04DF16836F9E}</x:author>
-    <x:author>tc={7F2D520E-EEB8-9B5B-A5FA-AC8684943CFC}</x:author>
-    <x:author>tc={99E54B8E-9A24-1D9B-D18D-A99CEE3073A9}</x:author>
-    <x:author>tc={E2408B08-DC23-E00C-ABC8-F8B0509D3010}</x:author>
-    <x:author>tc={04258BAD-A27F-91D5-78C7-2A8BA5B7C41F}</x:author>
-    <x:author>tc={ED6A5C66-C750-3738-9A68-F382389FA981}</x:author>
-    <x:author>tc={F9AF018B-7EE4-8405-B37E-D109D51BFAFF}</x:author>
-    <x:author>tc={51269B21-4255-FF54-E2AF-8E4098E64A3F}</x:author>
-    <x:author>tc={649E091F-A36A-D779-650E-6BBCA18ACD93}</x:author>
-    <x:author>tc={4E7BBEF9-CE9F-16C6-EDE8-5E5C7A9D23BD}</x:author>
-    <x:author>tc={1C2DA460-DAAE-BC6C-6F6F-B3EDEE0A4861}</x:author>
-    <x:author>tc={20437B8E-9FE6-66D8-BB72-40C14527F354}</x:author>
-    <x:author>tc={D749FECF-1A2E-3C4C-80B3-998EA745BA3E}</x:author>
-    <x:author>tc={E25AF189-AEEE-2810-9414-A95677204CDA}</x:author>
-    <x:author>tc={2525E799-85EE-FA6A-EE32-F00FF4E0A7B5}</x:author>
-    <x:author>tc={FFC2E545-B41D-A496-7326-AEAA054FC0A0}</x:author>
-    <x:author>tc={9CA82BEE-D657-5811-0AE1-EA4678C0CB1B}</x:author>
-    <x:author>tc={E71B444B-6DC1-88D6-1590-4082B5507BF4}</x:author>
-    <x:author>tc={AB5B8F92-786E-326A-1D64-8D139AAECF36}</x:author>
-    <x:author>tc={9AA7456A-20BE-E4F2-DA0E-556803D2059F}</x:author>
+    <x:author>tc={4621E60A-8035-BA73-3B5F-4819B7B702C6}</x:author>
+    <x:author>tc={162796F4-247C-2919-A562-B9397445C769}</x:author>
+    <x:author>tc={634CC515-1D2E-7411-C7E2-E57361E9A689}</x:author>
+    <x:author>tc={9672D852-1459-A87F-2C39-1EFA570D28E9}</x:author>
+    <x:author>tc={01A23984-C62A-08AD-B297-21A156BEEF06}</x:author>
+    <x:author>tc={794285E2-342A-BBA9-38EF-581EC582B5CF}</x:author>
+    <x:author>tc={29D9448F-3322-BC7C-5B0D-6D4A7A25E07E}</x:author>
+    <x:author>tc={C4D0E925-1F1E-33F1-FDCB-0C7448590B8C}</x:author>
+    <x:author>tc={ACBAEFE3-E08A-0B52-7201-E8AE738DF32E}</x:author>
+    <x:author>tc={7EF31889-764B-C98E-7E80-1407A7F2629D}</x:author>
+    <x:author>tc={9CDEA24C-B17C-97B7-DF28-9F23B53AE16B}</x:author>
+    <x:author>tc={B67EF076-E3E5-09FE-9C12-AB2A3F433819}</x:author>
+    <x:author>tc={1752A508-1C48-B3E9-BCB4-6547CE095D99}</x:author>
+    <x:author>tc={48796B4E-8B2E-5ED9-1CB8-81CB3ADA83B1}</x:author>
+    <x:author>tc={5FFC1694-755F-6CF5-9143-A034A133E846}</x:author>
+    <x:author>tc={658FF627-7EE0-96EC-57FB-FCCA21C7C319}</x:author>
+    <x:author>tc={365194B6-09B8-AF57-F099-8DB4BAA64557}</x:author>
+    <x:author>tc={DC14C814-516B-3F48-9313-B4D9EC42198E}</x:author>
+    <x:author>tc={D4038BF0-51FC-783E-2E95-3C0645EFE8AE}</x:author>
+    <x:author>tc={A20567BA-B53E-892F-E793-2980A3DF98C3}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="J5" authorId="0">
@@ -2060,7 +2060,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdfcace26e8534658"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8d5b88ebff6b44db"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2071,7 +2071,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{574C0617-F997-4DBE-9033-40879B9F29D3}"/>
+  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{040733F0-4A2E-4743-8B04-6908B11C5686}"/>
 </xltc:personList>
 </file>
 
@@ -2268,493 +2268,493 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="P5" dT="2026-08-15T14:42:13.3" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{27470C1F-3E86-8AB5-8DB2-4196211928B4}">
+  <xltc:threadedComment ref="P5" dT="2026-08-15T14:56:08.194" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{4DBD6BF6-10DC-C9AB-9CD1-709939978DBA}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P6" dT="2026-08-15T14:42:13.304" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{43B9B88D-1E17-4E9D-74E8-79D88964076A}">
+  <xltc:threadedComment ref="P6" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{BBA7CF7E-AC28-261A-8B13-2F207C1218A0}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P7" dT="2026-08-15T14:42:13.304" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{09C81470-7D1E-7221-B2D8-AA6FD4872EA8}">
+  <xltc:threadedComment ref="P7" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{72A601D1-876A-91CE-FFAD-4372EAC3B044}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P8" dT="2026-08-15T14:42:13.304" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B59682A6-6FDF-C9D6-870D-7DFF71907310}">
+  <xltc:threadedComment ref="P8" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{63AEFE69-E87F-CB50-C251-F53F91B5BC7D}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P9" dT="2026-08-15T14:42:13.304" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{A878EB5D-8AA5-15D0-1FA1-02C44890B262}">
+  <xltc:threadedComment ref="P9" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{34BD6919-CEFF-A072-C07C-DF821615DC08}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P10" dT="2026-08-15T14:42:13.304" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{95008EB4-3C0F-98C5-23B3-F71424269E1D}">
+  <xltc:threadedComment ref="P10" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{06E212B9-C215-9B55-79D0-3DCC68FDC5F2}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 119
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P11" dT="2026-08-15T14:42:13.304" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{6B501EBC-3B59-1C5A-6193-2997D84A5FBB}">
+  <xltc:threadedComment ref="P11" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{B3B2D943-46C7-7159-C4D2-5A2561471484}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 160
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P12" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{11DFB307-4A3F-3FDB-1070-4151518E0AEE}">
+  <xltc:threadedComment ref="P12" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{B7F42A5F-C7FD-3C66-478C-F3F30EC65E76}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P13" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{17A3383E-26CF-FF32-8293-53AA83273718}">
+  <xltc:threadedComment ref="P13" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{A4597E1D-F181-CFE5-0579-CB8E395D5F43}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P14" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{0895042D-2EC8-4E8E-011C-BD30B2542F82}">
+  <xltc:threadedComment ref="P14" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{15C385B1-3102-7CB9-2CC5-9E1619C28EFF}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P15" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{DE321951-CF60-2B51-28A6-7C21ECDC92A6}">
+  <xltc:threadedComment ref="P15" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{71943B6E-65A7-8FB9-D610-7EAAF042FB72}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P16" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{C5BB0CCC-B25B-84F6-9375-86524FB267AC}">
+  <xltc:threadedComment ref="P16" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{9C0C8A6E-1868-2889-498E-623A34106926}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P17" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{6412D127-5C7A-8179-ACAD-A754CB27998E}">
+  <xltc:threadedComment ref="P17" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{334D3079-E2A2-64EF-8548-37B4110F83CB}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P18" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{D1907D5E-7F3C-9668-216D-2F5A5682EBA9}">
+  <xltc:threadedComment ref="P18" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{E3828EA9-DCD7-589A-8909-33C5D206AAAB}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P19" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{8468B24A-1F34-D920-1D08-3C2BCB9FBF9C}">
+  <xltc:threadedComment ref="P19" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{7FDAF406-68E0-40BF-FF2E-810ED1C6B3AE}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P20" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{EE993572-ECCA-649C-B5F1-BEB76AC2CEAB}">
+  <xltc:threadedComment ref="P20" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{923B38B5-CB1F-C29F-3341-278DDD42C0D1}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 138
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P21" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{66E75104-6D85-7D8A-3B72-FE434D67D1E9}">
+  <xltc:threadedComment ref="P21" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{1A013CBB-E706-00DF-8726-CF619CEB3A04}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 212
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P22" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B7BFF56B-7F7A-1E49-543F-E2938CD11F48}">
+  <xltc:threadedComment ref="P22" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{EAC196E9-9494-9C63-D76F-35D9C8B67077}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P23" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{F131E133-4295-35BA-8C5E-AED07532BAFE}">
+  <xltc:threadedComment ref="P23" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{10D40289-30D1-453D-67F2-D072A488FDF3}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P24" dT="2026-08-15T14:42:13.305" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{5DD49923-5E31-F51D-F964-B00D6B7355DC}">
+  <xltc:threadedComment ref="P24" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{52EC0200-BA64-4464-226D-17C81EC16731}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P25" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{2ACC0BB8-7789-7C2D-2CFB-67C3CF3FD4F3}">
+  <xltc:threadedComment ref="P25" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{9CC16C61-D3B8-BFC6-1D65-26993EA95662}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P26" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B53DB07E-4BFC-B3DE-D0FF-6B25A369037B}">
+  <xltc:threadedComment ref="P26" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{87792696-2512-1D5F-88FE-607EFE850C91}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P27" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{65F3C94E-0D3D-417F-90E4-49B726CC0C03}">
+  <xltc:threadedComment ref="P27" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{4D963CBD-121C-D231-C8E6-271C69C09FBC}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 272
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P28" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{4B0328F8-ED35-E3C0-9FF9-3FCDCA19A578}">
+  <xltc:threadedComment ref="P28" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{7C7A7265-25A8-9CD8-BDFF-10D4C242D312}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P29" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{AEB20C69-FF92-1059-3CB3-67FB80E83B25}">
+  <xltc:threadedComment ref="P29" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{42EE7233-7324-8500-FA56-AE3756E9E833}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P30" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{CC51BCE6-9571-9338-4887-DFB1DDBE7CFE}">
+  <xltc:threadedComment ref="P30" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{4B348341-5383-CFE2-3931-37A2FB3A6796}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 158
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P31" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{57BF8223-B24F-CB96-C67D-FE3778AB7A98}">
+  <xltc:threadedComment ref="P31" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{1A3E9420-C80E-612F-6856-03663BE6B961}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P32" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{9DB71CD8-5F5A-D445-BA69-7431FF07F420}">
+  <xltc:threadedComment ref="P32" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{AA18FF0C-0609-3DC9-E3CB-79DB6840A473}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P33" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{BC682973-4495-F651-1E6B-5D638F213481}">
+  <xltc:threadedComment ref="P33" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{A69C99CA-A057-D8BB-284B-25BDF9CCEC33}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 72
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P34" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B29A439B-5573-E40C-A3F2-47DC01C114CA}">
+  <xltc:threadedComment ref="P34" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{D50807E6-8164-064B-B075-38383003CD54}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P35" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{27FB8DDD-912C-1E7A-7752-AC2705E606D1}">
+  <xltc:threadedComment ref="P35" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{BE002E50-346C-2ED1-02B3-A8794F3AB605}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P36" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{D64CC503-5D80-D76D-2203-9D94BA4D1DD6}">
+  <xltc:threadedComment ref="P36" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{B098C298-69AE-EEB7-D1C2-F7BC866E55B9}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 24
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P37" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{2D48482E-942F-70F1-9A1F-3042DF18F561}">
+  <xltc:threadedComment ref="P37" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{F3A4232B-B2F0-E38E-C4CD-27D2A497F98F}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P38" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{C6B6AE69-95AE-3428-95C7-F692D3F5D5E7}">
+  <xltc:threadedComment ref="P38" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{501C0B3C-E9F4-5518-C3B8-8CD0B037469A}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P39" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{8B99EECA-E1B0-BB8C-FDE3-12304B6E8837}">
+  <xltc:threadedComment ref="P39" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{BC165DAF-BA11-F405-6CBF-79578886B019}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 19
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P40" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{F0E086AD-557A-9367-4ADE-1174F432B4B0}">
+  <xltc:threadedComment ref="P40" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{580C07C1-9FAB-9F69-74D0-3B9278C97DDA}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P41" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{67850FFA-4D8D-12EF-F53E-9156F80A11A3}">
+  <xltc:threadedComment ref="P41" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{8CD97F42-50C5-7B2D-C42C-71A1179025FC}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P42" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{042B242A-E4E4-1CEA-BC47-62C535AD710E}">
+  <xltc:threadedComment ref="P42" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{6C0F0126-E58B-902E-A8E6-295BFBA74E7B}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P43" dT="2026-08-15T14:42:13.306" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{C18243BE-FBA2-E2DB-596C-F13761AAE732}">
+  <xltc:threadedComment ref="P43" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{D63E76FC-0272-8768-DE65-B5AF8778D0B0}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P44" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{48E8FE26-4F2B-76EF-9633-0159BA519100}">
+  <xltc:threadedComment ref="P44" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{B09B5ACD-368E-1E68-6052-475ECD03C5BF}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P45" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{587E4A9F-063E-97FE-91A7-D7AA3D4C7D0C}">
+  <xltc:threadedComment ref="P45" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{522883C0-51F3-52B3-5700-E265E06929EF}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P46" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{DD15F858-A966-B3D7-AE9F-F7E782BCF67F}">
+  <xltc:threadedComment ref="P46" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{54087D2A-D6F4-3D3A-D693-CAD90133167F}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P47" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{698148F6-A858-A2E4-43B4-090624731F08}">
+  <xltc:threadedComment ref="P47" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{5F18F3D5-8D17-8C4C-2D06-CDD09EA4D216}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P48" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{3C42F2E9-5177-361F-C391-72A553BBDCFD}">
+  <xltc:threadedComment ref="P48" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{13740A3D-A1FC-15E2-13DB-4FFB05B462BF}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P49" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{615871BF-6F97-376B-4041-7D4A2BE913E4}">
+  <xltc:threadedComment ref="P49" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{847A4145-4A0C-DA46-C37F-6096CA91F67D}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 118
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P50" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{29076D46-81AC-3DA1-E553-FB2CF9C5DB53}">
+  <xltc:threadedComment ref="P50" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{D6864198-192F-5FD4-B268-3D436B7AC010}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P51" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{640CFE87-0AB4-B553-BD22-210F6ED666FE}">
+  <xltc:threadedComment ref="P51" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{EBFCBED8-6CFC-ECB3-8C0A-7C4E9AD344F5}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P52" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{FF2EA90D-4615-E514-5382-8D7E2A36F5C8}">
+  <xltc:threadedComment ref="P52" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{9AD77AC5-C741-5D2F-DBAB-2B74EE25C270}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P53" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{26168C5B-79CB-D690-B1F7-4645EDB98430}">
+  <xltc:threadedComment ref="P53" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{ED12DAB1-3AFE-11C4-196F-7EE762522CAC}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-STF</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P54" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B7520A70-7331-EEF2-D384-8DA397742486}">
+  <xltc:threadedComment ref="P54" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{02AE57B2-7B9E-C2C4-B082-B19B326B3377}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P55" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{4A348036-AB29-AC77-7331-B011B8134AE2}">
+  <xltc:threadedComment ref="P55" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{675B19DD-8D0C-3276-6CE4-66346F83A194}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P56" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{4042F39D-46F4-EEDE-CCC8-9BBA2F58914E}">
+  <xltc:threadedComment ref="P56" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{762EADA7-A8B4-889D-2C9B-B45528872477}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 18
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P57" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{0AB46C1E-AB8F-81EA-04D0-66352A0116C5}">
+  <xltc:threadedComment ref="P57" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{EE508AFA-CBC9-9D04-C56A-ADE149A617D2}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P58" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{D210A386-4279-382A-0842-A075EAF7050A}">
+  <xltc:threadedComment ref="P58" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{7C3918C2-74FE-3B30-0011-76B90C31220D}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P59" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{D8EB7CCD-07F5-1D6D-9311-D9670A2252D0}">
+  <xltc:threadedComment ref="P59" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{B0FB2B0B-0E15-0FE4-7CE3-AD5EA4809E58}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P60" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{208C58C9-AD84-A1B7-1B1D-5E8F708B725B}">
+  <xltc:threadedComment ref="P60" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{D23A2CFB-B4DA-68EC-FAF4-DF302B3BF193}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P61" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{CDB5BC5C-C7CE-B2C9-6BC5-729C2FE78534}">
+  <xltc:threadedComment ref="P61" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{7AD41A11-0701-521D-0569-2ED6CDD82249}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P62" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B82F8D3D-4FA3-34A2-007F-93F66166FCE9}">
+  <xltc:threadedComment ref="P62" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{BCAC211D-B580-F9C0-E665-E57993EB833C}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P63" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{355858EA-94D6-A5F1-5963-0D4B997DA6C7}">
+  <xltc:threadedComment ref="P63" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{F6DDB6CD-A478-A288-D046-D50AE0A2F4F6}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P64" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{0A6E155D-B6F7-4B90-E2F6-8434C38B6F32}">
+  <xltc:threadedComment ref="P64" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{AB6399B6-CEFB-A3AE-273C-3B6F7674686D}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P65" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{8D39E17F-76E1-A06B-2B06-E442780A77FA}">
+  <xltc:threadedComment ref="P65" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{9194F186-D8EE-E399-BA03-2D260FE5AAA6}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 311
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P66" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{CB4D955D-631A-8D96-DA59-2A911C6CB46F}">
+  <xltc:threadedComment ref="P66" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{6FF53E52-37D4-CC19-3305-7182C053444B}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P67" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{1945AC02-CDAF-71E1-C7DC-047DA0EF251B}">
+  <xltc:threadedComment ref="P67" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{7C97B6C7-01FC-A9B4-6016-4EF64AFF88BA}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P68" dT="2026-08-15T14:42:13.307" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{DFA5B975-6AB1-8691-97D2-36BCCCC8EDC8}">
+  <xltc:threadedComment ref="P68" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{B2345AD4-1F0A-8132-33EE-B7AB8CFFBC6B}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 141
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P69" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{56DC07E0-8BA3-3FE7-E501-566B57DA91F2}">
+  <xltc:threadedComment ref="P69" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{8E4DE5D3-82C1-B07F-9C4A-9689FB42A15A}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P70" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{6B070A3A-232C-704C-5690-A92B4F27B006}">
+  <xltc:threadedComment ref="P70" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{3F4FFDE4-26EA-E657-F41C-D27365F25776}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P71" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{915CDFF3-212A-29C2-9707-BF1B51CEEF46}">
+  <xltc:threadedComment ref="P71" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{971388A1-D191-476F-30E3-CAF0BDF52814}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 33
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P72" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B63BE17A-0F55-CC42-213E-DA710F640E8E}">
+  <xltc:threadedComment ref="P72" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{87E9E59C-24D1-4B9B-2AAB-86BED77B3F37}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P73" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{47566A22-B4FC-24A0-4A33-5499E94221F3}">
+  <xltc:threadedComment ref="P73" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{4976AFE0-5E10-3595-15C3-A927BCBB7717}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P74" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{94F3B43E-34AA-D7D0-4C98-A0704157CD3B}">
+  <xltc:threadedComment ref="P74" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{1D183FA9-A787-A694-E39D-E98D2922412B}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 21
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P75" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{3746D14E-7E36-4093-679A-03CB636182CB}">
+  <xltc:threadedComment ref="P75" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{58AF00BE-79AC-4743-650E-E7324330A1BA}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P76" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{07D3A048-4A5B-9511-5E96-DA82AC82981A}">
+  <xltc:threadedComment ref="P76" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{D0EF5D59-18D7-6229-0688-54F1699A15EF}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P77" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{955769CA-F12C-6DE2-267A-2F9FA6FA447D}">
+  <xltc:threadedComment ref="P77" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{111F6C62-CBBA-BE4F-FF75-9BBDF71AE371}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 19
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P78" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{8B151F4C-CDFE-87DA-66A2-3019B71A46CA}">
+  <xltc:threadedComment ref="P78" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{EC36B2E5-7EB6-7E1B-F633-1386EF2A8501}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 43
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P79" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{E7294CE3-02B5-FE19-12E8-574930490330}">
+  <xltc:threadedComment ref="P79" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{94020BB4-4F25-D013-B6E5-BB7F36D27B62}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 44
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P80" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{351C48BB-DDEC-1F7B-E62E-199377745A55}">
+  <xltc:threadedComment ref="P80" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{FEF6468A-A138-F925-C425-925FC389C735}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 40
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P81" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{7B935A8A-05BF-F039-71E6-6CC5A47A6FF7}">
+  <xltc:threadedComment ref="P81" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{256ED2F9-711C-D379-9CF7-0C33127AB323}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P82" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{C98FDE63-8E41-FCB8-46F4-EB23F118E951}">
+  <xltc:threadedComment ref="P82" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{7FB9D626-25E8-1DBD-4F9B-E1D2D52EE7B2}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P83" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{B386906A-8267-D740-4904-2411DA5BE461}">
+  <xltc:threadedComment ref="P83" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{6A9B9A15-4C5F-9E87-6014-3970EF50A532}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 16
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P84" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{86940D5A-A9E3-91D3-D186-E09042CF5A01}">
+  <xltc:threadedComment ref="P84" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{BA8AB825-F19D-0BB0-BBFA-A0876A1836D0}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P85" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{F97DBEE1-5872-FF44-12BC-64BD321E1FD5}">
+  <xltc:threadedComment ref="P85" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{AC1C627A-2A35-C925-6C42-AE55C1F90C62}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P86" dT="2026-08-15T14:42:13.308" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{D60FA9C1-54B0-8F3B-C9BB-6E08D839AC43}">
+  <xltc:threadedComment ref="P86" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{2E768F64-774D-1D28-E9F7-5D8185ADD575}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 21
 Available: 2026-02-25
@@ -2765,64 +2765,64 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="J5" dT="2026-08-15T14:42:13.65" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{FF8E5068-65B0-98F7-06E8-04DF16836F9E}">
+  <xltc:threadedComment ref="J5" dT="2026-08-15T14:56:08.514" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{4621E60A-8035-BA73-3B5F-4819B7B702C6}">
     <xltc:text>Official source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J6" dT="2026-08-15T14:42:13.652" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{7F2D520E-EEB8-9B5B-A5FA-AC8684943CFC}">
+  <xltc:threadedComment ref="J6" dT="2026-08-15T14:56:08.517" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{162796F4-247C-2919-A562-B9397445C769}">
     <xltc:text>Official source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J7" dT="2026-08-15T14:42:13.654" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{99E54B8E-9A24-1D9B-D18D-A99CEE3073A9}">
+  <xltc:threadedComment ref="J7" dT="2026-08-15T14:56:08.52" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{634CC515-1D2E-7411-C7E2-E57361E9A689}">
     <xltc:text>Official source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J8" dT="2026-08-15T14:42:13.656" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{E2408B08-DC23-E00C-ABC8-F8B0509D3010}">
+  <xltc:threadedComment ref="J8" dT="2026-08-15T14:56:08.523" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{9672D852-1459-A87F-2C39-1EFA570D28E9}">
     <xltc:text>Official source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J9" dT="2026-08-15T14:42:13.658" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{04258BAD-A27F-91D5-78C7-2A8BA5B7C41F}">
+  <xltc:threadedComment ref="J9" dT="2026-08-15T14:56:08.525" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{01A23984-C62A-08AD-B297-21A156BEEF06}">
     <xltc:text>Official source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J10" dT="2026-08-15T14:42:13.661" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{ED6A5C66-C750-3738-9A68-F382389FA981}">
+  <xltc:threadedComment ref="J10" dT="2026-08-15T14:56:08.527" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{794285E2-342A-BBA9-38EF-581EC582B5CF}">
     <xltc:text>Official source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J11" dT="2026-08-15T14:42:13.663" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{F9AF018B-7EE4-8405-B37E-D109D51BFAFF}">
+  <xltc:threadedComment ref="J11" dT="2026-08-15T14:56:08.529" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{29D9448F-3322-BC7C-5B0D-6D4A7A25E07E}">
     <xltc:text>Official source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J12" dT="2026-08-15T14:42:13.664" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{51269B21-4255-FF54-E2AF-8E4098E64A3F}">
+  <xltc:threadedComment ref="J12" dT="2026-08-15T14:56:08.531" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{C4D0E925-1F1E-33F1-FDCB-0C7448590B8C}">
     <xltc:text>Official source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J13" dT="2026-08-15T14:42:13.666" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{649E091F-A36A-D779-650E-6BBCA18ACD93}">
+  <xltc:threadedComment ref="J13" dT="2026-08-15T14:56:08.534" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{ACBAEFE3-E08A-0B52-7201-E8AE738DF32E}">
     <xltc:text>Official source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J14" dT="2026-08-15T14:42:13.667" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{4E7BBEF9-CE9F-16C6-EDE8-5E5C7A9D23BD}">
+  <xltc:threadedComment ref="J14" dT="2026-08-15T14:56:08.536" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{7EF31889-764B-C98E-7E80-1407A7F2629D}">
     <xltc:text>Official source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J15" dT="2026-08-15T14:42:13.669" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{1C2DA460-DAAE-BC6C-6F6F-B3EDEE0A4861}">
+  <xltc:threadedComment ref="J15" dT="2026-08-15T14:56:08.538" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{9CDEA24C-B17C-97B7-DF28-9F23B53AE16B}">
     <xltc:text>Official source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J16" dT="2026-08-15T14:42:13.673" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{20437B8E-9FE6-66D8-BB72-40C14527F354}">
+  <xltc:threadedComment ref="J16" dT="2026-08-15T14:56:08.54" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{B67EF076-E3E5-09FE-9C12-AB2A3F433819}">
     <xltc:text>Official source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J17" dT="2026-08-15T14:42:13.674" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{D749FECF-1A2E-3C4C-80B3-998EA745BA3E}">
+  <xltc:threadedComment ref="J17" dT="2026-08-15T14:56:08.542" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{1752A508-1C48-B3E9-BCB4-6547CE095D99}">
     <xltc:text>Official source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J18" dT="2026-08-15T14:42:13.677" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{E25AF189-AEEE-2810-9414-A95677204CDA}">
+  <xltc:threadedComment ref="J18" dT="2026-08-15T14:56:08.546" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{48796B4E-8B2E-5ED9-1CB8-81CB3ADA83B1}">
     <xltc:text>Official source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J19" dT="2026-08-15T14:42:13.679" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{2525E799-85EE-FA6A-EE32-F00FF4E0A7B5}">
+  <xltc:threadedComment ref="J19" dT="2026-08-15T14:56:08.548" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{5FFC1694-755F-6CF5-9143-A034A133E846}">
     <xltc:text>Official source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J20" dT="2026-08-15T14:42:13.68" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{FFC2E545-B41D-A496-7326-AEAA054FC0A0}">
+  <xltc:threadedComment ref="J20" dT="2026-08-15T14:56:08.55" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{658FF627-7EE0-96EC-57FB-FCCA21C7C319}">
     <xltc:text>Official source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J21" dT="2026-08-15T14:42:13.682" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{9CA82BEE-D657-5811-0AE1-EA4678C0CB1B}">
+  <xltc:threadedComment ref="J21" dT="2026-08-15T14:56:08.552" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{365194B6-09B8-AF57-F099-8DB4BAA64557}">
     <xltc:text>Official source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J22" dT="2026-08-15T14:42:13.684" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{E71B444B-6DC1-88D6-1590-4082B5507BF4}">
+  <xltc:threadedComment ref="J22" dT="2026-08-15T14:56:08.554" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{DC14C814-516B-3F48-9313-B4D9EC42198E}">
     <xltc:text>Official source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J23" dT="2026-08-15T14:42:13.685" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{AB5B8F92-786E-326A-1D64-8D139AAECF36}">
+  <xltc:threadedComment ref="J23" dT="2026-08-15T14:56:08.556" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{D4038BF0-51FC-783E-2E95-3C0645EFE8AE}">
     <xltc:text>Official source: https://www.aspenpharma.com/download/annual-financial-statements-2/</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J24" dT="2026-08-15T14:42:13.687" personId="{574C0617-F997-4DBE-9033-40879B9F29D3}" id="{9AA7456A-20BE-E4F2-DA0E-556803D2059F}">
+  <xltc:threadedComment ref="J24" dT="2026-08-15T14:56:08.558" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{A20567BA-B53E-892F-E793-2980A3DF98C3}">
     <xltc:text>Official source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -3877,7 +3877,7 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5057e7e7dc734e7a"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70bd2a2cedd04f03"/>
 </x:worksheet>
 </file>
 
@@ -8611,7 +8611,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80794ba59efd42e3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e1b7f1952284071"/>
 </x:worksheet>
 </file>
 
@@ -9671,7 +9671,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re696f294952b47c0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf532b07fe2d41af"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Restamp final V3.2 portable release
</commit_message>
<xml_diff>
--- a/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
+++ b/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Refa4995be3d04ee7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R8af1eebdbf8d4e62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="R7f50b9fc52bc4285"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="R8e7a6f998fc742c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R6d10c4373f9a45d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="Ra17269f826874465"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Rd5f4997859c94c78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="Rf21410be4c814f8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="Rc712395c96ae4d64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="Rb1d41ec840144a46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R04a3fd164f384795"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R446d898fd8cb466b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="Rfbee45e282674bc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Rab888e9a2693495e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R77b2312b46be4a45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="Rbd702c155274446d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Rb087a52c07eb45e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="R49c2453e8b4c4cd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R93e8c8668f174eb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R6e68213158384451"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,88 +19,88 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={4DBD6BF6-10DC-C9AB-9CD1-709939978DBA}</x:author>
-    <x:author>tc={BBA7CF7E-AC28-261A-8B13-2F207C1218A0}</x:author>
-    <x:author>tc={72A601D1-876A-91CE-FFAD-4372EAC3B044}</x:author>
-    <x:author>tc={63AEFE69-E87F-CB50-C251-F53F91B5BC7D}</x:author>
-    <x:author>tc={34BD6919-CEFF-A072-C07C-DF821615DC08}</x:author>
-    <x:author>tc={06E212B9-C215-9B55-79D0-3DCC68FDC5F2}</x:author>
-    <x:author>tc={B3B2D943-46C7-7159-C4D2-5A2561471484}</x:author>
-    <x:author>tc={B7F42A5F-C7FD-3C66-478C-F3F30EC65E76}</x:author>
-    <x:author>tc={A4597E1D-F181-CFE5-0579-CB8E395D5F43}</x:author>
-    <x:author>tc={15C385B1-3102-7CB9-2CC5-9E1619C28EFF}</x:author>
-    <x:author>tc={71943B6E-65A7-8FB9-D610-7EAAF042FB72}</x:author>
-    <x:author>tc={9C0C8A6E-1868-2889-498E-623A34106926}</x:author>
-    <x:author>tc={334D3079-E2A2-64EF-8548-37B4110F83CB}</x:author>
-    <x:author>tc={E3828EA9-DCD7-589A-8909-33C5D206AAAB}</x:author>
-    <x:author>tc={7FDAF406-68E0-40BF-FF2E-810ED1C6B3AE}</x:author>
-    <x:author>tc={923B38B5-CB1F-C29F-3341-278DDD42C0D1}</x:author>
-    <x:author>tc={1A013CBB-E706-00DF-8726-CF619CEB3A04}</x:author>
-    <x:author>tc={EAC196E9-9494-9C63-D76F-35D9C8B67077}</x:author>
-    <x:author>tc={10D40289-30D1-453D-67F2-D072A488FDF3}</x:author>
-    <x:author>tc={52EC0200-BA64-4464-226D-17C81EC16731}</x:author>
-    <x:author>tc={9CC16C61-D3B8-BFC6-1D65-26993EA95662}</x:author>
-    <x:author>tc={87792696-2512-1D5F-88FE-607EFE850C91}</x:author>
-    <x:author>tc={4D963CBD-121C-D231-C8E6-271C69C09FBC}</x:author>
-    <x:author>tc={7C7A7265-25A8-9CD8-BDFF-10D4C242D312}</x:author>
-    <x:author>tc={42EE7233-7324-8500-FA56-AE3756E9E833}</x:author>
-    <x:author>tc={4B348341-5383-CFE2-3931-37A2FB3A6796}</x:author>
-    <x:author>tc={1A3E9420-C80E-612F-6856-03663BE6B961}</x:author>
-    <x:author>tc={AA18FF0C-0609-3DC9-E3CB-79DB6840A473}</x:author>
-    <x:author>tc={A69C99CA-A057-D8BB-284B-25BDF9CCEC33}</x:author>
-    <x:author>tc={D50807E6-8164-064B-B075-38383003CD54}</x:author>
-    <x:author>tc={BE002E50-346C-2ED1-02B3-A8794F3AB605}</x:author>
-    <x:author>tc={B098C298-69AE-EEB7-D1C2-F7BC866E55B9}</x:author>
-    <x:author>tc={F3A4232B-B2F0-E38E-C4CD-27D2A497F98F}</x:author>
-    <x:author>tc={501C0B3C-E9F4-5518-C3B8-8CD0B037469A}</x:author>
-    <x:author>tc={BC165DAF-BA11-F405-6CBF-79578886B019}</x:author>
-    <x:author>tc={580C07C1-9FAB-9F69-74D0-3B9278C97DDA}</x:author>
-    <x:author>tc={8CD97F42-50C5-7B2D-C42C-71A1179025FC}</x:author>
-    <x:author>tc={6C0F0126-E58B-902E-A8E6-295BFBA74E7B}</x:author>
-    <x:author>tc={D63E76FC-0272-8768-DE65-B5AF8778D0B0}</x:author>
-    <x:author>tc={B09B5ACD-368E-1E68-6052-475ECD03C5BF}</x:author>
-    <x:author>tc={522883C0-51F3-52B3-5700-E265E06929EF}</x:author>
-    <x:author>tc={54087D2A-D6F4-3D3A-D693-CAD90133167F}</x:author>
-    <x:author>tc={5F18F3D5-8D17-8C4C-2D06-CDD09EA4D216}</x:author>
-    <x:author>tc={13740A3D-A1FC-15E2-13DB-4FFB05B462BF}</x:author>
-    <x:author>tc={847A4145-4A0C-DA46-C37F-6096CA91F67D}</x:author>
-    <x:author>tc={D6864198-192F-5FD4-B268-3D436B7AC010}</x:author>
-    <x:author>tc={EBFCBED8-6CFC-ECB3-8C0A-7C4E9AD344F5}</x:author>
-    <x:author>tc={9AD77AC5-C741-5D2F-DBAB-2B74EE25C270}</x:author>
-    <x:author>tc={ED12DAB1-3AFE-11C4-196F-7EE762522CAC}</x:author>
-    <x:author>tc={02AE57B2-7B9E-C2C4-B082-B19B326B3377}</x:author>
-    <x:author>tc={675B19DD-8D0C-3276-6CE4-66346F83A194}</x:author>
-    <x:author>tc={762EADA7-A8B4-889D-2C9B-B45528872477}</x:author>
-    <x:author>tc={EE508AFA-CBC9-9D04-C56A-ADE149A617D2}</x:author>
-    <x:author>tc={7C3918C2-74FE-3B30-0011-76B90C31220D}</x:author>
-    <x:author>tc={B0FB2B0B-0E15-0FE4-7CE3-AD5EA4809E58}</x:author>
-    <x:author>tc={D23A2CFB-B4DA-68EC-FAF4-DF302B3BF193}</x:author>
-    <x:author>tc={7AD41A11-0701-521D-0569-2ED6CDD82249}</x:author>
-    <x:author>tc={BCAC211D-B580-F9C0-E665-E57993EB833C}</x:author>
-    <x:author>tc={F6DDB6CD-A478-A288-D046-D50AE0A2F4F6}</x:author>
-    <x:author>tc={AB6399B6-CEFB-A3AE-273C-3B6F7674686D}</x:author>
-    <x:author>tc={9194F186-D8EE-E399-BA03-2D260FE5AAA6}</x:author>
-    <x:author>tc={6FF53E52-37D4-CC19-3305-7182C053444B}</x:author>
-    <x:author>tc={7C97B6C7-01FC-A9B4-6016-4EF64AFF88BA}</x:author>
-    <x:author>tc={B2345AD4-1F0A-8132-33EE-B7AB8CFFBC6B}</x:author>
-    <x:author>tc={8E4DE5D3-82C1-B07F-9C4A-9689FB42A15A}</x:author>
-    <x:author>tc={3F4FFDE4-26EA-E657-F41C-D27365F25776}</x:author>
-    <x:author>tc={971388A1-D191-476F-30E3-CAF0BDF52814}</x:author>
-    <x:author>tc={87E9E59C-24D1-4B9B-2AAB-86BED77B3F37}</x:author>
-    <x:author>tc={4976AFE0-5E10-3595-15C3-A927BCBB7717}</x:author>
-    <x:author>tc={1D183FA9-A787-A694-E39D-E98D2922412B}</x:author>
-    <x:author>tc={58AF00BE-79AC-4743-650E-E7324330A1BA}</x:author>
-    <x:author>tc={D0EF5D59-18D7-6229-0688-54F1699A15EF}</x:author>
-    <x:author>tc={111F6C62-CBBA-BE4F-FF75-9BBDF71AE371}</x:author>
-    <x:author>tc={EC36B2E5-7EB6-7E1B-F633-1386EF2A8501}</x:author>
-    <x:author>tc={94020BB4-4F25-D013-B6E5-BB7F36D27B62}</x:author>
-    <x:author>tc={FEF6468A-A138-F925-C425-925FC389C735}</x:author>
-    <x:author>tc={256ED2F9-711C-D379-9CF7-0C33127AB323}</x:author>
-    <x:author>tc={7FB9D626-25E8-1DBD-4F9B-E1D2D52EE7B2}</x:author>
-    <x:author>tc={6A9B9A15-4C5F-9E87-6014-3970EF50A532}</x:author>
-    <x:author>tc={BA8AB825-F19D-0BB0-BBFA-A0876A1836D0}</x:author>
-    <x:author>tc={AC1C627A-2A35-C925-6C42-AE55C1F90C62}</x:author>
-    <x:author>tc={2E768F64-774D-1D28-E9F7-5D8185ADD575}</x:author>
+    <x:author>tc={2ED26A2B-7837-083D-9F91-2E1C1C9C804A}</x:author>
+    <x:author>tc={043405D0-022D-CE03-81D3-AF489ABD68A9}</x:author>
+    <x:author>tc={D34DFE13-CAE1-EB32-19DC-D3D61E45A130}</x:author>
+    <x:author>tc={F0CC0459-AC75-5733-37FD-D729BDC516EE}</x:author>
+    <x:author>tc={BBAB887A-8A65-8B92-424D-300C0145401F}</x:author>
+    <x:author>tc={1EE3C80A-BD61-F09D-5B89-C055910B21A8}</x:author>
+    <x:author>tc={071773AC-BAFA-9A1C-7CEC-858AE817169C}</x:author>
+    <x:author>tc={A64051D4-C4DD-3EAD-CAD5-DDCB5ED2D742}</x:author>
+    <x:author>tc={342DD7E3-64C9-FC39-8DEA-BB86036F486C}</x:author>
+    <x:author>tc={A5720320-9FF6-0861-0144-55CD868F0919}</x:author>
+    <x:author>tc={13F43D72-1AA3-0364-70A4-6A9B8423C7FE}</x:author>
+    <x:author>tc={0E8F289F-DFB0-8655-E6D1-D7FCF99AAB06}</x:author>
+    <x:author>tc={4B99CAD2-8EC9-BC88-3AFD-F1394BD6783F}</x:author>
+    <x:author>tc={010EBAEC-2F9D-B152-1556-960BE1725C4B}</x:author>
+    <x:author>tc={7333D144-0844-64FD-0AAB-4E413D2935D0}</x:author>
+    <x:author>tc={5518B81C-B0BC-B171-5762-AAA1625B3F0D}</x:author>
+    <x:author>tc={FE8B682C-7BBF-FB26-C52A-0567E7240CBA}</x:author>
+    <x:author>tc={3A15E6D2-B051-8834-4C93-A28DA909DDC7}</x:author>
+    <x:author>tc={2EA4B4F3-F741-14DC-D1D2-6FA54989E80C}</x:author>
+    <x:author>tc={F4DF57BE-F27A-2E50-A72C-5EF0B356A55E}</x:author>
+    <x:author>tc={31A0369D-1694-51B8-5DB4-35DB7F6AF63D}</x:author>
+    <x:author>tc={7B5F41ED-10A3-8B79-15C5-6A825FFFDDE4}</x:author>
+    <x:author>tc={46AE8608-356C-86B4-EC18-C1C6FE5CAAAD}</x:author>
+    <x:author>tc={7551C88D-E9F7-2348-0E76-9F80E57D2F60}</x:author>
+    <x:author>tc={ABF1018A-ABB9-7204-C90E-1105B94E814A}</x:author>
+    <x:author>tc={512B7354-5F2C-1AA7-CC3C-00CD42BBE0FC}</x:author>
+    <x:author>tc={AFFA6109-ADE2-4CE1-7C27-BAA3EFB317C9}</x:author>
+    <x:author>tc={D5144167-7AD8-57DF-B826-07D54D010D9C}</x:author>
+    <x:author>tc={B83DFD0F-794A-6C5E-1D58-744B039949BC}</x:author>
+    <x:author>tc={7B9E1B4B-9DCB-BECD-99F5-F055FB863E9C}</x:author>
+    <x:author>tc={8B2DC34E-17AF-DC22-540E-3A7428974B96}</x:author>
+    <x:author>tc={094E8309-B86F-1491-11B7-E843D5E63DAC}</x:author>
+    <x:author>tc={4513E577-194B-E888-43E5-01675E143F65}</x:author>
+    <x:author>tc={D063F1D2-2F95-2667-C7FF-CB2952CE7907}</x:author>
+    <x:author>tc={C9AF5DAB-FC5E-E759-C111-2F94BE966A52}</x:author>
+    <x:author>tc={5C3D6D9E-0399-3A1F-5FF8-7673B95728DC}</x:author>
+    <x:author>tc={40BAA6D9-7593-464B-9634-92C58D16225A}</x:author>
+    <x:author>tc={DA3A9B1C-4CB2-882E-946C-A1860B6BC64A}</x:author>
+    <x:author>tc={05CE38D1-9BF6-E417-141B-4027834AA96E}</x:author>
+    <x:author>tc={B6C35BC3-6F5F-B362-B79B-E7478D767EAB}</x:author>
+    <x:author>tc={A2136AA3-D60A-9CA4-782A-688014FA68CC}</x:author>
+    <x:author>tc={F9107F21-217D-6E1C-0F95-26D39A645301}</x:author>
+    <x:author>tc={6BDCC13B-4293-D80F-CDD9-0D914AF1E069}</x:author>
+    <x:author>tc={6FCD0DD5-A300-B061-80FD-E6DA09A1A00C}</x:author>
+    <x:author>tc={D33E4AF9-5B00-4D1E-2774-D1A03F8DAA00}</x:author>
+    <x:author>tc={B93F8331-7F4C-8F1E-6D00-D4F3F4DD941B}</x:author>
+    <x:author>tc={01017BE8-DAC5-0C0D-B269-33BF689C7906}</x:author>
+    <x:author>tc={0F0598D8-65DE-16CC-F316-558AAB8C206A}</x:author>
+    <x:author>tc={FD22F09B-1275-26C7-C5BC-CEBC26B724BD}</x:author>
+    <x:author>tc={50296461-F84A-5759-D5C7-3C73B6727E11}</x:author>
+    <x:author>tc={25FD297A-C8A3-7982-2A2A-6109869C428D}</x:author>
+    <x:author>tc={A01BC395-D63D-37E2-3702-F398D5D7D853}</x:author>
+    <x:author>tc={3CCE64FE-3C38-CB25-DAB1-1288A0B1E1D3}</x:author>
+    <x:author>tc={0381E4D2-1AB7-DC1B-5477-B3CE9858338D}</x:author>
+    <x:author>tc={0DB1B439-2233-2FF4-7F69-4CFB903C8BCE}</x:author>
+    <x:author>tc={702F1FDC-2B20-239C-C387-1F9994029E58}</x:author>
+    <x:author>tc={86BF3B4D-4C8B-94C5-2DF8-0E144D24162D}</x:author>
+    <x:author>tc={55FEB31D-AA64-C68B-21EB-2AD4013CA9D9}</x:author>
+    <x:author>tc={2120B059-1D9A-FB52-CB20-859A8A7B4431}</x:author>
+    <x:author>tc={DDAE0E6F-C9F0-E461-07EA-91968BE2E6D2}</x:author>
+    <x:author>tc={83232D14-7BAC-B848-7871-277E89FA684E}</x:author>
+    <x:author>tc={279DD734-DD6F-13E2-E0FD-18F5BF78E98D}</x:author>
+    <x:author>tc={0C0BEC61-5240-DC56-B9D0-4183924DDDA7}</x:author>
+    <x:author>tc={4B78E0A5-E835-82BC-95E0-9D6660CB0642}</x:author>
+    <x:author>tc={2AA3892A-F3E0-DCE4-4BA3-77C2298E4712}</x:author>
+    <x:author>tc={0BF67983-6F8F-9A8B-A733-988A5AE771CE}</x:author>
+    <x:author>tc={853E2097-1ED4-88BD-0FEF-BB1C45A97F6A}</x:author>
+    <x:author>tc={5437FE01-1237-5D55-7238-D3B41AD600A7}</x:author>
+    <x:author>tc={26525073-6162-76FE-6D24-B53B287B9745}</x:author>
+    <x:author>tc={BAC99CA3-3171-9911-60EA-9ADBAD9DAA89}</x:author>
+    <x:author>tc={4E489A6C-1C1A-971C-72AB-ACB53D354D17}</x:author>
+    <x:author>tc={280D1E73-5C17-150A-507B-D8086C4BA2AD}</x:author>
+    <x:author>tc={33816FEE-5341-8E14-F197-F3763F51C77B}</x:author>
+    <x:author>tc={0277E1E1-ACCD-F4A6-B8D9-B0F98C590404}</x:author>
+    <x:author>tc={F919CE15-F9D0-4C7F-A7F6-D4B6CEEDC7C3}</x:author>
+    <x:author>tc={70300967-130C-E9FC-5833-2A5E4C05B7E1}</x:author>
+    <x:author>tc={6A5C72F7-2A4F-E907-50AB-917C148A344A}</x:author>
+    <x:author>tc={0459789A-01BE-4F0D-BABB-8071C46032C0}</x:author>
+    <x:author>tc={AF3F7297-575B-2C4C-A9A0-434E38FE21C6}</x:author>
+    <x:author>tc={2DFC25D3-339D-7566-5DC3-205EE0DC70AC}</x:author>
+    <x:author>tc={326FB552-EB16-8CC1-A7BC-665356E8462C}</x:author>
+    <x:author>tc={5B218977-D8FC-2E26-E971-16C48C7A4A64}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="P5" authorId="0">
@@ -1176,26 +1176,26 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={4621E60A-8035-BA73-3B5F-4819B7B702C6}</x:author>
-    <x:author>tc={162796F4-247C-2919-A562-B9397445C769}</x:author>
-    <x:author>tc={634CC515-1D2E-7411-C7E2-E57361E9A689}</x:author>
-    <x:author>tc={9672D852-1459-A87F-2C39-1EFA570D28E9}</x:author>
-    <x:author>tc={01A23984-C62A-08AD-B297-21A156BEEF06}</x:author>
-    <x:author>tc={794285E2-342A-BBA9-38EF-581EC582B5CF}</x:author>
-    <x:author>tc={29D9448F-3322-BC7C-5B0D-6D4A7A25E07E}</x:author>
-    <x:author>tc={C4D0E925-1F1E-33F1-FDCB-0C7448590B8C}</x:author>
-    <x:author>tc={ACBAEFE3-E08A-0B52-7201-E8AE738DF32E}</x:author>
-    <x:author>tc={7EF31889-764B-C98E-7E80-1407A7F2629D}</x:author>
-    <x:author>tc={9CDEA24C-B17C-97B7-DF28-9F23B53AE16B}</x:author>
-    <x:author>tc={B67EF076-E3E5-09FE-9C12-AB2A3F433819}</x:author>
-    <x:author>tc={1752A508-1C48-B3E9-BCB4-6547CE095D99}</x:author>
-    <x:author>tc={48796B4E-8B2E-5ED9-1CB8-81CB3ADA83B1}</x:author>
-    <x:author>tc={5FFC1694-755F-6CF5-9143-A034A133E846}</x:author>
-    <x:author>tc={658FF627-7EE0-96EC-57FB-FCCA21C7C319}</x:author>
-    <x:author>tc={365194B6-09B8-AF57-F099-8DB4BAA64557}</x:author>
-    <x:author>tc={DC14C814-516B-3F48-9313-B4D9EC42198E}</x:author>
-    <x:author>tc={D4038BF0-51FC-783E-2E95-3C0645EFE8AE}</x:author>
-    <x:author>tc={A20567BA-B53E-892F-E793-2980A3DF98C3}</x:author>
+    <x:author>tc={5435A142-6F48-7F8E-AA2E-F52AAC279AE4}</x:author>
+    <x:author>tc={9CC18C9D-2A7E-BBA4-604E-47BA806E7B2F}</x:author>
+    <x:author>tc={085A4CDC-7E32-358A-62E3-4A77358D08F8}</x:author>
+    <x:author>tc={72DEC69B-94A9-1542-88CA-7EC24E89414E}</x:author>
+    <x:author>tc={EC00A534-D5BA-ED61-3F2B-8CB7D24617E1}</x:author>
+    <x:author>tc={BD623018-280B-401C-F592-908D468F1B42}</x:author>
+    <x:author>tc={5CF44951-8993-C254-E346-988F56277874}</x:author>
+    <x:author>tc={3383E0D9-5FB7-F9D0-946F-0F242015B017}</x:author>
+    <x:author>tc={C9F16D0A-4F5F-AB9A-2C26-F6275E8C8435}</x:author>
+    <x:author>tc={3722723F-FE60-9A5B-A3D7-6C5687C2A97E}</x:author>
+    <x:author>tc={8C0DCAC5-D72E-145A-C09F-EF8C4FAA42B1}</x:author>
+    <x:author>tc={BD872FF7-6078-B13F-D1F4-AA57675D46B6}</x:author>
+    <x:author>tc={6D17A93A-A61E-3F5B-A4A3-40F153329072}</x:author>
+    <x:author>tc={4891741C-0B9F-3D4F-9762-5EDE76F0468C}</x:author>
+    <x:author>tc={53C666BD-211F-1621-F3F0-ECA3FD5F446C}</x:author>
+    <x:author>tc={9FA26BA7-D49E-1A6C-C991-DF33DEA461B9}</x:author>
+    <x:author>tc={DDC71113-18C2-79AE-0740-24D3CBAE7A79}</x:author>
+    <x:author>tc={DDC034C5-42E6-D4B0-1111-EBFA516DC1A1}</x:author>
+    <x:author>tc={D6BA49A0-C68A-81AE-3743-C3D02B24476E}</x:author>
+    <x:author>tc={FB67F30A-6048-BB19-0884-B43E32B634A5}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="J5" authorId="0">
@@ -2060,7 +2060,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8d5b88ebff6b44db"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra6352f4be97f4ffa"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2071,7 +2071,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{040733F0-4A2E-4743-8B04-6908B11C5686}"/>
+  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}"/>
 </xltc:personList>
 </file>
 
@@ -2268,493 +2268,493 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="P5" dT="2026-08-15T14:56:08.194" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{4DBD6BF6-10DC-C9AB-9CD1-709939978DBA}">
+  <xltc:threadedComment ref="P5" dT="2026-08-15T15:09:01.88" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{2ED26A2B-7837-083D-9F91-2E1C1C9C804A}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P6" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{BBA7CF7E-AC28-261A-8B13-2F207C1218A0}">
+  <xltc:threadedComment ref="P6" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{043405D0-022D-CE03-81D3-AF489ABD68A9}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P7" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{72A601D1-876A-91CE-FFAD-4372EAC3B044}">
+  <xltc:threadedComment ref="P7" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{D34DFE13-CAE1-EB32-19DC-D3D61E45A130}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P8" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{63AEFE69-E87F-CB50-C251-F53F91B5BC7D}">
+  <xltc:threadedComment ref="P8" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{F0CC0459-AC75-5733-37FD-D729BDC516EE}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P9" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{34BD6919-CEFF-A072-C07C-DF821615DC08}">
+  <xltc:threadedComment ref="P9" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{BBAB887A-8A65-8B92-424D-300C0145401F}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P10" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{06E212B9-C215-9B55-79D0-3DCC68FDC5F2}">
+  <xltc:threadedComment ref="P10" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{1EE3C80A-BD61-F09D-5B89-C055910B21A8}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 119
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P11" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{B3B2D943-46C7-7159-C4D2-5A2561471484}">
+  <xltc:threadedComment ref="P11" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{071773AC-BAFA-9A1C-7CEC-858AE817169C}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 160
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P12" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{B7F42A5F-C7FD-3C66-478C-F3F30EC65E76}">
+  <xltc:threadedComment ref="P12" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{A64051D4-C4DD-3EAD-CAD5-DDCB5ED2D742}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P13" dT="2026-08-15T14:56:08.196" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{A4597E1D-F181-CFE5-0579-CB8E395D5F43}">
+  <xltc:threadedComment ref="P13" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{342DD7E3-64C9-FC39-8DEA-BB86036F486C}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P14" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{15C385B1-3102-7CB9-2CC5-9E1619C28EFF}">
+  <xltc:threadedComment ref="P14" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{A5720320-9FF6-0861-0144-55CD868F0919}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P15" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{71943B6E-65A7-8FB9-D610-7EAAF042FB72}">
+  <xltc:threadedComment ref="P15" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{13F43D72-1AA3-0364-70A4-6A9B8423C7FE}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P16" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{9C0C8A6E-1868-2889-498E-623A34106926}">
+  <xltc:threadedComment ref="P16" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0E8F289F-DFB0-8655-E6D1-D7FCF99AAB06}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P17" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{334D3079-E2A2-64EF-8548-37B4110F83CB}">
+  <xltc:threadedComment ref="P17" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{4B99CAD2-8EC9-BC88-3AFD-F1394BD6783F}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P18" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{E3828EA9-DCD7-589A-8909-33C5D206AAAB}">
+  <xltc:threadedComment ref="P18" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{010EBAEC-2F9D-B152-1556-960BE1725C4B}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P19" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{7FDAF406-68E0-40BF-FF2E-810ED1C6B3AE}">
+  <xltc:threadedComment ref="P19" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{7333D144-0844-64FD-0AAB-4E413D2935D0}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P20" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{923B38B5-CB1F-C29F-3341-278DDD42C0D1}">
+  <xltc:threadedComment ref="P20" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{5518B81C-B0BC-B171-5762-AAA1625B3F0D}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 138
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P21" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{1A013CBB-E706-00DF-8726-CF619CEB3A04}">
+  <xltc:threadedComment ref="P21" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{FE8B682C-7BBF-FB26-C52A-0567E7240CBA}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 212
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P22" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{EAC196E9-9494-9C63-D76F-35D9C8B67077}">
+  <xltc:threadedComment ref="P22" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{3A15E6D2-B051-8834-4C93-A28DA909DDC7}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P23" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{10D40289-30D1-453D-67F2-D072A488FDF3}">
+  <xltc:threadedComment ref="P23" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{2EA4B4F3-F741-14DC-D1D2-6FA54989E80C}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P24" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{52EC0200-BA64-4464-226D-17C81EC16731}">
+  <xltc:threadedComment ref="P24" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{F4DF57BE-F27A-2E50-A72C-5EF0B356A55E}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P25" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{9CC16C61-D3B8-BFC6-1D65-26993EA95662}">
+  <xltc:threadedComment ref="P25" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{31A0369D-1694-51B8-5DB4-35DB7F6AF63D}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P26" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{87792696-2512-1D5F-88FE-607EFE850C91}">
+  <xltc:threadedComment ref="P26" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{7B5F41ED-10A3-8B79-15C5-6A825FFFDDE4}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P27" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{4D963CBD-121C-D231-C8E6-271C69C09FBC}">
+  <xltc:threadedComment ref="P27" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{46AE8608-356C-86B4-EC18-C1C6FE5CAAAD}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 272
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P28" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{7C7A7265-25A8-9CD8-BDFF-10D4C242D312}">
+  <xltc:threadedComment ref="P28" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{7551C88D-E9F7-2348-0E76-9F80E57D2F60}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P29" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{42EE7233-7324-8500-FA56-AE3756E9E833}">
+  <xltc:threadedComment ref="P29" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{ABF1018A-ABB9-7204-C90E-1105B94E814A}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P30" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{4B348341-5383-CFE2-3931-37A2FB3A6796}">
+  <xltc:threadedComment ref="P30" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{512B7354-5F2C-1AA7-CC3C-00CD42BBE0FC}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 158
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P31" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{1A3E9420-C80E-612F-6856-03663BE6B961}">
+  <xltc:threadedComment ref="P31" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{AFFA6109-ADE2-4CE1-7C27-BAA3EFB317C9}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P32" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{AA18FF0C-0609-3DC9-E3CB-79DB6840A473}">
+  <xltc:threadedComment ref="P32" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{D5144167-7AD8-57DF-B826-07D54D010D9C}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P33" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{A69C99CA-A057-D8BB-284B-25BDF9CCEC33}">
+  <xltc:threadedComment ref="P33" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{B83DFD0F-794A-6C5E-1D58-744B039949BC}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 72
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P34" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{D50807E6-8164-064B-B075-38383003CD54}">
+  <xltc:threadedComment ref="P34" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{7B9E1B4B-9DCB-BECD-99F5-F055FB863E9C}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P35" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{BE002E50-346C-2ED1-02B3-A8794F3AB605}">
+  <xltc:threadedComment ref="P35" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{8B2DC34E-17AF-DC22-540E-3A7428974B96}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P36" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{B098C298-69AE-EEB7-D1C2-F7BC866E55B9}">
+  <xltc:threadedComment ref="P36" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{094E8309-B86F-1491-11B7-E843D5E63DAC}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 24
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P37" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{F3A4232B-B2F0-E38E-C4CD-27D2A497F98F}">
+  <xltc:threadedComment ref="P37" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{4513E577-194B-E888-43E5-01675E143F65}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P38" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{501C0B3C-E9F4-5518-C3B8-8CD0B037469A}">
+  <xltc:threadedComment ref="P38" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{D063F1D2-2F95-2667-C7FF-CB2952CE7907}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P39" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{BC165DAF-BA11-F405-6CBF-79578886B019}">
+  <xltc:threadedComment ref="P39" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{C9AF5DAB-FC5E-E759-C111-2F94BE966A52}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 19
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P40" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{580C07C1-9FAB-9F69-74D0-3B9278C97DDA}">
+  <xltc:threadedComment ref="P40" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{5C3D6D9E-0399-3A1F-5FF8-7673B95728DC}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P41" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{8CD97F42-50C5-7B2D-C42C-71A1179025FC}">
+  <xltc:threadedComment ref="P41" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{40BAA6D9-7593-464B-9634-92C58D16225A}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P42" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{6C0F0126-E58B-902E-A8E6-295BFBA74E7B}">
+  <xltc:threadedComment ref="P42" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{DA3A9B1C-4CB2-882E-946C-A1860B6BC64A}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P43" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{D63E76FC-0272-8768-DE65-B5AF8778D0B0}">
+  <xltc:threadedComment ref="P43" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{05CE38D1-9BF6-E417-141B-4027834AA96E}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P44" dT="2026-08-15T14:56:08.197" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{B09B5ACD-368E-1E68-6052-475ECD03C5BF}">
+  <xltc:threadedComment ref="P44" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{B6C35BC3-6F5F-B362-B79B-E7478D767EAB}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P45" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{522883C0-51F3-52B3-5700-E265E06929EF}">
+  <xltc:threadedComment ref="P45" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{A2136AA3-D60A-9CA4-782A-688014FA68CC}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P46" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{54087D2A-D6F4-3D3A-D693-CAD90133167F}">
+  <xltc:threadedComment ref="P46" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{F9107F21-217D-6E1C-0F95-26D39A645301}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P47" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{5F18F3D5-8D17-8C4C-2D06-CDD09EA4D216}">
+  <xltc:threadedComment ref="P47" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{6BDCC13B-4293-D80F-CDD9-0D914AF1E069}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P48" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{13740A3D-A1FC-15E2-13DB-4FFB05B462BF}">
+  <xltc:threadedComment ref="P48" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{6FCD0DD5-A300-B061-80FD-E6DA09A1A00C}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P49" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{847A4145-4A0C-DA46-C37F-6096CA91F67D}">
+  <xltc:threadedComment ref="P49" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{D33E4AF9-5B00-4D1E-2774-D1A03F8DAA00}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 118
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P50" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{D6864198-192F-5FD4-B268-3D436B7AC010}">
+  <xltc:threadedComment ref="P50" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{B93F8331-7F4C-8F1E-6D00-D4F3F4DD941B}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P51" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{EBFCBED8-6CFC-ECB3-8C0A-7C4E9AD344F5}">
+  <xltc:threadedComment ref="P51" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{01017BE8-DAC5-0C0D-B269-33BF689C7906}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P52" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{9AD77AC5-C741-5D2F-DBAB-2B74EE25C270}">
+  <xltc:threadedComment ref="P52" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0F0598D8-65DE-16CC-F316-558AAB8C206A}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P53" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{ED12DAB1-3AFE-11C4-196F-7EE762522CAC}">
+  <xltc:threadedComment ref="P53" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{FD22F09B-1275-26C7-C5BC-CEBC26B724BD}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-STF</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P54" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{02AE57B2-7B9E-C2C4-B082-B19B326B3377}">
+  <xltc:threadedComment ref="P54" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{50296461-F84A-5759-D5C7-3C73B6727E11}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P55" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{675B19DD-8D0C-3276-6CE4-66346F83A194}">
+  <xltc:threadedComment ref="P55" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{25FD297A-C8A3-7982-2A2A-6109869C428D}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P56" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{762EADA7-A8B4-889D-2C9B-B45528872477}">
+  <xltc:threadedComment ref="P56" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{A01BC395-D63D-37E2-3702-F398D5D7D853}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 18
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P57" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{EE508AFA-CBC9-9D04-C56A-ADE149A617D2}">
+  <xltc:threadedComment ref="P57" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{3CCE64FE-3C38-CB25-DAB1-1288A0B1E1D3}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P58" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{7C3918C2-74FE-3B30-0011-76B90C31220D}">
+  <xltc:threadedComment ref="P58" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0381E4D2-1AB7-DC1B-5477-B3CE9858338D}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P59" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{B0FB2B0B-0E15-0FE4-7CE3-AD5EA4809E58}">
+  <xltc:threadedComment ref="P59" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0DB1B439-2233-2FF4-7F69-4CFB903C8BCE}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P60" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{D23A2CFB-B4DA-68EC-FAF4-DF302B3BF193}">
+  <xltc:threadedComment ref="P60" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{702F1FDC-2B20-239C-C387-1F9994029E58}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P61" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{7AD41A11-0701-521D-0569-2ED6CDD82249}">
+  <xltc:threadedComment ref="P61" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{86BF3B4D-4C8B-94C5-2DF8-0E144D24162D}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P62" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{BCAC211D-B580-F9C0-E665-E57993EB833C}">
+  <xltc:threadedComment ref="P62" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{55FEB31D-AA64-C68B-21EB-2AD4013CA9D9}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P63" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{F6DDB6CD-A478-A288-D046-D50AE0A2F4F6}">
+  <xltc:threadedComment ref="P63" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{2120B059-1D9A-FB52-CB20-859A8A7B4431}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P64" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{AB6399B6-CEFB-A3AE-273C-3B6F7674686D}">
+  <xltc:threadedComment ref="P64" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{DDAE0E6F-C9F0-E461-07EA-91968BE2E6D2}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P65" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{9194F186-D8EE-E399-BA03-2D260FE5AAA6}">
+  <xltc:threadedComment ref="P65" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{83232D14-7BAC-B848-7871-277E89FA684E}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 311
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P66" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{6FF53E52-37D4-CC19-3305-7182C053444B}">
+  <xltc:threadedComment ref="P66" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{279DD734-DD6F-13E2-E0FD-18F5BF78E98D}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P67" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{7C97B6C7-01FC-A9B4-6016-4EF64AFF88BA}">
+  <xltc:threadedComment ref="P67" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0C0BEC61-5240-DC56-B9D0-4183924DDDA7}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P68" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{B2345AD4-1F0A-8132-33EE-B7AB8CFFBC6B}">
+  <xltc:threadedComment ref="P68" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{4B78E0A5-E835-82BC-95E0-9D6660CB0642}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 141
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P69" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{8E4DE5D3-82C1-B07F-9C4A-9689FB42A15A}">
+  <xltc:threadedComment ref="P69" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{2AA3892A-F3E0-DCE4-4BA3-77C2298E4712}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P70" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{3F4FFDE4-26EA-E657-F41C-D27365F25776}">
+  <xltc:threadedComment ref="P70" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0BF67983-6F8F-9A8B-A733-988A5AE771CE}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P71" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{971388A1-D191-476F-30E3-CAF0BDF52814}">
+  <xltc:threadedComment ref="P71" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{853E2097-1ED4-88BD-0FEF-BB1C45A97F6A}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 33
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P72" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{87E9E59C-24D1-4B9B-2AAB-86BED77B3F37}">
+  <xltc:threadedComment ref="P72" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{5437FE01-1237-5D55-7238-D3B41AD600A7}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P73" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{4976AFE0-5E10-3595-15C3-A927BCBB7717}">
+  <xltc:threadedComment ref="P73" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{26525073-6162-76FE-6D24-B53B287B9745}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P74" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{1D183FA9-A787-A694-E39D-E98D2922412B}">
+  <xltc:threadedComment ref="P74" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{BAC99CA3-3171-9911-60EA-9ADBAD9DAA89}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 21
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P75" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{58AF00BE-79AC-4743-650E-E7324330A1BA}">
+  <xltc:threadedComment ref="P75" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{4E489A6C-1C1A-971C-72AB-ACB53D354D17}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P76" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{D0EF5D59-18D7-6229-0688-54F1699A15EF}">
+  <xltc:threadedComment ref="P76" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{280D1E73-5C17-150A-507B-D8086C4BA2AD}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P77" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{111F6C62-CBBA-BE4F-FF75-9BBDF71AE371}">
+  <xltc:threadedComment ref="P77" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{33816FEE-5341-8E14-F197-F3763F51C77B}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 19
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P78" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{EC36B2E5-7EB6-7E1B-F633-1386EF2A8501}">
+  <xltc:threadedComment ref="P78" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0277E1E1-ACCD-F4A6-B8D9-B0F98C590404}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 43
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P79" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{94020BB4-4F25-D013-B6E5-BB7F36D27B62}">
+  <xltc:threadedComment ref="P79" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{F919CE15-F9D0-4C7F-A7F6-D4B6CEEDC7C3}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 44
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P80" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{FEF6468A-A138-F925-C425-925FC389C735}">
+  <xltc:threadedComment ref="P80" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{70300967-130C-E9FC-5833-2A5E4C05B7E1}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 40
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P81" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{256ED2F9-711C-D379-9CF7-0C33127AB323}">
+  <xltc:threadedComment ref="P81" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{6A5C72F7-2A4F-E907-50AB-917C148A344A}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P82" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{7FB9D626-25E8-1DBD-4F9B-E1D2D52EE7B2}">
+  <xltc:threadedComment ref="P82" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0459789A-01BE-4F0D-BABB-8071C46032C0}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P83" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{6A9B9A15-4C5F-9E87-6014-3970EF50A532}">
+  <xltc:threadedComment ref="P83" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{AF3F7297-575B-2C4C-A9A0-434E38FE21C6}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 16
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P84" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{BA8AB825-F19D-0BB0-BBFA-A0876A1836D0}">
+  <xltc:threadedComment ref="P84" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{2DFC25D3-339D-7566-5DC3-205EE0DC70AC}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P85" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{AC1C627A-2A35-C925-6C42-AE55C1F90C62}">
+  <xltc:threadedComment ref="P85" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{326FB552-EB16-8CC1-A7BC-665356E8462C}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P86" dT="2026-08-15T14:56:08.198" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{2E768F64-774D-1D28-E9F7-5D8185ADD575}">
+  <xltc:threadedComment ref="P86" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{5B218977-D8FC-2E26-E971-16C48C7A4A64}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 21
 Available: 2026-02-25
@@ -2765,64 +2765,64 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="J5" dT="2026-08-15T14:56:08.514" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{4621E60A-8035-BA73-3B5F-4819B7B702C6}">
+  <xltc:threadedComment ref="J5" dT="2026-08-15T15:09:02.238" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{5435A142-6F48-7F8E-AA2E-F52AAC279AE4}">
     <xltc:text>Official source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J6" dT="2026-08-15T14:56:08.517" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{162796F4-247C-2919-A562-B9397445C769}">
+  <xltc:threadedComment ref="J6" dT="2026-08-15T15:09:02.241" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{9CC18C9D-2A7E-BBA4-604E-47BA806E7B2F}">
     <xltc:text>Official source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J7" dT="2026-08-15T14:56:08.52" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{634CC515-1D2E-7411-C7E2-E57361E9A689}">
+  <xltc:threadedComment ref="J7" dT="2026-08-15T15:09:02.244" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{085A4CDC-7E32-358A-62E3-4A77358D08F8}">
     <xltc:text>Official source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J8" dT="2026-08-15T14:56:08.523" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{9672D852-1459-A87F-2C39-1EFA570D28E9}">
+  <xltc:threadedComment ref="J8" dT="2026-08-15T15:09:02.246" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{72DEC69B-94A9-1542-88CA-7EC24E89414E}">
     <xltc:text>Official source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J9" dT="2026-08-15T14:56:08.525" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{01A23984-C62A-08AD-B297-21A156BEEF06}">
+  <xltc:threadedComment ref="J9" dT="2026-08-15T15:09:02.249" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{EC00A534-D5BA-ED61-3F2B-8CB7D24617E1}">
     <xltc:text>Official source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J10" dT="2026-08-15T14:56:08.527" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{794285E2-342A-BBA9-38EF-581EC582B5CF}">
+  <xltc:threadedComment ref="J10" dT="2026-08-15T15:09:02.251" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{BD623018-280B-401C-F592-908D468F1B42}">
     <xltc:text>Official source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J11" dT="2026-08-15T14:56:08.529" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{29D9448F-3322-BC7C-5B0D-6D4A7A25E07E}">
+  <xltc:threadedComment ref="J11" dT="2026-08-15T15:09:02.253" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{5CF44951-8993-C254-E346-988F56277874}">
     <xltc:text>Official source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J12" dT="2026-08-15T14:56:08.531" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{C4D0E925-1F1E-33F1-FDCB-0C7448590B8C}">
+  <xltc:threadedComment ref="J12" dT="2026-08-15T15:09:02.256" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{3383E0D9-5FB7-F9D0-946F-0F242015B017}">
     <xltc:text>Official source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J13" dT="2026-08-15T14:56:08.534" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{ACBAEFE3-E08A-0B52-7201-E8AE738DF32E}">
+  <xltc:threadedComment ref="J13" dT="2026-08-15T15:09:02.259" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{C9F16D0A-4F5F-AB9A-2C26-F6275E8C8435}">
     <xltc:text>Official source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J14" dT="2026-08-15T14:56:08.536" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{7EF31889-764B-C98E-7E80-1407A7F2629D}">
+  <xltc:threadedComment ref="J14" dT="2026-08-15T15:09:02.26" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{3722723F-FE60-9A5B-A3D7-6C5687C2A97E}">
     <xltc:text>Official source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J15" dT="2026-08-15T14:56:08.538" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{9CDEA24C-B17C-97B7-DF28-9F23B53AE16B}">
+  <xltc:threadedComment ref="J15" dT="2026-08-15T15:09:02.262" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{8C0DCAC5-D72E-145A-C09F-EF8C4FAA42B1}">
     <xltc:text>Official source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J16" dT="2026-08-15T14:56:08.54" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{B67EF076-E3E5-09FE-9C12-AB2A3F433819}">
+  <xltc:threadedComment ref="J16" dT="2026-08-15T15:09:02.266" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{BD872FF7-6078-B13F-D1F4-AA57675D46B6}">
     <xltc:text>Official source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J17" dT="2026-08-15T14:56:08.542" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{1752A508-1C48-B3E9-BCB4-6547CE095D99}">
+  <xltc:threadedComment ref="J17" dT="2026-08-15T15:09:02.268" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{6D17A93A-A61E-3F5B-A4A3-40F153329072}">
     <xltc:text>Official source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J18" dT="2026-08-15T14:56:08.546" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{48796B4E-8B2E-5ED9-1CB8-81CB3ADA83B1}">
+  <xltc:threadedComment ref="J18" dT="2026-08-15T15:09:02.27" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{4891741C-0B9F-3D4F-9762-5EDE76F0468C}">
     <xltc:text>Official source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J19" dT="2026-08-15T14:56:08.548" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{5FFC1694-755F-6CF5-9143-A034A133E846}">
+  <xltc:threadedComment ref="J19" dT="2026-08-15T15:09:02.272" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{53C666BD-211F-1621-F3F0-ECA3FD5F446C}">
     <xltc:text>Official source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J20" dT="2026-08-15T14:56:08.55" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{658FF627-7EE0-96EC-57FB-FCCA21C7C319}">
+  <xltc:threadedComment ref="J20" dT="2026-08-15T15:09:02.275" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{9FA26BA7-D49E-1A6C-C991-DF33DEA461B9}">
     <xltc:text>Official source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J21" dT="2026-08-15T14:56:08.552" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{365194B6-09B8-AF57-F099-8DB4BAA64557}">
+  <xltc:threadedComment ref="J21" dT="2026-08-15T15:09:02.277" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{DDC71113-18C2-79AE-0740-24D3CBAE7A79}">
     <xltc:text>Official source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J22" dT="2026-08-15T14:56:08.554" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{DC14C814-516B-3F48-9313-B4D9EC42198E}">
+  <xltc:threadedComment ref="J22" dT="2026-08-15T15:09:02.279" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{DDC034C5-42E6-D4B0-1111-EBFA516DC1A1}">
     <xltc:text>Official source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J23" dT="2026-08-15T14:56:08.556" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{D4038BF0-51FC-783E-2E95-3C0645EFE8AE}">
+  <xltc:threadedComment ref="J23" dT="2026-08-15T15:09:02.281" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{D6BA49A0-C68A-81AE-3743-C3D02B24476E}">
     <xltc:text>Official source: https://www.aspenpharma.com/download/annual-financial-statements-2/</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J24" dT="2026-08-15T14:56:08.558" personId="{040733F0-4A2E-4743-8B04-6908B11C5686}" id="{A20567BA-B53E-892F-E793-2980A3DF98C3}">
+  <xltc:threadedComment ref="J24" dT="2026-08-15T15:09:02.282" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{FB67F30A-6048-BB19-0884-B43E32B634A5}">
     <xltc:text>Official source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -3877,7 +3877,7 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70bd2a2cedd04f03"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3932c49e3ae64aaa"/>
 </x:worksheet>
 </file>
 
@@ -8611,7 +8611,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e1b7f1952284071"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cc4b2c86cc4433c"/>
 </x:worksheet>
 </file>
 
@@ -9671,7 +9671,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf532b07fe2d41af"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d74c8a6f0f84da8"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Harden V3.2 hackathon submission coherence (#3)
* Harden V3.2 submission coherence

* Refresh V3.2 judging artifacts

* Make canonical artifact build convergent

* Bind V3.2 artifacts to final status authority

* Normalize cross-platform presentation provenance

* Use content-based submission drift checks

* Stamp final V3.2 submission artifacts

* Normalize golden-set hashes across platforms

* Restamp V3.2 artifacts after portable hash fix

* Preserve frozen digest and V3.2 status authority

* Restamp final V3.2 portable release
</commit_message>
<xml_diff>
--- a/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
+++ b/outputs/audit/Public-Facts-Anchor-Register-V3.2.0.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R380f9c27d3944774"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="Rfffcb405ec464c1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="R48c193a887c4416e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Rd66998ed3cc04402"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R49c40c130e0d45ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R631bd8a5e6674ca9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Rde69964a6bf84944"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="R858c58fbb73144bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="Rf02af7084cc44489"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R85030ef8203c4a51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R04a3fd164f384795"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R446d898fd8cb466b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="Rfbee45e282674bc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Rab888e9a2693495e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R77b2312b46be4a45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="Rbd702c155274446d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Rb087a52c07eb45e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion Readiness" sheetId="8" r:id="R49c2453e8b4c4cd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R93e8c8668f174eb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R6e68213158384451"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,88 +19,88 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={0AF4FEDA-AC03-3F9A-4677-E614750C0BE6}</x:author>
-    <x:author>tc={7B13601B-A686-D1F6-E2C3-2DEAACC41826}</x:author>
-    <x:author>tc={10B9DE82-DAAF-597E-4424-E67283E9A4F8}</x:author>
-    <x:author>tc={9DDF9D19-AAB7-35C6-6EAB-ADE447886907}</x:author>
-    <x:author>tc={CEC6EDDA-4333-DE39-19A1-CD6C28B0071E}</x:author>
-    <x:author>tc={9E0A3C03-F7F7-40B8-594C-1134A321AF12}</x:author>
-    <x:author>tc={6A469CC5-9E84-42E7-A4A2-5046B5EB797A}</x:author>
-    <x:author>tc={49F38930-D4FC-9148-B4AB-7B8868A6B1C4}</x:author>
-    <x:author>tc={6AE471B8-00A6-D8CA-E30E-F2F43B242CB2}</x:author>
-    <x:author>tc={070A3F26-F4D3-3501-5B26-B76E24181EE6}</x:author>
-    <x:author>tc={DB4AA7DC-83F7-AA9C-6650-AC0FBB081C37}</x:author>
-    <x:author>tc={E8A6B8CE-ACDD-0EA3-3036-3FEA4BE387E5}</x:author>
-    <x:author>tc={F5132FA4-62BD-C63C-B25A-A7E1FE946B04}</x:author>
-    <x:author>tc={924A75EC-79F9-BE2D-03E1-123D59F3BF71}</x:author>
-    <x:author>tc={7DFAAAEE-9F37-70B4-1295-82F48891DA0C}</x:author>
-    <x:author>tc={E2EA446D-49CF-67B3-25D3-448163193339}</x:author>
-    <x:author>tc={130AC7D8-E99A-FB9E-EC90-C0CC209F65EE}</x:author>
-    <x:author>tc={DFEDA6A7-98B9-D90B-F8E4-87463C1ABE71}</x:author>
-    <x:author>tc={F908D626-E856-7A2E-B578-6FFFAF10A067}</x:author>
-    <x:author>tc={4691BC9F-FA65-4FBB-BE88-C3485B37BF5B}</x:author>
-    <x:author>tc={54D1659D-A9A9-797D-09FE-9CCD3046EB3B}</x:author>
-    <x:author>tc={32021335-239B-D7CF-C593-02492073755E}</x:author>
-    <x:author>tc={2D4C52F2-DF0E-98A8-DBAD-465EFEA6430C}</x:author>
-    <x:author>tc={4F673CEB-0DB2-16EC-1BF9-E9916FC0D89C}</x:author>
-    <x:author>tc={8C766CE4-DCA4-0227-2719-EC43FBE4EB3E}</x:author>
-    <x:author>tc={030B07FB-3D16-4698-B4D5-9BFD808ED081}</x:author>
-    <x:author>tc={BB835A0A-AC15-BD40-37D2-BB2D5D7D1A29}</x:author>
-    <x:author>tc={ACE1C8E0-F10B-F24B-C4C3-09990BA1EAF5}</x:author>
-    <x:author>tc={89E2F11B-ECCC-3429-226F-74770117AB92}</x:author>
-    <x:author>tc={FE94A6DE-84F6-0201-3EFF-69B3D6B7D622}</x:author>
-    <x:author>tc={5FADB78B-442A-2857-7CCC-D525C440BCCF}</x:author>
-    <x:author>tc={33238565-3127-12AD-ACAF-5A83E4E3101E}</x:author>
-    <x:author>tc={DBA819E1-2CFB-40C0-8E60-4EBBB4963742}</x:author>
-    <x:author>tc={831BC617-DC59-E847-0D3A-95946FD8D988}</x:author>
-    <x:author>tc={9625D7E8-9A23-1EEE-66C1-3D1F41528532}</x:author>
-    <x:author>tc={36A13555-305E-B2C5-2B7A-87476C5BA766}</x:author>
-    <x:author>tc={69541CEA-6E11-BC48-6898-36AE3D548AB4}</x:author>
-    <x:author>tc={12AFE746-FDD9-963F-DCFD-DC968D22FFA6}</x:author>
-    <x:author>tc={425C83BD-D4DC-BDED-071D-487523F8AC3F}</x:author>
-    <x:author>tc={2D72A011-0216-7D35-09A3-D704E88BAEE3}</x:author>
-    <x:author>tc={86FBCAB8-88A0-F97B-4FA1-13C4BEAA369D}</x:author>
-    <x:author>tc={9185AC7C-5FA5-8BAE-5D74-F86F31883FC5}</x:author>
-    <x:author>tc={8F348568-9728-931E-D9B2-061F382ED13A}</x:author>
-    <x:author>tc={E5746BEC-90A8-ABA0-16B5-A6A9F11A2C96}</x:author>
-    <x:author>tc={4B1E6C62-4809-1469-5784-9EA7A65F2E2D}</x:author>
-    <x:author>tc={271EEFA8-492B-5EC5-67E3-8B28D1AE9871}</x:author>
-    <x:author>tc={3430FD27-2DAA-4633-A322-0688F2FCD467}</x:author>
-    <x:author>tc={8D7DF3C9-36A9-2E8C-6160-11B116238A97}</x:author>
-    <x:author>tc={31933AFB-CA47-471A-E7EB-D7E5B693D87A}</x:author>
-    <x:author>tc={CEB8E96A-F9CE-D6E4-1345-25BEA6D4853C}</x:author>
-    <x:author>tc={CE8B63E6-EC70-4885-EBBF-C61B84B9BD02}</x:author>
-    <x:author>tc={1236AB2A-50DD-58C5-F0CF-0A77396ECCB9}</x:author>
-    <x:author>tc={23B809AB-666E-3843-AA8B-2E06C9D6735C}</x:author>
-    <x:author>tc={F9218197-D7D7-96FC-5DEE-19E1B89C6668}</x:author>
-    <x:author>tc={49C564EF-C6E1-AA3E-BAE6-F9B6B7DAF702}</x:author>
-    <x:author>tc={6A34B57F-09E3-5DA4-9CDF-BDD9AFC15C62}</x:author>
-    <x:author>tc={EA67CC0C-3B7B-6001-4E9C-C907CB9A2E41}</x:author>
-    <x:author>tc={2C705125-9621-DC7B-9356-1AFFFB014183}</x:author>
-    <x:author>tc={4127462E-7049-10C8-6E6D-2726FCAFA040}</x:author>
-    <x:author>tc={DDC7860C-4BF8-FE8E-AB94-BF36F51E4742}</x:author>
-    <x:author>tc={355CD349-BEF2-1F91-3717-B7779FC267B7}</x:author>
-    <x:author>tc={BE707954-D4F8-3036-E784-0F6EF373E3B1}</x:author>
-    <x:author>tc={30C17E09-F415-E5D5-1412-983D6592AE59}</x:author>
-    <x:author>tc={946D1FE7-F4AA-6563-A358-3F55219C3AED}</x:author>
-    <x:author>tc={FF9DEADC-5F2B-2C71-0EDD-31A65A1DAC80}</x:author>
-    <x:author>tc={99FA21E2-86C5-2A76-2880-8215954AA3D4}</x:author>
-    <x:author>tc={901E21A1-49DD-A0DA-0A10-1EDE8076C1B3}</x:author>
-    <x:author>tc={FCB3C38E-B0AF-A412-700D-4D9A9D2C2741}</x:author>
-    <x:author>tc={9382A565-2A1D-550E-54B1-678F98943EC6}</x:author>
-    <x:author>tc={40576489-4A24-6AA0-06F2-24F75770098B}</x:author>
-    <x:author>tc={D80EF366-6BBD-D5AC-E71F-5666ED857ED8}</x:author>
-    <x:author>tc={8E28E375-5E9B-B43C-02D8-1D69B6DBCCB7}</x:author>
-    <x:author>tc={C52D303F-E26F-AEB2-82AD-C196257D053A}</x:author>
-    <x:author>tc={AD3CBF1C-654B-022F-1CCE-E3B6B02846E3}</x:author>
-    <x:author>tc={2EEF0622-B8D5-960E-069D-57BC28C46AE4}</x:author>
-    <x:author>tc={C7A17400-8C3D-04F3-BB45-75623A8D8379}</x:author>
-    <x:author>tc={9CB15BCB-A81F-4C51-B6D7-CA70F830A75F}</x:author>
-    <x:author>tc={9CDE5188-52E3-BEBE-AC4D-8F98AC717AA6}</x:author>
-    <x:author>tc={96D773F7-6FC9-4DF1-46BC-3C5A65EBE44A}</x:author>
-    <x:author>tc={69BF4FC0-9856-F2BC-F517-9DC02348AB96}</x:author>
-    <x:author>tc={EF1A8A33-3E41-8002-8157-23C7596AF4CA}</x:author>
-    <x:author>tc={CBA415B4-31A9-6F43-882D-D511ADAA6836}</x:author>
+    <x:author>tc={2ED26A2B-7837-083D-9F91-2E1C1C9C804A}</x:author>
+    <x:author>tc={043405D0-022D-CE03-81D3-AF489ABD68A9}</x:author>
+    <x:author>tc={D34DFE13-CAE1-EB32-19DC-D3D61E45A130}</x:author>
+    <x:author>tc={F0CC0459-AC75-5733-37FD-D729BDC516EE}</x:author>
+    <x:author>tc={BBAB887A-8A65-8B92-424D-300C0145401F}</x:author>
+    <x:author>tc={1EE3C80A-BD61-F09D-5B89-C055910B21A8}</x:author>
+    <x:author>tc={071773AC-BAFA-9A1C-7CEC-858AE817169C}</x:author>
+    <x:author>tc={A64051D4-C4DD-3EAD-CAD5-DDCB5ED2D742}</x:author>
+    <x:author>tc={342DD7E3-64C9-FC39-8DEA-BB86036F486C}</x:author>
+    <x:author>tc={A5720320-9FF6-0861-0144-55CD868F0919}</x:author>
+    <x:author>tc={13F43D72-1AA3-0364-70A4-6A9B8423C7FE}</x:author>
+    <x:author>tc={0E8F289F-DFB0-8655-E6D1-D7FCF99AAB06}</x:author>
+    <x:author>tc={4B99CAD2-8EC9-BC88-3AFD-F1394BD6783F}</x:author>
+    <x:author>tc={010EBAEC-2F9D-B152-1556-960BE1725C4B}</x:author>
+    <x:author>tc={7333D144-0844-64FD-0AAB-4E413D2935D0}</x:author>
+    <x:author>tc={5518B81C-B0BC-B171-5762-AAA1625B3F0D}</x:author>
+    <x:author>tc={FE8B682C-7BBF-FB26-C52A-0567E7240CBA}</x:author>
+    <x:author>tc={3A15E6D2-B051-8834-4C93-A28DA909DDC7}</x:author>
+    <x:author>tc={2EA4B4F3-F741-14DC-D1D2-6FA54989E80C}</x:author>
+    <x:author>tc={F4DF57BE-F27A-2E50-A72C-5EF0B356A55E}</x:author>
+    <x:author>tc={31A0369D-1694-51B8-5DB4-35DB7F6AF63D}</x:author>
+    <x:author>tc={7B5F41ED-10A3-8B79-15C5-6A825FFFDDE4}</x:author>
+    <x:author>tc={46AE8608-356C-86B4-EC18-C1C6FE5CAAAD}</x:author>
+    <x:author>tc={7551C88D-E9F7-2348-0E76-9F80E57D2F60}</x:author>
+    <x:author>tc={ABF1018A-ABB9-7204-C90E-1105B94E814A}</x:author>
+    <x:author>tc={512B7354-5F2C-1AA7-CC3C-00CD42BBE0FC}</x:author>
+    <x:author>tc={AFFA6109-ADE2-4CE1-7C27-BAA3EFB317C9}</x:author>
+    <x:author>tc={D5144167-7AD8-57DF-B826-07D54D010D9C}</x:author>
+    <x:author>tc={B83DFD0F-794A-6C5E-1D58-744B039949BC}</x:author>
+    <x:author>tc={7B9E1B4B-9DCB-BECD-99F5-F055FB863E9C}</x:author>
+    <x:author>tc={8B2DC34E-17AF-DC22-540E-3A7428974B96}</x:author>
+    <x:author>tc={094E8309-B86F-1491-11B7-E843D5E63DAC}</x:author>
+    <x:author>tc={4513E577-194B-E888-43E5-01675E143F65}</x:author>
+    <x:author>tc={D063F1D2-2F95-2667-C7FF-CB2952CE7907}</x:author>
+    <x:author>tc={C9AF5DAB-FC5E-E759-C111-2F94BE966A52}</x:author>
+    <x:author>tc={5C3D6D9E-0399-3A1F-5FF8-7673B95728DC}</x:author>
+    <x:author>tc={40BAA6D9-7593-464B-9634-92C58D16225A}</x:author>
+    <x:author>tc={DA3A9B1C-4CB2-882E-946C-A1860B6BC64A}</x:author>
+    <x:author>tc={05CE38D1-9BF6-E417-141B-4027834AA96E}</x:author>
+    <x:author>tc={B6C35BC3-6F5F-B362-B79B-E7478D767EAB}</x:author>
+    <x:author>tc={A2136AA3-D60A-9CA4-782A-688014FA68CC}</x:author>
+    <x:author>tc={F9107F21-217D-6E1C-0F95-26D39A645301}</x:author>
+    <x:author>tc={6BDCC13B-4293-D80F-CDD9-0D914AF1E069}</x:author>
+    <x:author>tc={6FCD0DD5-A300-B061-80FD-E6DA09A1A00C}</x:author>
+    <x:author>tc={D33E4AF9-5B00-4D1E-2774-D1A03F8DAA00}</x:author>
+    <x:author>tc={B93F8331-7F4C-8F1E-6D00-D4F3F4DD941B}</x:author>
+    <x:author>tc={01017BE8-DAC5-0C0D-B269-33BF689C7906}</x:author>
+    <x:author>tc={0F0598D8-65DE-16CC-F316-558AAB8C206A}</x:author>
+    <x:author>tc={FD22F09B-1275-26C7-C5BC-CEBC26B724BD}</x:author>
+    <x:author>tc={50296461-F84A-5759-D5C7-3C73B6727E11}</x:author>
+    <x:author>tc={25FD297A-C8A3-7982-2A2A-6109869C428D}</x:author>
+    <x:author>tc={A01BC395-D63D-37E2-3702-F398D5D7D853}</x:author>
+    <x:author>tc={3CCE64FE-3C38-CB25-DAB1-1288A0B1E1D3}</x:author>
+    <x:author>tc={0381E4D2-1AB7-DC1B-5477-B3CE9858338D}</x:author>
+    <x:author>tc={0DB1B439-2233-2FF4-7F69-4CFB903C8BCE}</x:author>
+    <x:author>tc={702F1FDC-2B20-239C-C387-1F9994029E58}</x:author>
+    <x:author>tc={86BF3B4D-4C8B-94C5-2DF8-0E144D24162D}</x:author>
+    <x:author>tc={55FEB31D-AA64-C68B-21EB-2AD4013CA9D9}</x:author>
+    <x:author>tc={2120B059-1D9A-FB52-CB20-859A8A7B4431}</x:author>
+    <x:author>tc={DDAE0E6F-C9F0-E461-07EA-91968BE2E6D2}</x:author>
+    <x:author>tc={83232D14-7BAC-B848-7871-277E89FA684E}</x:author>
+    <x:author>tc={279DD734-DD6F-13E2-E0FD-18F5BF78E98D}</x:author>
+    <x:author>tc={0C0BEC61-5240-DC56-B9D0-4183924DDDA7}</x:author>
+    <x:author>tc={4B78E0A5-E835-82BC-95E0-9D6660CB0642}</x:author>
+    <x:author>tc={2AA3892A-F3E0-DCE4-4BA3-77C2298E4712}</x:author>
+    <x:author>tc={0BF67983-6F8F-9A8B-A733-988A5AE771CE}</x:author>
+    <x:author>tc={853E2097-1ED4-88BD-0FEF-BB1C45A97F6A}</x:author>
+    <x:author>tc={5437FE01-1237-5D55-7238-D3B41AD600A7}</x:author>
+    <x:author>tc={26525073-6162-76FE-6D24-B53B287B9745}</x:author>
+    <x:author>tc={BAC99CA3-3171-9911-60EA-9ADBAD9DAA89}</x:author>
+    <x:author>tc={4E489A6C-1C1A-971C-72AB-ACB53D354D17}</x:author>
+    <x:author>tc={280D1E73-5C17-150A-507B-D8086C4BA2AD}</x:author>
+    <x:author>tc={33816FEE-5341-8E14-F197-F3763F51C77B}</x:author>
+    <x:author>tc={0277E1E1-ACCD-F4A6-B8D9-B0F98C590404}</x:author>
+    <x:author>tc={F919CE15-F9D0-4C7F-A7F6-D4B6CEEDC7C3}</x:author>
+    <x:author>tc={70300967-130C-E9FC-5833-2A5E4C05B7E1}</x:author>
+    <x:author>tc={6A5C72F7-2A4F-E907-50AB-917C148A344A}</x:author>
+    <x:author>tc={0459789A-01BE-4F0D-BABB-8071C46032C0}</x:author>
+    <x:author>tc={AF3F7297-575B-2C4C-A9A0-434E38FE21C6}</x:author>
+    <x:author>tc={2DFC25D3-339D-7566-5DC3-205EE0DC70AC}</x:author>
+    <x:author>tc={326FB552-EB16-8CC1-A7BC-665356E8462C}</x:author>
+    <x:author>tc={5B218977-D8FC-2E26-E971-16C48C7A4A64}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="P5" authorId="0">
@@ -1176,26 +1176,26 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={B01406AF-5C54-1385-E93F-8BC31DCEF046}</x:author>
-    <x:author>tc={6DD7D282-4D5B-6CEA-034D-91D0362B1489}</x:author>
-    <x:author>tc={B744CA31-60A8-7C0A-67C6-4F7042734E04}</x:author>
-    <x:author>tc={2CBFDB07-DAC4-1F7C-80B7-A9AE350E67F7}</x:author>
-    <x:author>tc={C6FFBF76-75E5-A885-90FC-7A4822669D85}</x:author>
-    <x:author>tc={48B6FC78-C54C-A341-9A8A-BAE4F532FF12}</x:author>
-    <x:author>tc={40834F88-B44F-30F0-0C1E-7A7EA53D4250}</x:author>
-    <x:author>tc={8C86F84D-BA29-E3DB-77BF-71A0444405B8}</x:author>
-    <x:author>tc={E119E111-72FF-3D54-C250-0ADC5886F9C3}</x:author>
-    <x:author>tc={82842CDD-4566-2F54-CBEE-B39CF6B61B97}</x:author>
-    <x:author>tc={87E8F4DE-0F6B-C100-170D-96C85EA2694F}</x:author>
-    <x:author>tc={327772B5-06F7-BF98-168C-1F90F7D50CBB}</x:author>
-    <x:author>tc={36BE7540-24E4-876F-B0E7-5753CB3F9B1F}</x:author>
-    <x:author>tc={3977E859-D6B3-767C-5E5F-B7BC8DA6835F}</x:author>
-    <x:author>tc={0EEA68E2-7763-CC47-F71C-8F260986727F}</x:author>
-    <x:author>tc={2E5078F9-9194-8A06-23A5-2ACD828EBE10}</x:author>
-    <x:author>tc={7D7BDFB5-CE3D-259A-6186-A2557641EECC}</x:author>
-    <x:author>tc={E14E0F78-126D-771B-A1F2-85F72686862D}</x:author>
-    <x:author>tc={9669977D-6EF4-2826-924E-2C0BB9D74365}</x:author>
-    <x:author>tc={0D86104F-0064-7B27-F768-D1C5A87ABBBB}</x:author>
+    <x:author>tc={5435A142-6F48-7F8E-AA2E-F52AAC279AE4}</x:author>
+    <x:author>tc={9CC18C9D-2A7E-BBA4-604E-47BA806E7B2F}</x:author>
+    <x:author>tc={085A4CDC-7E32-358A-62E3-4A77358D08F8}</x:author>
+    <x:author>tc={72DEC69B-94A9-1542-88CA-7EC24E89414E}</x:author>
+    <x:author>tc={EC00A534-D5BA-ED61-3F2B-8CB7D24617E1}</x:author>
+    <x:author>tc={BD623018-280B-401C-F592-908D468F1B42}</x:author>
+    <x:author>tc={5CF44951-8993-C254-E346-988F56277874}</x:author>
+    <x:author>tc={3383E0D9-5FB7-F9D0-946F-0F242015B017}</x:author>
+    <x:author>tc={C9F16D0A-4F5F-AB9A-2C26-F6275E8C8435}</x:author>
+    <x:author>tc={3722723F-FE60-9A5B-A3D7-6C5687C2A97E}</x:author>
+    <x:author>tc={8C0DCAC5-D72E-145A-C09F-EF8C4FAA42B1}</x:author>
+    <x:author>tc={BD872FF7-6078-B13F-D1F4-AA57675D46B6}</x:author>
+    <x:author>tc={6D17A93A-A61E-3F5B-A4A3-40F153329072}</x:author>
+    <x:author>tc={4891741C-0B9F-3D4F-9762-5EDE76F0468C}</x:author>
+    <x:author>tc={53C666BD-211F-1621-F3F0-ECA3FD5F446C}</x:author>
+    <x:author>tc={9FA26BA7-D49E-1A6C-C991-DF33DEA461B9}</x:author>
+    <x:author>tc={DDC71113-18C2-79AE-0740-24D3CBAE7A79}</x:author>
+    <x:author>tc={DDC034C5-42E6-D4B0-1111-EBFA516DC1A1}</x:author>
+    <x:author>tc={D6BA49A0-C68A-81AE-3743-C3D02B24476E}</x:author>
+    <x:author>tc={FB67F30A-6048-BB19-0884-B43E32B634A5}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="J5" authorId="0">
@@ -2060,7 +2060,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9c3b9377a8c64228"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra6352f4be97f4ffa"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2071,7 +2071,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}"/>
+  <xltc:person displayName="Corporate Wallet Digital Twin V3.2.0" id="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}"/>
 </xltc:personList>
 </file>
 
@@ -2268,493 +2268,493 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="P5" dT="2026-08-15T06:51:35.606" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{0AF4FEDA-AC03-3F9A-4677-E614750C0BE6}">
+  <xltc:threadedComment ref="P5" dT="2026-08-15T15:09:01.88" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{2ED26A2B-7837-083D-9F91-2E1C1C9C804A}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P6" dT="2026-08-15T06:51:35.608" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{7B13601B-A686-D1F6-E2C3-2DEAACC41826}">
+  <xltc:threadedComment ref="P6" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{043405D0-022D-CE03-81D3-AF489ABD68A9}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P7" dT="2026-08-15T06:51:35.608" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{10B9DE82-DAAF-597E-4424-E67283E9A4F8}">
+  <xltc:threadedComment ref="P7" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{D34DFE13-CAE1-EB32-19DC-D3D61E45A130}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P8" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9DDF9D19-AAB7-35C6-6EAB-ADE447886907}">
+  <xltc:threadedComment ref="P8" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{F0CC0459-AC75-5733-37FD-D729BDC516EE}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P9" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{CEC6EDDA-4333-DE39-19A1-CD6C28B0071E}">
+  <xltc:threadedComment ref="P9" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{BBAB887A-8A65-8B92-424D-300C0145401F}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P10" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9E0A3C03-F7F7-40B8-594C-1134A321AF12}">
+  <xltc:threadedComment ref="P10" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{1EE3C80A-BD61-F09D-5B89-C055910B21A8}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 119
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P11" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{6A469CC5-9E84-42E7-A4A2-5046B5EB797A}">
+  <xltc:threadedComment ref="P11" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{071773AC-BAFA-9A1C-7CEC-858AE817169C}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 160
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P12" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{49F38930-D4FC-9148-B4AB-7B8868A6B1C4}">
+  <xltc:threadedComment ref="P12" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{A64051D4-C4DD-3EAD-CAD5-DDCB5ED2D742}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P13" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{6AE471B8-00A6-D8CA-E30E-F2F43B242CB2}">
+  <xltc:threadedComment ref="P13" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{342DD7E3-64C9-FC39-8DEA-BB86036F486C}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P14" dT="2026-08-15T06:51:35.609" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{070A3F26-F4D3-3501-5B26-B76E24181EE6}">
+  <xltc:threadedComment ref="P14" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{A5720320-9FF6-0861-0144-55CD868F0919}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P15" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{DB4AA7DC-83F7-AA9C-6650-AC0FBB081C37}">
+  <xltc:threadedComment ref="P15" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{13F43D72-1AA3-0364-70A4-6A9B8423C7FE}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P16" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{E8A6B8CE-ACDD-0EA3-3036-3FEA4BE387E5}">
+  <xltc:threadedComment ref="P16" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0E8F289F-DFB0-8655-E6D1-D7FCF99AAB06}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P17" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{F5132FA4-62BD-C63C-B25A-A7E1FE946B04}">
+  <xltc:threadedComment ref="P17" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{4B99CAD2-8EC9-BC88-3AFD-F1394BD6783F}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P18" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{924A75EC-79F9-BE2D-03E1-123D59F3BF71}">
+  <xltc:threadedComment ref="P18" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{010EBAEC-2F9D-B152-1556-960BE1725C4B}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P19" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{7DFAAAEE-9F37-70B4-1295-82F48891DA0C}">
+  <xltc:threadedComment ref="P19" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{7333D144-0844-64FD-0AAB-4E413D2935D0}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P20" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{E2EA446D-49CF-67B3-25D3-448163193339}">
+  <xltc:threadedComment ref="P20" dT="2026-08-15T15:09:01.882" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{5518B81C-B0BC-B171-5762-AAA1625B3F0D}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 138
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P21" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{130AC7D8-E99A-FB9E-EC90-C0CC209F65EE}">
+  <xltc:threadedComment ref="P21" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{FE8B682C-7BBF-FB26-C52A-0567E7240CBA}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 212
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P22" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{DFEDA6A7-98B9-D90B-F8E4-87463C1ABE71}">
+  <xltc:threadedComment ref="P22" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{3A15E6D2-B051-8834-4C93-A28DA909DDC7}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P23" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{F908D626-E856-7A2E-B578-6FFFAF10A067}">
+  <xltc:threadedComment ref="P23" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{2EA4B4F3-F741-14DC-D1D2-6FA54989E80C}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P24" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{4691BC9F-FA65-4FBB-BE88-C3485B37BF5B}">
+  <xltc:threadedComment ref="P24" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{F4DF57BE-F27A-2E50-A72C-5EF0B356A55E}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P25" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{54D1659D-A9A9-797D-09FE-9CCD3046EB3B}">
+  <xltc:threadedComment ref="P25" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{31A0369D-1694-51B8-5DB4-35DB7F6AF63D}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P26" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{32021335-239B-D7CF-C593-02492073755E}">
+  <xltc:threadedComment ref="P26" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{7B5F41ED-10A3-8B79-15C5-6A825FFFDDE4}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P27" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2D4C52F2-DF0E-98A8-DBAD-465EFEA6430C}">
+  <xltc:threadedComment ref="P27" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{46AE8608-356C-86B4-EC18-C1C6FE5CAAAD}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 272
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P28" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{4F673CEB-0DB2-16EC-1BF9-E9916FC0D89C}">
+  <xltc:threadedComment ref="P28" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{7551C88D-E9F7-2348-0E76-9F80E57D2F60}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P29" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{8C766CE4-DCA4-0227-2719-EC43FBE4EB3E}">
+  <xltc:threadedComment ref="P29" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{ABF1018A-ABB9-7204-C90E-1105B94E814A}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P30" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{030B07FB-3D16-4698-B4D5-9BFD808ED081}">
+  <xltc:threadedComment ref="P30" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{512B7354-5F2C-1AA7-CC3C-00CD42BBE0FC}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 158
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P31" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{BB835A0A-AC15-BD40-37D2-BB2D5D7D1A29}">
+  <xltc:threadedComment ref="P31" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{AFFA6109-ADE2-4CE1-7C27-BAA3EFB317C9}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P32" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{ACE1C8E0-F10B-F24B-C4C3-09990BA1EAF5}">
+  <xltc:threadedComment ref="P32" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{D5144167-7AD8-57DF-B826-07D54D010D9C}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P33" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{89E2F11B-ECCC-3429-226F-74770117AB92}">
+  <xltc:threadedComment ref="P33" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{B83DFD0F-794A-6C5E-1D58-744B039949BC}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 72
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P34" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{FE94A6DE-84F6-0201-3EFF-69B3D6B7D622}">
+  <xltc:threadedComment ref="P34" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{7B9E1B4B-9DCB-BECD-99F5-F055FB863E9C}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P35" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{5FADB78B-442A-2857-7CCC-D525C440BCCF}">
+  <xltc:threadedComment ref="P35" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{8B2DC34E-17AF-DC22-540E-3A7428974B96}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P36" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{33238565-3127-12AD-ACAF-5A83E4E3101E}">
+  <xltc:threadedComment ref="P36" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{094E8309-B86F-1491-11B7-E843D5E63DAC}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 24
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P37" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{DBA819E1-2CFB-40C0-8E60-4EBBB4963742}">
+  <xltc:threadedComment ref="P37" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{4513E577-194B-E888-43E5-01675E143F65}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P38" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{831BC617-DC59-E847-0D3A-95946FD8D988}">
+  <xltc:threadedComment ref="P38" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{D063F1D2-2F95-2667-C7FF-CB2952CE7907}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P39" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9625D7E8-9A23-1EEE-66C1-3D1F41528532}">
+  <xltc:threadedComment ref="P39" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{C9AF5DAB-FC5E-E759-C111-2F94BE966A52}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 19
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P40" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{36A13555-305E-B2C5-2B7A-87476C5BA766}">
+  <xltc:threadedComment ref="P40" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{5C3D6D9E-0399-3A1F-5FF8-7673B95728DC}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P41" dT="2026-08-15T06:51:35.61" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{69541CEA-6E11-BC48-6898-36AE3D548AB4}">
+  <xltc:threadedComment ref="P41" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{40BAA6D9-7593-464B-9634-92C58D16225A}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P42" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{12AFE746-FDD9-963F-DCFD-DC968D22FFA6}">
+  <xltc:threadedComment ref="P42" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{DA3A9B1C-4CB2-882E-946C-A1860B6BC64A}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P43" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{425C83BD-D4DC-BDED-071D-487523F8AC3F}">
+  <xltc:threadedComment ref="P43" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{05CE38D1-9BF6-E417-141B-4027834AA96E}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P44" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2D72A011-0216-7D35-09A3-D704E88BAEE3}">
+  <xltc:threadedComment ref="P44" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{B6C35BC3-6F5F-B362-B79B-E7478D767EAB}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P45" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{86FBCAB8-88A0-F97B-4FA1-13C4BEAA369D}">
+  <xltc:threadedComment ref="P45" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{A2136AA3-D60A-9CA4-782A-688014FA68CC}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P46" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9185AC7C-5FA5-8BAE-5D74-F86F31883FC5}">
+  <xltc:threadedComment ref="P46" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{F9107F21-217D-6E1C-0F95-26D39A645301}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P47" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{8F348568-9728-931E-D9B2-061F382ED13A}">
+  <xltc:threadedComment ref="P47" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{6BDCC13B-4293-D80F-CDD9-0D914AF1E069}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P48" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{E5746BEC-90A8-ABA0-16B5-A6A9F11A2C96}">
+  <xltc:threadedComment ref="P48" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{6FCD0DD5-A300-B061-80FD-E6DA09A1A00C}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P49" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{4B1E6C62-4809-1469-5784-9EA7A65F2E2D}">
+  <xltc:threadedComment ref="P49" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{D33E4AF9-5B00-4D1E-2774-D1A03F8DAA00}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 118
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P50" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{271EEFA8-492B-5EC5-67E3-8B28D1AE9871}">
+  <xltc:threadedComment ref="P50" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{B93F8331-7F4C-8F1E-6D00-D4F3F4DD941B}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P51" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{3430FD27-2DAA-4633-A322-0688F2FCD467}">
+  <xltc:threadedComment ref="P51" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{01017BE8-DAC5-0C0D-B269-33BF689C7906}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P52" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{8D7DF3C9-36A9-2E8C-6160-11B116238A97}">
+  <xltc:threadedComment ref="P52" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0F0598D8-65DE-16CC-F316-558AAB8C206A}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P53" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{31933AFB-CA47-471A-E7EB-D7E5B693D87A}">
+  <xltc:threadedComment ref="P53" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{FD22F09B-1275-26C7-C5BC-CEBC26B724BD}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-STF</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P54" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{CEB8E96A-F9CE-D6E4-1345-25BEA6D4853C}">
+  <xltc:threadedComment ref="P54" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{50296461-F84A-5759-D5C7-3C73B6727E11}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P55" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{CE8B63E6-EC70-4885-EBBF-C61B84B9BD02}">
+  <xltc:threadedComment ref="P55" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{25FD297A-C8A3-7982-2A2A-6109869C428D}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P56" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{1236AB2A-50DD-58C5-F0CF-0A77396ECCB9}">
+  <xltc:threadedComment ref="P56" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{A01BC395-D63D-37E2-3702-F398D5D7D853}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 18
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P57" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{23B809AB-666E-3843-AA8B-2E06C9D6735C}">
+  <xltc:threadedComment ref="P57" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{3CCE64FE-3C38-CB25-DAB1-1288A0B1E1D3}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P58" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{F9218197-D7D7-96FC-5DEE-19E1B89C6668}">
+  <xltc:threadedComment ref="P58" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0381E4D2-1AB7-DC1B-5477-B3CE9858338D}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P59" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{49C564EF-C6E1-AA3E-BAE6-F9B6B7DAF702}">
+  <xltc:threadedComment ref="P59" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0DB1B439-2233-2FF4-7F69-4CFB903C8BCE}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P60" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{6A34B57F-09E3-5DA4-9CDF-BDD9AFC15C62}">
+  <xltc:threadedComment ref="P60" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{702F1FDC-2B20-239C-C387-1F9994029E58}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P61" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{EA67CC0C-3B7B-6001-4E9C-C907CB9A2E41}">
+  <xltc:threadedComment ref="P61" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{86BF3B4D-4C8B-94C5-2DF8-0E144D24162D}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P62" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2C705125-9621-DC7B-9356-1AFFFB014183}">
+  <xltc:threadedComment ref="P62" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{55FEB31D-AA64-C68B-21EB-2AD4013CA9D9}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P63" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{4127462E-7049-10C8-6E6D-2726FCAFA040}">
+  <xltc:threadedComment ref="P63" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{2120B059-1D9A-FB52-CB20-859A8A7B4431}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P64" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{DDC7860C-4BF8-FE8E-AB94-BF36F51E4742}">
+  <xltc:threadedComment ref="P64" dT="2026-08-15T15:09:01.883" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{DDAE0E6F-C9F0-E461-07EA-91968BE2E6D2}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P65" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{355CD349-BEF2-1F91-3717-B7779FC267B7}">
+  <xltc:threadedComment ref="P65" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{83232D14-7BAC-B848-7871-277E89FA684E}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 311
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P66" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{BE707954-D4F8-3036-E784-0F6EF373E3B1}">
+  <xltc:threadedComment ref="P66" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{279DD734-DD6F-13E2-E0FD-18F5BF78E98D}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P67" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{30C17E09-F415-E5D5-1412-983D6592AE59}">
+  <xltc:threadedComment ref="P67" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0C0BEC61-5240-DC56-B9D0-4183924DDDA7}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P68" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{946D1FE7-F4AA-6563-A358-3F55219C3AED}">
+  <xltc:threadedComment ref="P68" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{4B78E0A5-E835-82BC-95E0-9D6660CB0642}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 141
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P69" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{FF9DEADC-5F2B-2C71-0EDD-31A65A1DAC80}">
+  <xltc:threadedComment ref="P69" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{2AA3892A-F3E0-DCE4-4BA3-77C2298E4712}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P70" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{99FA21E2-86C5-2A76-2880-8215954AA3D4}">
+  <xltc:threadedComment ref="P70" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0BF67983-6F8F-9A8B-A733-988A5AE771CE}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P71" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{901E21A1-49DD-A0DA-0A10-1EDE8076C1B3}">
+  <xltc:threadedComment ref="P71" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{853E2097-1ED4-88BD-0FEF-BB1C45A97F6A}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 33
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P72" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{FCB3C38E-B0AF-A412-700D-4D9A9D2C2741}">
+  <xltc:threadedComment ref="P72" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{5437FE01-1237-5D55-7238-D3B41AD600A7}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P73" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9382A565-2A1D-550E-54B1-678F98943EC6}">
+  <xltc:threadedComment ref="P73" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{26525073-6162-76FE-6D24-B53B287B9745}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P74" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{40576489-4A24-6AA0-06F2-24F75770098B}">
+  <xltc:threadedComment ref="P74" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{BAC99CA3-3171-9911-60EA-9ADBAD9DAA89}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 21
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P75" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{D80EF366-6BBD-D5AC-E71F-5666ED857ED8}">
+  <xltc:threadedComment ref="P75" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{4E489A6C-1C1A-971C-72AB-ACB53D354D17}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P76" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{8E28E375-5E9B-B43C-02D8-1D69B6DBCCB7}">
+  <xltc:threadedComment ref="P76" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{280D1E73-5C17-150A-507B-D8086C4BA2AD}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P77" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{C52D303F-E26F-AEB2-82AD-C196257D053A}">
+  <xltc:threadedComment ref="P77" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{33816FEE-5341-8E14-F197-F3763F51C77B}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 19
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P78" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{AD3CBF1C-654B-022F-1CCE-E3B6B02846E3}">
+  <xltc:threadedComment ref="P78" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0277E1E1-ACCD-F4A6-B8D9-B0F98C590404}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 43
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P79" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2EEF0622-B8D5-960E-069D-57BC28C46AE4}">
+  <xltc:threadedComment ref="P79" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{F919CE15-F9D0-4C7F-A7F6-D4B6CEEDC7C3}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 44
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P80" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{C7A17400-8C3D-04F3-BB45-75623A8D8379}">
+  <xltc:threadedComment ref="P80" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{70300967-130C-E9FC-5833-2A5E4C05B7E1}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 40
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P81" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9CB15BCB-A81F-4C51-B6D7-CA70F830A75F}">
+  <xltc:threadedComment ref="P81" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{6A5C72F7-2A4F-E907-50AB-917C148A344A}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P82" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9CDE5188-52E3-BEBE-AC4D-8F98AC717AA6}">
+  <xltc:threadedComment ref="P82" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{0459789A-01BE-4F0D-BABB-8071C46032C0}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P83" dT="2026-08-15T06:51:35.611" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{96D773F7-6FC9-4DF1-46BC-3C5A65EBE44A}">
+  <xltc:threadedComment ref="P83" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{AF3F7297-575B-2C4C-A9A0-434E38FE21C6}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 16
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P84" dT="2026-08-15T06:51:35.612" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{69BF4FC0-9856-F2BC-F517-9DC02348AB96}">
+  <xltc:threadedComment ref="P84" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{2DFC25D3-339D-7566-5DC3-205EE0DC70AC}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P85" dT="2026-08-15T06:51:35.612" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{EF1A8A33-3E41-8002-8157-23C7596AF4CA}">
+  <xltc:threadedComment ref="P85" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{326FB552-EB16-8CC1-A7BC-665356E8462C}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P86" dT="2026-08-15T06:51:35.612" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{CBA415B4-31A9-6F43-882D-D511ADAA6836}">
+  <xltc:threadedComment ref="P86" dT="2026-08-15T15:09:01.884" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{5B218977-D8FC-2E26-E971-16C48C7A4A64}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 21
 Available: 2026-02-25
@@ -2765,64 +2765,64 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="J5" dT="2026-08-15T06:51:36.013" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{B01406AF-5C54-1385-E93F-8BC31DCEF046}">
+  <xltc:threadedComment ref="J5" dT="2026-08-15T15:09:02.238" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{5435A142-6F48-7F8E-AA2E-F52AAC279AE4}">
     <xltc:text>Official source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J6" dT="2026-08-15T06:51:36.015" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{6DD7D282-4D5B-6CEA-034D-91D0362B1489}">
+  <xltc:threadedComment ref="J6" dT="2026-08-15T15:09:02.241" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{9CC18C9D-2A7E-BBA4-604E-47BA806E7B2F}">
     <xltc:text>Official source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J7" dT="2026-08-15T06:51:36.019" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{B744CA31-60A8-7C0A-67C6-4F7042734E04}">
+  <xltc:threadedComment ref="J7" dT="2026-08-15T15:09:02.244" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{085A4CDC-7E32-358A-62E3-4A77358D08F8}">
     <xltc:text>Official source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J8" dT="2026-08-15T06:51:36.022" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2CBFDB07-DAC4-1F7C-80B7-A9AE350E67F7}">
+  <xltc:threadedComment ref="J8" dT="2026-08-15T15:09:02.246" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{72DEC69B-94A9-1542-88CA-7EC24E89414E}">
     <xltc:text>Official source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J9" dT="2026-08-15T06:51:36.025" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{C6FFBF76-75E5-A885-90FC-7A4822669D85}">
+  <xltc:threadedComment ref="J9" dT="2026-08-15T15:09:02.249" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{EC00A534-D5BA-ED61-3F2B-8CB7D24617E1}">
     <xltc:text>Official source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J10" dT="2026-08-15T06:51:36.029" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{48B6FC78-C54C-A341-9A8A-BAE4F532FF12}">
+  <xltc:threadedComment ref="J10" dT="2026-08-15T15:09:02.251" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{BD623018-280B-401C-F592-908D468F1B42}">
     <xltc:text>Official source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J11" dT="2026-08-15T06:51:36.031" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{40834F88-B44F-30F0-0C1E-7A7EA53D4250}">
+  <xltc:threadedComment ref="J11" dT="2026-08-15T15:09:02.253" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{5CF44951-8993-C254-E346-988F56277874}">
     <xltc:text>Official source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J12" dT="2026-08-15T06:51:36.033" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{8C86F84D-BA29-E3DB-77BF-71A0444405B8}">
+  <xltc:threadedComment ref="J12" dT="2026-08-15T15:09:02.256" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{3383E0D9-5FB7-F9D0-946F-0F242015B017}">
     <xltc:text>Official source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J13" dT="2026-08-15T06:51:36.035" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{E119E111-72FF-3D54-C250-0ADC5886F9C3}">
+  <xltc:threadedComment ref="J13" dT="2026-08-15T15:09:02.259" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{C9F16D0A-4F5F-AB9A-2C26-F6275E8C8435}">
     <xltc:text>Official source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J14" dT="2026-08-15T06:51:36.038" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{82842CDD-4566-2F54-CBEE-B39CF6B61B97}">
+  <xltc:threadedComment ref="J14" dT="2026-08-15T15:09:02.26" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{3722723F-FE60-9A5B-A3D7-6C5687C2A97E}">
     <xltc:text>Official source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J15" dT="2026-08-15T06:51:36.041" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{87E8F4DE-0F6B-C100-170D-96C85EA2694F}">
+  <xltc:threadedComment ref="J15" dT="2026-08-15T15:09:02.262" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{8C0DCAC5-D72E-145A-C09F-EF8C4FAA42B1}">
     <xltc:text>Official source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J16" dT="2026-08-15T06:51:36.043" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{327772B5-06F7-BF98-168C-1F90F7D50CBB}">
+  <xltc:threadedComment ref="J16" dT="2026-08-15T15:09:02.266" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{BD872FF7-6078-B13F-D1F4-AA57675D46B6}">
     <xltc:text>Official source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J17" dT="2026-08-15T06:51:36.045" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{36BE7540-24E4-876F-B0E7-5753CB3F9B1F}">
+  <xltc:threadedComment ref="J17" dT="2026-08-15T15:09:02.268" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{6D17A93A-A61E-3F5B-A4A3-40F153329072}">
     <xltc:text>Official source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J18" dT="2026-08-15T06:51:36.047" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{3977E859-D6B3-767C-5E5F-B7BC8DA6835F}">
+  <xltc:threadedComment ref="J18" dT="2026-08-15T15:09:02.27" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{4891741C-0B9F-3D4F-9762-5EDE76F0468C}">
     <xltc:text>Official source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J19" dT="2026-08-15T06:51:36.048" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{0EEA68E2-7763-CC47-F71C-8F260986727F}">
+  <xltc:threadedComment ref="J19" dT="2026-08-15T15:09:02.272" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{53C666BD-211F-1621-F3F0-ECA3FD5F446C}">
     <xltc:text>Official source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J20" dT="2026-08-15T06:51:36.054" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{2E5078F9-9194-8A06-23A5-2ACD828EBE10}">
+  <xltc:threadedComment ref="J20" dT="2026-08-15T15:09:02.275" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{9FA26BA7-D49E-1A6C-C991-DF33DEA461B9}">
     <xltc:text>Official source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J21" dT="2026-08-15T06:51:36.057" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{7D7BDFB5-CE3D-259A-6186-A2557641EECC}">
+  <xltc:threadedComment ref="J21" dT="2026-08-15T15:09:02.277" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{DDC71113-18C2-79AE-0740-24D3CBAE7A79}">
     <xltc:text>Official source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J22" dT="2026-08-15T06:51:36.059" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{E14E0F78-126D-771B-A1F2-85F72686862D}">
+  <xltc:threadedComment ref="J22" dT="2026-08-15T15:09:02.279" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{DDC034C5-42E6-D4B0-1111-EBFA516DC1A1}">
     <xltc:text>Official source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J23" dT="2026-08-15T06:51:36.061" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{9669977D-6EF4-2826-924E-2C0BB9D74365}">
+  <xltc:threadedComment ref="J23" dT="2026-08-15T15:09:02.281" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{D6BA49A0-C68A-81AE-3743-C3D02B24476E}">
     <xltc:text>Official source: https://www.aspenpharma.com/download/annual-financial-statements-2/</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J24" dT="2026-08-15T06:51:36.063" personId="{B2145340-41FB-4BFA-8AFB-959C37CD5CDE}" id="{0D86104F-0064-7B27-F768-D1C5A87ABBBB}">
+  <xltc:threadedComment ref="J24" dT="2026-08-15T15:09:02.282" personId="{B8989647-9DF0-489F-9A9C-0692D33C7BF0}" id="{FB67F30A-6048-BB19-0884-B43E32B634A5}">
     <xltc:text>Official source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -3877,7 +3877,7 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c7810c6b47b416f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3932c49e3ae64aaa"/>
 </x:worksheet>
 </file>
 
@@ -8611,7 +8611,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc12e983b47534b1a"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cc4b2c86cc4433c"/>
 </x:worksheet>
 </file>
 
@@ -9671,7 +9671,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R458cac95bef44c85"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d74c8a6f0f84da8"/>
 </x:worksheet>
 </file>
 

</xml_diff>